<commit_message>
Restore locally-graded bet results and Settings bankroll
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Slate" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Bet Log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Team Profiles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Model Comparison" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Slate" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bet Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Profiles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Comparison" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3569,6 +3569,11 @@
         <f>IF(I29="","",I29-#REF!)</f>
         <v/>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
       <c r="L29" s="11">
         <f>IF(K29="W",IF(G29&lt;0,H29*100/ABS(G29),H29*G29/100),IF(K29="L",-H29,0))</f>
         <v/>
@@ -3615,6 +3620,11 @@
         <f>IF(I30="","",I30-#REF!)</f>
         <v/>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
       <c r="L30" s="11">
         <f>IF(K30="W",IF(G30&lt;0,H30*100/ABS(G30),H30*G30/100),IF(K30="L",-H30,0))</f>
         <v/>
@@ -3658,6 +3668,11 @@
         <f>IF(I31="","",I31-#REF!)</f>
         <v/>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
       <c r="L31" s="11">
         <f>IF(K31="W",IF(G31&lt;0,H31*100/ABS(G31),H31*G31/100),IF(K31="L",-H31,0))</f>
         <v/>
@@ -3701,6 +3716,11 @@
         <f>IF(I32="","",I32-#REF!)</f>
         <v/>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
       <c r="L32" s="11">
         <f>IF(K32="W",IF(G32&lt;0,H32*100/ABS(G32),H32*G32/100),IF(K32="L",-H32,0))</f>
         <v/>
@@ -3711,7 +3731,44 @@
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Maryland @ Uconn</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Uconn</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
       <c r="J33" s="6" t="n"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="L33" s="11">
         <f>IF(K33="W",IF(G33&lt;0,H33*100/ABS(G33),H33*G33/100),IF(K33="L",-H33,0))</f>
         <v/>
@@ -3722,9 +3779,43 @@
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ohio State @ Texas</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>500</v>
+      </c>
+      <c r="H34" t="n">
+        <v>40</v>
+      </c>
       <c r="J34" s="6">
         <f>IF(I34="","",I34-F34)</f>
         <v/>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
       </c>
       <c r="L34" s="11">
         <f>IF(K34="W",IF(G34&lt;0,H34*100/ABS(G34),H34*G34/100),IF(K34="L",-H34,0))</f>

</xml_diff>

<commit_message>
Update either data or bets
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -3893,6 +3893,38 @@
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Wyoming @ Central Michigan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Central Michigan</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
       <c r="J35" s="6">
         <f>IF(I35="","",I35-F35)</f>
         <v/>
@@ -3907,6 +3939,38 @@
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Wyoming @ Central Michigan</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Central Michigan</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
       <c r="J36" s="6">
         <f>IF(I36="","",I36-F36)</f>
         <v/>
@@ -3921,6 +3985,38 @@
       </c>
     </row>
     <row r="37" ht="14.25" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Sacramento State @ North Dakota State</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>North Dakota State</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>-27.5</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
       <c r="J37" s="6">
         <f>IF(I37="","",I37-F37)</f>
         <v/>

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-09-20 16:08 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -953,28 +953,25 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>UNLV</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Central Michigan</t>
+          <t>Akron</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-9.300000000000001</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.2</v>
+        <v>3.9</v>
       </c>
       <c r="G2" s="6">
         <f>F2-E2</f>
@@ -985,10 +982,7 @@
         <v/>
       </c>
       <c r="I2" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="J2" t="n">
-        <v>38.8</v>
+        <v>49.1</v>
       </c>
       <c r="K2" s="6">
         <f>I2-J2</f>
@@ -1011,28 +1005,25 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UTEP</t>
+          <t>Northern Illinois</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Georgia State</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-29.7</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-34.8</v>
+        <v>-7.8</v>
       </c>
       <c r="G3" s="6">
         <f>F3-E3</f>
@@ -1043,10 +1034,7 @@
         <v/>
       </c>
       <c r="I3" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="J3" t="n">
-        <v>48.5</v>
+        <v>43.3</v>
       </c>
       <c r="K3" s="6">
         <f>I3-J3</f>
@@ -1067,28 +1055,25 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nevada</t>
+          <t>Hawai'i</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Middle Tennessee</t>
+          <t>Wyoming</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="F4" t="n">
-        <v>3.8</v>
+        <v>1.9</v>
       </c>
       <c r="G4" s="6">
         <f>F4-E4</f>
@@ -1099,10 +1084,7 @@
         <v/>
       </c>
       <c r="I4" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="J4" t="n">
-        <v>50.5</v>
+        <v>42.9</v>
       </c>
       <c r="K4" s="6">
         <f>I4-J4</f>
@@ -1123,11 +1105,11 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1137,14 +1119,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>New Mexico State</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>-10.8</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-21.8</v>
+        <v>18.8</v>
       </c>
       <c r="G5" s="6">
         <f>F5-E5</f>
@@ -1155,10 +1134,7 @@
         <v/>
       </c>
       <c r="I5" t="n">
-        <v>37</v>
-      </c>
-      <c r="J5" t="n">
-        <v>45.5</v>
+        <v>47.1</v>
       </c>
       <c r="K5" s="6">
         <f>I5-J5</f>
@@ -1184,28 +1160,25 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>North Dakota State</t>
+          <t>Oregon State</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sacramento State</t>
+          <t>UTEP</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="F6" t="n">
-        <v>27</v>
+        <v>10.5</v>
       </c>
       <c r="G6" s="6">
         <f>F6-E6</f>
@@ -1216,10 +1189,7 @@
         <v/>
       </c>
       <c r="I6" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="J6" t="n">
-        <v>50.5</v>
+        <v>49</v>
       </c>
       <c r="K6" s="6">
         <f>I6-J6</f>
@@ -1245,29 +1215,27 @@
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Northern Illinois</t>
+          <t>Air Force</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Nevada</t>
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>-30.9</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>-33.8</v>
-      </c>
+        <v>1.7</v>
+      </c>
+      <c r="F7" s="10" t="n"/>
       <c r="G7" s="10">
         <f>F7-E7</f>
         <v/>
@@ -1277,11 +1245,9 @@
         <v/>
       </c>
       <c r="I7" s="10" t="n">
-        <v>36.8</v>
-      </c>
-      <c r="J7" s="10" t="n">
-        <v>50.2</v>
-      </c>
+        <v>47.2</v>
+      </c>
+      <c r="J7" s="10" t="n"/>
       <c r="K7" s="10">
         <f>I7-J7</f>
         <v/>
@@ -1305,30 +1271,6 @@
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Fresno State</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>San José State</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>6.5</v>
-      </c>
       <c r="G8" s="6">
         <f>F8-E8</f>
         <v/>
@@ -1336,12 +1278,6 @@
       <c r="H8" s="6">
         <f>IF(G8=0,"Pick'em",IF(G8&gt;0,"Home","Away"))</f>
         <v/>
-      </c>
-      <c r="I8" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="J8" t="n">
-        <v>49.8</v>
       </c>
       <c r="K8" s="6">
         <f>I8-J8</f>
@@ -5418,7 +5354,7 @@
         </is>
       </c>
       <c r="D2" s="9" t="n">
-        <v>1748.4</v>
+        <v>1760.7</v>
       </c>
       <c r="E2" s="9" t="n">
         <v>4.2</v>
@@ -5492,7 +5428,7 @@
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>1589.7</v>
+        <v>1575.5</v>
       </c>
       <c r="E4" s="9" t="n">
         <v>5</v>
@@ -5603,7 +5539,7 @@
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>1417.7</v>
+        <v>1399.2</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>-13.7</v>
@@ -5640,7 +5576,7 @@
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>1394.7</v>
+        <v>1385.2</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>-16.9</v>
@@ -5677,7 +5613,7 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1451.7</v>
+        <v>1428.8</v>
       </c>
       <c r="E9" s="9" t="n">
         <v>-12.5</v>
@@ -5714,7 +5650,7 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>1411.8</v>
+        <v>1393.9</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>-7.6</v>
@@ -5751,7 +5687,7 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>1382.6</v>
+        <v>1375.4</v>
       </c>
       <c r="E11" s="9" t="n">
         <v>-16.2</v>

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-09-22 19:01 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="F2" t="n">
         <v>13.5</v>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-7.8</v>
+        <v>-7.7</v>
       </c>
       <c r="F3" t="n">
         <v>-10</v>
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="F5" t="n">
         <v>12.8</v>

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-09-27 01:46 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -1287,7 +1287,7 @@
         <v/>
       </c>
       <c r="I6" t="n">
-        <v>51</v>
+        <v>50.9</v>
       </c>
       <c r="J6" t="n">
         <v>56.2</v>
@@ -1348,7 +1348,7 @@
         <v/>
       </c>
       <c r="I7" s="10" t="n">
-        <v>46.4</v>
+        <v>46.5</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>50.5</v>
@@ -17475,20 +17475,20 @@
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>Ole Miss</t>
+          <t>Utah</t>
         </is>
       </c>
       <c r="B10" s="35" t="n">
-        <v>84.90000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="C10" s="35" t="n">
-        <v>84</v>
+        <v>83.5</v>
       </c>
       <c r="D10" s="35" t="n">
-        <v>84.5</v>
+        <v>84.2</v>
       </c>
       <c r="E10" s="35" t="n">
-        <v>84.5</v>
+        <v>84.3</v>
       </c>
       <c r="V10" s="37" t="inlineStr">
         <is>
@@ -17499,58 +17499,58 @@
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="B11" s="35" t="n">
-        <v>81.59999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="C11" s="35" t="n">
-        <v>83.5</v>
+        <v>80.2</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>84.2</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="E11" s="35" t="n">
-        <v>84.3</v>
+        <v>83.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="B12" s="35" t="n">
-        <v>81.2</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="C12" s="35" t="n">
-        <v>80.2</v>
+        <v>82.3</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>84.59999999999999</v>
+        <v>82.2</v>
       </c>
       <c r="E12" s="35" t="n">
-        <v>83.7</v>
+        <v>82.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="B13" s="35" t="n">
-        <v>80.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="C13" s="35" t="n">
-        <v>82.3</v>
+        <v>83.2</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>82.2</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="E13" s="35" t="n">
-        <v>82.2</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="14">
@@ -17575,226 +17575,226 @@
     <row r="15">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Penn State</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="B15" s="35" t="n">
-        <v>80.90000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="C15" s="35" t="n">
-        <v>80.3</v>
+        <v>79</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>81.2</v>
+        <v>78.7</v>
       </c>
       <c r="E15" s="35" t="n">
-        <v>81.2</v>
+        <v>81.59999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="35" t="inlineStr">
         <is>
-          <t>South Carolina</t>
+          <t>Ole Miss</t>
         </is>
       </c>
       <c r="B16" s="35" t="n">
-        <v>75.09999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="C16" s="35" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D16" s="35" t="n">
-        <v>81</v>
+        <v>84.5</v>
       </c>
       <c r="E16" s="35" t="n">
-        <v>81</v>
+        <v>81.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="35" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>South Carolina</t>
         </is>
       </c>
       <c r="B17" s="35" t="n">
-        <v>75</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="C17" s="35" t="n">
-        <v>74.8</v>
+        <v>81</v>
       </c>
       <c r="D17" s="35" t="n">
-        <v>76.2</v>
+        <v>81</v>
       </c>
       <c r="E17" s="35" t="n">
-        <v>80.5</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="B18" s="35" t="n">
-        <v>76.8</v>
+        <v>75</v>
       </c>
       <c r="C18" s="35" t="n">
-        <v>77.8</v>
+        <v>74.8</v>
       </c>
       <c r="D18" s="35" t="n">
-        <v>78.90000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="E18" s="35" t="n">
-        <v>80.2</v>
+        <v>80.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="35" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Penn State</t>
         </is>
       </c>
       <c r="B19" s="35" t="n">
-        <v>79.2</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="C19" s="35" t="n">
-        <v>83.2</v>
+        <v>80.3</v>
       </c>
       <c r="D19" s="35" t="n">
-        <v>80.09999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="E19" s="35" t="n">
-        <v>80.09999999999999</v>
+        <v>80.40000000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="B20" s="35" t="n">
-        <v>79.09999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="C20" s="35" t="n">
-        <v>78.3</v>
+        <v>77.8</v>
       </c>
       <c r="D20" s="35" t="n">
-        <v>80</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="E20" s="35" t="n">
-        <v>80</v>
+        <v>80.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="35" t="inlineStr">
         <is>
-          <t>LSU</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="B21" s="35" t="n">
         <v>79.09999999999999</v>
       </c>
       <c r="C21" s="35" t="n">
-        <v>80.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="D21" s="35" t="n">
-        <v>79.7</v>
+        <v>80</v>
       </c>
       <c r="E21" s="35" t="n">
-        <v>79.7</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="35" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>LSU</t>
         </is>
       </c>
       <c r="B22" s="35" t="n">
-        <v>75.3</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C22" s="35" t="n">
-        <v>74.7</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="D22" s="35" t="n">
-        <v>74.09999999999999</v>
+        <v>79.7</v>
       </c>
       <c r="E22" s="35" t="n">
-        <v>79.09999999999999</v>
+        <v>79.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="35" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="B23" s="35" t="n">
-        <v>80.40000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="C23" s="35" t="n">
-        <v>78.8</v>
+        <v>74.7</v>
       </c>
       <c r="D23" s="35" t="n">
-        <v>78.8</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="E23" s="35" t="n">
-        <v>78.8</v>
+        <v>79.09999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="35" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>BYU</t>
         </is>
       </c>
       <c r="B24" s="35" t="n">
-        <v>75.2</v>
+        <v>78.3</v>
       </c>
       <c r="C24" s="35" t="n">
         <v>79</v>
       </c>
       <c r="D24" s="35" t="n">
-        <v>78.7</v>
+        <v>78.5</v>
       </c>
       <c r="E24" s="35" t="n">
-        <v>78.7</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="35" t="inlineStr">
         <is>
-          <t>BYU</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B25" s="35" t="n">
-        <v>78.3</v>
+        <v>74.7</v>
       </c>
       <c r="C25" s="35" t="n">
-        <v>79</v>
+        <v>78.8</v>
       </c>
       <c r="D25" s="35" t="n">
-        <v>78.5</v>
+        <v>79.8</v>
       </c>
       <c r="E25" s="35" t="n">
-        <v>78.5</v>
+        <v>77.90000000000001</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="35" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>SMU</t>
         </is>
       </c>
       <c r="B26" s="35" t="n">
-        <v>74.7</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="C26" s="35" t="n">
-        <v>78.8</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D26" s="35" t="n">
-        <v>79.8</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="E26" s="35" t="n">
         <v>77.90000000000001</v>
@@ -17803,17 +17803,17 @@
     <row r="27">
       <c r="A27" s="35" t="inlineStr">
         <is>
-          <t>SMU</t>
+          <t>Oklahoma</t>
         </is>
       </c>
       <c r="B27" s="35" t="n">
-        <v>75.40000000000001</v>
+        <v>81.2</v>
       </c>
       <c r="C27" s="35" t="n">
-        <v>78.90000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="D27" s="35" t="n">
-        <v>77.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="E27" s="35" t="n">
         <v>77.90000000000001</v>
@@ -17822,36 +17822,36 @@
     <row r="28">
       <c r="A28" s="35" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="B28" s="35" t="n">
-        <v>81.2</v>
+        <v>78</v>
       </c>
       <c r="C28" s="35" t="n">
-        <v>79.5</v>
+        <v>77.5</v>
       </c>
       <c r="D28" s="35" t="n">
-        <v>80</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>77.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="35" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="B29" s="35" t="n">
-        <v>78</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="C29" s="35" t="n">
-        <v>77.5</v>
+        <v>78.8</v>
       </c>
       <c r="D29" s="35" t="n">
-        <v>77.40000000000001</v>
+        <v>78.8</v>
       </c>
       <c r="E29" s="35" t="n">
         <v>77.40000000000001</v>
@@ -17860,39 +17860,39 @@
     <row r="30">
       <c r="A30" s="35" t="inlineStr">
         <is>
-          <t>James Madison</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="B30" s="35" t="n">
-        <v>67.8</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="C30" s="35" t="n">
-        <v>76.8</v>
+        <v>74.7</v>
       </c>
       <c r="D30" s="35" t="n">
-        <v>77.09999999999999</v>
+        <v>76.3</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>77.09999999999999</v>
+        <v>77.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="35" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>James Madison</t>
         </is>
       </c>
       <c r="B31" s="35" t="n">
-        <v>72.09999999999999</v>
+        <v>67.8</v>
       </c>
       <c r="C31" s="35" t="n">
-        <v>74.7</v>
+        <v>76.8</v>
       </c>
       <c r="D31" s="35" t="n">
-        <v>76.3</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="E31" s="35" t="n">
-        <v>76.3</v>
+        <v>77.09999999999999</v>
       </c>
     </row>
     <row r="32">
@@ -17930,7 +17930,7 @@
         <v>75.8</v>
       </c>
       <c r="E33" s="35" t="n">
-        <v>75.8</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="34">
@@ -18126,58 +18126,58 @@
     <row r="44">
       <c r="A44" s="35" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Auburn</t>
         </is>
       </c>
       <c r="B44" s="35" t="n">
-        <v>73.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="C44" s="35" t="n">
-        <v>72.7</v>
+        <v>71.2</v>
       </c>
       <c r="D44" s="35" t="n">
-        <v>72.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="E44" s="35" t="n">
-        <v>72.59999999999999</v>
+        <v>72.90000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="35" t="inlineStr">
         <is>
-          <t>New Mexico</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="B45" s="35" t="n">
-        <v>66.59999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="C45" s="35" t="n">
         <v>72.7</v>
       </c>
       <c r="D45" s="35" t="n">
-        <v>72.09999999999999</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="E45" s="35" t="n">
-        <v>72.3</v>
+        <v>72.59999999999999</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="35" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>New Mexico</t>
         </is>
       </c>
       <c r="B46" s="35" t="n">
-        <v>68.2</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="C46" s="35" t="n">
-        <v>68.3</v>
+        <v>72.7</v>
       </c>
       <c r="D46" s="35" t="n">
-        <v>72</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="E46" s="35" t="n">
-        <v>72</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="47">
@@ -18221,36 +18221,36 @@
     <row r="49">
       <c r="A49" s="35" t="inlineStr">
         <is>
-          <t>Auburn</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="B49" s="35" t="n">
-        <v>69.40000000000001</v>
+        <v>63.8</v>
       </c>
       <c r="C49" s="35" t="n">
-        <v>71.2</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="D49" s="35" t="n">
-        <v>71.5</v>
+        <v>66.7</v>
       </c>
       <c r="E49" s="35" t="n">
-        <v>71.5</v>
+        <v>71.3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="35" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Mississippi State</t>
         </is>
       </c>
       <c r="B50" s="35" t="n">
-        <v>63.8</v>
+        <v>68.8</v>
       </c>
       <c r="C50" s="35" t="n">
-        <v>65.90000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="D50" s="35" t="n">
-        <v>66.7</v>
+        <v>71.3</v>
       </c>
       <c r="E50" s="35" t="n">
         <v>71.3</v>
@@ -18259,20 +18259,20 @@
     <row r="51">
       <c r="A51" s="35" t="inlineStr">
         <is>
-          <t>Mississippi State</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="B51" s="35" t="n">
-        <v>68.8</v>
+        <v>68.2</v>
       </c>
       <c r="C51" s="35" t="n">
-        <v>71.3</v>
+        <v>68.3</v>
       </c>
       <c r="D51" s="35" t="n">
-        <v>71.3</v>
+        <v>72</v>
       </c>
       <c r="E51" s="35" t="n">
-        <v>71.3</v>
+        <v>70</v>
       </c>
     </row>
     <row r="52">
@@ -18316,58 +18316,58 @@
     <row r="54">
       <c r="A54" s="35" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="B54" s="35" t="n">
-        <v>69.8</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="C54" s="35" t="n">
         <v>67.2</v>
       </c>
       <c r="D54" s="35" t="n">
-        <v>69.5</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="E54" s="35" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="35" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Minnesota</t>
         </is>
       </c>
       <c r="B55" s="35" t="n">
-        <v>67.8</v>
+        <v>69.8</v>
       </c>
       <c r="C55" s="35" t="n">
-        <v>68.2</v>
+        <v>67.2</v>
       </c>
       <c r="D55" s="35" t="n">
-        <v>68.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="E55" s="35" t="n">
-        <v>69.3</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="35" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="B56" s="35" t="n">
-        <v>64.59999999999999</v>
+        <v>67.8</v>
       </c>
       <c r="C56" s="35" t="n">
-        <v>67.2</v>
+        <v>68.2</v>
       </c>
       <c r="D56" s="35" t="n">
-        <v>68.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="E56" s="35" t="n">
-        <v>68.90000000000001</v>
+        <v>69.3</v>
       </c>
     </row>
     <row r="57">
@@ -18525,20 +18525,20 @@
     <row r="65">
       <c r="A65" s="35" t="inlineStr">
         <is>
-          <t>Michigan State</t>
+          <t>East Carolina</t>
         </is>
       </c>
       <c r="B65" s="35" t="n">
-        <v>66</v>
+        <v>64.8</v>
       </c>
       <c r="C65" s="35" t="n">
-        <v>66.90000000000001</v>
+        <v>63</v>
       </c>
       <c r="D65" s="35" t="n">
-        <v>67.5</v>
+        <v>63.9</v>
       </c>
       <c r="E65" s="35" t="n">
-        <v>67.5</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="66">
@@ -18582,191 +18582,191 @@
     <row r="68">
       <c r="A68" s="35" t="inlineStr">
         <is>
-          <t>West Virginia</t>
+          <t>Michigan State</t>
         </is>
       </c>
       <c r="B68" s="35" t="n">
-        <v>58.2</v>
+        <v>66</v>
       </c>
       <c r="C68" s="35" t="n">
-        <v>63.2</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="D68" s="35" t="n">
-        <v>66.3</v>
+        <v>67.5</v>
       </c>
       <c r="E68" s="35" t="n">
-        <v>66.3</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="35" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>West Virginia</t>
         </is>
       </c>
       <c r="B69" s="35" t="n">
-        <v>65.7</v>
+        <v>58.2</v>
       </c>
       <c r="C69" s="35" t="n">
-        <v>65.40000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="D69" s="35" t="n">
-        <v>65.7</v>
+        <v>66.3</v>
       </c>
       <c r="E69" s="35" t="n">
-        <v>65.7</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="35" t="inlineStr">
         <is>
-          <t>UTSA</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="B70" s="35" t="n">
-        <v>66.59999999999999</v>
+        <v>65.7</v>
       </c>
       <c r="C70" s="35" t="n">
-        <v>66.40000000000001</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D70" s="35" t="n">
-        <v>66</v>
+        <v>65.7</v>
       </c>
       <c r="E70" s="35" t="n">
-        <v>65.59999999999999</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="35" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>UTSA</t>
         </is>
       </c>
       <c r="B71" s="35" t="n">
-        <v>62.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="C71" s="35" t="n">
-        <v>63</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="D71" s="35" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E71" s="35" t="n">
-        <v>65.09999999999999</v>
+        <v>65.59999999999999</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="35" t="inlineStr">
         <is>
-          <t>North Texas</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="B72" s="35" t="n">
-        <v>63.9</v>
+        <v>62.3</v>
       </c>
       <c r="C72" s="35" t="n">
-        <v>67.40000000000001</v>
+        <v>63</v>
       </c>
       <c r="D72" s="35" t="n">
-        <v>64.90000000000001</v>
+        <v>63</v>
       </c>
       <c r="E72" s="35" t="n">
-        <v>64.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="35" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>North Texas</t>
         </is>
       </c>
       <c r="B73" s="35" t="n">
-        <v>61.3</v>
+        <v>63.9</v>
       </c>
       <c r="C73" s="35" t="n">
-        <v>64.7</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="D73" s="35" t="n">
-        <v>64.5</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="E73" s="35" t="n">
-        <v>64.5</v>
+        <v>64.90000000000001</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="35" t="inlineStr">
         <is>
-          <t>Army</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="B74" s="35" t="n">
-        <v>64.5</v>
+        <v>61.3</v>
       </c>
       <c r="C74" s="35" t="n">
-        <v>64.5</v>
+        <v>64.7</v>
       </c>
       <c r="D74" s="35" t="n">
         <v>64.5</v>
       </c>
       <c r="E74" s="35" t="n">
-        <v>64.3</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="35" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Army</t>
         </is>
       </c>
       <c r="B75" s="35" t="n">
-        <v>64.90000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="C75" s="35" t="n">
-        <v>68</v>
+        <v>64.5</v>
       </c>
       <c r="D75" s="35" t="n">
-        <v>64.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="E75" s="35" t="n">
-        <v>64.2</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="35" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="B76" s="35" t="n">
-        <v>66.90000000000001</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="C76" s="35" t="n">
-        <v>65.09999999999999</v>
+        <v>68</v>
       </c>
       <c r="D76" s="35" t="n">
-        <v>64</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="E76" s="35" t="n">
-        <v>64</v>
+        <v>64.2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="35" t="inlineStr">
         <is>
-          <t>East Carolina</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="B77" s="35" t="n">
-        <v>64.8</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="C77" s="35" t="n">
-        <v>63</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="D77" s="35" t="n">
-        <v>63.9</v>
+        <v>64</v>
       </c>
       <c r="E77" s="35" t="n">
-        <v>63.9</v>
+        <v>64</v>
       </c>
     </row>
     <row r="78">
@@ -19114,36 +19114,36 @@
     <row r="96">
       <c r="A96" s="35" t="inlineStr">
         <is>
-          <t>Delaware</t>
+          <t>Boston College</t>
         </is>
       </c>
       <c r="B96" s="35" t="n">
-        <v>56.1</v>
+        <v>57.5</v>
       </c>
       <c r="C96" s="35" t="n">
-        <v>57.6</v>
+        <v>56.6</v>
       </c>
       <c r="D96" s="35" t="n">
-        <v>58.3</v>
+        <v>57.9</v>
       </c>
       <c r="E96" s="35" t="n">
-        <v>58.3</v>
+        <v>58</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="35" t="inlineStr">
         <is>
-          <t>Boston College</t>
+          <t>Florida International</t>
         </is>
       </c>
       <c r="B97" s="35" t="n">
-        <v>57.5</v>
+        <v>55.5</v>
       </c>
       <c r="C97" s="35" t="n">
-        <v>56.6</v>
+        <v>56.4</v>
       </c>
       <c r="D97" s="35" t="n">
-        <v>57.9</v>
+        <v>55.5</v>
       </c>
       <c r="E97" s="35" t="n">
         <v>58</v>
@@ -19266,77 +19266,77 @@
     <row r="104">
       <c r="A104" s="35" t="inlineStr">
         <is>
-          <t>Colorado State</t>
+          <t>Delaware</t>
         </is>
       </c>
       <c r="B104" s="35" t="n">
-        <v>51</v>
+        <v>56.1</v>
       </c>
       <c r="C104" s="35" t="n">
-        <v>55.7</v>
+        <v>57.6</v>
       </c>
       <c r="D104" s="35" t="n">
-        <v>56.1</v>
+        <v>58.3</v>
       </c>
       <c r="E104" s="35" t="n">
-        <v>56.5</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="35" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Colorado State</t>
         </is>
       </c>
       <c r="B105" s="35" t="n">
-        <v>56.7</v>
+        <v>51</v>
       </c>
       <c r="C105" s="35" t="n">
-        <v>57.9</v>
+        <v>55.7</v>
       </c>
       <c r="D105" s="35" t="n">
-        <v>57.2</v>
+        <v>56.1</v>
       </c>
       <c r="E105" s="35" t="n">
-        <v>56.4</v>
+        <v>56.5</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="35" t="inlineStr">
         <is>
-          <t>Georgia Southern</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="B106" s="35" t="n">
-        <v>56.1</v>
+        <v>56.7</v>
       </c>
       <c r="C106" s="35" t="n">
-        <v>55.8</v>
+        <v>57.9</v>
       </c>
       <c r="D106" s="35" t="n">
-        <v>55.6</v>
+        <v>57.2</v>
       </c>
       <c r="E106" s="35" t="n">
-        <v>55.6</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="35" t="inlineStr">
         <is>
-          <t>Florida International</t>
+          <t>Georgia Southern</t>
         </is>
       </c>
       <c r="B107" s="35" t="n">
-        <v>55.5</v>
+        <v>56.1</v>
       </c>
       <c r="C107" s="35" t="n">
-        <v>56.4</v>
+        <v>55.8</v>
       </c>
       <c r="D107" s="35" t="n">
-        <v>55.5</v>
+        <v>55.6</v>
       </c>
       <c r="E107" s="35" t="n">
-        <v>55.5</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="108">
@@ -19836,33 +19836,33 @@
     <row r="134">
       <c r="A134" s="35" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Bowling Green</t>
         </is>
       </c>
       <c r="B134" s="35" t="n">
-        <v>44</v>
+        <v>48.8</v>
       </c>
       <c r="C134" s="35" t="n">
-        <v>44.9</v>
+        <v>46.2</v>
       </c>
       <c r="D134" s="35" t="n">
-        <v>45</v>
+        <v>43.7</v>
       </c>
       <c r="E134" s="35" t="n">
-        <v>45</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="35" t="inlineStr">
         <is>
-          <t>UL Monroe</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="B135" s="35" t="n">
-        <v>42.9</v>
+        <v>44</v>
       </c>
       <c r="C135" s="35" t="n">
-        <v>43.3</v>
+        <v>44.9</v>
       </c>
       <c r="D135" s="35" t="n">
         <v>45</v>
@@ -19874,58 +19874,58 @@
     <row r="136">
       <c r="A136" s="35" t="inlineStr">
         <is>
-          <t>Northern Illinois</t>
+          <t>UL Monroe</t>
         </is>
       </c>
       <c r="B136" s="35" t="n">
-        <v>44.3</v>
+        <v>42.9</v>
       </c>
       <c r="C136" s="35" t="n">
-        <v>45.8</v>
+        <v>43.3</v>
       </c>
       <c r="D136" s="35" t="n">
-        <v>45.9</v>
+        <v>45</v>
       </c>
       <c r="E136" s="35" t="n">
-        <v>44.2</v>
+        <v>45</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="35" t="inlineStr">
         <is>
-          <t>Ball State</t>
+          <t>Northern Illinois</t>
         </is>
       </c>
       <c r="B137" s="35" t="n">
-        <v>43</v>
+        <v>44.3</v>
       </c>
       <c r="C137" s="35" t="n">
-        <v>47.5</v>
+        <v>45.8</v>
       </c>
       <c r="D137" s="35" t="n">
-        <v>44.9</v>
+        <v>45.9</v>
       </c>
       <c r="E137" s="35" t="n">
-        <v>43.9</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="35" t="inlineStr">
         <is>
-          <t>Bowling Green</t>
+          <t>Ball State</t>
         </is>
       </c>
       <c r="B138" s="35" t="n">
-        <v>48.8</v>
+        <v>43</v>
       </c>
       <c r="C138" s="35" t="n">
-        <v>46.2</v>
+        <v>47.5</v>
       </c>
       <c r="D138" s="35" t="n">
-        <v>43.7</v>
+        <v>44.9</v>
       </c>
       <c r="E138" s="35" t="n">
-        <v>43.7</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="139">

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-09-27 03:40 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -17341,7 +17341,7 @@
         <v>91.40000000000001</v>
       </c>
       <c r="E4" s="35" t="n">
-        <v>91.40000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="V4" s="35" t="inlineStr">
         <is>
@@ -17395,7 +17395,7 @@
         <v>89.7</v>
       </c>
       <c r="E6" s="35" t="n">
-        <v>89.7</v>
+        <v>89.5</v>
       </c>
     </row>
     <row r="7">
@@ -17499,77 +17499,77 @@
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="B11" s="35" t="n">
-        <v>81.2</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="C11" s="35" t="n">
-        <v>80.2</v>
+        <v>82.3</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>84.59999999999999</v>
+        <v>82.2</v>
       </c>
       <c r="E11" s="35" t="n">
-        <v>83.7</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="B12" s="35" t="n">
-        <v>80.90000000000001</v>
+        <v>81.2</v>
       </c>
       <c r="C12" s="35" t="n">
-        <v>82.3</v>
+        <v>80.2</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>82.2</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="E12" s="35" t="n">
-        <v>82.2</v>
+        <v>83.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>LSU</t>
         </is>
       </c>
       <c r="B13" s="35" t="n">
-        <v>79.2</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C13" s="35" t="n">
-        <v>83.2</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>80.09999999999999</v>
+        <v>79.7</v>
       </c>
       <c r="E13" s="35" t="n">
-        <v>81.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="35" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="B14" s="35" t="n">
-        <v>82.8</v>
+        <v>79.2</v>
       </c>
       <c r="C14" s="35" t="n">
-        <v>84.3</v>
+        <v>83.2</v>
       </c>
       <c r="D14" s="35" t="n">
-        <v>81.7</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="E14" s="35" t="n">
-        <v>81.7</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="15">
@@ -17613,115 +17613,115 @@
     <row r="17">
       <c r="A17" s="35" t="inlineStr">
         <is>
-          <t>South Carolina</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="B17" s="35" t="n">
-        <v>75.09999999999999</v>
+        <v>75</v>
       </c>
       <c r="C17" s="35" t="n">
-        <v>81</v>
+        <v>74.8</v>
       </c>
       <c r="D17" s="35" t="n">
-        <v>81</v>
+        <v>76.2</v>
       </c>
       <c r="E17" s="35" t="n">
-        <v>81</v>
+        <v>80.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Penn State</t>
         </is>
       </c>
       <c r="B18" s="35" t="n">
-        <v>75</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="C18" s="35" t="n">
-        <v>74.8</v>
+        <v>80.3</v>
       </c>
       <c r="D18" s="35" t="n">
-        <v>76.2</v>
+        <v>81.2</v>
       </c>
       <c r="E18" s="35" t="n">
-        <v>80.5</v>
+        <v>80.40000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="35" t="inlineStr">
         <is>
-          <t>Penn State</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="B19" s="35" t="n">
-        <v>80.90000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="C19" s="35" t="n">
-        <v>80.3</v>
+        <v>77.8</v>
       </c>
       <c r="D19" s="35" t="n">
-        <v>81.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="E19" s="35" t="n">
-        <v>80.40000000000001</v>
+        <v>80.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="B20" s="35" t="n">
-        <v>76.8</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C20" s="35" t="n">
-        <v>77.8</v>
+        <v>78.3</v>
       </c>
       <c r="D20" s="35" t="n">
-        <v>78.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="E20" s="35" t="n">
-        <v>80.2</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="35" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>South Carolina</t>
         </is>
       </c>
       <c r="B21" s="35" t="n">
-        <v>79.09999999999999</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="C21" s="35" t="n">
-        <v>78.3</v>
+        <v>81</v>
       </c>
       <c r="D21" s="35" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E21" s="35" t="n">
-        <v>80</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="35" t="inlineStr">
         <is>
-          <t>LSU</t>
+          <t>James Madison</t>
         </is>
       </c>
       <c r="B22" s="35" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="C22" s="35" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="D22" s="35" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="E22" s="35" t="n">
         <v>79.09999999999999</v>
-      </c>
-      <c r="C22" s="35" t="n">
-        <v>80.09999999999999</v>
-      </c>
-      <c r="D22" s="35" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="E22" s="35" t="n">
-        <v>79.7</v>
       </c>
     </row>
     <row r="23">
@@ -17746,55 +17746,55 @@
     <row r="24">
       <c r="A24" s="35" t="inlineStr">
         <is>
-          <t>BYU</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="B24" s="35" t="n">
-        <v>78.3</v>
+        <v>82.8</v>
       </c>
       <c r="C24" s="35" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="D24" s="35" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="E24" s="35" t="n">
         <v>79</v>
-      </c>
-      <c r="D24" s="35" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="E24" s="35" t="n">
-        <v>78.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="35" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>BYU</t>
         </is>
       </c>
       <c r="B25" s="35" t="n">
-        <v>74.7</v>
+        <v>78.3</v>
       </c>
       <c r="C25" s="35" t="n">
-        <v>78.8</v>
+        <v>79</v>
       </c>
       <c r="D25" s="35" t="n">
-        <v>79.8</v>
+        <v>78.5</v>
       </c>
       <c r="E25" s="35" t="n">
-        <v>77.90000000000001</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="35" t="inlineStr">
         <is>
-          <t>SMU</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B26" s="35" t="n">
-        <v>75.40000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="C26" s="35" t="n">
-        <v>78.90000000000001</v>
+        <v>78.8</v>
       </c>
       <c r="D26" s="35" t="n">
-        <v>77.90000000000001</v>
+        <v>79.8</v>
       </c>
       <c r="E26" s="35" t="n">
         <v>77.90000000000001</v>
@@ -17803,17 +17803,17 @@
     <row r="27">
       <c r="A27" s="35" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>SMU</t>
         </is>
       </c>
       <c r="B27" s="35" t="n">
-        <v>81.2</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="C27" s="35" t="n">
-        <v>79.5</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D27" s="35" t="n">
-        <v>80</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="E27" s="35" t="n">
         <v>77.90000000000001</v>
@@ -17822,77 +17822,77 @@
     <row r="28">
       <c r="A28" s="35" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>Oklahoma</t>
         </is>
       </c>
       <c r="B28" s="35" t="n">
-        <v>78</v>
+        <v>81.2</v>
       </c>
       <c r="C28" s="35" t="n">
-        <v>77.5</v>
+        <v>79.5</v>
       </c>
       <c r="D28" s="35" t="n">
-        <v>77.40000000000001</v>
+        <v>80</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>77.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="35" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>USC</t>
         </is>
       </c>
       <c r="B29" s="35" t="n">
-        <v>80.40000000000001</v>
+        <v>78</v>
       </c>
       <c r="C29" s="35" t="n">
-        <v>78.8</v>
+        <v>77.5</v>
       </c>
       <c r="D29" s="35" t="n">
-        <v>78.8</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="E29" s="35" t="n">
-        <v>77.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="35" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="B30" s="35" t="n">
-        <v>72.09999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="C30" s="35" t="n">
-        <v>74.7</v>
+        <v>78.8</v>
       </c>
       <c r="D30" s="35" t="n">
-        <v>76.3</v>
+        <v>78.8</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>77.2</v>
+        <v>77.40000000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="35" t="inlineStr">
         <is>
-          <t>James Madison</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="B31" s="35" t="n">
-        <v>67.8</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="C31" s="35" t="n">
-        <v>76.8</v>
+        <v>74.7</v>
       </c>
       <c r="D31" s="35" t="n">
-        <v>77.09999999999999</v>
+        <v>76.3</v>
       </c>
       <c r="E31" s="35" t="n">
-        <v>77.09999999999999</v>
+        <v>77.2</v>
       </c>
     </row>
     <row r="32">
@@ -17993,131 +17993,131 @@
     <row r="37">
       <c r="A37" s="35" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>Illinois</t>
         </is>
       </c>
       <c r="B37" s="35" t="n">
-        <v>67.2</v>
+        <v>71</v>
       </c>
       <c r="C37" s="35" t="n">
-        <v>74.2</v>
+        <v>71.2</v>
       </c>
       <c r="D37" s="35" t="n">
         <v>74.3</v>
       </c>
       <c r="E37" s="35" t="n">
-        <v>74.3</v>
+        <v>73.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="35" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>Northwestern</t>
         </is>
       </c>
       <c r="B38" s="35" t="n">
-        <v>74.59999999999999</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="C38" s="35" t="n">
-        <v>74.90000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="D38" s="35" t="n">
-        <v>74</v>
+        <v>71.5</v>
       </c>
       <c r="E38" s="35" t="n">
-        <v>74</v>
+        <v>73.59999999999999</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="35" t="inlineStr">
         <is>
-          <t>Illinois</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="B39" s="35" t="n">
-        <v>71</v>
+        <v>69.3</v>
       </c>
       <c r="C39" s="35" t="n">
-        <v>71.2</v>
+        <v>74</v>
       </c>
       <c r="D39" s="35" t="n">
-        <v>74.3</v>
+        <v>73</v>
       </c>
       <c r="E39" s="35" t="n">
-        <v>73.8</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="35" t="inlineStr">
         <is>
-          <t>Northwestern</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="B40" s="35" t="n">
-        <v>68.09999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="C40" s="35" t="n">
-        <v>68.09999999999999</v>
+        <v>72.7</v>
       </c>
       <c r="D40" s="35" t="n">
-        <v>71.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="E40" s="35" t="n">
-        <v>73.59999999999999</v>
+        <v>73.2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="35" t="inlineStr">
         <is>
-          <t>Kansas State</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="B41" s="35" t="n">
-        <v>70.7</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C41" s="35" t="n">
-        <v>73.2</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="D41" s="35" t="n">
-        <v>73.40000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="E41" s="35" t="n">
-        <v>73.40000000000001</v>
+        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="35" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>Kansas State</t>
         </is>
       </c>
       <c r="B42" s="35" t="n">
-        <v>69.09999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="C42" s="35" t="n">
-        <v>74.09999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="D42" s="35" t="n">
-        <v>75.09999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="E42" s="35" t="n">
-        <v>73.09999999999999</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="35" t="inlineStr">
         <is>
-          <t>Cincinnati</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="B43" s="35" t="n">
-        <v>69.3</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="C43" s="35" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="D43" s="35" t="n">
         <v>74</v>
-      </c>
-      <c r="D43" s="35" t="n">
-        <v>73</v>
       </c>
       <c r="E43" s="35" t="n">
         <v>73</v>
@@ -18126,17 +18126,17 @@
     <row r="44">
       <c r="A44" s="35" t="inlineStr">
         <is>
-          <t>Auburn</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="B44" s="35" t="n">
-        <v>69.40000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="C44" s="35" t="n">
-        <v>71.2</v>
+        <v>74.2</v>
       </c>
       <c r="D44" s="35" t="n">
-        <v>71.5</v>
+        <v>74.3</v>
       </c>
       <c r="E44" s="35" t="n">
         <v>72.90000000000001</v>
@@ -18145,20 +18145,20 @@
     <row r="45">
       <c r="A45" s="35" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Auburn</t>
         </is>
       </c>
       <c r="B45" s="35" t="n">
-        <v>73.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="C45" s="35" t="n">
-        <v>72.7</v>
+        <v>71.2</v>
       </c>
       <c r="D45" s="35" t="n">
-        <v>72.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="E45" s="35" t="n">
-        <v>72.59999999999999</v>
+        <v>72.90000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -18183,74 +18183,74 @@
     <row r="47">
       <c r="A47" s="35" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>Mississippi State</t>
         </is>
       </c>
       <c r="B47" s="35" t="n">
-        <v>66.8</v>
+        <v>68.8</v>
       </c>
       <c r="C47" s="35" t="n">
-        <v>71.2</v>
+        <v>71.3</v>
       </c>
       <c r="D47" s="35" t="n">
-        <v>71.5</v>
+        <v>71.3</v>
       </c>
       <c r="E47" s="35" t="n">
-        <v>72</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="35" t="inlineStr">
         <is>
-          <t>Iowa State</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="B48" s="35" t="n">
-        <v>68.3</v>
+        <v>66.8</v>
       </c>
       <c r="C48" s="35" t="n">
-        <v>69.3</v>
+        <v>71.2</v>
       </c>
       <c r="D48" s="35" t="n">
-        <v>71.8</v>
+        <v>71.5</v>
       </c>
       <c r="E48" s="35" t="n">
-        <v>71.7</v>
+        <v>72</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="35" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Iowa State</t>
         </is>
       </c>
       <c r="B49" s="35" t="n">
-        <v>63.8</v>
+        <v>68.3</v>
       </c>
       <c r="C49" s="35" t="n">
-        <v>65.90000000000001</v>
+        <v>69.3</v>
       </c>
       <c r="D49" s="35" t="n">
-        <v>66.7</v>
+        <v>71.8</v>
       </c>
       <c r="E49" s="35" t="n">
-        <v>71.3</v>
+        <v>71.7</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="35" t="inlineStr">
         <is>
-          <t>Mississippi State</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="B50" s="35" t="n">
-        <v>68.8</v>
+        <v>63.8</v>
       </c>
       <c r="C50" s="35" t="n">
-        <v>71.3</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="D50" s="35" t="n">
-        <v>71.3</v>
+        <v>66.7</v>
       </c>
       <c r="E50" s="35" t="n">
         <v>71.3</v>
@@ -18278,17 +18278,17 @@
     <row r="52">
       <c r="A52" s="35" t="inlineStr">
         <is>
-          <t>Florida State</t>
+          <t>North Texas</t>
         </is>
       </c>
       <c r="B52" s="35" t="n">
-        <v>67.2</v>
+        <v>63.9</v>
       </c>
       <c r="C52" s="35" t="n">
-        <v>67.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="D52" s="35" t="n">
-        <v>67.3</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="E52" s="35" t="n">
         <v>69.7</v>
@@ -18297,36 +18297,36 @@
     <row r="53">
       <c r="A53" s="35" t="inlineStr">
         <is>
-          <t>Georgia Tech</t>
+          <t>Florida State</t>
         </is>
       </c>
       <c r="B53" s="35" t="n">
-        <v>67.7</v>
+        <v>67.2</v>
       </c>
       <c r="C53" s="35" t="n">
-        <v>66.59999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="D53" s="35" t="n">
-        <v>69.59999999999999</v>
+        <v>67.3</v>
       </c>
       <c r="E53" s="35" t="n">
-        <v>69.59999999999999</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="35" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="B54" s="35" t="n">
-        <v>64.59999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="C54" s="35" t="n">
-        <v>67.2</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="D54" s="35" t="n">
-        <v>68.90000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E54" s="35" t="n">
         <v>69.59999999999999</v>
@@ -18335,150 +18335,150 @@
     <row r="55">
       <c r="A55" s="35" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="B55" s="35" t="n">
-        <v>69.8</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="C55" s="35" t="n">
         <v>67.2</v>
       </c>
       <c r="D55" s="35" t="n">
-        <v>69.5</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="E55" s="35" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="35" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Minnesota</t>
         </is>
       </c>
       <c r="B56" s="35" t="n">
-        <v>67.8</v>
+        <v>69.8</v>
       </c>
       <c r="C56" s="35" t="n">
-        <v>68.2</v>
+        <v>67.2</v>
       </c>
       <c r="D56" s="35" t="n">
-        <v>68.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="E56" s="35" t="n">
-        <v>69.3</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="35" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="B57" s="35" t="n">
-        <v>66.5</v>
+        <v>67.8</v>
       </c>
       <c r="C57" s="35" t="n">
-        <v>65.2</v>
+        <v>68.2</v>
       </c>
       <c r="D57" s="35" t="n">
-        <v>67.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="E57" s="35" t="n">
-        <v>68.7</v>
+        <v>69.3</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="35" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Texas State</t>
         </is>
       </c>
       <c r="B58" s="35" t="n">
-        <v>62.1</v>
+        <v>60.5</v>
       </c>
       <c r="C58" s="35" t="n">
-        <v>67.59999999999999</v>
+        <v>60.7</v>
       </c>
       <c r="D58" s="35" t="n">
-        <v>66.59999999999999</v>
+        <v>63.2</v>
       </c>
       <c r="E58" s="35" t="n">
-        <v>68.59999999999999</v>
+        <v>68.90000000000001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="35" t="inlineStr">
         <is>
-          <t>Old Dominion</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="B59" s="35" t="n">
-        <v>72.59999999999999</v>
+        <v>66.5</v>
       </c>
       <c r="C59" s="35" t="n">
-        <v>69.5</v>
+        <v>65.2</v>
       </c>
       <c r="D59" s="35" t="n">
-        <v>68.5</v>
+        <v>67.7</v>
       </c>
       <c r="E59" s="35" t="n">
-        <v>68.5</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="35" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Toledo</t>
         </is>
       </c>
       <c r="B60" s="35" t="n">
-        <v>68.2</v>
+        <v>62.1</v>
       </c>
       <c r="C60" s="35" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="D60" s="35" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="D60" s="35" t="n">
-        <v>68.2</v>
-      </c>
       <c r="E60" s="35" t="n">
-        <v>68.2</v>
+        <v>68.59999999999999</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="35" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="B61" s="35" t="n">
-        <v>72.2</v>
+        <v>68.2</v>
       </c>
       <c r="C61" s="35" t="n">
-        <v>69.40000000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="D61" s="35" t="n">
-        <v>69.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="E61" s="35" t="n">
-        <v>67.8</v>
+        <v>68.2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="35" t="inlineStr">
         <is>
-          <t>Washington State</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="B62" s="35" t="n">
-        <v>66.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C62" s="35" t="n">
-        <v>63.7</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D62" s="35" t="n">
-        <v>67.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="E62" s="35" t="n">
         <v>67.8</v>
@@ -18544,267 +18544,267 @@
     <row r="66">
       <c r="A66" s="35" t="inlineStr">
         <is>
-          <t>Rutgers</t>
+          <t>Washington State</t>
         </is>
       </c>
       <c r="B66" s="35" t="n">
-        <v>61.1</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="C66" s="35" t="n">
-        <v>62</v>
+        <v>63.7</v>
       </c>
       <c r="D66" s="35" t="n">
-        <v>62.1</v>
+        <v>67.8</v>
       </c>
       <c r="E66" s="35" t="n">
-        <v>67.09999999999999</v>
+        <v>67.2</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="35" t="inlineStr">
         <is>
-          <t>Western Michigan</t>
+          <t>Rutgers</t>
         </is>
       </c>
       <c r="B67" s="35" t="n">
-        <v>68.09999999999999</v>
+        <v>61.1</v>
       </c>
       <c r="C67" s="35" t="n">
-        <v>71.09999999999999</v>
+        <v>62</v>
       </c>
       <c r="D67" s="35" t="n">
-        <v>69.3</v>
+        <v>62.1</v>
       </c>
       <c r="E67" s="35" t="n">
-        <v>66.90000000000001</v>
+        <v>67.09999999999999</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="35" t="inlineStr">
         <is>
-          <t>Michigan State</t>
+          <t>Western Michigan</t>
         </is>
       </c>
       <c r="B68" s="35" t="n">
-        <v>66</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="C68" s="35" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="D68" s="35" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="E68" s="35" t="n">
         <v>66.90000000000001</v>
-      </c>
-      <c r="D68" s="35" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="E68" s="35" t="n">
-        <v>66.5</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="35" t="inlineStr">
         <is>
-          <t>West Virginia</t>
+          <t>Michigan State</t>
         </is>
       </c>
       <c r="B69" s="35" t="n">
-        <v>58.2</v>
+        <v>66</v>
       </c>
       <c r="C69" s="35" t="n">
-        <v>63.2</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="D69" s="35" t="n">
-        <v>66.3</v>
+        <v>67.5</v>
       </c>
       <c r="E69" s="35" t="n">
-        <v>66.3</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="35" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Old Dominion</t>
         </is>
       </c>
       <c r="B70" s="35" t="n">
-        <v>65.7</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C70" s="35" t="n">
-        <v>65.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="D70" s="35" t="n">
-        <v>65.7</v>
+        <v>68.5</v>
       </c>
       <c r="E70" s="35" t="n">
-        <v>65.7</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="35" t="inlineStr">
         <is>
-          <t>UTSA</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="B71" s="35" t="n">
-        <v>66.59999999999999</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="C71" s="35" t="n">
-        <v>66.40000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="D71" s="35" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E71" s="35" t="n">
-        <v>65.59999999999999</v>
+        <v>66.2</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="35" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="B72" s="35" t="n">
-        <v>62.3</v>
+        <v>65.7</v>
       </c>
       <c r="C72" s="35" t="n">
-        <v>63</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D72" s="35" t="n">
-        <v>63</v>
+        <v>65.7</v>
       </c>
       <c r="E72" s="35" t="n">
-        <v>65.09999999999999</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="35" t="inlineStr">
         <is>
-          <t>North Texas</t>
+          <t>UTSA</t>
         </is>
       </c>
       <c r="B73" s="35" t="n">
-        <v>63.9</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="C73" s="35" t="n">
-        <v>67.40000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="D73" s="35" t="n">
-        <v>64.90000000000001</v>
+        <v>66</v>
       </c>
       <c r="E73" s="35" t="n">
-        <v>64.90000000000001</v>
+        <v>65.59999999999999</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="35" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="B74" s="35" t="n">
-        <v>61.3</v>
+        <v>62.3</v>
       </c>
       <c r="C74" s="35" t="n">
-        <v>64.7</v>
+        <v>63</v>
       </c>
       <c r="D74" s="35" t="n">
-        <v>64.5</v>
+        <v>63</v>
       </c>
       <c r="E74" s="35" t="n">
-        <v>64.5</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="35" t="inlineStr">
         <is>
-          <t>Army</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="B75" s="35" t="n">
-        <v>64.5</v>
+        <v>61.3</v>
       </c>
       <c r="C75" s="35" t="n">
-        <v>64.5</v>
+        <v>64.7</v>
       </c>
       <c r="D75" s="35" t="n">
         <v>64.5</v>
       </c>
       <c r="E75" s="35" t="n">
-        <v>64.3</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="35" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Army</t>
         </is>
       </c>
       <c r="B76" s="35" t="n">
-        <v>64.90000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="C76" s="35" t="n">
-        <v>68</v>
+        <v>64.5</v>
       </c>
       <c r="D76" s="35" t="n">
-        <v>64.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="E76" s="35" t="n">
-        <v>64.2</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="35" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>West Virginia</t>
         </is>
       </c>
       <c r="B77" s="35" t="n">
-        <v>66.90000000000001</v>
+        <v>58.2</v>
       </c>
       <c r="C77" s="35" t="n">
-        <v>65.09999999999999</v>
+        <v>63.2</v>
       </c>
       <c r="D77" s="35" t="n">
-        <v>64</v>
+        <v>66.3</v>
       </c>
       <c r="E77" s="35" t="n">
-        <v>64</v>
+        <v>64.2</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="35" t="inlineStr">
         <is>
-          <t>Texas State</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="B78" s="35" t="n">
-        <v>60.5</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="C78" s="35" t="n">
-        <v>60.7</v>
+        <v>68</v>
       </c>
       <c r="D78" s="35" t="n">
-        <v>63.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="E78" s="35" t="n">
-        <v>63.2</v>
+        <v>64.2</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="35" t="inlineStr">
         <is>
-          <t>Tulane</t>
+          <t>Oklahoma State</t>
         </is>
       </c>
       <c r="B79" s="35" t="n">
-        <v>63.9</v>
+        <v>50.2</v>
       </c>
       <c r="C79" s="35" t="n">
-        <v>63.1</v>
+        <v>54.5</v>
       </c>
       <c r="D79" s="35" t="n">
-        <v>62.9</v>
+        <v>61.5</v>
       </c>
       <c r="E79" s="35" t="n">
-        <v>62.9</v>
+        <v>63.6</v>
       </c>
     </row>
     <row r="80">
@@ -18829,77 +18829,77 @@
     <row r="81">
       <c r="A81" s="35" t="inlineStr">
         <is>
-          <t>Liberty</t>
+          <t>Utah State</t>
         </is>
       </c>
       <c r="B81" s="35" t="n">
-        <v>57.2</v>
+        <v>60.9</v>
       </c>
       <c r="C81" s="35" t="n">
-        <v>58</v>
+        <v>61.7</v>
       </c>
       <c r="D81" s="35" t="n">
-        <v>60.5</v>
+        <v>61</v>
       </c>
       <c r="E81" s="35" t="n">
-        <v>61.7</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="35" t="inlineStr">
         <is>
-          <t>Oklahoma State</t>
+          <t>Tulane</t>
         </is>
       </c>
       <c r="B82" s="35" t="n">
-        <v>50.2</v>
+        <v>63.9</v>
       </c>
       <c r="C82" s="35" t="n">
-        <v>54.5</v>
+        <v>63.1</v>
       </c>
       <c r="D82" s="35" t="n">
-        <v>61.5</v>
+        <v>62.9</v>
       </c>
       <c r="E82" s="35" t="n">
-        <v>61.5</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="35" t="inlineStr">
         <is>
-          <t>Ohio</t>
+          <t>Liberty</t>
         </is>
       </c>
       <c r="B83" s="35" t="n">
-        <v>58.8</v>
+        <v>57.2</v>
       </c>
       <c r="C83" s="35" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D83" s="35" t="n">
-        <v>58.2</v>
+        <v>60.5</v>
       </c>
       <c r="E83" s="35" t="n">
-        <v>61.3</v>
+        <v>61.7</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="35" t="inlineStr">
         <is>
-          <t>Utah State</t>
+          <t>Ohio</t>
         </is>
       </c>
       <c r="B84" s="35" t="n">
-        <v>60.9</v>
+        <v>58.8</v>
       </c>
       <c r="C84" s="35" t="n">
-        <v>61.7</v>
+        <v>59</v>
       </c>
       <c r="D84" s="35" t="n">
-        <v>61</v>
+        <v>58.2</v>
       </c>
       <c r="E84" s="35" t="n">
-        <v>61</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="85">
@@ -19038,20 +19038,20 @@
     <row r="92">
       <c r="A92" s="35" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Western Kentucky</t>
         </is>
       </c>
       <c r="B92" s="35" t="n">
-        <v>55.3</v>
+        <v>56.1</v>
       </c>
       <c r="C92" s="35" t="n">
-        <v>54.8</v>
+        <v>53.9</v>
       </c>
       <c r="D92" s="35" t="n">
-        <v>59.9</v>
+        <v>54.6</v>
       </c>
       <c r="E92" s="35" t="n">
-        <v>59.9</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="93">
@@ -19089,7 +19089,7 @@
         <v>59.1</v>
       </c>
       <c r="E94" s="35" t="n">
-        <v>59.1</v>
+        <v>58.9</v>
       </c>
     </row>
     <row r="95">
@@ -19165,45 +19165,45 @@
         <v>57.9</v>
       </c>
       <c r="E98" s="35" t="n">
-        <v>57.9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="35" t="inlineStr">
         <is>
-          <t>UConn</t>
+          <t>Tulsa</t>
         </is>
       </c>
       <c r="B99" s="35" t="n">
-        <v>57.3</v>
+        <v>55.3</v>
       </c>
       <c r="C99" s="35" t="n">
-        <v>54.5</v>
+        <v>54.8</v>
       </c>
       <c r="D99" s="35" t="n">
-        <v>57.1</v>
+        <v>59.9</v>
       </c>
       <c r="E99" s="35" t="n">
-        <v>57.2</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="35" t="inlineStr">
         <is>
-          <t>Central Michigan</t>
+          <t>UConn</t>
         </is>
       </c>
       <c r="B100" s="35" t="n">
-        <v>55</v>
+        <v>57.3</v>
       </c>
       <c r="C100" s="35" t="n">
-        <v>56.2</v>
+        <v>54.5</v>
       </c>
       <c r="D100" s="35" t="n">
         <v>57.1</v>
       </c>
       <c r="E100" s="35" t="n">
-        <v>57.1</v>
+        <v>57.2</v>
       </c>
     </row>
     <row r="101">
@@ -19228,33 +19228,33 @@
     <row r="102">
       <c r="A102" s="35" t="inlineStr">
         <is>
-          <t>Syracuse</t>
+          <t>Louisiana</t>
         </is>
       </c>
       <c r="B102" s="35" t="n">
-        <v>55.7</v>
+        <v>54.3</v>
       </c>
       <c r="C102" s="35" t="n">
-        <v>56.3</v>
+        <v>54.7</v>
       </c>
       <c r="D102" s="35" t="n">
-        <v>56.8</v>
+        <v>55.2</v>
       </c>
       <c r="E102" s="35" t="n">
-        <v>56.8</v>
+        <v>56.9</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="35" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Syracuse</t>
         </is>
       </c>
       <c r="B103" s="35" t="n">
-        <v>53.1</v>
+        <v>55.7</v>
       </c>
       <c r="C103" s="35" t="n">
-        <v>55.9</v>
+        <v>56.3</v>
       </c>
       <c r="D103" s="35" t="n">
         <v>56.8</v>
@@ -19342,93 +19342,93 @@
     <row r="108">
       <c r="A108" s="35" t="inlineStr">
         <is>
-          <t>Louisiana</t>
+          <t>Florida Atlantic</t>
         </is>
       </c>
       <c r="B108" s="35" t="n">
-        <v>54.3</v>
+        <v>50.4</v>
       </c>
       <c r="C108" s="35" t="n">
-        <v>54.7</v>
+        <v>53.3</v>
       </c>
       <c r="D108" s="35" t="n">
-        <v>55.2</v>
+        <v>54.2</v>
       </c>
       <c r="E108" s="35" t="n">
-        <v>55.2</v>
+        <v>56.1</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="35" t="inlineStr">
         <is>
-          <t>Missouri State</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="B109" s="35" t="n">
-        <v>50.7</v>
+        <v>53.1</v>
       </c>
       <c r="C109" s="35" t="n">
-        <v>55.6</v>
+        <v>55.9</v>
       </c>
       <c r="D109" s="35" t="n">
-        <v>54.7</v>
+        <v>56.8</v>
       </c>
       <c r="E109" s="35" t="n">
-        <v>54.7</v>
+        <v>55.9</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="35" t="inlineStr">
         <is>
-          <t>Western Kentucky</t>
+          <t>Central Michigan</t>
         </is>
       </c>
       <c r="B110" s="35" t="n">
-        <v>56.1</v>
+        <v>55</v>
       </c>
       <c r="C110" s="35" t="n">
-        <v>53.9</v>
+        <v>56.2</v>
       </c>
       <c r="D110" s="35" t="n">
-        <v>54.6</v>
+        <v>57.1</v>
       </c>
       <c r="E110" s="35" t="n">
-        <v>54.6</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="35" t="inlineStr">
         <is>
-          <t>Coastal Carolina</t>
+          <t>Missouri State</t>
         </is>
       </c>
       <c r="B111" s="35" t="n">
-        <v>51</v>
+        <v>50.7</v>
       </c>
       <c r="C111" s="35" t="n">
-        <v>56.1</v>
+        <v>55.6</v>
       </c>
       <c r="D111" s="35" t="n">
-        <v>55.4</v>
+        <v>54.7</v>
       </c>
       <c r="E111" s="35" t="n">
-        <v>54.2</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="35" t="inlineStr">
         <is>
-          <t>Florida Atlantic</t>
+          <t>Coastal Carolina</t>
         </is>
       </c>
       <c r="B112" s="35" t="n">
-        <v>50.4</v>
+        <v>51</v>
       </c>
       <c r="C112" s="35" t="n">
-        <v>53.3</v>
+        <v>56.1</v>
       </c>
       <c r="D112" s="35" t="n">
-        <v>54.2</v>
+        <v>55.4</v>
       </c>
       <c r="E112" s="35" t="n">
         <v>54.2</v>
@@ -19545,7 +19545,7 @@
         <v>52.6</v>
       </c>
       <c r="E118" s="35" t="n">
-        <v>52.6</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="119">
@@ -19570,77 +19570,77 @@
     <row r="120">
       <c r="A120" s="35" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>App State</t>
         </is>
       </c>
       <c r="B120" s="35" t="n">
-        <v>48.6</v>
+        <v>49.2</v>
       </c>
       <c r="C120" s="35" t="n">
-        <v>50.9</v>
+        <v>51.1</v>
       </c>
       <c r="D120" s="35" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E120" s="35" t="n">
-        <v>51.9</v>
+        <v>52.3</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="35" t="inlineStr">
         <is>
-          <t>Georgia State</t>
+          <t>Wyoming</t>
         </is>
       </c>
       <c r="B121" s="35" t="n">
-        <v>47.4</v>
+        <v>48.6</v>
       </c>
       <c r="C121" s="35" t="n">
-        <v>49.7</v>
+        <v>50.9</v>
       </c>
       <c r="D121" s="35" t="n">
-        <v>49.6</v>
+        <v>50</v>
       </c>
       <c r="E121" s="35" t="n">
-        <v>51.3</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="35" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Georgia State</t>
         </is>
       </c>
       <c r="B122" s="35" t="n">
-        <v>51.5</v>
+        <v>47.4</v>
       </c>
       <c r="C122" s="35" t="n">
-        <v>50.6</v>
+        <v>49.7</v>
       </c>
       <c r="D122" s="35" t="n">
-        <v>49.8</v>
+        <v>49.6</v>
       </c>
       <c r="E122" s="35" t="n">
-        <v>51.2</v>
+        <v>51.3</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="35" t="inlineStr">
         <is>
-          <t>App State</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="B123" s="35" t="n">
-        <v>49.2</v>
+        <v>51.5</v>
       </c>
       <c r="C123" s="35" t="n">
-        <v>51.1</v>
+        <v>50.6</v>
       </c>
       <c r="D123" s="35" t="n">
-        <v>51</v>
+        <v>49.8</v>
       </c>
       <c r="E123" s="35" t="n">
-        <v>51</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="124">
@@ -19659,7 +19659,7 @@
         <v>49.9</v>
       </c>
       <c r="E124" s="35" t="n">
-        <v>49.9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="125">
@@ -19855,77 +19855,77 @@
     <row r="135">
       <c r="A135" s="35" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Northern Illinois</t>
         </is>
       </c>
       <c r="B135" s="35" t="n">
-        <v>44</v>
+        <v>44.3</v>
       </c>
       <c r="C135" s="35" t="n">
-        <v>44.9</v>
+        <v>45.8</v>
       </c>
       <c r="D135" s="35" t="n">
-        <v>45</v>
+        <v>45.9</v>
       </c>
       <c r="E135" s="35" t="n">
-        <v>45</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="35" t="inlineStr">
         <is>
-          <t>UL Monroe</t>
+          <t>Ball State</t>
         </is>
       </c>
       <c r="B136" s="35" t="n">
-        <v>42.9</v>
+        <v>43</v>
       </c>
       <c r="C136" s="35" t="n">
-        <v>43.3</v>
+        <v>47.5</v>
       </c>
       <c r="D136" s="35" t="n">
-        <v>45</v>
+        <v>44.9</v>
       </c>
       <c r="E136" s="35" t="n">
-        <v>45</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="35" t="inlineStr">
         <is>
-          <t>Northern Illinois</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="B137" s="35" t="n">
-        <v>44.3</v>
+        <v>44</v>
       </c>
       <c r="C137" s="35" t="n">
-        <v>45.8</v>
+        <v>44.9</v>
       </c>
       <c r="D137" s="35" t="n">
-        <v>45.9</v>
+        <v>45</v>
       </c>
       <c r="E137" s="35" t="n">
-        <v>44.2</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="35" t="inlineStr">
         <is>
-          <t>Ball State</t>
+          <t>UL Monroe</t>
         </is>
       </c>
       <c r="B138" s="35" t="n">
-        <v>43</v>
+        <v>42.9</v>
       </c>
       <c r="C138" s="35" t="n">
-        <v>47.5</v>
+        <v>43.3</v>
       </c>
       <c r="D138" s="35" t="n">
-        <v>44.9</v>
+        <v>45</v>
       </c>
       <c r="E138" s="35" t="n">
-        <v>43.9</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="139">

</xml_diff>

<commit_message>
Regenerate site data with Line column populated
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deene\Mountain Dub Handicapping\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E43BEDF-AE36-40AF-AEA3-18C866DD2CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17BDA28C-B9EF-4C07-9B16-E533F78130FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6827,9 +6827,6 @@
       <c r="E57" t="s">
         <v>73</v>
       </c>
-      <c r="F57">
-        <v>0</v>
-      </c>
       <c r="G57">
         <v>116</v>
       </c>
@@ -12388,11 +12385,11 @@
     </row>
     <row r="450" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J450" s="12" t="str">
-        <f t="shared" ref="J450:J513" si="14">IF(I450="","",I450-F450)</f>
+        <f t="shared" ref="J450:J500" si="14">IF(I450="","",I450-F450)</f>
         <v/>
       </c>
       <c r="L450" s="11">
-        <f t="shared" ref="L450:L513" si="15">IF(K450="W",IF(G450&lt;0,H450*100/ABS(G450),H450*G450/100),IF(K450="L",-H450,0))</f>
+        <f t="shared" ref="L450:L500" si="15">IF(K450="W",IF(G450&lt;0,H450*100/ABS(G450),H450*G450/100),IF(K450="L",-H450,0))</f>
         <v>0</v>
       </c>
       <c r="M450" s="11">

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-09-29 20:10 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -938,7 +938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18628,7 +18628,7 @@
         </is>
       </c>
       <c r="C88" s="33" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D88" s="33" t="n">
         <v>83</v>

</xml_diff>

<commit_message>
Widen Tracking page and Excel ATS record to all FBS conferences
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -1442,7 +1442,7 @@
     <row r="5">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>UAB</t>
+          <t>North Texas</t>
         </is>
       </c>
       <c r="B5" s="35" t="n">
@@ -1455,7 +1455,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" s="35" t="n">
         <v>2</v>
@@ -1464,40 +1464,42 @@
     <row r="6">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>Army</t>
+          <t>UAB</t>
         </is>
       </c>
       <c r="B6" s="35" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="35" t="n">
         <v>1</v>
-      </c>
-      <c r="D6" s="35" t="n">
-        <v>0.5</v>
       </c>
       <c r="E6" s="35" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Army</t>
         </is>
       </c>
       <c r="B7" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="35" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="35" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D7" s="35" t="n">
+        <v>0.5</v>
+      </c>
       <c r="E7" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="35" t="n">
         <v>1</v>
@@ -1506,7 +1508,7 @@
     <row r="8">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="B8" s="35" t="n">
@@ -1546,18 +1548,20 @@
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>East Carolina</t>
+          <t>Tulsa</t>
         </is>
       </c>
       <c r="B10" s="35" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="35" t="n"/>
       <c r="E10" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="35" t="n">
         <v>2</v>
@@ -1566,7 +1570,7 @@
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>North Texas</t>
+          <t>East Carolina</t>
         </is>
       </c>
       <c r="B11" s="35" t="n">
@@ -2700,27 +2704,29 @@
     <row r="4">
       <c r="A4" s="35" t="inlineStr">
         <is>
-          <t>Liberty</t>
+          <t>New Mexico State</t>
         </is>
       </c>
       <c r="B4" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="35" t="n"/>
+      <c r="D4" s="35" t="n">
+        <v>1</v>
+      </c>
       <c r="E4" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="35" t="n">
         <v>3</v>
-      </c>
-      <c r="F4" s="35" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="35" t="inlineStr">
         <is>
-          <t>Delaware</t>
+          <t>Liberty</t>
         </is>
       </c>
       <c r="B5" s="35" t="n">
@@ -2731,16 +2737,16 @@
       </c>
       <c r="D5" s="35" t="n"/>
       <c r="E5" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" s="35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="35" t="inlineStr">
         <is>
-          <t>Florida International</t>
+          <t>Delaware</t>
         </is>
       </c>
       <c r="B6" s="35" t="n">
@@ -2760,18 +2766,16 @@
     <row r="7">
       <c r="A7" s="35" t="inlineStr">
         <is>
-          <t>Middle Tennessee</t>
+          <t>Florida International</t>
         </is>
       </c>
       <c r="B7" s="35" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="D7" s="35" t="n"/>
       <c r="E7" s="35" t="n">
         <v>2</v>
       </c>
@@ -2782,27 +2786,29 @@
     <row r="8">
       <c r="A8" s="35" t="inlineStr">
         <is>
-          <t>Kennesaw State</t>
+          <t>Middle Tennessee</t>
         </is>
       </c>
       <c r="B8" s="35" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="35" t="n"/>
       <c r="E8" s="35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>Missouri State</t>
+          <t>Kennesaw State</t>
         </is>
       </c>
       <c r="B9" s="35" t="n">
@@ -2822,7 +2828,7 @@
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>New Mexico State</t>
+          <t>Missouri State</t>
         </is>
       </c>
       <c r="B10" s="35" t="n">
@@ -2869,14 +2875,16 @@
         <v>0</v>
       </c>
       <c r="C12" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="35" t="n"/>
       <c r="E12" s="35" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" ht="26.5" customHeight="1">
@@ -4800,7 +4808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4929,7 +4937,7 @@
         <v>5.2</v>
       </c>
       <c r="F2" t="n">
-        <v>-3</v>
+        <v>-3.2</v>
       </c>
       <c r="G2" s="6">
         <f>F2-E2</f>
@@ -4943,7 +4951,7 @@
         <v>55.1</v>
       </c>
       <c r="J2" t="n">
-        <v>45.8</v>
+        <v>45.5</v>
       </c>
       <c r="K2" s="6">
         <f>I2-J2</f>
@@ -4987,7 +4995,7 @@
         <v>-30.3</v>
       </c>
       <c r="F3" t="n">
-        <v>-18.2</v>
+        <v>-17.2</v>
       </c>
       <c r="G3" s="6">
         <f>F3-E3</f>
@@ -5001,7 +5009,7 @@
         <v>46.7</v>
       </c>
       <c r="J3" t="n">
-        <v>45.5</v>
+        <v>44.5</v>
       </c>
       <c r="K3" s="6">
         <f>I3-J3</f>
@@ -5043,7 +5051,7 @@
         <v>-5.3</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.5</v>
+        <v>-2.8</v>
       </c>
       <c r="G4" s="6">
         <f>F4-E4</f>
@@ -5113,7 +5121,7 @@
         <v>43.7</v>
       </c>
       <c r="J5" t="n">
-        <v>48.5</v>
+        <v>47.8</v>
       </c>
       <c r="K5" s="6">
         <f>I5-J5</f>
@@ -5174,7 +5182,7 @@
         <v>48.5</v>
       </c>
       <c r="J6" t="n">
-        <v>51.5</v>
+        <v>50.5</v>
       </c>
       <c r="K6" s="6">
         <f>I6-J6</f>
@@ -15832,6 +15840,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
   </cols>
@@ -15862,6 +15871,11 @@
           <t>Week 4</t>
         </is>
       </c>
+      <c r="F1" s="33" t="inlineStr">
+        <is>
+          <t>Week 5</t>
+        </is>
+      </c>
       <c r="V1" s="34" t="inlineStr">
         <is>
           <t>Matchup Spread Calculator</t>
@@ -15886,6 +15900,9 @@
       <c r="E2" s="35" t="n">
         <v>94.90000000000001</v>
       </c>
+      <c r="F2" s="35" t="n">
+        <v>94.59999999999999</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="35" t="inlineStr">
@@ -15905,6 +15922,9 @@
       <c r="E3" s="35" t="n">
         <v>94</v>
       </c>
+      <c r="F3" s="35" t="n">
+        <v>94</v>
+      </c>
       <c r="V3" s="35" t="inlineStr">
         <is>
           <t>Home Team</t>
@@ -15934,6 +15954,9 @@
       <c r="E4" s="35" t="n">
         <v>90.40000000000001</v>
       </c>
+      <c r="F4" s="35" t="n">
+        <v>90.40000000000001</v>
+      </c>
       <c r="V4" s="35" t="inlineStr">
         <is>
           <t>Away Team</t>
@@ -15963,6 +15986,9 @@
       <c r="E5" s="35" t="n">
         <v>89.40000000000001</v>
       </c>
+      <c r="F5" s="35" t="n">
+        <v>89.40000000000001</v>
+      </c>
       <c r="V5" s="35" t="inlineStr">
         <is>
           <t>Neutral Site? (Y/N)</t>
@@ -15992,6 +16018,9 @@
       <c r="E6" s="35" t="n">
         <v>89</v>
       </c>
+      <c r="F6" s="35" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="35" t="inlineStr">
@@ -16011,6 +16040,9 @@
       <c r="E7" s="35" t="n">
         <v>88</v>
       </c>
+      <c r="F7" s="35" t="n">
+        <v>88</v>
+      </c>
       <c r="V7" s="35" t="inlineStr">
         <is>
           <t>HFA (model constant)</t>
@@ -16038,53 +16070,62 @@
       <c r="E8" s="35" t="n">
         <v>85.59999999999999</v>
       </c>
+      <c r="F8" s="35" t="n">
+        <v>85.59999999999999</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>Texas Tech</t>
+          <t>Utah</t>
         </is>
       </c>
       <c r="B9" s="35" t="n">
-        <v>87.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="C9" s="35" t="n">
-        <v>85.09999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="D9" s="35" t="n">
-        <v>84.7</v>
+        <v>84.2</v>
       </c>
       <c r="E9" s="35" t="n">
         <v>84.3</v>
       </c>
+      <c r="F9" s="35" t="n">
+        <v>84.3</v>
+      </c>
       <c r="V9" s="36" t="inlineStr">
         <is>
           <t>Predicted Spread (Home)</t>
         </is>
       </c>
       <c r="W9" s="36">
-        <f>IF(OR(W3="",W4=""),"",INDEX($E$2:$E$139,MATCH(W4,$A$2:$A$139,0))-INDEX($E$2:$E$139,MATCH(W3,$A$2:$A$139,0))-IF(UPPER(W5)="Y",0,W7))</f>
+        <f>IF(OR(W3="",W4=""),"",INDEX($F$2:$F$139,MATCH(W4,$A$2:$A$139,0))-INDEX($F$2:$F$139,MATCH(W3,$A$2:$A$139,0))-IF(UPPER(W5)="Y",0,W7))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Texas Tech</t>
         </is>
       </c>
       <c r="B10" s="35" t="n">
-        <v>81.59999999999999</v>
+        <v>87.3</v>
       </c>
       <c r="C10" s="35" t="n">
-        <v>83.5</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="D10" s="35" t="n">
-        <v>84.2</v>
+        <v>84.7</v>
       </c>
       <c r="E10" s="35" t="n">
         <v>84.3</v>
       </c>
+      <c r="F10" s="35" t="n">
+        <v>84.3</v>
+      </c>
       <c r="V10" s="37" t="inlineStr">
         <is>
           <t>(negative = home team favored, e.g. "Home -6.5")</t>
@@ -16109,6 +16150,9 @@
       <c r="E11" s="35" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="F11" s="35" t="n">
+        <v>83.90000000000001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
@@ -16128,6 +16172,9 @@
       <c r="E12" s="35" t="n">
         <v>82.5</v>
       </c>
+      <c r="F12" s="35" t="n">
+        <v>82.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
@@ -16147,6 +16194,9 @@
       <c r="E13" s="35" t="n">
         <v>81.3</v>
       </c>
+      <c r="F13" s="35" t="n">
+        <v>81.40000000000001</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="35" t="inlineStr">
@@ -16166,6 +16216,9 @@
       <c r="E14" s="35" t="n">
         <v>81.09999999999999</v>
       </c>
+      <c r="F14" s="35" t="n">
+        <v>81.09999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="35" t="inlineStr">
@@ -16185,6 +16238,9 @@
       <c r="E15" s="35" t="n">
         <v>80.2</v>
       </c>
+      <c r="F15" s="35" t="n">
+        <v>80.2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="35" t="inlineStr">
@@ -16204,6 +16260,9 @@
       <c r="E16" s="35" t="n">
         <v>79.7</v>
       </c>
+      <c r="F16" s="35" t="n">
+        <v>79.7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="35" t="inlineStr">
@@ -16223,6 +16282,9 @@
       <c r="E17" s="35" t="n">
         <v>79.5</v>
       </c>
+      <c r="F17" s="35" t="n">
+        <v>79.59999999999999</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
@@ -16242,6 +16304,9 @@
       <c r="E18" s="35" t="n">
         <v>79.5</v>
       </c>
+      <c r="F18" s="35" t="n">
+        <v>79.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="35" t="inlineStr">
@@ -16261,6 +16326,9 @@
       <c r="E19" s="35" t="n">
         <v>78.90000000000001</v>
       </c>
+      <c r="F19" s="35" t="n">
+        <v>78.90000000000001</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
@@ -16280,6 +16348,9 @@
       <c r="E20" s="35" t="n">
         <v>78.2</v>
       </c>
+      <c r="F20" s="35" t="n">
+        <v>78.2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="35" t="inlineStr">
@@ -16299,6 +16370,9 @@
       <c r="E21" s="35" t="n">
         <v>78.09999999999999</v>
       </c>
+      <c r="F21" s="35" t="n">
+        <v>78.2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="35" t="inlineStr">
@@ -16318,6 +16392,9 @@
       <c r="E22" s="35" t="n">
         <v>77.7</v>
       </c>
+      <c r="F22" s="35" t="n">
+        <v>77.59999999999999</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="35" t="inlineStr">
@@ -16337,6 +16414,9 @@
       <c r="E23" s="35" t="n">
         <v>77.5</v>
       </c>
+      <c r="F23" s="35" t="n">
+        <v>77.5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="35" t="inlineStr">
@@ -16356,6 +16436,9 @@
       <c r="E24" s="35" t="n">
         <v>77.5</v>
       </c>
+      <c r="F24" s="35" t="n">
+        <v>77.5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="35" t="inlineStr">
@@ -16375,6 +16458,9 @@
       <c r="E25" s="35" t="n">
         <v>77.2</v>
       </c>
+      <c r="F25" s="35" t="n">
+        <v>77.2</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="35" t="inlineStr">
@@ -16394,6 +16480,9 @@
       <c r="E26" s="35" t="n">
         <v>77</v>
       </c>
+      <c r="F26" s="35" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="35" t="inlineStr">
@@ -16413,6 +16502,9 @@
       <c r="E27" s="35" t="n">
         <v>76.59999999999999</v>
       </c>
+      <c r="F27" s="35" t="n">
+        <v>76.7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="35" t="inlineStr">
@@ -16432,6 +16524,9 @@
       <c r="E28" s="35" t="n">
         <v>76.3</v>
       </c>
+      <c r="F28" s="35" t="n">
+        <v>76.3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="35" t="inlineStr">
@@ -16451,6 +16546,9 @@
       <c r="E29" s="35" t="n">
         <v>76.09999999999999</v>
       </c>
+      <c r="F29" s="35" t="n">
+        <v>76.2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="35" t="inlineStr">
@@ -16470,6 +16568,9 @@
       <c r="E30" s="35" t="n">
         <v>76</v>
       </c>
+      <c r="F30" s="35" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="35" t="inlineStr">
@@ -16489,6 +16590,9 @@
       <c r="E31" s="35" t="n">
         <v>75.3</v>
       </c>
+      <c r="F31" s="35" t="n">
+        <v>75.3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="35" t="inlineStr">
@@ -16508,6 +16612,9 @@
       <c r="E32" s="35" t="n">
         <v>74.40000000000001</v>
       </c>
+      <c r="F32" s="35" t="n">
+        <v>74.40000000000001</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="35" t="inlineStr">
@@ -16527,6 +16634,9 @@
       <c r="E33" s="35" t="n">
         <v>74.09999999999999</v>
       </c>
+      <c r="F33" s="35" t="n">
+        <v>74.09999999999999</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="35" t="inlineStr">
@@ -16546,6 +16656,9 @@
       <c r="E34" s="35" t="n">
         <v>73.2</v>
       </c>
+      <c r="F34" s="35" t="n">
+        <v>73.2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="35" t="inlineStr">
@@ -16565,6 +16678,9 @@
       <c r="E35" s="35" t="n">
         <v>72.90000000000001</v>
       </c>
+      <c r="F35" s="35" t="n">
+        <v>72.90000000000001</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="35" t="inlineStr">
@@ -16584,6 +16700,9 @@
       <c r="E36" s="35" t="n">
         <v>72.90000000000001</v>
       </c>
+      <c r="F36" s="35" t="n">
+        <v>72.90000000000001</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="35" t="inlineStr">
@@ -16603,6 +16722,9 @@
       <c r="E37" s="35" t="n">
         <v>72.8</v>
       </c>
+      <c r="F37" s="35" t="n">
+        <v>72.8</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="35" t="inlineStr">
@@ -16622,6 +16744,9 @@
       <c r="E38" s="35" t="n">
         <v>72.8</v>
       </c>
+      <c r="F38" s="35" t="n">
+        <v>72.8</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="35" t="inlineStr">
@@ -16641,6 +16766,9 @@
       <c r="E39" s="35" t="n">
         <v>72.7</v>
       </c>
+      <c r="F39" s="35" t="n">
+        <v>72.7</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="35" t="inlineStr">
@@ -16660,6 +16788,9 @@
       <c r="E40" s="35" t="n">
         <v>72.40000000000001</v>
       </c>
+      <c r="F40" s="35" t="n">
+        <v>72.40000000000001</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="35" t="inlineStr">
@@ -16679,6 +16810,9 @@
       <c r="E41" s="35" t="n">
         <v>72.2</v>
       </c>
+      <c r="F41" s="35" t="n">
+        <v>72.3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="35" t="inlineStr">
@@ -16698,6 +16832,9 @@
       <c r="E42" s="35" t="n">
         <v>71.90000000000001</v>
       </c>
+      <c r="F42" s="35" t="n">
+        <v>71.90000000000001</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="35" t="inlineStr">
@@ -16717,6 +16854,9 @@
       <c r="E43" s="35" t="n">
         <v>71.90000000000001</v>
       </c>
+      <c r="F43" s="35" t="n">
+        <v>71.90000000000001</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="35" t="inlineStr">
@@ -16736,6 +16876,9 @@
       <c r="E44" s="35" t="n">
         <v>71.7</v>
       </c>
+      <c r="F44" s="35" t="n">
+        <v>71.8</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="35" t="inlineStr">
@@ -16755,6 +16898,9 @@
       <c r="E45" s="35" t="n">
         <v>71.7</v>
       </c>
+      <c r="F45" s="35" t="n">
+        <v>71.7</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="35" t="inlineStr">
@@ -16774,6 +16920,9 @@
       <c r="E46" s="35" t="n">
         <v>71.40000000000001</v>
       </c>
+      <c r="F46" s="35" t="n">
+        <v>71.40000000000001</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="35" t="inlineStr">
@@ -16793,6 +16942,9 @@
       <c r="E47" s="35" t="n">
         <v>70.90000000000001</v>
       </c>
+      <c r="F47" s="35" t="n">
+        <v>70.90000000000001</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="35" t="inlineStr">
@@ -16812,6 +16964,9 @@
       <c r="E48" s="35" t="n">
         <v>70.7</v>
       </c>
+      <c r="F48" s="35" t="n">
+        <v>70.7</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="35" t="inlineStr">
@@ -16831,6 +16986,9 @@
       <c r="E49" s="35" t="n">
         <v>70.40000000000001</v>
       </c>
+      <c r="F49" s="35" t="n">
+        <v>70.2</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="35" t="inlineStr">
@@ -16850,6 +17008,9 @@
       <c r="E50" s="35" t="n">
         <v>70.2</v>
       </c>
+      <c r="F50" s="35" t="n">
+        <v>70.2</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="35" t="inlineStr">
@@ -16869,6 +17030,9 @@
       <c r="E51" s="35" t="n">
         <v>69.40000000000001</v>
       </c>
+      <c r="F51" s="35" t="n">
+        <v>69.40000000000001</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="35" t="inlineStr">
@@ -16888,6 +17052,9 @@
       <c r="E52" s="35" t="n">
         <v>68.8</v>
       </c>
+      <c r="F52" s="35" t="n">
+        <v>68.8</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="35" t="inlineStr">
@@ -16907,6 +17074,9 @@
       <c r="E53" s="35" t="n">
         <v>68.59999999999999</v>
       </c>
+      <c r="F53" s="35" t="n">
+        <v>68.59999999999999</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="35" t="inlineStr">
@@ -16926,6 +17096,9 @@
       <c r="E54" s="35" t="n">
         <v>67.8</v>
       </c>
+      <c r="F54" s="35" t="n">
+        <v>67.8</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="35" t="inlineStr">
@@ -16945,6 +17118,9 @@
       <c r="E55" s="35" t="n">
         <v>67.7</v>
       </c>
+      <c r="F55" s="35" t="n">
+        <v>67.7</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="35" t="inlineStr">
@@ -16964,6 +17140,9 @@
       <c r="E56" s="35" t="n">
         <v>67.7</v>
       </c>
+      <c r="F56" s="35" t="n">
+        <v>67.7</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="35" t="inlineStr">
@@ -16983,6 +17162,9 @@
       <c r="E57" s="35" t="n">
         <v>67.59999999999999</v>
       </c>
+      <c r="F57" s="35" t="n">
+        <v>67.5</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="35" t="inlineStr">
@@ -17002,6 +17184,9 @@
       <c r="E58" s="35" t="n">
         <v>67.3</v>
       </c>
+      <c r="F58" s="35" t="n">
+        <v>67.2</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="35" t="inlineStr">
@@ -17021,6 +17206,9 @@
       <c r="E59" s="35" t="n">
         <v>67.2</v>
       </c>
+      <c r="F59" s="35" t="n">
+        <v>67.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="35" t="inlineStr">
@@ -17040,118 +17228,139 @@
       <c r="E60" s="35" t="n">
         <v>67.09999999999999</v>
       </c>
+      <c r="F60" s="35" t="n">
+        <v>67.09999999999999</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="35" t="inlineStr">
         <is>
-          <t>North Texas</t>
+          <t>Michigan State</t>
         </is>
       </c>
       <c r="B61" s="35" t="n">
-        <v>63.9</v>
+        <v>66</v>
       </c>
       <c r="C61" s="35" t="n">
-        <v>67.40000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="D61" s="35" t="n">
-        <v>64.8</v>
+        <v>67.5</v>
       </c>
       <c r="E61" s="35" t="n">
-        <v>66.90000000000001</v>
+        <v>66.40000000000001</v>
+      </c>
+      <c r="F61" s="35" t="n">
+        <v>66.40000000000001</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="35" t="inlineStr">
         <is>
-          <t>Michigan State</t>
+          <t>Toledo</t>
         </is>
       </c>
       <c r="B62" s="35" t="n">
-        <v>66</v>
+        <v>62.1</v>
       </c>
       <c r="C62" s="35" t="n">
-        <v>66.90000000000001</v>
+        <v>65</v>
       </c>
       <c r="D62" s="35" t="n">
-        <v>67.5</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="E62" s="35" t="n">
-        <v>66.40000000000001</v>
+        <v>66.3</v>
+      </c>
+      <c r="F62" s="35" t="n">
+        <v>66.3</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="35" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Old Dominion</t>
         </is>
       </c>
       <c r="B63" s="35" t="n">
-        <v>62.1</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C63" s="35" t="n">
-        <v>65</v>
+        <v>69.5</v>
       </c>
       <c r="D63" s="35" t="n">
-        <v>64.09999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="E63" s="35" t="n">
         <v>66.3</v>
       </c>
+      <c r="F63" s="35" t="n">
+        <v>66.3</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="35" t="inlineStr">
         <is>
-          <t>Old Dominion</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="B64" s="35" t="n">
-        <v>72.59999999999999</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="C64" s="35" t="n">
-        <v>69.5</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="D64" s="35" t="n">
-        <v>68.5</v>
+        <v>64</v>
       </c>
       <c r="E64" s="35" t="n">
-        <v>66.3</v>
+        <v>65.90000000000001</v>
+      </c>
+      <c r="F64" s="35" t="n">
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="35" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="B65" s="35" t="n">
-        <v>66.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="C65" s="35" t="n">
-        <v>65.09999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="D65" s="35" t="n">
-        <v>64</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E65" s="35" t="n">
-        <v>66</v>
+        <v>65.8</v>
+      </c>
+      <c r="F65" s="35" t="n">
+        <v>65.8</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="35" t="inlineStr">
         <is>
-          <t>Georgia Tech</t>
+          <t>North Texas</t>
         </is>
       </c>
       <c r="B66" s="35" t="n">
-        <v>67.7</v>
+        <v>63.9</v>
       </c>
       <c r="C66" s="35" t="n">
-        <v>66.7</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="D66" s="35" t="n">
-        <v>67.40000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="E66" s="35" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="F66" s="35" t="n">
         <v>65.8</v>
       </c>
     </row>
@@ -17173,6 +17382,9 @@
       <c r="E67" s="35" t="n">
         <v>65.7</v>
       </c>
+      <c r="F67" s="35" t="n">
+        <v>65.7</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="35" t="inlineStr">
@@ -17192,6 +17404,9 @@
       <c r="E68" s="35" t="n">
         <v>65.40000000000001</v>
       </c>
+      <c r="F68" s="35" t="n">
+        <v>65.40000000000001</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="35" t="inlineStr">
@@ -17211,6 +17426,9 @@
       <c r="E69" s="35" t="n">
         <v>65.09999999999999</v>
       </c>
+      <c r="F69" s="35" t="n">
+        <v>65.09999999999999</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="35" t="inlineStr">
@@ -17230,6 +17448,9 @@
       <c r="E70" s="35" t="n">
         <v>65.09999999999999</v>
       </c>
+      <c r="F70" s="35" t="n">
+        <v>65.09999999999999</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="35" t="inlineStr">
@@ -17249,44 +17470,53 @@
       <c r="E71" s="35" t="n">
         <v>64.7</v>
       </c>
+      <c r="F71" s="35" t="n">
+        <v>64.7</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="35" t="inlineStr">
         <is>
-          <t>Rutgers</t>
+          <t>UTSA</t>
         </is>
       </c>
       <c r="B72" s="35" t="n">
-        <v>61.1</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="C72" s="35" t="n">
-        <v>62</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D72" s="35" t="n">
-        <v>62.1</v>
+        <v>65.2</v>
       </c>
       <c r="E72" s="35" t="n">
         <v>64.7</v>
       </c>
+      <c r="F72" s="35" t="n">
+        <v>64.7</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="35" t="inlineStr">
         <is>
-          <t>UTSA</t>
+          <t>Rutgers</t>
         </is>
       </c>
       <c r="B73" s="35" t="n">
-        <v>66.59999999999999</v>
+        <v>61.1</v>
       </c>
       <c r="C73" s="35" t="n">
-        <v>65.59999999999999</v>
+        <v>62</v>
       </c>
       <c r="D73" s="35" t="n">
-        <v>65.2</v>
+        <v>62.1</v>
       </c>
       <c r="E73" s="35" t="n">
         <v>64.7</v>
       </c>
+      <c r="F73" s="35" t="n">
+        <v>64.3</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="35" t="inlineStr">
@@ -17306,6 +17536,9 @@
       <c r="E74" s="35" t="n">
         <v>64.2</v>
       </c>
+      <c r="F74" s="35" t="n">
+        <v>64.2</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="35" t="inlineStr">
@@ -17325,6 +17558,9 @@
       <c r="E75" s="35" t="n">
         <v>63.9</v>
       </c>
+      <c r="F75" s="35" t="n">
+        <v>63.9</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="35" t="inlineStr">
@@ -17344,6 +17580,9 @@
       <c r="E76" s="35" t="n">
         <v>62.3</v>
       </c>
+      <c r="F76" s="35" t="n">
+        <v>62.3</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="35" t="inlineStr">
@@ -17363,6 +17602,9 @@
       <c r="E77" s="35" t="n">
         <v>62.2</v>
       </c>
+      <c r="F77" s="35" t="n">
+        <v>62.2</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="35" t="inlineStr">
@@ -17382,6 +17624,9 @@
       <c r="E78" s="35" t="n">
         <v>61.7</v>
       </c>
+      <c r="F78" s="35" t="n">
+        <v>61.7</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="35" t="inlineStr">
@@ -17401,6 +17646,9 @@
       <c r="E79" s="35" t="n">
         <v>61.5</v>
       </c>
+      <c r="F79" s="35" t="n">
+        <v>61.5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="35" t="inlineStr">
@@ -17420,6 +17668,9 @@
       <c r="E80" s="35" t="n">
         <v>61.4</v>
       </c>
+      <c r="F80" s="35" t="n">
+        <v>61.4</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="35" t="inlineStr">
@@ -17439,44 +17690,53 @@
       <c r="E81" s="35" t="n">
         <v>61.4</v>
       </c>
+      <c r="F81" s="35" t="n">
+        <v>61.4</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="35" t="inlineStr">
         <is>
-          <t>UNLV</t>
+          <t>West Virginia</t>
         </is>
       </c>
       <c r="B82" s="35" t="n">
-        <v>62.6</v>
+        <v>58.2</v>
       </c>
       <c r="C82" s="35" t="n">
-        <v>59</v>
+        <v>60.5</v>
       </c>
       <c r="D82" s="35" t="n">
-        <v>59</v>
+        <v>63.4</v>
       </c>
       <c r="E82" s="35" t="n">
         <v>60.9</v>
       </c>
+      <c r="F82" s="35" t="n">
+        <v>60.9</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="35" t="inlineStr">
         <is>
-          <t>West Virginia</t>
+          <t>UNLV</t>
         </is>
       </c>
       <c r="B83" s="35" t="n">
-        <v>58.2</v>
+        <v>62.6</v>
       </c>
       <c r="C83" s="35" t="n">
-        <v>60.5</v>
+        <v>59</v>
       </c>
       <c r="D83" s="35" t="n">
-        <v>63.4</v>
+        <v>59</v>
       </c>
       <c r="E83" s="35" t="n">
         <v>60.9</v>
       </c>
+      <c r="F83" s="35" t="n">
+        <v>60.9</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="35" t="inlineStr">
@@ -17496,6 +17756,9 @@
       <c r="E84" s="35" t="n">
         <v>60.2</v>
       </c>
+      <c r="F84" s="35" t="n">
+        <v>60.2</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="35" t="inlineStr">
@@ -17515,6 +17778,9 @@
       <c r="E85" s="35" t="n">
         <v>60.1</v>
       </c>
+      <c r="F85" s="35" t="n">
+        <v>60.1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="35" t="inlineStr">
@@ -17534,6 +17800,9 @@
       <c r="E86" s="35" t="n">
         <v>59.9</v>
       </c>
+      <c r="F86" s="35" t="n">
+        <v>59.9</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="35" t="inlineStr">
@@ -17553,62 +17822,74 @@
       <c r="E87" s="35" t="n">
         <v>59.7</v>
       </c>
+      <c r="F87" s="35" t="n">
+        <v>59.7</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="35" t="inlineStr">
         <is>
-          <t>Ohio</t>
+          <t>Oklahoma State</t>
         </is>
       </c>
       <c r="B88" s="35" t="n">
-        <v>58.8</v>
+        <v>50.2</v>
       </c>
       <c r="C88" s="35" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D88" s="35" t="n">
-        <v>58.2</v>
+        <v>57.8</v>
       </c>
       <c r="E88" s="35" t="n">
         <v>59.6</v>
       </c>
+      <c r="F88" s="35" t="n">
+        <v>59.6</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="35" t="inlineStr">
         <is>
-          <t>Oklahoma State</t>
+          <t>California</t>
         </is>
       </c>
       <c r="B89" s="35" t="n">
-        <v>50.2</v>
+        <v>60.4</v>
       </c>
       <c r="C89" s="35" t="n">
-        <v>54</v>
+        <v>59.8</v>
       </c>
       <c r="D89" s="35" t="n">
-        <v>57.8</v>
+        <v>60.5</v>
       </c>
       <c r="E89" s="35" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="F89" s="35" t="n">
         <v>59.6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="35" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>Ohio</t>
         </is>
       </c>
       <c r="B90" s="35" t="n">
-        <v>60.4</v>
+        <v>58.8</v>
       </c>
       <c r="C90" s="35" t="n">
-        <v>59.8</v>
+        <v>59</v>
       </c>
       <c r="D90" s="35" t="n">
-        <v>60.6</v>
+        <v>58.2</v>
       </c>
       <c r="E90" s="35" t="n">
-        <v>59.5</v>
+        <v>59.6</v>
+      </c>
+      <c r="F90" s="35" t="n">
+        <v>59.4</v>
       </c>
     </row>
     <row r="91">
@@ -17629,6 +17910,9 @@
       <c r="E91" s="35" t="n">
         <v>59.2</v>
       </c>
+      <c r="F91" s="35" t="n">
+        <v>59.1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="35" t="inlineStr">
@@ -17648,6 +17932,9 @@
       <c r="E92" s="35" t="n">
         <v>58.7</v>
       </c>
+      <c r="F92" s="35" t="n">
+        <v>58.7</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="35" t="inlineStr">
@@ -17667,6 +17954,9 @@
       <c r="E93" s="35" t="n">
         <v>58.5</v>
       </c>
+      <c r="F93" s="35" t="n">
+        <v>58.5</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="35" t="inlineStr">
@@ -17686,43 +17976,52 @@
       <c r="E94" s="35" t="n">
         <v>58</v>
       </c>
+      <c r="F94" s="35" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="35" t="inlineStr">
         <is>
-          <t>Western Kentucky</t>
+          <t>Louisiana</t>
         </is>
       </c>
       <c r="B95" s="35" t="n">
-        <v>56.1</v>
+        <v>54.3</v>
       </c>
       <c r="C95" s="35" t="n">
-        <v>53.9</v>
+        <v>54.8</v>
       </c>
       <c r="D95" s="35" t="n">
-        <v>54.4</v>
+        <v>55.3</v>
       </c>
       <c r="E95" s="35" t="n">
-        <v>57.1</v>
+        <v>57</v>
+      </c>
+      <c r="F95" s="35" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="35" t="inlineStr">
         <is>
-          <t>Louisiana</t>
+          <t>Tulsa</t>
         </is>
       </c>
       <c r="B96" s="35" t="n">
-        <v>54.3</v>
+        <v>55.3</v>
       </c>
       <c r="C96" s="35" t="n">
-        <v>54.8</v>
+        <v>55.4</v>
       </c>
       <c r="D96" s="35" t="n">
-        <v>55.3</v>
+        <v>58.2</v>
       </c>
       <c r="E96" s="35" t="n">
-        <v>57</v>
+        <v>55.9</v>
+      </c>
+      <c r="F96" s="35" t="n">
+        <v>56.9</v>
       </c>
     </row>
     <row r="97">
@@ -17743,6 +18042,9 @@
       <c r="E97" s="35" t="n">
         <v>56.8</v>
       </c>
+      <c r="F97" s="35" t="n">
+        <v>56.8</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="35" t="inlineStr">
@@ -17762,6 +18064,9 @@
       <c r="E98" s="35" t="n">
         <v>56.7</v>
       </c>
+      <c r="F98" s="35" t="n">
+        <v>56.7</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="35" t="inlineStr">
@@ -17781,6 +18086,9 @@
       <c r="E99" s="35" t="n">
         <v>56.6</v>
       </c>
+      <c r="F99" s="35" t="n">
+        <v>56.6</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="35" t="inlineStr">
@@ -17800,6 +18108,9 @@
       <c r="E100" s="35" t="n">
         <v>56.5</v>
       </c>
+      <c r="F100" s="35" t="n">
+        <v>56.5</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="35" t="inlineStr">
@@ -17819,6 +18130,9 @@
       <c r="E101" s="35" t="n">
         <v>56</v>
       </c>
+      <c r="F101" s="35" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="35" t="inlineStr">
@@ -17838,6 +18152,9 @@
       <c r="E102" s="35" t="n">
         <v>55.9</v>
       </c>
+      <c r="F102" s="35" t="n">
+        <v>55.9</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="35" t="inlineStr">
@@ -17857,6 +18174,9 @@
       <c r="E103" s="35" t="n">
         <v>55.8</v>
       </c>
+      <c r="F103" s="35" t="n">
+        <v>55.8</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="35" t="inlineStr">
@@ -17876,6 +18196,9 @@
       <c r="E104" s="35" t="n">
         <v>55.6</v>
       </c>
+      <c r="F104" s="35" t="n">
+        <v>55.3</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="35" t="inlineStr">
@@ -17895,81 +18218,96 @@
       <c r="E105" s="35" t="n">
         <v>55.2</v>
       </c>
+      <c r="F105" s="35" t="n">
+        <v>55.3</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="35" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>UConn</t>
         </is>
       </c>
       <c r="B106" s="35" t="n">
-        <v>55.3</v>
+        <v>57.3</v>
       </c>
       <c r="C106" s="35" t="n">
-        <v>54.8</v>
+        <v>54.7</v>
       </c>
       <c r="D106" s="35" t="n">
-        <v>57.6</v>
+        <v>57.3</v>
       </c>
       <c r="E106" s="35" t="n">
-        <v>55.2</v>
+        <v>54.4</v>
+      </c>
+      <c r="F106" s="35" t="n">
+        <v>54.4</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="35" t="inlineStr">
         <is>
-          <t>UConn</t>
+          <t>Colorado State</t>
         </is>
       </c>
       <c r="B107" s="35" t="n">
-        <v>57.3</v>
+        <v>51</v>
       </c>
       <c r="C107" s="35" t="n">
-        <v>54.7</v>
+        <v>53.6</v>
       </c>
       <c r="D107" s="35" t="n">
-        <v>57.3</v>
+        <v>53.8</v>
       </c>
       <c r="E107" s="35" t="n">
-        <v>54.4</v>
+        <v>54.3</v>
+      </c>
+      <c r="F107" s="35" t="n">
+        <v>54.3</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="35" t="inlineStr">
         <is>
-          <t>Colorado State</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="B108" s="35" t="n">
-        <v>51</v>
+        <v>53.1</v>
       </c>
       <c r="C108" s="35" t="n">
-        <v>53.6</v>
+        <v>53.7</v>
       </c>
       <c r="D108" s="35" t="n">
-        <v>53.8</v>
+        <v>54.6</v>
       </c>
       <c r="E108" s="35" t="n">
-        <v>54.3</v>
+        <v>54.2</v>
+      </c>
+      <c r="F108" s="35" t="n">
+        <v>54.2</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="35" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Western Kentucky</t>
         </is>
       </c>
       <c r="B109" s="35" t="n">
-        <v>53.1</v>
+        <v>56.1</v>
       </c>
       <c r="C109" s="35" t="n">
-        <v>53.7</v>
+        <v>53.9</v>
       </c>
       <c r="D109" s="35" t="n">
-        <v>54.6</v>
+        <v>54.4</v>
       </c>
       <c r="E109" s="35" t="n">
-        <v>54.2</v>
+        <v>57.1</v>
+      </c>
+      <c r="F109" s="35" t="n">
+        <v>53.9</v>
       </c>
     </row>
     <row r="110">
@@ -17990,6 +18328,9 @@
       <c r="E110" s="35" t="n">
         <v>53.9</v>
       </c>
+      <c r="F110" s="35" t="n">
+        <v>53.5</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="35" t="inlineStr">
@@ -18009,6 +18350,9 @@
       <c r="E111" s="35" t="n">
         <v>53.3</v>
       </c>
+      <c r="F111" s="35" t="n">
+        <v>53.3</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="35" t="inlineStr">
@@ -18028,6 +18372,9 @@
       <c r="E112" s="35" t="n">
         <v>53.2</v>
       </c>
+      <c r="F112" s="35" t="n">
+        <v>53.2</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="35" t="inlineStr">
@@ -18047,6 +18394,9 @@
       <c r="E113" s="35" t="n">
         <v>53.1</v>
       </c>
+      <c r="F113" s="35" t="n">
+        <v>53.1</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="35" t="inlineStr">
@@ -18066,6 +18416,9 @@
       <c r="E114" s="35" t="n">
         <v>52.5</v>
       </c>
+      <c r="F114" s="35" t="n">
+        <v>52.5</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="35" t="inlineStr">
@@ -18085,6 +18438,9 @@
       <c r="E115" s="35" t="n">
         <v>52.3</v>
       </c>
+      <c r="F115" s="35" t="n">
+        <v>52.3</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="35" t="inlineStr">
@@ -18104,6 +18460,9 @@
       <c r="E116" s="35" t="n">
         <v>52.1</v>
       </c>
+      <c r="F116" s="35" t="n">
+        <v>52.1</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="35" t="inlineStr">
@@ -18123,138 +18482,162 @@
       <c r="E117" s="35" t="n">
         <v>51.9</v>
       </c>
+      <c r="F117" s="35" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="35" t="inlineStr">
         <is>
-          <t>Coastal Carolina</t>
+          <t>New Mexico State</t>
         </is>
       </c>
       <c r="B118" s="35" t="n">
-        <v>51</v>
+        <v>50.6</v>
       </c>
       <c r="C118" s="35" t="n">
-        <v>54.1</v>
+        <v>49.5</v>
       </c>
       <c r="D118" s="35" t="n">
-        <v>53</v>
+        <v>49.5</v>
       </c>
       <c r="E118" s="35" t="n">
-        <v>51.7</v>
+        <v>49.1</v>
+      </c>
+      <c r="F118" s="35" t="n">
+        <v>51.9</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="35" t="inlineStr">
         <is>
-          <t>Marshall</t>
+          <t>Coastal Carolina</t>
         </is>
       </c>
       <c r="B119" s="35" t="n">
-        <v>52.1</v>
+        <v>51</v>
       </c>
       <c r="C119" s="35" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="D119" s="35" t="n">
+        <v>53</v>
+      </c>
+      <c r="E119" s="35" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="F119" s="35" t="n">
         <v>51.8</v>
-      </c>
-      <c r="D119" s="35" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="E119" s="35" t="n">
-        <v>51.4</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="35" t="inlineStr">
         <is>
-          <t>Southern Miss</t>
+          <t>Marshall</t>
         </is>
       </c>
       <c r="B120" s="35" t="n">
-        <v>54.4</v>
+        <v>52.1</v>
       </c>
       <c r="C120" s="35" t="n">
-        <v>52.7</v>
+        <v>51.8</v>
       </c>
       <c r="D120" s="35" t="n">
-        <v>50.1</v>
+        <v>52.5</v>
       </c>
       <c r="E120" s="35" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="F120" s="35" t="n">
         <v>51.3</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="35" t="inlineStr">
         <is>
-          <t>Georgia State</t>
+          <t>Southern Miss</t>
         </is>
       </c>
       <c r="B121" s="35" t="n">
-        <v>47.4</v>
+        <v>54.4</v>
       </c>
       <c r="C121" s="35" t="n">
-        <v>49.7</v>
+        <v>52.7</v>
       </c>
       <c r="D121" s="35" t="n">
-        <v>49.6</v>
+        <v>50.1</v>
       </c>
       <c r="E121" s="35" t="n">
-        <v>51.2</v>
+        <v>51.3</v>
+      </c>
+      <c r="F121" s="35" t="n">
+        <v>51.3</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="35" t="inlineStr">
         <is>
-          <t>San José State</t>
+          <t>Georgia State</t>
         </is>
       </c>
       <c r="B122" s="35" t="n">
-        <v>51.7</v>
+        <v>47.4</v>
       </c>
       <c r="C122" s="35" t="n">
-        <v>51.6</v>
+        <v>49.7</v>
       </c>
       <c r="D122" s="35" t="n">
-        <v>50.5</v>
+        <v>49.6</v>
       </c>
       <c r="E122" s="35" t="n">
-        <v>50.4</v>
+        <v>51.2</v>
+      </c>
+      <c r="F122" s="35" t="n">
+        <v>51.2</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="35" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>San José State</t>
         </is>
       </c>
       <c r="B123" s="35" t="n">
-        <v>48.6</v>
+        <v>51.7</v>
       </c>
       <c r="C123" s="35" t="n">
-        <v>48.8</v>
+        <v>51.6</v>
       </c>
       <c r="D123" s="35" t="n">
-        <v>47.5</v>
+        <v>50.5</v>
       </c>
       <c r="E123" s="35" t="n">
-        <v>49.6</v>
+        <v>50.4</v>
+      </c>
+      <c r="F123" s="35" t="n">
+        <v>50.4</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="35" t="inlineStr">
         <is>
-          <t>New Mexico State</t>
+          <t>Wyoming</t>
         </is>
       </c>
       <c r="B124" s="35" t="n">
-        <v>50.6</v>
+        <v>48.6</v>
       </c>
       <c r="C124" s="35" t="n">
-        <v>49.5</v>
+        <v>48.8</v>
       </c>
       <c r="D124" s="35" t="n">
-        <v>49.5</v>
+        <v>47.5</v>
       </c>
       <c r="E124" s="35" t="n">
-        <v>49.1</v>
+        <v>49.6</v>
+      </c>
+      <c r="F124" s="35" t="n">
+        <v>49.6</v>
       </c>
     </row>
     <row r="125">
@@ -18275,6 +18658,9 @@
       <c r="E125" s="35" t="n">
         <v>48.8</v>
       </c>
+      <c r="F125" s="35" t="n">
+        <v>48.6</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="35" t="inlineStr">
@@ -18294,42 +18680,51 @@
       <c r="E126" s="35" t="n">
         <v>48.5</v>
       </c>
+      <c r="F126" s="35" t="n">
+        <v>48.5</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="35" t="inlineStr">
         <is>
-          <t>Akron</t>
+          <t>Rice</t>
         </is>
       </c>
       <c r="B127" s="35" t="n">
-        <v>48.5</v>
+        <v>46.8</v>
       </c>
       <c r="C127" s="35" t="n">
-        <v>51.5</v>
+        <v>45.8</v>
       </c>
       <c r="D127" s="35" t="n">
-        <v>49.3</v>
+        <v>47.4</v>
       </c>
       <c r="E127" s="35" t="n">
-        <v>47.4</v>
+        <v>47.3</v>
+      </c>
+      <c r="F127" s="35" t="n">
+        <v>47.3</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="35" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>Akron</t>
         </is>
       </c>
       <c r="B128" s="35" t="n">
-        <v>46.8</v>
+        <v>48.5</v>
       </c>
       <c r="C128" s="35" t="n">
-        <v>45.8</v>
+        <v>51.5</v>
       </c>
       <c r="D128" s="35" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="E128" s="35" t="n">
         <v>47.4</v>
       </c>
-      <c r="E128" s="35" t="n">
+      <c r="F128" s="35" t="n">
         <v>47.3</v>
       </c>
     </row>
@@ -18351,80 +18746,95 @@
       <c r="E129" s="35" t="n">
         <v>46.8</v>
       </c>
+      <c r="F129" s="35" t="n">
+        <v>46.4</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="35" t="inlineStr">
         <is>
-          <t>Sam Houston</t>
+          <t>Kent State</t>
         </is>
       </c>
       <c r="B130" s="35" t="n">
-        <v>41.1</v>
+        <v>45.6</v>
       </c>
       <c r="C130" s="35" t="n">
-        <v>41.7</v>
+        <v>47.5</v>
       </c>
       <c r="D130" s="35" t="n">
-        <v>47</v>
+        <v>45.5</v>
       </c>
       <c r="E130" s="35" t="n">
-        <v>46.7</v>
+        <v>46.3</v>
+      </c>
+      <c r="F130" s="35" t="n">
+        <v>46.3</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="35" t="inlineStr">
         <is>
-          <t>Kent State</t>
+          <t>Sam Houston</t>
         </is>
       </c>
       <c r="B131" s="35" t="n">
-        <v>45.6</v>
+        <v>41.1</v>
       </c>
       <c r="C131" s="35" t="n">
-        <v>47.5</v>
+        <v>41.1</v>
       </c>
       <c r="D131" s="35" t="n">
-        <v>45.5</v>
+        <v>46.5</v>
       </c>
       <c r="E131" s="35" t="n">
-        <v>46.3</v>
+        <v>46.2</v>
+      </c>
+      <c r="F131" s="35" t="n">
+        <v>46.2</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="35" t="inlineStr">
         <is>
-          <t>Massachusetts</t>
+          <t>Bowling Green</t>
         </is>
       </c>
       <c r="B132" s="35" t="n">
-        <v>37.6</v>
+        <v>48.8</v>
       </c>
       <c r="C132" s="35" t="n">
-        <v>41.2</v>
+        <v>46.2</v>
       </c>
       <c r="D132" s="35" t="n">
-        <v>41.1</v>
+        <v>43.7</v>
       </c>
       <c r="E132" s="35" t="n">
-        <v>45.6</v>
+        <v>45.4</v>
+      </c>
+      <c r="F132" s="35" t="n">
+        <v>45.4</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="35" t="inlineStr">
         <is>
-          <t>Bowling Green</t>
+          <t>Massachusetts</t>
         </is>
       </c>
       <c r="B133" s="35" t="n">
-        <v>48.8</v>
+        <v>37.6</v>
       </c>
       <c r="C133" s="35" t="n">
-        <v>46.2</v>
+        <v>41.2</v>
       </c>
       <c r="D133" s="35" t="n">
-        <v>43.7</v>
+        <v>41.1</v>
       </c>
       <c r="E133" s="35" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="F133" s="35" t="n">
         <v>45.4</v>
       </c>
     </row>
@@ -18446,6 +18856,9 @@
       <c r="E134" s="35" t="n">
         <v>43.3</v>
       </c>
+      <c r="F134" s="35" t="n">
+        <v>43.3</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="35" t="inlineStr">
@@ -18465,6 +18878,9 @@
       <c r="E135" s="35" t="n">
         <v>42.6</v>
       </c>
+      <c r="F135" s="35" t="n">
+        <v>42.6</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="35" t="inlineStr">
@@ -18484,6 +18900,9 @@
       <c r="E136" s="35" t="n">
         <v>42.3</v>
       </c>
+      <c r="F136" s="35" t="n">
+        <v>42.3</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="35" t="inlineStr">
@@ -18503,6 +18922,9 @@
       <c r="E137" s="35" t="n">
         <v>41.2</v>
       </c>
+      <c r="F137" s="35" t="n">
+        <v>41.2</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="35" t="inlineStr">
@@ -18522,6 +18944,9 @@
       <c r="E138" s="35" t="n">
         <v>40.7</v>
       </c>
+      <c r="F138" s="35" t="n">
+        <v>40.7</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="35" t="inlineStr">
@@ -18540,6 +18965,9 @@
       </c>
       <c r="E139" s="35" t="n">
         <v>37.3</v>
+      </c>
+      <c r="F139" s="35" t="n">
+        <v>37.2</v>
       </c>
     </row>
   </sheetData>
@@ -20895,10 +21323,10 @@
         <v>1622.5</v>
       </c>
       <c r="F24" s="35" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G24" s="42" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
@@ -21111,10 +21539,10 @@
         <v>1415.3</v>
       </c>
       <c r="F32" s="35" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G32" s="42" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="33">
@@ -21714,34 +22142,34 @@
     <row r="55">
       <c r="A55" s="35" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>North Texas</t>
         </is>
       </c>
       <c r="B55" s="35" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C55" s="35" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="D55" s="35" t="n">
         <v>50</v>
       </c>
       <c r="E55" s="35" t="n">
-        <v>1656.2</v>
+        <v>1625.5</v>
       </c>
       <c r="F55" s="35" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G55" s="35" t="n">
-        <v>-24</v>
+        <v>-14</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="35" t="inlineStr">
         <is>
-          <t>New Mexico</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="B56" s="35" t="inlineStr">
@@ -21756,19 +22184,19 @@
         <v>51</v>
       </c>
       <c r="E56" s="35" t="n">
-        <v>1597.5</v>
+        <v>1656.2</v>
       </c>
       <c r="F56" s="35" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="G56" s="35" t="n">
-        <v>2</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="35" t="inlineStr">
         <is>
-          <t>App State</t>
+          <t>New Mexico</t>
         </is>
       </c>
       <c r="B57" s="35" t="inlineStr">
@@ -21777,84 +22205,84 @@
         </is>
       </c>
       <c r="C57" s="35" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="D57" s="35" t="n">
         <v>52</v>
       </c>
       <c r="E57" s="35" t="n">
-        <v>1505.1</v>
+        <v>1597.5</v>
       </c>
       <c r="F57" s="35" t="n">
-        <v>87</v>
-      </c>
-      <c r="G57" s="42" t="n">
-        <v>35</v>
+        <v>53</v>
+      </c>
+      <c r="G57" s="35" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="35" t="inlineStr">
         <is>
-          <t>Idaho State</t>
+          <t>App State</t>
         </is>
       </c>
       <c r="B58" s="35" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="C58" s="35" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="D58" s="35" t="n">
         <v>53</v>
       </c>
       <c r="E58" s="35" t="n">
-        <v>1459.7</v>
+        <v>1505.1</v>
       </c>
       <c r="F58" s="35" t="n">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="G58" s="42" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="35" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Idaho State</t>
         </is>
       </c>
       <c r="B59" s="35" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="C59" s="35" t="n">
-        <v>0.51</v>
+        <v>0.57</v>
       </c>
       <c r="D59" s="35" t="n">
         <v>54</v>
       </c>
       <c r="E59" s="35" t="n">
-        <v>1596.4</v>
+        <v>1459.7</v>
       </c>
       <c r="F59" s="35" t="n">
-        <v>54</v>
-      </c>
-      <c r="G59" s="35" t="n">
-        <v>0</v>
+        <v>118</v>
+      </c>
+      <c r="G59" s="42" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="35" t="inlineStr">
         <is>
-          <t>Montana State</t>
+          <t>Minnesota</t>
         </is>
       </c>
       <c r="B60" s="35" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="C60" s="35" t="n">
@@ -21864,24 +22292,24 @@
         <v>55</v>
       </c>
       <c r="E60" s="35" t="n">
-        <v>1505.4</v>
+        <v>1596.4</v>
       </c>
       <c r="F60" s="35" t="n">
-        <v>86</v>
-      </c>
-      <c r="G60" s="42" t="n">
-        <v>31</v>
+        <v>54</v>
+      </c>
+      <c r="G60" s="35" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="35" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Montana State</t>
         </is>
       </c>
       <c r="B61" s="35" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="C61" s="35" t="n">
@@ -21891,19 +22319,19 @@
         <v>56</v>
       </c>
       <c r="E61" s="35" t="n">
-        <v>1622.7</v>
+        <v>1505.4</v>
       </c>
       <c r="F61" s="35" t="n">
-        <v>37</v>
-      </c>
-      <c r="G61" s="35" t="n">
-        <v>-19</v>
+        <v>85</v>
+      </c>
+      <c r="G61" s="42" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="35" t="inlineStr">
         <is>
-          <t>Georgia State</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="B62" s="35" t="inlineStr">
@@ -21918,132 +22346,132 @@
         <v>57</v>
       </c>
       <c r="E62" s="35" t="n">
-        <v>1440.6</v>
+        <v>1622.7</v>
       </c>
       <c r="F62" s="35" t="n">
-        <v>143</v>
-      </c>
-      <c r="G62" s="42" t="n">
-        <v>86</v>
+        <v>38</v>
+      </c>
+      <c r="G62" s="35" t="n">
+        <v>-19</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="35" t="inlineStr">
         <is>
-          <t>Tarleton State</t>
+          <t>Georgia State</t>
         </is>
       </c>
       <c r="B63" s="35" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="C63" s="35" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="D63" s="35" t="n">
         <v>58</v>
       </c>
       <c r="E63" s="35" t="n">
-        <v>1505.7</v>
+        <v>1440.6</v>
       </c>
       <c r="F63" s="35" t="n">
+        <v>143</v>
+      </c>
+      <c r="G63" s="42" t="n">
         <v>85</v>
-      </c>
-      <c r="G63" s="42" t="n">
-        <v>27</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="35" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Tarleton State</t>
         </is>
       </c>
       <c r="B64" s="35" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="C64" s="35" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="D64" s="35" t="n">
         <v>59</v>
       </c>
       <c r="E64" s="35" t="n">
-        <v>1461.8</v>
+        <v>1505.7</v>
       </c>
       <c r="F64" s="35" t="n">
-        <v>115</v>
+        <v>84</v>
       </c>
       <c r="G64" s="42" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="35" t="inlineStr">
         <is>
-          <t>Illinois State</t>
+          <t>Stanford</t>
         </is>
       </c>
       <c r="B65" s="35" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C65" s="35" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="D65" s="35" t="n">
         <v>60</v>
       </c>
       <c r="E65" s="35" t="n">
-        <v>1460.9</v>
+        <v>1461.8</v>
       </c>
       <c r="F65" s="35" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G65" s="42" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="35" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>Illinois State</t>
         </is>
       </c>
       <c r="B66" s="35" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="C66" s="35" t="n">
-        <v>0.43</v>
+        <v>0.47</v>
       </c>
       <c r="D66" s="35" t="n">
         <v>61</v>
       </c>
       <c r="E66" s="35" t="n">
-        <v>1640</v>
+        <v>1460.9</v>
       </c>
       <c r="F66" s="35" t="n">
-        <v>32</v>
-      </c>
-      <c r="G66" s="35" t="n">
-        <v>-29</v>
+        <v>116</v>
+      </c>
+      <c r="G66" s="42" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="35" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Oklahoma</t>
         </is>
       </c>
       <c r="B67" s="35" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C67" s="35" t="n">
@@ -22053,46 +22481,46 @@
         <v>62</v>
       </c>
       <c r="E67" s="35" t="n">
-        <v>1503.2</v>
+        <v>1640</v>
       </c>
       <c r="F67" s="35" t="n">
-        <v>89</v>
-      </c>
-      <c r="G67" s="42" t="n">
-        <v>27</v>
+        <v>32</v>
+      </c>
+      <c r="G67" s="35" t="n">
+        <v>-30</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="35" t="inlineStr">
         <is>
-          <t>Louisiana</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="B68" s="35" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="C68" s="35" t="n">
-        <v>0.41</v>
+        <v>0.43</v>
       </c>
       <c r="D68" s="35" t="n">
         <v>63</v>
       </c>
       <c r="E68" s="35" t="n">
-        <v>1553</v>
+        <v>1503.2</v>
       </c>
       <c r="F68" s="35" t="n">
-        <v>72</v>
-      </c>
-      <c r="G68" s="35" t="n">
-        <v>9</v>
+        <v>88</v>
+      </c>
+      <c r="G68" s="42" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="35" t="inlineStr">
         <is>
-          <t>West Virginia</t>
+          <t>Louisiana</t>
         </is>
       </c>
       <c r="B69" s="35" t="inlineStr">
@@ -22101,25 +22529,25 @@
         </is>
       </c>
       <c r="C69" s="35" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="D69" s="35" t="n">
         <v>64</v>
       </c>
       <c r="E69" s="35" t="n">
-        <v>1515.8</v>
+        <v>1553</v>
       </c>
       <c r="F69" s="35" t="n">
-        <v>83</v>
-      </c>
-      <c r="G69" s="42" t="n">
-        <v>19</v>
+        <v>72</v>
+      </c>
+      <c r="G69" s="35" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="35" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>West Virginia</t>
         </is>
       </c>
       <c r="B70" s="35" t="inlineStr">
@@ -22128,25 +22556,25 @@
         </is>
       </c>
       <c r="C70" s="35" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="D70" s="35" t="n">
         <v>65</v>
       </c>
       <c r="E70" s="35" t="n">
-        <v>1667.5</v>
+        <v>1515.8</v>
       </c>
       <c r="F70" s="35" t="n">
-        <v>24</v>
-      </c>
-      <c r="G70" s="35" t="n">
-        <v>-41</v>
+        <v>82</v>
+      </c>
+      <c r="G70" s="42" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="35" t="inlineStr">
         <is>
-          <t>Baylor</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="B71" s="35" t="inlineStr">
@@ -22161,24 +22589,24 @@
         <v>66</v>
       </c>
       <c r="E71" s="35" t="n">
-        <v>1565.6</v>
+        <v>1667.5</v>
       </c>
       <c r="F71" s="35" t="n">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="G71" s="35" t="n">
-        <v>0</v>
+        <v>-42</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="35" t="inlineStr">
         <is>
-          <t>UNLV</t>
+          <t>Baylor</t>
         </is>
       </c>
       <c r="B72" s="35" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="C72" s="35" t="n">
@@ -22188,73 +22616,73 @@
         <v>67</v>
       </c>
       <c r="E72" s="35" t="n">
-        <v>1606.6</v>
+        <v>1565.6</v>
       </c>
       <c r="F72" s="35" t="n">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="G72" s="35" t="n">
-        <v>-22</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="35" t="inlineStr">
         <is>
-          <t>The Citadel</t>
+          <t>UNLV</t>
         </is>
       </c>
       <c r="B73" s="35" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C73" s="35" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="D73" s="35" t="n">
         <v>68</v>
       </c>
       <c r="E73" s="35" t="n">
-        <v>1459.6</v>
+        <v>1606.6</v>
       </c>
       <c r="F73" s="35" t="n">
-        <v>119</v>
-      </c>
-      <c r="G73" s="42" t="n">
-        <v>51</v>
+        <v>45</v>
+      </c>
+      <c r="G73" s="35" t="n">
+        <v>-23</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="35" t="inlineStr">
         <is>
-          <t>Arizona State</t>
+          <t>The Citadel</t>
         </is>
       </c>
       <c r="B74" s="35" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="C74" s="35" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="D74" s="35" t="n">
         <v>69</v>
       </c>
       <c r="E74" s="35" t="n">
-        <v>1606</v>
+        <v>1459.6</v>
       </c>
       <c r="F74" s="35" t="n">
-        <v>47</v>
-      </c>
-      <c r="G74" s="35" t="n">
-        <v>-22</v>
+        <v>119</v>
+      </c>
+      <c r="G74" s="42" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="35" t="inlineStr">
         <is>
-          <t>Northwestern</t>
+          <t>Arizona State</t>
         </is>
       </c>
       <c r="B75" s="35" t="inlineStr">
@@ -22263,57 +22691,57 @@
         </is>
       </c>
       <c r="C75" s="35" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="D75" s="35" t="n">
         <v>70</v>
       </c>
       <c r="E75" s="35" t="n">
-        <v>1573.7</v>
+        <v>1606</v>
       </c>
       <c r="F75" s="35" t="n">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="G75" s="35" t="n">
-        <v>-6</v>
+        <v>-23</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="35" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Northwestern</t>
         </is>
       </c>
       <c r="B76" s="35" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="C76" s="35" t="n">
-        <v>0.29</v>
+        <v>0.31</v>
       </c>
       <c r="D76" s="35" t="n">
         <v>71</v>
       </c>
       <c r="E76" s="35" t="n">
-        <v>1600.6</v>
+        <v>1573.7</v>
       </c>
       <c r="F76" s="35" t="n">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="G76" s="35" t="n">
-        <v>-20</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="35" t="inlineStr">
         <is>
-          <t>Jacksonville State</t>
+          <t>Toledo</t>
         </is>
       </c>
       <c r="B77" s="35" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="C77" s="35" t="n">
@@ -22323,19 +22751,19 @@
         <v>72</v>
       </c>
       <c r="E77" s="35" t="n">
-        <v>1579.4</v>
+        <v>1600.6</v>
       </c>
       <c r="F77" s="35" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G77" s="35" t="n">
-        <v>-11</v>
+        <v>-21</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="35" t="inlineStr">
         <is>
-          <t>Michigan State</t>
+          <t>Jacksonville State</t>
         </is>
       </c>
       <c r="B78" s="35" t="inlineStr">
@@ -22344,46 +22772,46 @@
         </is>
       </c>
       <c r="C78" s="35" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="D78" s="35" t="n">
         <v>73</v>
       </c>
       <c r="E78" s="35" t="n">
-        <v>1471.5</v>
+        <v>1579.4</v>
       </c>
       <c r="F78" s="35" t="n">
-        <v>110</v>
-      </c>
-      <c r="G78" s="42" t="n">
-        <v>37</v>
+        <v>61</v>
+      </c>
+      <c r="G78" s="35" t="n">
+        <v>-12</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="35" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Michigan State</t>
         </is>
       </c>
       <c r="B79" s="35" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C79" s="35" t="n">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="D79" s="35" t="n">
         <v>74</v>
       </c>
       <c r="E79" s="35" t="n">
-        <v>1430.6</v>
+        <v>1471.5</v>
       </c>
       <c r="F79" s="35" t="n">
-        <v>161</v>
+        <v>110</v>
       </c>
       <c r="G79" s="42" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
     </row>
     <row r="80">
@@ -22434,10 +22862,10 @@
         <v>1502.2</v>
       </c>
       <c r="F81" s="35" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G81" s="35" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="82">
@@ -22470,7 +22898,7 @@
     <row r="83">
       <c r="A83" s="35" t="inlineStr">
         <is>
-          <t>North Texas</t>
+          <t>Utah State</t>
         </is>
       </c>
       <c r="B83" s="35" t="inlineStr">
@@ -22485,100 +22913,100 @@
         <v>78</v>
       </c>
       <c r="E83" s="35" t="n">
-        <v>1621.2</v>
+        <v>1466.7</v>
       </c>
       <c r="F83" s="35" t="n">
-        <v>39</v>
-      </c>
-      <c r="G83" s="35" t="n">
-        <v>-39</v>
+        <v>113</v>
+      </c>
+      <c r="G83" s="42" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="35" t="inlineStr">
         <is>
-          <t>Utah State</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="B84" s="35" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C84" s="35" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="D84" s="35" t="n">
         <v>79</v>
       </c>
       <c r="E84" s="35" t="n">
-        <v>1466.7</v>
+        <v>1638.9</v>
       </c>
       <c r="F84" s="35" t="n">
-        <v>113</v>
-      </c>
-      <c r="G84" s="42" t="n">
-        <v>34</v>
+        <v>33</v>
+      </c>
+      <c r="G84" s="35" t="n">
+        <v>-46</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="35" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Army</t>
         </is>
       </c>
       <c r="B85" s="35" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="C85" s="35" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="D85" s="35" t="n">
         <v>80</v>
       </c>
       <c r="E85" s="35" t="n">
-        <v>1638.9</v>
+        <v>1610.1</v>
       </c>
       <c r="F85" s="35" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G85" s="35" t="n">
-        <v>-47</v>
+        <v>-37</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="35" t="inlineStr">
         <is>
-          <t>Army</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="B86" s="35" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C86" s="35" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="D86" s="35" t="n">
         <v>81</v>
       </c>
       <c r="E86" s="35" t="n">
-        <v>1610.1</v>
+        <v>1460</v>
       </c>
       <c r="F86" s="35" t="n">
-        <v>43</v>
-      </c>
-      <c r="G86" s="35" t="n">
-        <v>-38</v>
+        <v>117</v>
+      </c>
+      <c r="G86" s="42" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="35" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Texas State</t>
         </is>
       </c>
       <c r="B87" s="35" t="inlineStr">
@@ -22587,25 +23015,25 @@
         </is>
       </c>
       <c r="C87" s="35" t="n">
-        <v>0.02</v>
+        <v>-0</v>
       </c>
       <c r="D87" s="35" t="n">
         <v>82</v>
       </c>
       <c r="E87" s="35" t="n">
-        <v>1460</v>
+        <v>1588.2</v>
       </c>
       <c r="F87" s="35" t="n">
-        <v>117</v>
-      </c>
-      <c r="G87" s="42" t="n">
-        <v>35</v>
+        <v>58</v>
+      </c>
+      <c r="G87" s="35" t="n">
+        <v>-24</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="35" t="inlineStr">
         <is>
-          <t>Texas State</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B88" s="35" t="inlineStr">
@@ -22614,25 +23042,25 @@
         </is>
       </c>
       <c r="C88" s="35" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="D88" s="35" t="n">
         <v>83</v>
       </c>
       <c r="E88" s="35" t="n">
-        <v>1588.2</v>
+        <v>1658.8</v>
       </c>
       <c r="F88" s="35" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G88" s="35" t="n">
-        <v>-25</v>
+        <v>-58</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="35" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="B89" s="35" t="inlineStr">
@@ -22641,25 +23069,25 @@
         </is>
       </c>
       <c r="C89" s="35" t="n">
-        <v>-0.01</v>
+        <v>-0.04</v>
       </c>
       <c r="D89" s="35" t="n">
         <v>84</v>
       </c>
       <c r="E89" s="35" t="n">
-        <v>1658.8</v>
+        <v>1504.3</v>
       </c>
       <c r="F89" s="35" t="n">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="G89" s="35" t="n">
-        <v>-59</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="35" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>South Alabama</t>
         </is>
       </c>
       <c r="B90" s="35" t="inlineStr">
@@ -22668,25 +23096,25 @@
         </is>
       </c>
       <c r="C90" s="35" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="D90" s="35" t="n">
         <v>85</v>
       </c>
       <c r="E90" s="35" t="n">
-        <v>1504.3</v>
+        <v>1493.6</v>
       </c>
       <c r="F90" s="35" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="G90" s="35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="35" t="inlineStr">
         <is>
-          <t>South Alabama</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="B91" s="35" t="inlineStr">
@@ -22701,19 +23129,19 @@
         <v>86</v>
       </c>
       <c r="E91" s="35" t="n">
-        <v>1493.6</v>
+        <v>1592.5</v>
       </c>
       <c r="F91" s="35" t="n">
-        <v>95</v>
+        <v>57</v>
       </c>
       <c r="G91" s="35" t="n">
-        <v>9</v>
+        <v>-29</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="35" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>East Carolina</t>
         </is>
       </c>
       <c r="B92" s="35" t="inlineStr">
@@ -22722,79 +23150,79 @@
         </is>
       </c>
       <c r="C92" s="35" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="D92" s="35" t="n">
         <v>87</v>
       </c>
       <c r="E92" s="35" t="n">
-        <v>1592.5</v>
+        <v>1593.3</v>
       </c>
       <c r="F92" s="35" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G92" s="35" t="n">
-        <v>-30</v>
+        <v>-32</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="35" t="inlineStr">
         <is>
-          <t>East Carolina</t>
+          <t>SE Louisiana</t>
         </is>
       </c>
       <c r="B93" s="35" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="C93" s="35" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="D93" s="35" t="n">
         <v>88</v>
       </c>
       <c r="E93" s="35" t="n">
-        <v>1593.3</v>
+        <v>1412.1</v>
       </c>
       <c r="F93" s="35" t="n">
-        <v>55</v>
-      </c>
-      <c r="G93" s="35" t="n">
-        <v>-33</v>
+        <v>202</v>
+      </c>
+      <c r="G93" s="42" t="n">
+        <v>114</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="35" t="inlineStr">
         <is>
-          <t>SE Louisiana</t>
+          <t>Delaware</t>
         </is>
       </c>
       <c r="B94" s="35" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C94" s="35" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="D94" s="35" t="n">
         <v>89</v>
       </c>
       <c r="E94" s="35" t="n">
-        <v>1412.1</v>
+        <v>1496</v>
       </c>
       <c r="F94" s="35" t="n">
-        <v>201</v>
-      </c>
-      <c r="G94" s="42" t="n">
-        <v>112</v>
+        <v>93</v>
+      </c>
+      <c r="G94" s="35" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="35" t="inlineStr">
         <is>
-          <t>Delaware</t>
+          <t>Arkansas State</t>
         </is>
       </c>
       <c r="B95" s="35" t="inlineStr">
@@ -22803,25 +23231,25 @@
         </is>
       </c>
       <c r="C95" s="35" t="n">
-        <v>-0.1</v>
+        <v>-0.12</v>
       </c>
       <c r="D95" s="35" t="n">
         <v>90</v>
       </c>
       <c r="E95" s="35" t="n">
-        <v>1496</v>
+        <v>1509.2</v>
       </c>
       <c r="F95" s="35" t="n">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="G95" s="35" t="n">
-        <v>4</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="35" t="inlineStr">
         <is>
-          <t>Arkansas State</t>
+          <t>Western Michigan</t>
         </is>
       </c>
       <c r="B96" s="35" t="inlineStr">
@@ -22836,24 +23264,24 @@
         <v>91</v>
       </c>
       <c r="E96" s="35" t="n">
-        <v>1509.2</v>
+        <v>1579.5</v>
       </c>
       <c r="F96" s="35" t="n">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="G96" s="35" t="n">
-        <v>-7</v>
+        <v>-31</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="35" t="inlineStr">
         <is>
-          <t>Western Michigan</t>
+          <t>Tennessee State</t>
         </is>
       </c>
       <c r="B97" s="35" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C97" s="35" t="n">
@@ -22863,127 +23291,127 @@
         <v>92</v>
       </c>
       <c r="E97" s="35" t="n">
-        <v>1579.5</v>
+        <v>1447.4</v>
       </c>
       <c r="F97" s="35" t="n">
-        <v>60</v>
-      </c>
-      <c r="G97" s="35" t="n">
-        <v>-32</v>
+        <v>132</v>
+      </c>
+      <c r="G97" s="42" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="35" t="inlineStr">
         <is>
-          <t>Tennessee State</t>
+          <t>Miami (OH)</t>
         </is>
       </c>
       <c r="B98" s="35" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C98" s="35" t="n">
-        <v>-0.12</v>
+        <v>-0.13</v>
       </c>
       <c r="D98" s="35" t="n">
         <v>93</v>
       </c>
       <c r="E98" s="35" t="n">
-        <v>1447.4</v>
+        <v>1536.7</v>
       </c>
       <c r="F98" s="35" t="n">
-        <v>132</v>
-      </c>
-      <c r="G98" s="42" t="n">
-        <v>39</v>
+        <v>76</v>
+      </c>
+      <c r="G98" s="35" t="n">
+        <v>-17</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="35" t="inlineStr">
         <is>
-          <t>Miami (OH)</t>
+          <t>Florida A&amp;M</t>
         </is>
       </c>
       <c r="B99" s="35" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C99" s="35" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="D99" s="35" t="n">
         <v>94</v>
       </c>
       <c r="E99" s="35" t="n">
-        <v>1536.7</v>
+        <v>1414.3</v>
       </c>
       <c r="F99" s="35" t="n">
-        <v>76</v>
-      </c>
-      <c r="G99" s="35" t="n">
-        <v>-18</v>
+        <v>191</v>
+      </c>
+      <c r="G99" s="42" t="n">
+        <v>97</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="35" t="inlineStr">
         <is>
-          <t>Florida A&amp;M</t>
+          <t>Central Michigan</t>
         </is>
       </c>
       <c r="B100" s="35" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C100" s="35" t="n">
-        <v>-0.14</v>
+        <v>-0.16</v>
       </c>
       <c r="D100" s="35" t="n">
         <v>95</v>
       </c>
       <c r="E100" s="35" t="n">
-        <v>1414.3</v>
+        <v>1466.3</v>
       </c>
       <c r="F100" s="35" t="n">
-        <v>190</v>
+        <v>114</v>
       </c>
       <c r="G100" s="42" t="n">
-        <v>95</v>
+        <v>19</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="35" t="inlineStr">
         <is>
-          <t>Central Michigan</t>
+          <t>Abilene Christian</t>
         </is>
       </c>
       <c r="B101" s="35" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C101" s="35" t="n">
-        <v>-0.16</v>
+        <v>-0.17</v>
       </c>
       <c r="D101" s="35" t="n">
         <v>96</v>
       </c>
       <c r="E101" s="35" t="n">
-        <v>1466.3</v>
+        <v>1414.3</v>
       </c>
       <c r="F101" s="35" t="n">
-        <v>114</v>
+        <v>192</v>
       </c>
       <c r="G101" s="42" t="n">
-        <v>18</v>
+        <v>96</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="35" t="inlineStr">
         <is>
-          <t>Abilene Christian</t>
+          <t>UC Davis</t>
         </is>
       </c>
       <c r="B102" s="35" t="inlineStr">
@@ -22992,25 +23420,25 @@
         </is>
       </c>
       <c r="C102" s="35" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="D102" s="35" t="n">
         <v>97</v>
       </c>
       <c r="E102" s="35" t="n">
-        <v>1414.3</v>
+        <v>1449.9</v>
       </c>
       <c r="F102" s="35" t="n">
-        <v>191</v>
+        <v>129</v>
       </c>
       <c r="G102" s="42" t="n">
-        <v>94</v>
+        <v>32</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="35" t="inlineStr">
         <is>
-          <t>UC Davis</t>
+          <t>Idaho</t>
         </is>
       </c>
       <c r="B103" s="35" t="inlineStr">
@@ -23025,19 +23453,19 @@
         <v>98</v>
       </c>
       <c r="E103" s="35" t="n">
-        <v>1449.9</v>
+        <v>1459.1</v>
       </c>
       <c r="F103" s="35" t="n">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="G103" s="42" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="35" t="inlineStr">
         <is>
-          <t>Idaho</t>
+          <t>Northern Iowa</t>
         </is>
       </c>
       <c r="B104" s="35" t="inlineStr">
@@ -23052,24 +23480,24 @@
         <v>99</v>
       </c>
       <c r="E104" s="35" t="n">
-        <v>1459.1</v>
+        <v>1411.5</v>
       </c>
       <c r="F104" s="35" t="n">
-        <v>121</v>
+        <v>204</v>
       </c>
       <c r="G104" s="42" t="n">
-        <v>22</v>
+        <v>105</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="35" t="inlineStr">
         <is>
-          <t>Northern Iowa</t>
+          <t>San José State</t>
         </is>
       </c>
       <c r="B105" s="35" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C105" s="35" t="n">
@@ -23079,40 +23507,40 @@
         <v>100</v>
       </c>
       <c r="E105" s="35" t="n">
-        <v>1411.5</v>
+        <v>1428.8</v>
       </c>
       <c r="F105" s="35" t="n">
-        <v>203</v>
+        <v>165</v>
       </c>
       <c r="G105" s="42" t="n">
-        <v>103</v>
+        <v>65</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="35" t="inlineStr">
         <is>
-          <t>San José State</t>
+          <t>Tulsa</t>
         </is>
       </c>
       <c r="B106" s="35" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C106" s="35" t="n">
-        <v>-0.18</v>
+        <v>-0.19</v>
       </c>
       <c r="D106" s="35" t="n">
         <v>101</v>
       </c>
       <c r="E106" s="35" t="n">
-        <v>1428.8</v>
+        <v>1426.3</v>
       </c>
       <c r="F106" s="35" t="n">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="G106" s="42" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="107">
@@ -23244,10 +23672,10 @@
         <v>1406.9</v>
       </c>
       <c r="F111" s="35" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G111" s="42" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="112">
@@ -23298,10 +23726,10 @@
         <v>1519.1</v>
       </c>
       <c r="F113" s="35" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G113" s="35" t="n">
-        <v>-26</v>
+        <v>-27</v>
       </c>
     </row>
     <row r="114">
@@ -23460,10 +23888,10 @@
         <v>1412.3</v>
       </c>
       <c r="F119" s="35" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G119" s="42" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="120">
@@ -23487,10 +23915,10 @@
         <v>1429.6</v>
       </c>
       <c r="F120" s="35" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G120" s="42" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="121">
@@ -23568,10 +23996,10 @@
         <v>1427.9</v>
       </c>
       <c r="F123" s="35" t="n">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G123" s="42" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="124">
@@ -23595,10 +24023,10 @@
         <v>1422.7</v>
       </c>
       <c r="F124" s="35" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G124" s="42" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="125">
@@ -23730,10 +24158,10 @@
         <v>1414.2</v>
       </c>
       <c r="F129" s="35" t="n">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G129" s="42" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="130">
@@ -23757,10 +24185,10 @@
         <v>1418.5</v>
       </c>
       <c r="F130" s="35" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G130" s="42" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="131">
@@ -23811,10 +24239,10 @@
         <v>1422.8</v>
       </c>
       <c r="F132" s="35" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G132" s="42" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="133">
@@ -23892,10 +24320,10 @@
         <v>1429.2</v>
       </c>
       <c r="F135" s="35" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G135" s="42" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="136">
@@ -23973,10 +24401,10 @@
         <v>1405.5</v>
       </c>
       <c r="F138" s="35" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G138" s="42" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="139">
@@ -24000,10 +24428,10 @@
         <v>1413.9</v>
       </c>
       <c r="F139" s="35" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G139" s="42" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="140">
@@ -24027,10 +24455,10 @@
         <v>1403.3</v>
       </c>
       <c r="F140" s="35" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G140" s="42" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="141">
@@ -24054,10 +24482,10 @@
         <v>1409.5</v>
       </c>
       <c r="F141" s="35" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G141" s="42" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="142">
@@ -24081,10 +24509,10 @@
         <v>1428.8</v>
       </c>
       <c r="F142" s="35" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G142" s="42" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="143">
@@ -24108,10 +24536,10 @@
         <v>1420.7</v>
       </c>
       <c r="F143" s="35" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G143" s="42" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="144">
@@ -24162,10 +24590,10 @@
         <v>1491.6</v>
       </c>
       <c r="F145" s="35" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G145" s="35" t="n">
-        <v>-43</v>
+        <v>-44</v>
       </c>
     </row>
     <row r="146">
@@ -24189,10 +24617,10 @@
         <v>1411.7</v>
       </c>
       <c r="F146" s="35" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G146" s="42" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="147">
@@ -24243,10 +24671,10 @@
         <v>1412.8</v>
       </c>
       <c r="F148" s="35" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G148" s="42" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="149">
@@ -24297,10 +24725,10 @@
         <v>1398.8</v>
       </c>
       <c r="F150" s="35" t="n">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G150" s="42" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="151">
@@ -24378,10 +24806,10 @@
         <v>1414.9</v>
       </c>
       <c r="F153" s="35" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G153" s="42" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="154">
@@ -24432,10 +24860,10 @@
         <v>1488.5</v>
       </c>
       <c r="F155" s="35" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G155" s="35" t="n">
-        <v>-50</v>
+        <v>-51</v>
       </c>
     </row>
     <row r="156">
@@ -24459,10 +24887,10 @@
         <v>1429.6</v>
       </c>
       <c r="F156" s="35" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G156" s="35" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="157">
@@ -24486,10 +24914,10 @@
         <v>1387.5</v>
       </c>
       <c r="F157" s="35" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G157" s="42" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="158">
@@ -24513,10 +24941,10 @@
         <v>1400.8</v>
       </c>
       <c r="F158" s="35" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G158" s="42" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="159">
@@ -24675,10 +25103,10 @@
         <v>1520.2</v>
       </c>
       <c r="F164" s="35" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G164" s="35" t="n">
-        <v>-78</v>
+        <v>-79</v>
       </c>
     </row>
     <row r="165">
@@ -24702,10 +25130,10 @@
         <v>1402.8</v>
       </c>
       <c r="F165" s="35" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G165" s="42" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="166">
@@ -24729,10 +25157,10 @@
         <v>1417.1</v>
       </c>
       <c r="F166" s="35" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G166" s="42" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="167">
@@ -24783,10 +25211,10 @@
         <v>1391.8</v>
       </c>
       <c r="F168" s="35" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G168" s="42" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="169">
@@ -24810,10 +25238,10 @@
         <v>1411.1</v>
       </c>
       <c r="F169" s="35" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G169" s="42" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="170">
@@ -24891,10 +25319,10 @@
         <v>1422</v>
       </c>
       <c r="F172" s="35" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G172" s="35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="173">
@@ -24945,10 +25373,10 @@
         <v>1404.2</v>
       </c>
       <c r="F174" s="35" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G174" s="42" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="175">
@@ -24972,10 +25400,10 @@
         <v>1413.6</v>
       </c>
       <c r="F175" s="35" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G175" s="42" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="176">
@@ -24999,10 +25427,10 @@
         <v>1624</v>
       </c>
       <c r="F176" s="35" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G176" s="35" t="n">
-        <v>-135</v>
+        <v>-134</v>
       </c>
     </row>
     <row r="177">
@@ -25026,10 +25454,10 @@
         <v>1418.7</v>
       </c>
       <c r="F177" s="35" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G177" s="35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="178">
@@ -25053,10 +25481,10 @@
         <v>1420.6</v>
       </c>
       <c r="F178" s="35" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G178" s="35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="179">
@@ -25080,10 +25508,10 @@
         <v>1416.7</v>
       </c>
       <c r="F179" s="35" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G179" s="35" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="180">
@@ -25134,10 +25562,10 @@
         <v>1393.9</v>
       </c>
       <c r="F181" s="35" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G181" s="42" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="182">
@@ -25188,10 +25616,10 @@
         <v>1412.2</v>
       </c>
       <c r="F183" s="35" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G183" s="42" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="184">
@@ -25242,10 +25670,10 @@
         <v>1388</v>
       </c>
       <c r="F185" s="35" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G185" s="42" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="186">
@@ -25269,10 +25697,10 @@
         <v>1395</v>
       </c>
       <c r="F186" s="35" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G186" s="42" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="187">
@@ -25323,10 +25751,10 @@
         <v>1417.9</v>
       </c>
       <c r="F188" s="35" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G188" s="35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="189">
@@ -25350,10 +25778,10 @@
         <v>1397.7</v>
       </c>
       <c r="F189" s="35" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G189" s="42" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="190">
@@ -25377,10 +25805,10 @@
         <v>1501.2</v>
       </c>
       <c r="F190" s="35" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G190" s="35" t="n">
-        <v>-94</v>
+        <v>-95</v>
       </c>
     </row>
     <row r="191">
@@ -25404,10 +25832,10 @@
         <v>1413.3</v>
       </c>
       <c r="F191" s="35" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G191" s="35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="192">
@@ -25566,43 +25994,43 @@
         <v>1427.1</v>
       </c>
       <c r="F197" s="35" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G197" s="35" t="n">
-        <v>-22</v>
+        <v>-23</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="35" t="inlineStr">
         <is>
-          <t>Western Kentucky</t>
+          <t>Gardner-Webb</t>
         </is>
       </c>
       <c r="B198" s="35" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="C198" s="35" t="n">
-        <v>-0.77</v>
+        <v>-0.78</v>
       </c>
       <c r="D198" s="35" t="n">
         <v>193</v>
       </c>
       <c r="E198" s="35" t="n">
-        <v>1521.5</v>
+        <v>1421.6</v>
       </c>
       <c r="F198" s="35" t="n">
-        <v>79</v>
+        <v>179</v>
       </c>
       <c r="G198" s="35" t="n">
-        <v>-114</v>
+        <v>-14</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="35" t="inlineStr">
         <is>
-          <t>Gardner-Webb</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="B199" s="35" t="inlineStr">
@@ -25611,25 +26039,25 @@
         </is>
       </c>
       <c r="C199" s="35" t="n">
-        <v>-0.78</v>
+        <v>-0.79</v>
       </c>
       <c r="D199" s="35" t="n">
         <v>194</v>
       </c>
       <c r="E199" s="35" t="n">
-        <v>1421.6</v>
+        <v>1501</v>
       </c>
       <c r="F199" s="35" t="n">
-        <v>178</v>
+        <v>91</v>
       </c>
       <c r="G199" s="35" t="n">
-        <v>-16</v>
+        <v>-103</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="35" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Houston Christian</t>
         </is>
       </c>
       <c r="B200" s="35" t="inlineStr">
@@ -25638,25 +26066,25 @@
         </is>
       </c>
       <c r="C200" s="35" t="n">
-        <v>-0.79</v>
+        <v>-0.8</v>
       </c>
       <c r="D200" s="35" t="n">
         <v>195</v>
       </c>
       <c r="E200" s="35" t="n">
-        <v>1501</v>
+        <v>1392.6</v>
       </c>
       <c r="F200" s="35" t="n">
-        <v>92</v>
-      </c>
-      <c r="G200" s="35" t="n">
-        <v>-103</v>
+        <v>230</v>
+      </c>
+      <c r="G200" s="42" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="35" t="inlineStr">
         <is>
-          <t>Houston Christian</t>
+          <t>Duquesne</t>
         </is>
       </c>
       <c r="B201" s="35" t="inlineStr">
@@ -25671,19 +26099,19 @@
         <v>196</v>
       </c>
       <c r="E201" s="35" t="n">
-        <v>1392.6</v>
+        <v>1359.3</v>
       </c>
       <c r="F201" s="35" t="n">
-        <v>229</v>
+        <v>247</v>
       </c>
       <c r="G201" s="42" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="35" t="inlineStr">
         <is>
-          <t>Duquesne</t>
+          <t>West Georgia</t>
         </is>
       </c>
       <c r="B202" s="35" t="inlineStr">
@@ -25692,25 +26120,25 @@
         </is>
       </c>
       <c r="C202" s="35" t="n">
-        <v>-0.8</v>
+        <v>-0.82</v>
       </c>
       <c r="D202" s="35" t="n">
         <v>197</v>
       </c>
       <c r="E202" s="35" t="n">
-        <v>1359.3</v>
+        <v>1442.3</v>
       </c>
       <c r="F202" s="35" t="n">
-        <v>247</v>
-      </c>
-      <c r="G202" s="42" t="n">
-        <v>50</v>
+        <v>141</v>
+      </c>
+      <c r="G202" s="35" t="n">
+        <v>-56</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="35" t="inlineStr">
         <is>
-          <t>West Georgia</t>
+          <t>Long Island University</t>
         </is>
       </c>
       <c r="B203" s="35" t="inlineStr">
@@ -25719,73 +26147,73 @@
         </is>
       </c>
       <c r="C203" s="35" t="n">
-        <v>-0.82</v>
+        <v>-0.83</v>
       </c>
       <c r="D203" s="35" t="n">
         <v>198</v>
       </c>
       <c r="E203" s="35" t="n">
-        <v>1442.3</v>
+        <v>1409.7</v>
       </c>
       <c r="F203" s="35" t="n">
-        <v>141</v>
+        <v>206</v>
       </c>
       <c r="G203" s="35" t="n">
-        <v>-57</v>
+        <v>8</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="35" t="inlineStr">
         <is>
-          <t>Long Island University</t>
+          <t>Rice</t>
         </is>
       </c>
       <c r="B204" s="35" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>0-3</t>
         </is>
       </c>
       <c r="C204" s="35" t="n">
-        <v>-0.83</v>
+        <v>-0.84</v>
       </c>
       <c r="D204" s="35" t="n">
         <v>199</v>
       </c>
       <c r="E204" s="35" t="n">
-        <v>1409.7</v>
+        <v>1413.7</v>
       </c>
       <c r="F204" s="35" t="n">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="G204" s="35" t="n">
-        <v>6</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="35" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>New Mexico State</t>
         </is>
       </c>
       <c r="B205" s="35" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C205" s="35" t="n">
-        <v>-0.84</v>
+        <v>-0.88</v>
       </c>
       <c r="D205" s="35" t="n">
         <v>200</v>
       </c>
       <c r="E205" s="35" t="n">
-        <v>1413.7</v>
+        <v>1423</v>
       </c>
       <c r="F205" s="35" t="n">
-        <v>194</v>
+        <v>175</v>
       </c>
       <c r="G205" s="35" t="n">
-        <v>-6</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="206">
@@ -25836,10 +26264,10 @@
         <v>1520.6</v>
       </c>
       <c r="F207" s="35" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G207" s="35" t="n">
-        <v>-122</v>
+        <v>-123</v>
       </c>
     </row>
     <row r="208">
@@ -25890,10 +26318,10 @@
         <v>1388.5</v>
       </c>
       <c r="F209" s="35" t="n">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G209" s="42" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="210">
@@ -26025,10 +26453,10 @@
         <v>1499.6</v>
       </c>
       <c r="F214" s="35" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G214" s="35" t="n">
-        <v>-116</v>
+        <v>-117</v>
       </c>
     </row>
     <row r="215">
@@ -26052,10 +26480,10 @@
         <v>1402.2</v>
       </c>
       <c r="F215" s="35" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G215" s="35" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="216">
@@ -26079,10 +26507,10 @@
         <v>1399.2</v>
       </c>
       <c r="F216" s="35" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G216" s="35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="217">
@@ -26133,10 +26561,10 @@
         <v>1491.5</v>
       </c>
       <c r="F218" s="35" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G218" s="35" t="n">
-        <v>-115</v>
+        <v>-116</v>
       </c>
     </row>
     <row r="219">
@@ -26160,10 +26588,10 @@
         <v>1396.1</v>
       </c>
       <c r="F219" s="35" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G219" s="35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="220">
@@ -26187,10 +26615,10 @@
         <v>1427.8</v>
       </c>
       <c r="F220" s="35" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G220" s="35" t="n">
-        <v>-46</v>
+        <v>-47</v>
       </c>
     </row>
     <row r="221">
@@ -26295,10 +26723,10 @@
         <v>1393.2</v>
       </c>
       <c r="F224" s="35" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G224" s="35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="225">
@@ -26322,10 +26750,10 @@
         <v>1419.1</v>
       </c>
       <c r="F225" s="35" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G225" s="35" t="n">
-        <v>-39</v>
+        <v>-38</v>
       </c>
     </row>
     <row r="226">
@@ -26376,10 +26804,10 @@
         <v>1406.7</v>
       </c>
       <c r="F227" s="35" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G227" s="35" t="n">
-        <v>-12</v>
+        <v>-11</v>
       </c>
     </row>
     <row r="228">
@@ -26457,10 +26885,10 @@
         <v>1389.7</v>
       </c>
       <c r="F230" s="35" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G230" s="35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="231">
@@ -26484,16 +26912,16 @@
         <v>1414.7</v>
       </c>
       <c r="F231" s="35" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G231" s="35" t="n">
-        <v>-37</v>
+        <v>-36</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="35" t="inlineStr">
         <is>
-          <t>New Mexico State</t>
+          <t>Kennesaw State</t>
         </is>
       </c>
       <c r="B232" s="35" t="inlineStr">
@@ -26502,30 +26930,30 @@
         </is>
       </c>
       <c r="C232" s="35" t="n">
-        <v>-1.31</v>
+        <v>-1.34</v>
       </c>
       <c r="D232" s="35" t="n">
         <v>227</v>
       </c>
       <c r="E232" s="35" t="n">
-        <v>1387.2</v>
+        <v>1480.8</v>
       </c>
       <c r="F232" s="35" t="n">
-        <v>235</v>
+        <v>101</v>
       </c>
       <c r="G232" s="35" t="n">
-        <v>8</v>
+        <v>-126</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="35" t="inlineStr">
         <is>
-          <t>Kennesaw State</t>
+          <t>Western Kentucky</t>
         </is>
       </c>
       <c r="B233" s="35" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="C233" s="35" t="n">
@@ -26535,13 +26963,13 @@
         <v>228</v>
       </c>
       <c r="E233" s="35" t="n">
-        <v>1480.8</v>
+        <v>1485.6</v>
       </c>
       <c r="F233" s="35" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G233" s="35" t="n">
-        <v>-127</v>
+        <v>-128</v>
       </c>
     </row>
     <row r="234">
@@ -26673,10 +27101,10 @@
         <v>1404.9</v>
       </c>
       <c r="F238" s="35" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G238" s="35" t="n">
-        <v>-21</v>
+        <v>-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-10-07 20:49 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -13946,26 +13946,26 @@
       </c>
       <c r="B3" s="38" t="inlineStr">
         <is>
-          <t>33-26-1</t>
+          <t>33-27-1</t>
         </is>
       </c>
       <c r="C3" s="41" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>Weekly ATS (Wk 5)</t>
+          <t>Weekly ATS (Wk 6)</t>
         </is>
       </c>
       <c r="B4" s="38" t="inlineStr">
         <is>
-          <t>3-3-0</t>
+          <t>0-1-0</t>
         </is>
       </c>
       <c r="C4" s="41" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="15.6" customHeight="1">
@@ -14098,7 +14098,7 @@
     <row r="12">
       <c r="A12" s="38" t="inlineStr">
         <is>
-          <t>Georgia Southern</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="B12" s="38" t="n">
@@ -14111,69 +14111,71 @@
         <v>1</v>
       </c>
       <c r="E12" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="38" t="n">
         <v>2</v>
-      </c>
-      <c r="F12" s="38" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="38" t="inlineStr">
         <is>
-          <t>App State</t>
+          <t>Georgia Southern</t>
         </is>
       </c>
       <c r="B13" s="38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="38" t="n"/>
+      <c r="D13" s="38" t="n">
+        <v>1</v>
+      </c>
       <c r="E13" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="38" t="n">
         <v>3</v>
-      </c>
-      <c r="F13" s="38" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t>Marshall</t>
+          <t>App State</t>
         </is>
       </c>
       <c r="B14" s="38" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="38" t="n">
         <v>0</v>
       </c>
+      <c r="D14" s="38" t="n"/>
       <c r="E14" s="38" t="n">
         <v>3</v>
       </c>
       <c r="F14" s="38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
         <is>
-          <t>Louisiana Tech</t>
+          <t>Marshall</t>
         </is>
       </c>
       <c r="B15" s="38" t="n">
         <v>0</v>
       </c>
       <c r="C15" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="38" t="n"/>
       <c r="E15" s="38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="38" t="n">
         <v>2</v>
@@ -14182,7 +14184,7 @@
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Louisiana Tech</t>
         </is>
       </c>
       <c r="B16" s="38" t="n">
@@ -14224,34 +14226,36 @@
     <row r="18" ht="26.45" customHeight="1">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>Southern Miss</t>
+          <t>Coastal Carolina</t>
         </is>
       </c>
       <c r="B18" s="38" t="n">
         <v>0</v>
       </c>
       <c r="C18" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="38" t="n"/>
       <c r="E18" s="38" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="38" t="inlineStr">
         <is>
-          <t>Coastal Carolina</t>
+          <t>Old Dominion</t>
         </is>
       </c>
       <c r="B19" s="38" t="n">
         <v>0</v>
       </c>
       <c r="C19" s="38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="38" t="n">
         <v>0</v>
@@ -14266,14 +14270,14 @@
     <row r="20">
       <c r="A20" s="38" t="inlineStr">
         <is>
-          <t>Old Dominion</t>
+          <t>Southern Miss</t>
         </is>
       </c>
       <c r="B20" s="38" t="n">
         <v>0</v>
       </c>
       <c r="C20" s="38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="38" t="n">
         <v>0</v>
@@ -14454,9 +14458,17 @@
       <c r="N25" s="38" t="n">
         <v>0.3</v>
       </c>
-      <c r="O25" s="38" t="n"/>
-      <c r="P25" s="38" t="n"/>
-      <c r="Q25" s="38" t="n"/>
+      <c r="O25" s="38" t="n">
+        <v>34</v>
+      </c>
+      <c r="P25" s="38" t="n">
+        <v>55</v>
+      </c>
+      <c r="Q25" s="43" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="38" t="n">
@@ -25448,7 +25460,7 @@
         <v/>
       </c>
       <c r="I3" t="n">
-        <v>45.6</v>
+        <v>45.7</v>
       </c>
       <c r="J3" t="n">
         <v>43.5</v>
@@ -25560,7 +25572,7 @@
         <v/>
       </c>
       <c r="I5" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="J5" t="n">
         <v>49.5</v>
@@ -36639,6 +36651,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
   </cols>
@@ -36674,6 +36687,11 @@
           <t>Week 5</t>
         </is>
       </c>
+      <c r="G1" s="36" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
       <c r="V1" s="37" t="inlineStr">
         <is>
           <t>Matchup Spread Calculator</t>
@@ -36701,6 +36719,9 @@
       <c r="F2" s="38" t="n">
         <v>94.59999999999999</v>
       </c>
+      <c r="G2" s="38" t="n">
+        <v>94.59999999999999</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="38" t="inlineStr">
@@ -36723,6 +36744,9 @@
       <c r="F3" s="38" t="n">
         <v>94.2</v>
       </c>
+      <c r="G3" s="38" t="n">
+        <v>94.3</v>
+      </c>
       <c r="V3" s="38" t="inlineStr">
         <is>
           <t>Home Team</t>
@@ -36755,6 +36779,9 @@
       <c r="F4" s="38" t="n">
         <v>90.40000000000001</v>
       </c>
+      <c r="G4" s="38" t="n">
+        <v>90.5</v>
+      </c>
       <c r="V4" s="38" t="inlineStr">
         <is>
           <t>Away Team</t>
@@ -36787,6 +36814,9 @@
       <c r="F5" s="38" t="n">
         <v>89.2</v>
       </c>
+      <c r="G5" s="38" t="n">
+        <v>89.2</v>
+      </c>
       <c r="V5" s="38" t="inlineStr">
         <is>
           <t>Neutral Site? (Y/N)</t>
@@ -36819,6 +36849,9 @@
       <c r="F6" s="38" t="n">
         <v>88</v>
       </c>
+      <c r="G6" s="38" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="38" t="inlineStr">
@@ -36841,6 +36874,9 @@
       <c r="F7" s="38" t="n">
         <v>87.8</v>
       </c>
+      <c r="G7" s="38" t="n">
+        <v>87.8</v>
+      </c>
       <c r="V7" s="38" t="inlineStr">
         <is>
           <t>HFA (model constant)</t>
@@ -36871,6 +36907,9 @@
       <c r="F8" s="38" t="n">
         <v>85.8</v>
       </c>
+      <c r="G8" s="38" t="n">
+        <v>85.8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="38" t="inlineStr">
@@ -36893,13 +36932,16 @@
       <c r="F9" s="38" t="n">
         <v>85.7</v>
       </c>
+      <c r="G9" s="38" t="n">
+        <v>85.7</v>
+      </c>
       <c r="V9" s="39" t="inlineStr">
         <is>
           <t>Predicted Spread (Home)</t>
         </is>
       </c>
       <c r="W9" s="39">
-        <f>IF(OR(W3="",W4=""),"",INDEX($F$2:$F$139,MATCH(W4,$A$2:$A$139,0))-INDEX($F$2:$F$139,MATCH(W3,$A$2:$A$139,0))-IF(UPPER(W5)="Y",0,W7))</f>
+        <f>IF(OR(W3="",W4=""),"",INDEX($G$2:$G$139,MATCH(W4,$A$2:$A$139,0))-INDEX($G$2:$G$139,MATCH(W3,$A$2:$A$139,0))-IF(UPPER(W5)="Y",0,W7))</f>
         <v/>
       </c>
     </row>
@@ -36924,6 +36966,9 @@
       <c r="F10" s="38" t="n">
         <v>84.5</v>
       </c>
+      <c r="G10" s="38" t="n">
+        <v>84.5</v>
+      </c>
       <c r="V10" s="40" t="inlineStr">
         <is>
           <t>(negative = home team favored, e.g. "Home -6.5")</t>
@@ -36951,6 +36996,9 @@
       <c r="F11" s="38" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="G11" s="38" t="n">
+        <v>84.09999999999999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="38" t="inlineStr">
@@ -36973,6 +37021,9 @@
       <c r="F12" s="38" t="n">
         <v>83</v>
       </c>
+      <c r="G12" s="38" t="n">
+        <v>83.2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="38" t="inlineStr">
@@ -36995,6 +37046,9 @@
       <c r="F13" s="38" t="n">
         <v>81.2</v>
       </c>
+      <c r="G13" s="38" t="n">
+        <v>81.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="38" t="inlineStr">
@@ -37017,6 +37071,9 @@
       <c r="F14" s="38" t="n">
         <v>81.09999999999999</v>
       </c>
+      <c r="G14" s="38" t="n">
+        <v>81.09999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="38" t="inlineStr">
@@ -37039,6 +37096,9 @@
       <c r="F15" s="38" t="n">
         <v>80.7</v>
       </c>
+      <c r="G15" s="38" t="n">
+        <v>80.7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="38" t="inlineStr">
@@ -37061,6 +37121,9 @@
       <c r="F16" s="38" t="n">
         <v>80.40000000000001</v>
       </c>
+      <c r="G16" s="38" t="n">
+        <v>80.40000000000001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="38" t="inlineStr">
@@ -37083,6 +37146,9 @@
       <c r="F17" s="38" t="n">
         <v>79.8</v>
       </c>
+      <c r="G17" s="38" t="n">
+        <v>79.8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="inlineStr">
@@ -37105,6 +37171,9 @@
       <c r="F18" s="38" t="n">
         <v>78.8</v>
       </c>
+      <c r="G18" s="38" t="n">
+        <v>78.8</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="38" t="inlineStr">
@@ -37127,6 +37196,9 @@
       <c r="F19" s="38" t="n">
         <v>78.2</v>
       </c>
+      <c r="G19" s="38" t="n">
+        <v>78.2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="38" t="inlineStr">
@@ -37149,6 +37221,9 @@
       <c r="F20" s="38" t="n">
         <v>78</v>
       </c>
+      <c r="G20" s="38" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="38" t="inlineStr">
@@ -37171,6 +37246,9 @@
       <c r="F21" s="38" t="n">
         <v>77.8</v>
       </c>
+      <c r="G21" s="38" t="n">
+        <v>77.8</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="38" t="inlineStr">
@@ -37193,6 +37271,9 @@
       <c r="F22" s="38" t="n">
         <v>77.59999999999999</v>
       </c>
+      <c r="G22" s="38" t="n">
+        <v>77.59999999999999</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="38" t="inlineStr">
@@ -37215,6 +37296,9 @@
       <c r="F23" s="38" t="n">
         <v>77.59999999999999</v>
       </c>
+      <c r="G23" s="38" t="n">
+        <v>77.59999999999999</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="inlineStr">
@@ -37237,6 +37321,9 @@
       <c r="F24" s="38" t="n">
         <v>77.5</v>
       </c>
+      <c r="G24" s="38" t="n">
+        <v>77.5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="38" t="inlineStr">
@@ -37259,6 +37346,9 @@
       <c r="F25" s="38" t="n">
         <v>77.40000000000001</v>
       </c>
+      <c r="G25" s="38" t="n">
+        <v>77.40000000000001</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="38" t="inlineStr">
@@ -37281,6 +37371,9 @@
       <c r="F26" s="38" t="n">
         <v>76.90000000000001</v>
       </c>
+      <c r="G26" s="38" t="n">
+        <v>76.90000000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="38" t="inlineStr">
@@ -37303,50 +37396,59 @@
       <c r="F27" s="38" t="n">
         <v>76.59999999999999</v>
       </c>
+      <c r="G27" s="38" t="n">
+        <v>76.59999999999999</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="38" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>James Madison</t>
         </is>
       </c>
       <c r="B28" s="38" t="n">
-        <v>73.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="C28" s="38" t="n">
-        <v>72.7</v>
+        <v>73.5</v>
       </c>
       <c r="D28" s="38" t="n">
-        <v>72.5</v>
+        <v>74.2</v>
       </c>
       <c r="E28" s="38" t="n">
-        <v>73</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="F28" s="38" t="n">
         <v>76.5</v>
       </c>
+      <c r="G28" s="38" t="n">
+        <v>76.59999999999999</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="38" t="inlineStr">
         <is>
-          <t>James Madison</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="B29" s="38" t="n">
-        <v>67.8</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="C29" s="38" t="n">
-        <v>73.5</v>
+        <v>72.7</v>
       </c>
       <c r="D29" s="38" t="n">
-        <v>74.2</v>
+        <v>72.5</v>
       </c>
       <c r="E29" s="38" t="n">
-        <v>76.09999999999999</v>
+        <v>73</v>
       </c>
       <c r="F29" s="38" t="n">
         <v>76.5</v>
       </c>
+      <c r="G29" s="38" t="n">
+        <v>76.5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="38" t="inlineStr">
@@ -37369,6 +37471,9 @@
       <c r="F30" s="38" t="n">
         <v>76.3</v>
       </c>
+      <c r="G30" s="38" t="n">
+        <v>76.3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="38" t="inlineStr">
@@ -37391,6 +37496,9 @@
       <c r="F31" s="38" t="n">
         <v>76.2</v>
       </c>
+      <c r="G31" s="38" t="n">
+        <v>76.2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
@@ -37413,6 +37521,9 @@
       <c r="F32" s="38" t="n">
         <v>76.09999999999999</v>
       </c>
+      <c r="G32" s="38" t="n">
+        <v>76.09999999999999</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="38" t="inlineStr">
@@ -37435,6 +37546,9 @@
       <c r="F33" s="38" t="n">
         <v>75.2</v>
       </c>
+      <c r="G33" s="38" t="n">
+        <v>75.3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="38" t="inlineStr">
@@ -37457,6 +37571,9 @@
       <c r="F34" s="38" t="n">
         <v>75.2</v>
       </c>
+      <c r="G34" s="38" t="n">
+        <v>75.2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="38" t="inlineStr">
@@ -37479,6 +37596,9 @@
       <c r="F35" s="38" t="n">
         <v>75.09999999999999</v>
       </c>
+      <c r="G35" s="38" t="n">
+        <v>75.09999999999999</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="38" t="inlineStr">
@@ -37501,6 +37621,9 @@
       <c r="F36" s="38" t="n">
         <v>74.8</v>
       </c>
+      <c r="G36" s="38" t="n">
+        <v>74.8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="38" t="inlineStr">
@@ -37523,6 +37646,9 @@
       <c r="F37" s="38" t="n">
         <v>73.7</v>
       </c>
+      <c r="G37" s="38" t="n">
+        <v>73.8</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="38" t="inlineStr">
@@ -37545,6 +37671,9 @@
       <c r="F38" s="38" t="n">
         <v>73.7</v>
       </c>
+      <c r="G38" s="38" t="n">
+        <v>73.7</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="38" t="inlineStr">
@@ -37567,6 +37696,9 @@
       <c r="F39" s="38" t="n">
         <v>73.09999999999999</v>
       </c>
+      <c r="G39" s="38" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="38" t="inlineStr">
@@ -37589,6 +37721,9 @@
       <c r="F40" s="38" t="n">
         <v>73.09999999999999</v>
       </c>
+      <c r="G40" s="38" t="n">
+        <v>73.09999999999999</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="38" t="inlineStr">
@@ -37611,6 +37746,9 @@
       <c r="F41" s="38" t="n">
         <v>72.90000000000001</v>
       </c>
+      <c r="G41" s="38" t="n">
+        <v>72.90000000000001</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="38" t="inlineStr">
@@ -37633,6 +37771,9 @@
       <c r="F42" s="38" t="n">
         <v>72.8</v>
       </c>
+      <c r="G42" s="38" t="n">
+        <v>72.8</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
@@ -37655,6 +37796,9 @@
       <c r="F43" s="38" t="n">
         <v>72.09999999999999</v>
       </c>
+      <c r="G43" s="38" t="n">
+        <v>72.09999999999999</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="38" t="inlineStr">
@@ -37677,6 +37821,9 @@
       <c r="F44" s="38" t="n">
         <v>71.5</v>
       </c>
+      <c r="G44" s="38" t="n">
+        <v>71.5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="38" t="inlineStr">
@@ -37699,6 +37846,9 @@
       <c r="F45" s="38" t="n">
         <v>71.40000000000001</v>
       </c>
+      <c r="G45" s="38" t="n">
+        <v>71.40000000000001</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="38" t="inlineStr">
@@ -37721,6 +37871,9 @@
       <c r="F46" s="38" t="n">
         <v>71.3</v>
       </c>
+      <c r="G46" s="38" t="n">
+        <v>71.3</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="38" t="inlineStr">
@@ -37743,6 +37896,9 @@
       <c r="F47" s="38" t="n">
         <v>71.09999999999999</v>
       </c>
+      <c r="G47" s="38" t="n">
+        <v>71.09999999999999</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="38" t="inlineStr">
@@ -37765,6 +37921,9 @@
       <c r="F48" s="38" t="n">
         <v>71</v>
       </c>
+      <c r="G48" s="38" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="38" t="inlineStr">
@@ -37787,6 +37946,9 @@
       <c r="F49" s="38" t="n">
         <v>70.3</v>
       </c>
+      <c r="G49" s="38" t="n">
+        <v>70.3</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="38" t="inlineStr">
@@ -37809,6 +37971,9 @@
       <c r="F50" s="38" t="n">
         <v>70.2</v>
       </c>
+      <c r="G50" s="38" t="n">
+        <v>70.2</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="38" t="inlineStr">
@@ -37831,6 +37996,9 @@
       <c r="F51" s="38" t="n">
         <v>69.7</v>
       </c>
+      <c r="G51" s="38" t="n">
+        <v>69.7</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="38" t="inlineStr">
@@ -37853,6 +38021,9 @@
       <c r="F52" s="38" t="n">
         <v>69.5</v>
       </c>
+      <c r="G52" s="38" t="n">
+        <v>69.5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="38" t="inlineStr">
@@ -37875,6 +38046,9 @@
       <c r="F53" s="38" t="n">
         <v>69.3</v>
       </c>
+      <c r="G53" s="38" t="n">
+        <v>69.3</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="38" t="inlineStr">
@@ -37897,6 +38071,9 @@
       <c r="F54" s="38" t="n">
         <v>68.5</v>
       </c>
+      <c r="G54" s="38" t="n">
+        <v>68.5</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="38" t="inlineStr">
@@ -37919,6 +38096,9 @@
       <c r="F55" s="38" t="n">
         <v>68.3</v>
       </c>
+      <c r="G55" s="38" t="n">
+        <v>68.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="38" t="inlineStr">
@@ -37941,6 +38121,9 @@
       <c r="F56" s="38" t="n">
         <v>68.2</v>
       </c>
+      <c r="G56" s="38" t="n">
+        <v>68.2</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="38" t="inlineStr">
@@ -37963,6 +38146,9 @@
       <c r="F57" s="38" t="n">
         <v>67.3</v>
       </c>
+      <c r="G57" s="38" t="n">
+        <v>67.3</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="38" t="inlineStr">
@@ -37985,6 +38171,9 @@
       <c r="F58" s="38" t="n">
         <v>67</v>
       </c>
+      <c r="G58" s="38" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="38" t="inlineStr">
@@ -38007,6 +38196,9 @@
       <c r="F59" s="38" t="n">
         <v>66.90000000000001</v>
       </c>
+      <c r="G59" s="38" t="n">
+        <v>66.90000000000001</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="38" t="inlineStr">
@@ -38029,6 +38221,9 @@
       <c r="F60" s="38" t="n">
         <v>66.40000000000001</v>
       </c>
+      <c r="G60" s="38" t="n">
+        <v>66.40000000000001</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="38" t="inlineStr">
@@ -38051,6 +38246,9 @@
       <c r="F61" s="38" t="n">
         <v>65.8</v>
       </c>
+      <c r="G61" s="38" t="n">
+        <v>65.8</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="38" t="inlineStr">
@@ -38073,6 +38271,9 @@
       <c r="F62" s="38" t="n">
         <v>65.59999999999999</v>
       </c>
+      <c r="G62" s="38" t="n">
+        <v>65.7</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="38" t="inlineStr">
@@ -38095,6 +38296,9 @@
       <c r="F63" s="38" t="n">
         <v>65.2</v>
       </c>
+      <c r="G63" s="38" t="n">
+        <v>65.2</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="38" t="inlineStr">
@@ -38117,6 +38321,9 @@
       <c r="F64" s="38" t="n">
         <v>65.09999999999999</v>
       </c>
+      <c r="G64" s="38" t="n">
+        <v>65.09999999999999</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="38" t="inlineStr">
@@ -38139,6 +38346,9 @@
       <c r="F65" s="38" t="n">
         <v>65</v>
       </c>
+      <c r="G65" s="38" t="n">
+        <v>65.09999999999999</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="38" t="inlineStr">
@@ -38161,6 +38371,9 @@
       <c r="F66" s="38" t="n">
         <v>64.7</v>
       </c>
+      <c r="G66" s="38" t="n">
+        <v>64.7</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="38" t="inlineStr">
@@ -38183,6 +38396,9 @@
       <c r="F67" s="38" t="n">
         <v>64.7</v>
       </c>
+      <c r="G67" s="38" t="n">
+        <v>64.7</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="38" t="inlineStr">
@@ -38205,6 +38421,9 @@
       <c r="F68" s="38" t="n">
         <v>64.5</v>
       </c>
+      <c r="G68" s="38" t="n">
+        <v>64.5</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="38" t="inlineStr">
@@ -38227,6 +38446,9 @@
       <c r="F69" s="38" t="n">
         <v>64.09999999999999</v>
       </c>
+      <c r="G69" s="38" t="n">
+        <v>64.09999999999999</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="38" t="inlineStr">
@@ -38249,6 +38471,9 @@
       <c r="F70" s="38" t="n">
         <v>63.9</v>
       </c>
+      <c r="G70" s="38" t="n">
+        <v>63.9</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="38" t="inlineStr">
@@ -38271,6 +38496,9 @@
       <c r="F71" s="38" t="n">
         <v>63.6</v>
       </c>
+      <c r="G71" s="38" t="n">
+        <v>63.7</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="38" t="inlineStr">
@@ -38293,6 +38521,9 @@
       <c r="F72" s="38" t="n">
         <v>63.6</v>
       </c>
+      <c r="G72" s="38" t="n">
+        <v>63.6</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="38" t="inlineStr">
@@ -38315,6 +38546,9 @@
       <c r="F73" s="38" t="n">
         <v>62.6</v>
       </c>
+      <c r="G73" s="38" t="n">
+        <v>62.6</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="38" t="inlineStr">
@@ -38337,6 +38571,9 @@
       <c r="F74" s="38" t="n">
         <v>62.5</v>
       </c>
+      <c r="G74" s="38" t="n">
+        <v>62.6</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="38" t="inlineStr">
@@ -38359,6 +38596,9 @@
       <c r="F75" s="38" t="n">
         <v>62.5</v>
       </c>
+      <c r="G75" s="38" t="n">
+        <v>62.5</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="38" t="inlineStr">
@@ -38381,6 +38621,9 @@
       <c r="F76" s="38" t="n">
         <v>62.2</v>
       </c>
+      <c r="G76" s="38" t="n">
+        <v>62.2</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="38" t="inlineStr">
@@ -38403,6 +38646,9 @@
       <c r="F77" s="38" t="n">
         <v>62</v>
       </c>
+      <c r="G77" s="38" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="38" t="inlineStr">
@@ -38425,6 +38671,9 @@
       <c r="F78" s="38" t="n">
         <v>61.7</v>
       </c>
+      <c r="G78" s="38" t="n">
+        <v>61.7</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="38" t="inlineStr">
@@ -38447,6 +38696,9 @@
       <c r="F79" s="38" t="n">
         <v>61.7</v>
       </c>
+      <c r="G79" s="38" t="n">
+        <v>61.7</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="38" t="inlineStr">
@@ -38469,6 +38721,9 @@
       <c r="F80" s="38" t="n">
         <v>61.6</v>
       </c>
+      <c r="G80" s="38" t="n">
+        <v>61.7</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="38" t="inlineStr">
@@ -38491,6 +38746,9 @@
       <c r="F81" s="38" t="n">
         <v>61.6</v>
       </c>
+      <c r="G81" s="38" t="n">
+        <v>61.6</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="38" t="inlineStr">
@@ -38513,6 +38771,9 @@
       <c r="F82" s="38" t="n">
         <v>61.4</v>
       </c>
+      <c r="G82" s="38" t="n">
+        <v>61.5</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="38" t="inlineStr">
@@ -38535,6 +38796,9 @@
       <c r="F83" s="38" t="n">
         <v>61.4</v>
       </c>
+      <c r="G83" s="38" t="n">
+        <v>61.4</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="38" t="inlineStr">
@@ -38557,6 +38821,9 @@
       <c r="F84" s="38" t="n">
         <v>61.3</v>
       </c>
+      <c r="G84" s="38" t="n">
+        <v>61.3</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="38" t="inlineStr">
@@ -38579,6 +38846,9 @@
       <c r="F85" s="38" t="n">
         <v>60.7</v>
       </c>
+      <c r="G85" s="38" t="n">
+        <v>60.7</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="38" t="inlineStr">
@@ -38601,6 +38871,9 @@
       <c r="F86" s="38" t="n">
         <v>60.6</v>
       </c>
+      <c r="G86" s="38" t="n">
+        <v>60.6</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="38" t="inlineStr">
@@ -38623,6 +38896,9 @@
       <c r="F87" s="38" t="n">
         <v>59.7</v>
       </c>
+      <c r="G87" s="38" t="n">
+        <v>59.7</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="38" t="inlineStr">
@@ -38645,6 +38921,9 @@
       <c r="F88" s="38" t="n">
         <v>59.6</v>
       </c>
+      <c r="G88" s="38" t="n">
+        <v>59.6</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="38" t="inlineStr">
@@ -38667,6 +38946,9 @@
       <c r="F89" s="38" t="n">
         <v>59.5</v>
       </c>
+      <c r="G89" s="38" t="n">
+        <v>59.5</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="38" t="inlineStr">
@@ -38689,92 +38971,107 @@
       <c r="F90" s="38" t="n">
         <v>59.3</v>
       </c>
+      <c r="G90" s="38" t="n">
+        <v>59.3</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="38" t="inlineStr">
         <is>
-          <t>Florida Atlantic</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="B91" s="38" t="n">
-        <v>50.4</v>
+        <v>56.7</v>
       </c>
       <c r="C91" s="38" t="n">
-        <v>53.3</v>
+        <v>57.9</v>
       </c>
       <c r="D91" s="38" t="n">
-        <v>54.2</v>
+        <v>57</v>
       </c>
       <c r="E91" s="38" t="n">
-        <v>55.8</v>
+        <v>56.5</v>
       </c>
       <c r="F91" s="38" t="n">
         <v>58.6</v>
       </c>
+      <c r="G91" s="38" t="n">
+        <v>58.6</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="38" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Ohio</t>
         </is>
       </c>
       <c r="B92" s="38" t="n">
-        <v>56.7</v>
+        <v>58.8</v>
       </c>
       <c r="C92" s="38" t="n">
-        <v>57.9</v>
+        <v>59</v>
       </c>
       <c r="D92" s="38" t="n">
-        <v>57</v>
+        <v>58.2</v>
       </c>
       <c r="E92" s="38" t="n">
-        <v>56.5</v>
+        <v>59.6</v>
       </c>
       <c r="F92" s="38" t="n">
-        <v>58.6</v>
+        <v>58.4</v>
+      </c>
+      <c r="G92" s="38" t="n">
+        <v>58.5</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="38" t="inlineStr">
         <is>
-          <t>Ohio</t>
+          <t>California</t>
         </is>
       </c>
       <c r="B93" s="38" t="n">
-        <v>58.8</v>
+        <v>60.4</v>
       </c>
       <c r="C93" s="38" t="n">
-        <v>59</v>
+        <v>59.4</v>
       </c>
       <c r="D93" s="38" t="n">
-        <v>58.2</v>
+        <v>60.2</v>
       </c>
       <c r="E93" s="38" t="n">
-        <v>59.6</v>
+        <v>59.2</v>
       </c>
       <c r="F93" s="38" t="n">
         <v>58.4</v>
       </c>
+      <c r="G93" s="38" t="n">
+        <v>58.4</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="38" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>Florida Atlantic</t>
         </is>
       </c>
       <c r="B94" s="38" t="n">
-        <v>60.4</v>
+        <v>50.4</v>
       </c>
       <c r="C94" s="38" t="n">
-        <v>59.4</v>
+        <v>53.3</v>
       </c>
       <c r="D94" s="38" t="n">
-        <v>60.2</v>
+        <v>54.2</v>
       </c>
       <c r="E94" s="38" t="n">
-        <v>59.2</v>
+        <v>55.8</v>
       </c>
       <c r="F94" s="38" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="G94" s="38" t="n">
         <v>58.4</v>
       </c>
     </row>
@@ -38799,6 +39096,9 @@
       <c r="F95" s="38" t="n">
         <v>58</v>
       </c>
+      <c r="G95" s="38" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="38" t="inlineStr">
@@ -38821,6 +39121,9 @@
       <c r="F96" s="38" t="n">
         <v>57.5</v>
       </c>
+      <c r="G96" s="38" t="n">
+        <v>57.5</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="38" t="inlineStr">
@@ -38843,6 +39146,9 @@
       <c r="F97" s="38" t="n">
         <v>57.4</v>
       </c>
+      <c r="G97" s="38" t="n">
+        <v>57.4</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="38" t="inlineStr">
@@ -38865,6 +39171,9 @@
       <c r="F98" s="38" t="n">
         <v>57.2</v>
       </c>
+      <c r="G98" s="38" t="n">
+        <v>57.2</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="38" t="inlineStr">
@@ -38887,6 +39196,9 @@
       <c r="F99" s="38" t="n">
         <v>56.8</v>
       </c>
+      <c r="G99" s="38" t="n">
+        <v>56.9</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="38" t="inlineStr">
@@ -38909,6 +39221,9 @@
       <c r="F100" s="38" t="n">
         <v>56.7</v>
       </c>
+      <c r="G100" s="38" t="n">
+        <v>56.7</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="38" t="inlineStr">
@@ -38931,6 +39246,9 @@
       <c r="F101" s="38" t="n">
         <v>56.5</v>
       </c>
+      <c r="G101" s="38" t="n">
+        <v>56.6</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="38" t="inlineStr">
@@ -38953,6 +39271,9 @@
       <c r="F102" s="38" t="n">
         <v>56.1</v>
       </c>
+      <c r="G102" s="38" t="n">
+        <v>56.1</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="38" t="inlineStr">
@@ -38975,137 +39296,158 @@
       <c r="F103" s="38" t="n">
         <v>56</v>
       </c>
+      <c r="G103" s="38" t="n">
+        <v>56.1</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="38" t="inlineStr">
         <is>
-          <t>Georgia State</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="B104" s="38" t="n">
-        <v>47.4</v>
+        <v>53.1</v>
       </c>
       <c r="C104" s="38" t="n">
-        <v>49.7</v>
+        <v>53.7</v>
       </c>
       <c r="D104" s="38" t="n">
-        <v>49.6</v>
+        <v>54.6</v>
       </c>
       <c r="E104" s="38" t="n">
-        <v>51.2</v>
+        <v>54.2</v>
       </c>
       <c r="F104" s="38" t="n">
-        <v>55.9</v>
+        <v>54.2</v>
+      </c>
+      <c r="G104" s="38" t="n">
+        <v>56</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="38" t="inlineStr">
         <is>
-          <t>Delaware</t>
+          <t>Georgia State</t>
         </is>
       </c>
       <c r="B105" s="38" t="n">
-        <v>56.1</v>
+        <v>47.4</v>
       </c>
       <c r="C105" s="38" t="n">
-        <v>57.4</v>
+        <v>49.7</v>
       </c>
       <c r="D105" s="38" t="n">
-        <v>57.8</v>
+        <v>49.6</v>
       </c>
       <c r="E105" s="38" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="F105" s="38" t="n">
         <v>55.9</v>
       </c>
-      <c r="F105" s="38" t="n">
-        <v>55.5</v>
+      <c r="G105" s="38" t="n">
+        <v>55.9</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="38" t="inlineStr">
         <is>
-          <t>Florida International</t>
+          <t>Delaware</t>
         </is>
       </c>
       <c r="B106" s="38" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="C106" s="38" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="D106" s="38" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="E106" s="38" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="F106" s="38" t="n">
         <v>55.5</v>
       </c>
-      <c r="C106" s="38" t="n">
-        <v>56.4</v>
-      </c>
-      <c r="D106" s="38" t="n">
+      <c r="G106" s="38" t="n">
         <v>55.5</v>
-      </c>
-      <c r="E106" s="38" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="F106" s="38" t="n">
-        <v>55.3</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="38" t="inlineStr">
         <is>
-          <t>UConn</t>
+          <t>Florida International</t>
         </is>
       </c>
       <c r="B107" s="38" t="n">
-        <v>57.3</v>
+        <v>55.5</v>
       </c>
       <c r="C107" s="38" t="n">
-        <v>54.4</v>
+        <v>56.4</v>
       </c>
       <c r="D107" s="38" t="n">
-        <v>57</v>
+        <v>55.5</v>
       </c>
       <c r="E107" s="38" t="n">
-        <v>54.2</v>
+        <v>55.6</v>
       </c>
       <c r="F107" s="38" t="n">
-        <v>54.9</v>
+        <v>55.3</v>
+      </c>
+      <c r="G107" s="38" t="n">
+        <v>55.3</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="38" t="inlineStr">
         <is>
-          <t>Central Michigan</t>
+          <t>UConn</t>
         </is>
       </c>
       <c r="B108" s="38" t="n">
-        <v>55</v>
+        <v>57.3</v>
       </c>
       <c r="C108" s="38" t="n">
-        <v>53.8</v>
+        <v>54.4</v>
       </c>
       <c r="D108" s="38" t="n">
-        <v>54.6</v>
+        <v>57</v>
       </c>
       <c r="E108" s="38" t="n">
-        <v>53</v>
+        <v>54.2</v>
       </c>
       <c r="F108" s="38" t="n">
-        <v>54.5</v>
+        <v>54.9</v>
+      </c>
+      <c r="G108" s="38" t="n">
+        <v>54.9</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="38" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Central Michigan</t>
         </is>
       </c>
       <c r="B109" s="38" t="n">
-        <v>53.1</v>
+        <v>55</v>
       </c>
       <c r="C109" s="38" t="n">
-        <v>53.7</v>
+        <v>53.8</v>
       </c>
       <c r="D109" s="38" t="n">
         <v>54.6</v>
       </c>
       <c r="E109" s="38" t="n">
-        <v>54.2</v>
+        <v>53</v>
       </c>
       <c r="F109" s="38" t="n">
-        <v>54.2</v>
+        <v>54.5</v>
+      </c>
+      <c r="G109" s="38" t="n">
+        <v>54.5</v>
       </c>
     </row>
     <row r="110">
@@ -39129,6 +39471,9 @@
       <c r="F110" s="38" t="n">
         <v>53.9</v>
       </c>
+      <c r="G110" s="38" t="n">
+        <v>53.9</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="38" t="inlineStr">
@@ -39151,6 +39496,9 @@
       <c r="F111" s="38" t="n">
         <v>53.8</v>
       </c>
+      <c r="G111" s="38" t="n">
+        <v>53.7</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="38" t="inlineStr">
@@ -39173,6 +39521,9 @@
       <c r="F112" s="38" t="n">
         <v>53.5</v>
       </c>
+      <c r="G112" s="38" t="n">
+        <v>53.5</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="38" t="inlineStr">
@@ -39195,6 +39546,9 @@
       <c r="F113" s="38" t="n">
         <v>52.9</v>
       </c>
+      <c r="G113" s="38" t="n">
+        <v>52.9</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="38" t="inlineStr">
@@ -39217,6 +39571,9 @@
       <c r="F114" s="38" t="n">
         <v>52.6</v>
       </c>
+      <c r="G114" s="38" t="n">
+        <v>52.7</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="38" t="inlineStr">
@@ -39239,6 +39596,9 @@
       <c r="F115" s="38" t="n">
         <v>52.5</v>
       </c>
+      <c r="G115" s="38" t="n">
+        <v>52.5</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="38" t="inlineStr">
@@ -39261,6 +39621,9 @@
       <c r="F116" s="38" t="n">
         <v>52.4</v>
       </c>
+      <c r="G116" s="38" t="n">
+        <v>52.4</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="38" t="inlineStr">
@@ -39283,6 +39646,9 @@
       <c r="F117" s="38" t="n">
         <v>52</v>
       </c>
+      <c r="G117" s="38" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="38" t="inlineStr">
@@ -39305,6 +39671,9 @@
       <c r="F118" s="38" t="n">
         <v>51.9</v>
       </c>
+      <c r="G118" s="38" t="n">
+        <v>51.9</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="38" t="inlineStr">
@@ -39327,6 +39696,9 @@
       <c r="F119" s="38" t="n">
         <v>51.8</v>
       </c>
+      <c r="G119" s="38" t="n">
+        <v>51.8</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="38" t="inlineStr">
@@ -39349,114 +39721,132 @@
       <c r="F120" s="38" t="n">
         <v>51.6</v>
       </c>
+      <c r="G120" s="38" t="n">
+        <v>51.6</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="38" t="inlineStr">
         <is>
-          <t>Southern Miss</t>
+          <t>San José State</t>
         </is>
       </c>
       <c r="B121" s="38" t="n">
-        <v>54.4</v>
+        <v>51.7</v>
       </c>
       <c r="C121" s="38" t="n">
-        <v>52.7</v>
+        <v>51.6</v>
       </c>
       <c r="D121" s="38" t="n">
-        <v>50.1</v>
+        <v>50.5</v>
       </c>
       <c r="E121" s="38" t="n">
-        <v>51.2</v>
+        <v>50.4</v>
       </c>
       <c r="F121" s="38" t="n">
-        <v>51.2</v>
+        <v>51.1</v>
+      </c>
+      <c r="G121" s="38" t="n">
+        <v>51.1</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="38" t="inlineStr">
         <is>
-          <t>San José State</t>
+          <t>Marshall</t>
         </is>
       </c>
       <c r="B122" s="38" t="n">
-        <v>51.7</v>
+        <v>52.1</v>
       </c>
       <c r="C122" s="38" t="n">
-        <v>51.6</v>
+        <v>51.8</v>
       </c>
       <c r="D122" s="38" t="n">
-        <v>50.5</v>
+        <v>52.5</v>
       </c>
       <c r="E122" s="38" t="n">
-        <v>50.4</v>
+        <v>51.5</v>
       </c>
       <c r="F122" s="38" t="n">
-        <v>51.1</v>
+        <v>51</v>
+      </c>
+      <c r="G122" s="38" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="38" t="inlineStr">
         <is>
-          <t>Marshall</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="B123" s="38" t="n">
-        <v>52.1</v>
+        <v>51.5</v>
       </c>
       <c r="C123" s="38" t="n">
-        <v>51.8</v>
+        <v>50.6</v>
       </c>
       <c r="D123" s="38" t="n">
-        <v>52.5</v>
+        <v>49.7</v>
       </c>
       <c r="E123" s="38" t="n">
-        <v>51.5</v>
+        <v>48.8</v>
       </c>
       <c r="F123" s="38" t="n">
-        <v>51</v>
+        <v>50.2</v>
+      </c>
+      <c r="G123" s="38" t="n">
+        <v>50.2</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="38" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Eastern Michigan</t>
         </is>
       </c>
       <c r="B124" s="38" t="n">
-        <v>51.5</v>
+        <v>47.2</v>
       </c>
       <c r="C124" s="38" t="n">
-        <v>50.6</v>
+        <v>46.4</v>
       </c>
       <c r="D124" s="38" t="n">
-        <v>49.7</v>
+        <v>44.8</v>
       </c>
       <c r="E124" s="38" t="n">
-        <v>48.8</v>
+        <v>47.4</v>
       </c>
       <c r="F124" s="38" t="n">
-        <v>50.2</v>
+        <v>49.4</v>
+      </c>
+      <c r="G124" s="38" t="n">
+        <v>49.4</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="38" t="inlineStr">
         <is>
-          <t>Eastern Michigan</t>
+          <t>Southern Miss</t>
         </is>
       </c>
       <c r="B125" s="38" t="n">
-        <v>47.2</v>
+        <v>54.4</v>
       </c>
       <c r="C125" s="38" t="n">
-        <v>46.4</v>
+        <v>52.7</v>
       </c>
       <c r="D125" s="38" t="n">
-        <v>44.8</v>
+        <v>50.1</v>
       </c>
       <c r="E125" s="38" t="n">
-        <v>47.4</v>
+        <v>51.2</v>
       </c>
       <c r="F125" s="38" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="G125" s="38" t="n">
         <v>49.4</v>
       </c>
     </row>
@@ -39481,6 +39871,9 @@
       <c r="F126" s="38" t="n">
         <v>49.2</v>
       </c>
+      <c r="G126" s="38" t="n">
+        <v>49.2</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="38" t="inlineStr">
@@ -39503,6 +39896,9 @@
       <c r="F127" s="38" t="n">
         <v>48.8</v>
       </c>
+      <c r="G127" s="38" t="n">
+        <v>48.8</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="38" t="inlineStr">
@@ -39525,6 +39921,9 @@
       <c r="F128" s="38" t="n">
         <v>47</v>
       </c>
+      <c r="G128" s="38" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="38" t="inlineStr">
@@ -39547,6 +39946,9 @@
       <c r="F129" s="38" t="n">
         <v>46.2</v>
       </c>
+      <c r="G129" s="38" t="n">
+        <v>46.2</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="38" t="inlineStr">
@@ -39569,6 +39971,9 @@
       <c r="F130" s="38" t="n">
         <v>45.8</v>
       </c>
+      <c r="G130" s="38" t="n">
+        <v>45.8</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="38" t="inlineStr">
@@ -39591,6 +39996,9 @@
       <c r="F131" s="38" t="n">
         <v>45.3</v>
       </c>
+      <c r="G131" s="38" t="n">
+        <v>45.4</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="38" t="inlineStr">
@@ -39613,6 +40021,9 @@
       <c r="F132" s="38" t="n">
         <v>44.1</v>
       </c>
+      <c r="G132" s="38" t="n">
+        <v>44.1</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="38" t="inlineStr">
@@ -39635,6 +40046,9 @@
       <c r="F133" s="38" t="n">
         <v>42.9</v>
       </c>
+      <c r="G133" s="38" t="n">
+        <v>42.9</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="38" t="inlineStr">
@@ -39657,6 +40071,9 @@
       <c r="F134" s="38" t="n">
         <v>42.6</v>
       </c>
+      <c r="G134" s="38" t="n">
+        <v>42.6</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="38" t="inlineStr">
@@ -39679,6 +40096,9 @@
       <c r="F135" s="38" t="n">
         <v>42.5</v>
       </c>
+      <c r="G135" s="38" t="n">
+        <v>42.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="38" t="inlineStr">
@@ -39701,6 +40121,9 @@
       <c r="F136" s="38" t="n">
         <v>40.5</v>
       </c>
+      <c r="G136" s="38" t="n">
+        <v>40.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="38" t="inlineStr">
@@ -39723,6 +40146,9 @@
       <c r="F137" s="38" t="n">
         <v>40.1</v>
       </c>
+      <c r="G137" s="38" t="n">
+        <v>40.2</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="38" t="inlineStr">
@@ -39745,6 +40171,9 @@
       <c r="F138" s="38" t="n">
         <v>39.5</v>
       </c>
+      <c r="G138" s="38" t="n">
+        <v>39.3</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="38" t="inlineStr">
@@ -39765,6 +40194,9 @@
         <v>37.3</v>
       </c>
       <c r="F139" s="38" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="G139" s="38" t="n">
         <v>37.2</v>
       </c>
     </row>
@@ -43324,10 +43756,10 @@
         <v>1521.6</v>
       </c>
       <c r="F57" s="38" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G57" s="45" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="58">
@@ -43783,10 +44215,10 @@
         <v>1528.5</v>
       </c>
       <c r="F74" s="38" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G74" s="38" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="75">
@@ -44467,34 +44899,34 @@
     <row r="100">
       <c r="A100" s="38" t="inlineStr">
         <is>
-          <t>UC Davis</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="B100" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C100" s="38" t="n">
-        <v>-0.18</v>
+        <v>-0.17</v>
       </c>
       <c r="D100" s="38" t="n">
         <v>95</v>
       </c>
       <c r="E100" s="38" t="n">
-        <v>1449.9</v>
+        <v>1535.2</v>
       </c>
       <c r="F100" s="38" t="n">
-        <v>128</v>
-      </c>
-      <c r="G100" s="45" t="n">
-        <v>33</v>
+        <v>75</v>
+      </c>
+      <c r="G100" s="38" t="n">
+        <v>-20</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="38" t="inlineStr">
         <is>
-          <t>Idaho</t>
+          <t>UC Davis</t>
         </is>
       </c>
       <c r="B101" s="38" t="inlineStr">
@@ -44509,19 +44941,19 @@
         <v>96</v>
       </c>
       <c r="E101" s="38" t="n">
-        <v>1459.1</v>
+        <v>1449.9</v>
       </c>
       <c r="F101" s="38" t="n">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="G101" s="45" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="38" t="inlineStr">
         <is>
-          <t>Northern Iowa</t>
+          <t>Idaho</t>
         </is>
       </c>
       <c r="B102" s="38" t="inlineStr">
@@ -44536,51 +44968,51 @@
         <v>97</v>
       </c>
       <c r="E102" s="38" t="n">
-        <v>1411.5</v>
+        <v>1459.1</v>
       </c>
       <c r="F102" s="38" t="n">
-        <v>203</v>
+        <v>119</v>
       </c>
       <c r="G102" s="45" t="n">
-        <v>106</v>
+        <v>22</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="38" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Northern Iowa</t>
         </is>
       </c>
       <c r="B103" s="38" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C103" s="38" t="n">
-        <v>-0.19</v>
+        <v>-0.18</v>
       </c>
       <c r="D103" s="38" t="n">
         <v>98</v>
       </c>
       <c r="E103" s="38" t="n">
-        <v>1426.3</v>
+        <v>1411.5</v>
       </c>
       <c r="F103" s="38" t="n">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="G103" s="45" t="n">
-        <v>71</v>
+        <v>105</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="38" t="inlineStr">
         <is>
-          <t>Utah Tech</t>
+          <t>Tulsa</t>
         </is>
       </c>
       <c r="B104" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C104" s="38" t="n">
@@ -44590,19 +45022,19 @@
         <v>99</v>
       </c>
       <c r="E104" s="38" t="n">
-        <v>1439.6</v>
+        <v>1426.3</v>
       </c>
       <c r="F104" s="38" t="n">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="G104" s="45" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="38" t="inlineStr">
         <is>
-          <t>Eastern Washington</t>
+          <t>Utah Tech</t>
         </is>
       </c>
       <c r="B105" s="38" t="inlineStr">
@@ -44611,25 +45043,25 @@
         </is>
       </c>
       <c r="C105" s="38" t="n">
-        <v>-0.2</v>
+        <v>-0.19</v>
       </c>
       <c r="D105" s="38" t="n">
         <v>100</v>
       </c>
       <c r="E105" s="38" t="n">
-        <v>1433.4</v>
+        <v>1439.6</v>
       </c>
       <c r="F105" s="38" t="n">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="G105" s="45" t="n">
-        <v>59</v>
+        <v>48</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="38" t="inlineStr">
         <is>
-          <t>William &amp; Mary</t>
+          <t>Eastern Washington</t>
         </is>
       </c>
       <c r="B106" s="38" t="inlineStr">
@@ -44644,19 +45076,19 @@
         <v>101</v>
       </c>
       <c r="E106" s="38" t="n">
-        <v>1440</v>
+        <v>1433.4</v>
       </c>
       <c r="F106" s="38" t="n">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="G106" s="45" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="38" t="inlineStr">
         <is>
-          <t>McNeese</t>
+          <t>William &amp; Mary</t>
         </is>
       </c>
       <c r="B107" s="38" t="inlineStr">
@@ -44665,25 +45097,25 @@
         </is>
       </c>
       <c r="C107" s="38" t="n">
-        <v>-0.21</v>
+        <v>-0.2</v>
       </c>
       <c r="D107" s="38" t="n">
         <v>102</v>
       </c>
       <c r="E107" s="38" t="n">
-        <v>1417.4</v>
+        <v>1440</v>
       </c>
       <c r="F107" s="38" t="n">
-        <v>186</v>
+        <v>147</v>
       </c>
       <c r="G107" s="45" t="n">
-        <v>84</v>
+        <v>45</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="38" t="inlineStr">
         <is>
-          <t>Austin Peay</t>
+          <t>McNeese</t>
         </is>
       </c>
       <c r="B108" s="38" t="inlineStr">
@@ -44692,25 +45124,25 @@
         </is>
       </c>
       <c r="C108" s="38" t="n">
-        <v>-0.23</v>
+        <v>-0.21</v>
       </c>
       <c r="D108" s="38" t="n">
         <v>103</v>
       </c>
       <c r="E108" s="38" t="n">
-        <v>1470.1</v>
+        <v>1417.4</v>
       </c>
       <c r="F108" s="38" t="n">
-        <v>109</v>
-      </c>
-      <c r="G108" s="38" t="n">
-        <v>6</v>
+        <v>186</v>
+      </c>
+      <c r="G108" s="45" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="38" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Austin Peay</t>
         </is>
       </c>
       <c r="B109" s="38" t="inlineStr">
@@ -44725,19 +45157,19 @@
         <v>104</v>
       </c>
       <c r="E109" s="38" t="n">
-        <v>1456.2</v>
+        <v>1470.1</v>
       </c>
       <c r="F109" s="38" t="n">
-        <v>122</v>
-      </c>
-      <c r="G109" s="45" t="n">
-        <v>18</v>
+        <v>109</v>
+      </c>
+      <c r="G109" s="38" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="38" t="inlineStr">
         <is>
-          <t>Furman</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="B110" s="38" t="inlineStr">
@@ -44746,30 +45178,30 @@
         </is>
       </c>
       <c r="C110" s="38" t="n">
-        <v>-0.25</v>
+        <v>-0.23</v>
       </c>
       <c r="D110" s="38" t="n">
         <v>105</v>
       </c>
       <c r="E110" s="38" t="n">
-        <v>1444.8</v>
+        <v>1456.2</v>
       </c>
       <c r="F110" s="38" t="n">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="G110" s="45" t="n">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="38" t="inlineStr">
         <is>
-          <t>Syracuse</t>
+          <t>Furman</t>
         </is>
       </c>
       <c r="B111" s="38" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C111" s="38" t="n">
@@ -44779,24 +45211,24 @@
         <v>106</v>
       </c>
       <c r="E111" s="38" t="n">
-        <v>1464.9</v>
+        <v>1444.8</v>
       </c>
       <c r="F111" s="38" t="n">
-        <v>113</v>
-      </c>
-      <c r="G111" s="38" t="n">
-        <v>7</v>
+        <v>139</v>
+      </c>
+      <c r="G111" s="45" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="38" t="inlineStr">
         <is>
-          <t>South Dakota</t>
+          <t>Syracuse</t>
         </is>
       </c>
       <c r="B112" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C112" s="38" t="n">
@@ -44806,24 +45238,24 @@
         <v>107</v>
       </c>
       <c r="E112" s="38" t="n">
-        <v>1445.5</v>
+        <v>1464.9</v>
       </c>
       <c r="F112" s="38" t="n">
-        <v>138</v>
-      </c>
-      <c r="G112" s="45" t="n">
-        <v>31</v>
+        <v>113</v>
+      </c>
+      <c r="G112" s="38" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="38" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>South Dakota</t>
         </is>
       </c>
       <c r="B113" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C113" s="38" t="n">
@@ -44833,24 +45265,24 @@
         <v>108</v>
       </c>
       <c r="E113" s="38" t="n">
-        <v>1447</v>
+        <v>1445.5</v>
       </c>
       <c r="F113" s="38" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G113" s="45" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="38" t="inlineStr">
         <is>
-          <t>Delaware State</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="B114" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C114" s="38" t="n">
@@ -44860,19 +45292,19 @@
         <v>109</v>
       </c>
       <c r="E114" s="38" t="n">
-        <v>1412.3</v>
+        <v>1447</v>
       </c>
       <c r="F114" s="38" t="n">
-        <v>199</v>
+        <v>134</v>
       </c>
       <c r="G114" s="45" t="n">
-        <v>90</v>
+        <v>25</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="38" t="inlineStr">
         <is>
-          <t>Grambling</t>
+          <t>Delaware State</t>
         </is>
       </c>
       <c r="B115" s="38" t="inlineStr">
@@ -44881,25 +45313,25 @@
         </is>
       </c>
       <c r="C115" s="38" t="n">
-        <v>-0.26</v>
+        <v>-0.25</v>
       </c>
       <c r="D115" s="38" t="n">
         <v>110</v>
       </c>
       <c r="E115" s="38" t="n">
-        <v>1429.6</v>
+        <v>1412.3</v>
       </c>
       <c r="F115" s="38" t="n">
-        <v>164</v>
+        <v>199</v>
       </c>
       <c r="G115" s="45" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="38" t="inlineStr">
         <is>
-          <t>Bucknell</t>
+          <t>Grambling</t>
         </is>
       </c>
       <c r="B116" s="38" t="inlineStr">
@@ -44914,19 +45346,19 @@
         <v>111</v>
       </c>
       <c r="E116" s="38" t="n">
-        <v>1431.1</v>
+        <v>1429.6</v>
       </c>
       <c r="F116" s="38" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="G116" s="45" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="38" t="inlineStr">
         <is>
-          <t>Northern Arizona</t>
+          <t>Bucknell</t>
         </is>
       </c>
       <c r="B117" s="38" t="inlineStr">
@@ -44941,19 +45373,19 @@
         <v>112</v>
       </c>
       <c r="E117" s="38" t="n">
-        <v>1447.5</v>
+        <v>1431.1</v>
       </c>
       <c r="F117" s="38" t="n">
-        <v>132</v>
+        <v>161</v>
       </c>
       <c r="G117" s="45" t="n">
-        <v>20</v>
+        <v>49</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="38" t="inlineStr">
         <is>
-          <t>Arkansas-Pine Bluff</t>
+          <t>Northern Arizona</t>
         </is>
       </c>
       <c r="B118" s="38" t="inlineStr">
@@ -44968,19 +45400,19 @@
         <v>113</v>
       </c>
       <c r="E118" s="38" t="n">
-        <v>1422.7</v>
+        <v>1447.5</v>
       </c>
       <c r="F118" s="38" t="n">
-        <v>176</v>
+        <v>132</v>
       </c>
       <c r="G118" s="45" t="n">
-        <v>63</v>
+        <v>19</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="38" t="inlineStr">
         <is>
-          <t>Southeast Missouri State</t>
+          <t>Arkansas-Pine Bluff</t>
         </is>
       </c>
       <c r="B119" s="38" t="inlineStr">
@@ -44989,25 +45421,25 @@
         </is>
       </c>
       <c r="C119" s="38" t="n">
-        <v>-0.27</v>
+        <v>-0.26</v>
       </c>
       <c r="D119" s="38" t="n">
         <v>114</v>
       </c>
       <c r="E119" s="38" t="n">
-        <v>1436.8</v>
+        <v>1422.7</v>
       </c>
       <c r="F119" s="38" t="n">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="G119" s="45" t="n">
-        <v>37</v>
+        <v>62</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="38" t="inlineStr">
         <is>
-          <t>Bryant</t>
+          <t>Southeast Missouri State</t>
         </is>
       </c>
       <c r="B120" s="38" t="inlineStr">
@@ -45016,30 +45448,30 @@
         </is>
       </c>
       <c r="C120" s="38" t="n">
-        <v>-0.28</v>
+        <v>-0.27</v>
       </c>
       <c r="D120" s="38" t="n">
         <v>115</v>
       </c>
       <c r="E120" s="38" t="n">
-        <v>1434.1</v>
+        <v>1436.8</v>
       </c>
       <c r="F120" s="38" t="n">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="G120" s="45" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="38" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Bryant</t>
         </is>
       </c>
       <c r="B121" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C121" s="38" t="n">
@@ -45049,24 +45481,24 @@
         <v>116</v>
       </c>
       <c r="E121" s="38" t="n">
-        <v>1489.6</v>
+        <v>1434.1</v>
       </c>
       <c r="F121" s="38" t="n">
-        <v>99</v>
-      </c>
-      <c r="G121" s="38" t="n">
-        <v>-17</v>
+        <v>156</v>
+      </c>
+      <c r="G121" s="45" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="38" t="inlineStr">
         <is>
-          <t>Southern Illinois</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="B122" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C122" s="38" t="n">
@@ -45076,19 +45508,19 @@
         <v>117</v>
       </c>
       <c r="E122" s="38" t="n">
-        <v>1436.5</v>
+        <v>1489.6</v>
       </c>
       <c r="F122" s="38" t="n">
-        <v>152</v>
-      </c>
-      <c r="G122" s="45" t="n">
-        <v>35</v>
+        <v>99</v>
+      </c>
+      <c r="G122" s="38" t="n">
+        <v>-18</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="38" t="inlineStr">
         <is>
-          <t>Morgan State</t>
+          <t>Southern Illinois</t>
         </is>
       </c>
       <c r="B123" s="38" t="inlineStr">
@@ -45097,25 +45529,25 @@
         </is>
       </c>
       <c r="C123" s="38" t="n">
-        <v>-0.29</v>
+        <v>-0.28</v>
       </c>
       <c r="D123" s="38" t="n">
         <v>118</v>
       </c>
       <c r="E123" s="38" t="n">
-        <v>1414.2</v>
+        <v>1436.5</v>
       </c>
       <c r="F123" s="38" t="n">
-        <v>193</v>
+        <v>152</v>
       </c>
       <c r="G123" s="45" t="n">
-        <v>75</v>
+        <v>34</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="38" t="inlineStr">
         <is>
-          <t>Eastern Illinois</t>
+          <t>Morgan State</t>
         </is>
       </c>
       <c r="B124" s="38" t="inlineStr">
@@ -45130,19 +45562,19 @@
         <v>119</v>
       </c>
       <c r="E124" s="38" t="n">
-        <v>1418.5</v>
+        <v>1414.2</v>
       </c>
       <c r="F124" s="38" t="n">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="G124" s="45" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="38" t="inlineStr">
         <is>
-          <t>Monmouth</t>
+          <t>Eastern Illinois</t>
         </is>
       </c>
       <c r="B125" s="38" t="inlineStr">
@@ -45151,30 +45583,30 @@
         </is>
       </c>
       <c r="C125" s="38" t="n">
-        <v>-0.3</v>
+        <v>-0.29</v>
       </c>
       <c r="D125" s="38" t="n">
         <v>120</v>
       </c>
       <c r="E125" s="38" t="n">
-        <v>1438.9</v>
+        <v>1418.5</v>
       </c>
       <c r="F125" s="38" t="n">
-        <v>150</v>
+        <v>184</v>
       </c>
       <c r="G125" s="45" t="n">
-        <v>30</v>
+        <v>64</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="38" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="B126" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C126" s="38" t="n">
@@ -45184,24 +45616,24 @@
         <v>121</v>
       </c>
       <c r="E126" s="38" t="n">
-        <v>1644.9</v>
+        <v>1438.9</v>
       </c>
       <c r="F126" s="38" t="n">
+        <v>150</v>
+      </c>
+      <c r="G126" s="45" t="n">
         <v>29</v>
-      </c>
-      <c r="G126" s="38" t="n">
-        <v>-92</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="38" t="inlineStr">
         <is>
-          <t>Southern</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B127" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C127" s="38" t="n">
@@ -45211,19 +45643,19 @@
         <v>122</v>
       </c>
       <c r="E127" s="38" t="n">
-        <v>1422.8</v>
+        <v>1644.9</v>
       </c>
       <c r="F127" s="38" t="n">
-        <v>175</v>
-      </c>
-      <c r="G127" s="45" t="n">
-        <v>53</v>
+        <v>29</v>
+      </c>
+      <c r="G127" s="38" t="n">
+        <v>-93</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="38" t="inlineStr">
         <is>
-          <t>UT Rio Grande Valley</t>
+          <t>Southern</t>
         </is>
       </c>
       <c r="B128" s="38" t="inlineStr">
@@ -45238,19 +45670,19 @@
         <v>123</v>
       </c>
       <c r="E128" s="38" t="n">
-        <v>1480.7</v>
+        <v>1422.8</v>
       </c>
       <c r="F128" s="38" t="n">
-        <v>104</v>
-      </c>
-      <c r="G128" s="38" t="n">
-        <v>-19</v>
+        <v>175</v>
+      </c>
+      <c r="G128" s="45" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="38" t="inlineStr">
         <is>
-          <t>North Dakota</t>
+          <t>UT Rio Grande Valley</t>
         </is>
       </c>
       <c r="B129" s="38" t="inlineStr">
@@ -45265,24 +45697,24 @@
         <v>124</v>
       </c>
       <c r="E129" s="38" t="n">
-        <v>1451</v>
+        <v>1480.7</v>
       </c>
       <c r="F129" s="38" t="n">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="G129" s="38" t="n">
-        <v>3</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="38" t="inlineStr">
         <is>
-          <t>Temple</t>
+          <t>North Dakota</t>
         </is>
       </c>
       <c r="B130" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C130" s="38" t="n">
@@ -45292,46 +45724,46 @@
         <v>125</v>
       </c>
       <c r="E130" s="38" t="n">
-        <v>1451.6</v>
+        <v>1451</v>
       </c>
       <c r="F130" s="38" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G130" s="38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="38" t="inlineStr">
         <is>
-          <t>North Carolina Central</t>
+          <t>Temple</t>
         </is>
       </c>
       <c r="B131" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C131" s="38" t="n">
-        <v>-0.31</v>
+        <v>-0.3</v>
       </c>
       <c r="D131" s="38" t="n">
         <v>126</v>
       </c>
       <c r="E131" s="38" t="n">
-        <v>1429.2</v>
+        <v>1451.6</v>
       </c>
       <c r="F131" s="38" t="n">
-        <v>165</v>
-      </c>
-      <c r="G131" s="45" t="n">
-        <v>39</v>
+        <v>126</v>
+      </c>
+      <c r="G131" s="38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="38" t="inlineStr">
         <is>
-          <t>Incarnate Word</t>
+          <t>North Carolina Central</t>
         </is>
       </c>
       <c r="B132" s="38" t="inlineStr">
@@ -45340,25 +45772,25 @@
         </is>
       </c>
       <c r="C132" s="38" t="n">
-        <v>-0.32</v>
+        <v>-0.31</v>
       </c>
       <c r="D132" s="38" t="n">
         <v>127</v>
       </c>
       <c r="E132" s="38" t="n">
-        <v>1441.2</v>
+        <v>1429.2</v>
       </c>
       <c r="F132" s="38" t="n">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="G132" s="45" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="38" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Incarnate Word</t>
         </is>
       </c>
       <c r="B133" s="38" t="inlineStr">
@@ -45373,19 +45805,19 @@
         <v>128</v>
       </c>
       <c r="E133" s="38" t="n">
-        <v>1425.1</v>
+        <v>1441.2</v>
       </c>
       <c r="F133" s="38" t="n">
-        <v>172</v>
+        <v>146</v>
       </c>
       <c r="G133" s="45" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="38" t="inlineStr">
         <is>
-          <t>Lafayette</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="B134" s="38" t="inlineStr">
@@ -45400,19 +45832,19 @@
         <v>129</v>
       </c>
       <c r="E134" s="38" t="n">
-        <v>1405.5</v>
+        <v>1425.1</v>
       </c>
       <c r="F134" s="38" t="n">
-        <v>211</v>
+        <v>172</v>
       </c>
       <c r="G134" s="45" t="n">
-        <v>82</v>
+        <v>43</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="38" t="inlineStr">
         <is>
-          <t>Campbell</t>
+          <t>Lafayette</t>
         </is>
       </c>
       <c r="B135" s="38" t="inlineStr">
@@ -45421,25 +45853,25 @@
         </is>
       </c>
       <c r="C135" s="38" t="n">
-        <v>-0.33</v>
+        <v>-0.32</v>
       </c>
       <c r="D135" s="38" t="n">
         <v>130</v>
       </c>
       <c r="E135" s="38" t="n">
-        <v>1413.9</v>
+        <v>1405.5</v>
       </c>
       <c r="F135" s="38" t="n">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="G135" s="45" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="38" t="inlineStr">
         <is>
-          <t>Central Connecticut</t>
+          <t>Campbell</t>
         </is>
       </c>
       <c r="B136" s="38" t="inlineStr">
@@ -45454,19 +45886,19 @@
         <v>131</v>
       </c>
       <c r="E136" s="38" t="n">
-        <v>1403.3</v>
+        <v>1413.9</v>
       </c>
       <c r="F136" s="38" t="n">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="G136" s="45" t="n">
-        <v>85</v>
+        <v>63</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="38" t="inlineStr">
         <is>
-          <t>Eastern Kentucky</t>
+          <t>Central Connecticut</t>
         </is>
       </c>
       <c r="B137" s="38" t="inlineStr">
@@ -45475,30 +45907,30 @@
         </is>
       </c>
       <c r="C137" s="38" t="n">
-        <v>-0.34</v>
+        <v>-0.33</v>
       </c>
       <c r="D137" s="38" t="n">
         <v>132</v>
       </c>
       <c r="E137" s="38" t="n">
-        <v>1409.5</v>
+        <v>1403.3</v>
       </c>
       <c r="F137" s="38" t="n">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="G137" s="45" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="38" t="inlineStr">
         <is>
-          <t>Bowling Green</t>
+          <t>Eastern Kentucky</t>
         </is>
       </c>
       <c r="B138" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C138" s="38" t="n">
@@ -45508,24 +45940,24 @@
         <v>133</v>
       </c>
       <c r="E138" s="38" t="n">
-        <v>1400.7</v>
+        <v>1409.5</v>
       </c>
       <c r="F138" s="38" t="n">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="G138" s="45" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="38" t="inlineStr">
         <is>
-          <t>Army</t>
+          <t>Bowling Green</t>
         </is>
       </c>
       <c r="B139" s="38" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C139" s="38" t="n">
@@ -45535,51 +45967,51 @@
         <v>134</v>
       </c>
       <c r="E139" s="38" t="n">
-        <v>1598</v>
+        <v>1400.7</v>
       </c>
       <c r="F139" s="38" t="n">
-        <v>53</v>
-      </c>
-      <c r="G139" s="38" t="n">
-        <v>-81</v>
+        <v>219</v>
+      </c>
+      <c r="G139" s="45" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="38" t="inlineStr">
         <is>
-          <t>Alabama State</t>
+          <t>Army</t>
         </is>
       </c>
       <c r="B140" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C140" s="38" t="n">
-        <v>-0.35</v>
+        <v>-0.34</v>
       </c>
       <c r="D140" s="38" t="n">
         <v>135</v>
       </c>
       <c r="E140" s="38" t="n">
-        <v>1428.8</v>
+        <v>1598</v>
       </c>
       <c r="F140" s="38" t="n">
-        <v>166</v>
-      </c>
-      <c r="G140" s="45" t="n">
-        <v>31</v>
+        <v>53</v>
+      </c>
+      <c r="G140" s="38" t="n">
+        <v>-82</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="38" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Alabama State</t>
         </is>
       </c>
       <c r="B141" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C141" s="38" t="n">
@@ -45589,24 +46021,24 @@
         <v>136</v>
       </c>
       <c r="E141" s="38" t="n">
-        <v>1426.7</v>
+        <v>1428.8</v>
       </c>
       <c r="F141" s="38" t="n">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G141" s="45" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="38" t="inlineStr">
         <is>
-          <t>Western Carolina</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="B142" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C142" s="38" t="n">
@@ -45616,19 +46048,19 @@
         <v>137</v>
       </c>
       <c r="E142" s="38" t="n">
-        <v>1420.7</v>
+        <v>1426.7</v>
       </c>
       <c r="F142" s="38" t="n">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="G142" s="45" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="38" t="inlineStr">
         <is>
-          <t>Mercer</t>
+          <t>Western Carolina</t>
         </is>
       </c>
       <c r="B143" s="38" t="inlineStr">
@@ -45637,25 +46069,25 @@
         </is>
       </c>
       <c r="C143" s="38" t="n">
-        <v>-0.36</v>
+        <v>-0.35</v>
       </c>
       <c r="D143" s="38" t="n">
         <v>138</v>
       </c>
       <c r="E143" s="38" t="n">
-        <v>1430.9</v>
+        <v>1420.7</v>
       </c>
       <c r="F143" s="38" t="n">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="G143" s="45" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="38" t="inlineStr">
         <is>
-          <t>South Dakota State</t>
+          <t>Mercer</t>
         </is>
       </c>
       <c r="B144" s="38" t="inlineStr">
@@ -45670,19 +46102,19 @@
         <v>139</v>
       </c>
       <c r="E144" s="38" t="n">
-        <v>1491.6</v>
+        <v>1430.9</v>
       </c>
       <c r="F144" s="38" t="n">
-        <v>97</v>
-      </c>
-      <c r="G144" s="38" t="n">
-        <v>-42</v>
+        <v>162</v>
+      </c>
+      <c r="G144" s="45" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="38" t="inlineStr">
         <is>
-          <t>Charleston Southern</t>
+          <t>South Dakota State</t>
         </is>
       </c>
       <c r="B145" s="38" t="inlineStr">
@@ -45691,25 +46123,25 @@
         </is>
       </c>
       <c r="C145" s="38" t="n">
-        <v>-0.37</v>
+        <v>-0.36</v>
       </c>
       <c r="D145" s="38" t="n">
         <v>140</v>
       </c>
       <c r="E145" s="38" t="n">
-        <v>1411.7</v>
+        <v>1491.6</v>
       </c>
       <c r="F145" s="38" t="n">
-        <v>202</v>
-      </c>
-      <c r="G145" s="45" t="n">
-        <v>62</v>
+        <v>97</v>
+      </c>
+      <c r="G145" s="38" t="n">
+        <v>-43</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="38" t="inlineStr">
         <is>
-          <t>Northwestern State</t>
+          <t>Charleston Southern</t>
         </is>
       </c>
       <c r="B146" s="38" t="inlineStr">
@@ -45718,25 +46150,25 @@
         </is>
       </c>
       <c r="C146" s="38" t="n">
-        <v>-0.38</v>
+        <v>-0.37</v>
       </c>
       <c r="D146" s="38" t="n">
         <v>141</v>
       </c>
       <c r="E146" s="38" t="n">
-        <v>1382.5</v>
+        <v>1411.7</v>
       </c>
       <c r="F146" s="38" t="n">
-        <v>237</v>
+        <v>202</v>
       </c>
       <c r="G146" s="45" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="38" t="inlineStr">
         <is>
-          <t>Lamar</t>
+          <t>Northwestern State</t>
         </is>
       </c>
       <c r="B147" s="38" t="inlineStr">
@@ -45751,19 +46183,19 @@
         <v>142</v>
       </c>
       <c r="E147" s="38" t="n">
-        <v>1412.8</v>
+        <v>1382.5</v>
       </c>
       <c r="F147" s="38" t="n">
-        <v>197</v>
+        <v>237</v>
       </c>
       <c r="G147" s="45" t="n">
-        <v>55</v>
+        <v>95</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="38" t="inlineStr">
         <is>
-          <t>Youngstown State</t>
+          <t>Lamar</t>
         </is>
       </c>
       <c r="B148" s="38" t="inlineStr">
@@ -45772,25 +46204,25 @@
         </is>
       </c>
       <c r="C148" s="38" t="n">
-        <v>-0.39</v>
+        <v>-0.38</v>
       </c>
       <c r="D148" s="38" t="n">
         <v>143</v>
       </c>
       <c r="E148" s="38" t="n">
-        <v>1425.9</v>
+        <v>1412.8</v>
       </c>
       <c r="F148" s="38" t="n">
-        <v>170</v>
+        <v>197</v>
       </c>
       <c r="G148" s="45" t="n">
-        <v>27</v>
+        <v>54</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="38" t="inlineStr">
         <is>
-          <t>Holy Cross</t>
+          <t>Youngstown State</t>
         </is>
       </c>
       <c r="B149" s="38" t="inlineStr">
@@ -45805,19 +46237,19 @@
         <v>144</v>
       </c>
       <c r="E149" s="38" t="n">
-        <v>1444.4</v>
+        <v>1425.9</v>
       </c>
       <c r="F149" s="38" t="n">
-        <v>141</v>
-      </c>
-      <c r="G149" s="38" t="n">
-        <v>-3</v>
+        <v>170</v>
+      </c>
+      <c r="G149" s="45" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="38" t="inlineStr">
         <is>
-          <t>Prairie View A&amp;M</t>
+          <t>Holy Cross</t>
         </is>
       </c>
       <c r="B150" s="38" t="inlineStr">
@@ -45826,57 +46258,57 @@
         </is>
       </c>
       <c r="C150" s="38" t="n">
-        <v>-0.4</v>
+        <v>-0.39</v>
       </c>
       <c r="D150" s="38" t="n">
         <v>145</v>
       </c>
       <c r="E150" s="38" t="n">
-        <v>1414.9</v>
+        <v>1444.4</v>
       </c>
       <c r="F150" s="38" t="n">
-        <v>189</v>
-      </c>
-      <c r="G150" s="45" t="n">
-        <v>44</v>
+        <v>141</v>
+      </c>
+      <c r="G150" s="38" t="n">
+        <v>-4</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="38" t="inlineStr">
         <is>
-          <t>Texas State</t>
+          <t>Prairie View A&amp;M</t>
         </is>
       </c>
       <c r="B151" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C151" s="38" t="n">
-        <v>-0.41</v>
+        <v>-0.4</v>
       </c>
       <c r="D151" s="38" t="n">
         <v>146</v>
       </c>
       <c r="E151" s="38" t="n">
-        <v>1576.6</v>
+        <v>1414.9</v>
       </c>
       <c r="F151" s="38" t="n">
-        <v>62</v>
-      </c>
-      <c r="G151" s="38" t="n">
-        <v>-84</v>
+        <v>189</v>
+      </c>
+      <c r="G151" s="45" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="38" t="inlineStr">
         <is>
-          <t>Central Arkansas</t>
+          <t>Texas State</t>
         </is>
       </c>
       <c r="B152" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C152" s="38" t="n">
@@ -45886,51 +46318,51 @@
         <v>147</v>
       </c>
       <c r="E152" s="38" t="n">
-        <v>1433.8</v>
+        <v>1576.6</v>
       </c>
       <c r="F152" s="38" t="n">
-        <v>157</v>
+        <v>62</v>
       </c>
       <c r="G152" s="38" t="n">
-        <v>10</v>
+        <v>-85</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="38" t="inlineStr">
         <is>
-          <t>Florida International</t>
+          <t>Central Arkansas</t>
         </is>
       </c>
       <c r="B153" s="38" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C153" s="38" t="n">
-        <v>-0.42</v>
+        <v>-0.41</v>
       </c>
       <c r="D153" s="38" t="n">
         <v>148</v>
       </c>
       <c r="E153" s="38" t="n">
-        <v>1488.5</v>
+        <v>1433.8</v>
       </c>
       <c r="F153" s="38" t="n">
-        <v>100</v>
+        <v>157</v>
       </c>
       <c r="G153" s="38" t="n">
-        <v>-48</v>
+        <v>9</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="38" t="inlineStr">
         <is>
-          <t>East Tennessee State</t>
+          <t>Florida International</t>
         </is>
       </c>
       <c r="B154" s="38" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="C154" s="38" t="n">
@@ -45940,19 +46372,19 @@
         <v>149</v>
       </c>
       <c r="E154" s="38" t="n">
-        <v>1429.6</v>
+        <v>1488.5</v>
       </c>
       <c r="F154" s="38" t="n">
-        <v>163</v>
+        <v>100</v>
       </c>
       <c r="G154" s="38" t="n">
-        <v>14</v>
+        <v>-49</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="38" t="inlineStr">
         <is>
-          <t>Western Illinois</t>
+          <t>East Tennessee State</t>
         </is>
       </c>
       <c r="B155" s="38" t="inlineStr">
@@ -45967,19 +46399,19 @@
         <v>150</v>
       </c>
       <c r="E155" s="38" t="n">
-        <v>1387.5</v>
+        <v>1429.6</v>
       </c>
       <c r="F155" s="38" t="n">
-        <v>233</v>
-      </c>
-      <c r="G155" s="45" t="n">
-        <v>83</v>
+        <v>163</v>
+      </c>
+      <c r="G155" s="38" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="38" t="inlineStr">
         <is>
-          <t>Merrimack</t>
+          <t>Western Illinois</t>
         </is>
       </c>
       <c r="B156" s="38" t="inlineStr">
@@ -45988,25 +46420,25 @@
         </is>
       </c>
       <c r="C156" s="38" t="n">
-        <v>-0.43</v>
+        <v>-0.42</v>
       </c>
       <c r="D156" s="38" t="n">
         <v>151</v>
       </c>
       <c r="E156" s="38" t="n">
-        <v>1400.8</v>
+        <v>1387.5</v>
       </c>
       <c r="F156" s="38" t="n">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="G156" s="45" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="38" t="inlineStr">
         <is>
-          <t>Bethune-Cookman</t>
+          <t>Merrimack</t>
         </is>
       </c>
       <c r="B157" s="38" t="inlineStr">
@@ -46021,19 +46453,19 @@
         <v>152</v>
       </c>
       <c r="E157" s="38" t="n">
-        <v>1379</v>
+        <v>1400.8</v>
       </c>
       <c r="F157" s="38" t="n">
-        <v>239</v>
+        <v>218</v>
       </c>
       <c r="G157" s="45" t="n">
-        <v>87</v>
+        <v>66</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="38" t="inlineStr">
         <is>
-          <t>North Alabama</t>
+          <t>Bethune-Cookman</t>
         </is>
       </c>
       <c r="B158" s="38" t="inlineStr">
@@ -46048,19 +46480,19 @@
         <v>153</v>
       </c>
       <c r="E158" s="38" t="n">
-        <v>1434.2</v>
+        <v>1379</v>
       </c>
       <c r="F158" s="38" t="n">
-        <v>155</v>
-      </c>
-      <c r="G158" s="38" t="n">
-        <v>2</v>
+        <v>239</v>
+      </c>
+      <c r="G158" s="45" t="n">
+        <v>86</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="38" t="inlineStr">
         <is>
-          <t>Weber State</t>
+          <t>North Alabama</t>
         </is>
       </c>
       <c r="B159" s="38" t="inlineStr">
@@ -46069,25 +46501,25 @@
         </is>
       </c>
       <c r="C159" s="38" t="n">
-        <v>-0.45</v>
+        <v>-0.43</v>
       </c>
       <c r="D159" s="38" t="n">
         <v>154</v>
       </c>
       <c r="E159" s="38" t="n">
-        <v>1433.7</v>
+        <v>1434.2</v>
       </c>
       <c r="F159" s="38" t="n">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="G159" s="38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="38" t="inlineStr">
         <is>
-          <t>UAlbany</t>
+          <t>Weber State</t>
         </is>
       </c>
       <c r="B160" s="38" t="inlineStr">
@@ -46102,24 +46534,24 @@
         <v>155</v>
       </c>
       <c r="E160" s="38" t="n">
-        <v>1435.7</v>
+        <v>1433.7</v>
       </c>
       <c r="F160" s="38" t="n">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G160" s="38" t="n">
-        <v>-2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="38" t="inlineStr">
         <is>
-          <t>Arkansas State</t>
+          <t>UAlbany</t>
         </is>
       </c>
       <c r="B161" s="38" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="C161" s="38" t="n">
@@ -46129,24 +46561,24 @@
         <v>156</v>
       </c>
       <c r="E161" s="38" t="n">
-        <v>1500</v>
+        <v>1435.7</v>
       </c>
       <c r="F161" s="38" t="n">
-        <v>91</v>
+        <v>153</v>
       </c>
       <c r="G161" s="38" t="n">
-        <v>-65</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="38" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Arkansas State</t>
         </is>
       </c>
       <c r="B162" s="38" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="C162" s="38" t="n">
@@ -46156,13 +46588,13 @@
         <v>157</v>
       </c>
       <c r="E162" s="38" t="n">
-        <v>1520.2</v>
+        <v>1500</v>
       </c>
       <c r="F162" s="38" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G162" s="38" t="n">
-        <v>-77</v>
+        <v>-66</v>
       </c>
     </row>
     <row r="163">
@@ -46213,10 +46645,10 @@
         <v>1402.8</v>
       </c>
       <c r="F164" s="38" t="n">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G164" s="45" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="165">
@@ -46294,10 +46726,10 @@
         <v>1391.8</v>
       </c>
       <c r="F167" s="38" t="n">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G167" s="45" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="168">
@@ -46402,10 +46834,10 @@
         <v>1404.2</v>
       </c>
       <c r="F171" s="38" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G171" s="45" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="172">
@@ -46483,10 +46915,10 @@
         <v>1521.7</v>
       </c>
       <c r="F174" s="38" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G174" s="38" t="n">
-        <v>-91</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="175">
@@ -46591,10 +47023,10 @@
         <v>1393.9</v>
       </c>
       <c r="F178" s="38" t="n">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G178" s="45" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="179">
@@ -46753,10 +47185,10 @@
         <v>1395</v>
       </c>
       <c r="F184" s="38" t="n">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G184" s="45" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="185">
@@ -46834,10 +47266,10 @@
         <v>1397.7</v>
       </c>
       <c r="F187" s="38" t="n">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G187" s="45" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="188">
@@ -46942,10 +47374,10 @@
         <v>1398.4</v>
       </c>
       <c r="F191" s="38" t="n">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G191" s="45" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="192">
@@ -47239,10 +47671,10 @@
         <v>1392.6</v>
       </c>
       <c r="F202" s="38" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G202" s="45" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="203">
@@ -47536,10 +47968,10 @@
         <v>1530.9</v>
       </c>
       <c r="F213" s="38" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G213" s="38" t="n">
-        <v>-132</v>
+        <v>-131</v>
       </c>
     </row>
     <row r="214">
@@ -47617,10 +48049,10 @@
         <v>1402.2</v>
       </c>
       <c r="F216" s="38" t="n">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G216" s="38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="217">
@@ -47644,10 +48076,10 @@
         <v>1399.2</v>
       </c>
       <c r="F217" s="38" t="n">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G217" s="38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="218">
@@ -47761,7 +48193,7 @@
     <row r="222">
       <c r="A222" s="38" t="inlineStr">
         <is>
-          <t>Southern Miss</t>
+          <t>Sam Houston</t>
         </is>
       </c>
       <c r="B222" s="38" t="inlineStr">
@@ -47770,138 +48202,138 @@
         </is>
       </c>
       <c r="C222" s="38" t="n">
-        <v>-1.17</v>
+        <v>-1.23</v>
       </c>
       <c r="D222" s="38" t="n">
         <v>217</v>
       </c>
       <c r="E222" s="38" t="n">
-        <v>1406.7</v>
+        <v>1389.7</v>
       </c>
       <c r="F222" s="38" t="n">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="G222" s="38" t="n">
-        <v>-7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="38" t="inlineStr">
         <is>
-          <t>Sam Houston</t>
+          <t>Rice</t>
         </is>
       </c>
       <c r="B223" s="38" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="C223" s="38" t="n">
-        <v>-1.23</v>
+        <v>-1.27</v>
       </c>
       <c r="D223" s="38" t="n">
         <v>218</v>
       </c>
       <c r="E223" s="38" t="n">
-        <v>1389.7</v>
+        <v>1407.2</v>
       </c>
       <c r="F223" s="38" t="n">
-        <v>230</v>
+        <v>207</v>
       </c>
       <c r="G223" s="38" t="n">
-        <v>12</v>
+        <v>-11</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="38" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>Mercyhurst</t>
         </is>
       </c>
       <c r="B224" s="38" t="inlineStr">
         <is>
-          <t>0-4</t>
+          <t>0-3</t>
         </is>
       </c>
       <c r="C224" s="38" t="n">
-        <v>-1.27</v>
+        <v>-1.3</v>
       </c>
       <c r="D224" s="38" t="n">
         <v>219</v>
       </c>
       <c r="E224" s="38" t="n">
-        <v>1407.2</v>
+        <v>1414.7</v>
       </c>
       <c r="F224" s="38" t="n">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="G224" s="38" t="n">
-        <v>-12</v>
+        <v>-29</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="38" t="inlineStr">
         <is>
-          <t>Mercyhurst</t>
+          <t>Washington State</t>
         </is>
       </c>
       <c r="B225" s="38" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="C225" s="38" t="n">
-        <v>-1.3</v>
+        <v>-1.32</v>
       </c>
       <c r="D225" s="38" t="n">
         <v>220</v>
       </c>
       <c r="E225" s="38" t="n">
-        <v>1414.7</v>
+        <v>1492.5</v>
       </c>
       <c r="F225" s="38" t="n">
-        <v>190</v>
+        <v>95</v>
       </c>
       <c r="G225" s="38" t="n">
-        <v>-30</v>
+        <v>-125</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="38" t="inlineStr">
         <is>
-          <t>Washington State</t>
+          <t>Kennesaw State</t>
         </is>
       </c>
       <c r="B226" s="38" t="inlineStr">
         <is>
-          <t>0-4</t>
+          <t>0-3</t>
         </is>
       </c>
       <c r="C226" s="38" t="n">
-        <v>-1.32</v>
+        <v>-1.34</v>
       </c>
       <c r="D226" s="38" t="n">
         <v>221</v>
       </c>
       <c r="E226" s="38" t="n">
-        <v>1492.5</v>
+        <v>1480.8</v>
       </c>
       <c r="F226" s="38" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G226" s="38" t="n">
-        <v>-126</v>
+        <v>-118</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="38" t="inlineStr">
         <is>
-          <t>Kennesaw State</t>
+          <t>Western Kentucky</t>
         </is>
       </c>
       <c r="B227" s="38" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="C227" s="38" t="n">
@@ -47911,19 +48343,19 @@
         <v>222</v>
       </c>
       <c r="E227" s="38" t="n">
-        <v>1480.8</v>
+        <v>1485.6</v>
       </c>
       <c r="F227" s="38" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G227" s="38" t="n">
-        <v>-119</v>
+        <v>-121</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="38" t="inlineStr">
         <is>
-          <t>Western Kentucky</t>
+          <t>UTEP</t>
         </is>
       </c>
       <c r="B228" s="38" t="inlineStr">
@@ -47932,57 +48364,57 @@
         </is>
       </c>
       <c r="C228" s="38" t="n">
-        <v>-1.34</v>
+        <v>-1.41</v>
       </c>
       <c r="D228" s="38" t="n">
         <v>223</v>
       </c>
       <c r="E228" s="38" t="n">
-        <v>1485.6</v>
+        <v>1331.5</v>
       </c>
       <c r="F228" s="38" t="n">
-        <v>101</v>
-      </c>
-      <c r="G228" s="38" t="n">
-        <v>-122</v>
+        <v>250</v>
+      </c>
+      <c r="G228" s="45" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="38" t="inlineStr">
         <is>
-          <t>UTEP</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="B229" s="38" t="inlineStr">
         <is>
-          <t>0-4</t>
+          <t>0-3</t>
         </is>
       </c>
       <c r="C229" s="38" t="n">
-        <v>-1.41</v>
+        <v>-1.5</v>
       </c>
       <c r="D229" s="38" t="n">
         <v>224</v>
       </c>
       <c r="E229" s="38" t="n">
-        <v>1331.5</v>
+        <v>1581.9</v>
       </c>
       <c r="F229" s="38" t="n">
-        <v>250</v>
-      </c>
-      <c r="G229" s="45" t="n">
-        <v>26</v>
+        <v>59</v>
+      </c>
+      <c r="G229" s="38" t="n">
+        <v>-165</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="38" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="B230" s="38" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="C230" s="38" t="n">
@@ -47992,67 +48424,67 @@
         <v>225</v>
       </c>
       <c r="E230" s="38" t="n">
-        <v>1581.9</v>
+        <v>1274.2</v>
       </c>
       <c r="F230" s="38" t="n">
-        <v>59</v>
-      </c>
-      <c r="G230" s="38" t="n">
-        <v>-166</v>
+        <v>252</v>
+      </c>
+      <c r="G230" s="45" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="38" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="B231" s="38" t="inlineStr">
         <is>
-          <t>0-4</t>
+          <t>0-3</t>
         </is>
       </c>
       <c r="C231" s="38" t="n">
-        <v>-1.5</v>
+        <v>-1.53</v>
       </c>
       <c r="D231" s="38" t="n">
         <v>226</v>
       </c>
       <c r="E231" s="38" t="n">
-        <v>1274.2</v>
+        <v>1532.4</v>
       </c>
       <c r="F231" s="38" t="n">
-        <v>252</v>
-      </c>
-      <c r="G231" s="45" t="n">
-        <v>26</v>
+        <v>76</v>
+      </c>
+      <c r="G231" s="38" t="n">
+        <v>-150</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="38" t="inlineStr">
         <is>
-          <t>Georgia Tech</t>
+          <t>Southern Miss</t>
         </is>
       </c>
       <c r="B232" s="38" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="C232" s="38" t="n">
-        <v>-1.53</v>
+        <v>-1.55</v>
       </c>
       <c r="D232" s="38" t="n">
         <v>227</v>
       </c>
       <c r="E232" s="38" t="n">
-        <v>1532.4</v>
+        <v>1391.6</v>
       </c>
       <c r="F232" s="38" t="n">
-        <v>75</v>
+        <v>228</v>
       </c>
       <c r="G232" s="38" t="n">
-        <v>-152</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233">
@@ -48157,10 +48589,10 @@
         <v>1404.9</v>
       </c>
       <c r="F236" s="38" t="n">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G236" s="38" t="n">
-        <v>-19</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="237">
@@ -48336,26 +48768,26 @@
       </c>
       <c r="B3" s="38" t="inlineStr">
         <is>
-          <t>207-178-5</t>
+          <t>207-179-5</t>
         </is>
       </c>
       <c r="C3" s="41" t="n">
-        <v>0.538</v>
+        <v>0.536</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>Weekly ATS (Wk 5)</t>
+          <t>Weekly ATS (Wk 6)</t>
         </is>
       </c>
       <c r="B4" s="38" t="inlineStr">
         <is>
-          <t>28-30-1</t>
+          <t>0-1-0</t>
         </is>
       </c>
       <c r="C4" s="41" t="n">
-        <v>0.483</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="26.45" customHeight="1">
@@ -51469,9 +51901,17 @@
       <c r="N60" s="38" t="n">
         <v>0.3</v>
       </c>
-      <c r="O60" s="38" t="n"/>
-      <c r="P60" s="38" t="n"/>
-      <c r="Q60" s="38" t="n"/>
+      <c r="O60" s="38" t="n">
+        <v>34</v>
+      </c>
+      <c r="P60" s="38" t="n">
+        <v>55</v>
+      </c>
+      <c r="Q60" s="43" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="38" t="n">

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-10-13 19:23 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -1624,7 +1624,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>8.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -1680,7 +1680,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-33.1</v>
+        <v>-33.4</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -1744,7 +1744,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-9.300000000000001</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -1808,7 +1808,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-17.6</v>
+        <v>-16.9</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -1864,7 +1864,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-13.2</v>
+        <v>-13</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -1920,7 +1920,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-30.3</v>
+        <v>-29.9</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -1976,7 +1976,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>8.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -2088,7 +2088,7 @@
       <c r="P37" s="42" t="n"/>
       <c r="Q37" s="42" t="n"/>
       <c r="R37" s="42" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="S37" s="51" t="n"/>
       <c r="T37" s="51" t="n"/>
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-4.5</v>
+        <v>-5.4</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="S42" s="53" t="inlineStr">
         <is>
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
       <c r="S43" s="52" t="inlineStr">
         <is>
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-1.3</v>
+        <v>-1.7</v>
       </c>
       <c r="S44" s="53" t="inlineStr">
         <is>
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>-13.4</v>
+        <v>-13.5</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-4.7</v>
+        <v>-4.8</v>
       </c>
       <c r="S46" s="52" t="inlineStr">
         <is>
@@ -2808,7 +2808,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-37.8</v>
+        <v>-36.9</v>
       </c>
       <c r="S47" s="52" t="inlineStr">
         <is>
@@ -2820,9 +2820,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U47" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U47" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V47" s="52" t="inlineStr">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-1.1</v>
+        <v>-0.3</v>
       </c>
       <c r="S51" s="53" t="inlineStr">
         <is>
@@ -3027,9 +3027,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U51" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U51" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V51" s="53" t="inlineStr">
@@ -3102,7 +3102,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R52" s="42" t="n"/>
+      <c r="R52" s="42" t="n">
+        <v>6.7</v>
+      </c>
       <c r="S52" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -3113,7 +3115,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U52" s="51" t="n"/>
+      <c r="U52" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V52" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -3185,7 +3191,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
@@ -3273,7 +3279,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-1.3</v>
+        <v>-1.4</v>
       </c>
       <c r="S54" s="52" t="inlineStr">
         <is>
@@ -3361,7 +3367,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="S55" s="52" t="inlineStr">
         <is>
@@ -3449,7 +3455,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>-20.8</v>
+        <v>-20.1</v>
       </c>
       <c r="S56" s="52" t="inlineStr">
         <is>
@@ -3461,9 +3467,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U56" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U56" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V56" s="53" t="inlineStr">
@@ -3537,7 +3543,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>-8</v>
+        <v>-8.1</v>
       </c>
       <c r="S57" s="53" t="inlineStr">
         <is>
@@ -3625,7 +3631,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>-6.2</v>
+        <v>-6.8</v>
       </c>
       <c r="S58" s="53" t="inlineStr">
         <is>
@@ -3713,7 +3719,7 @@
         </is>
       </c>
       <c r="R59" s="42" t="n">
-        <v>-6.8</v>
+        <v>-7</v>
       </c>
       <c r="S59" s="53" t="inlineStr">
         <is>
@@ -4360,7 +4366,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -4416,7 +4422,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>-2.4</v>
+        <v>-2.6</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -4472,7 +4478,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -4528,7 +4534,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -4584,7 +4590,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-15.7</v>
+        <v>-14.8</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -4640,7 +4646,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-11.4</v>
+        <v>-10.9</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -4696,7 +4702,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-11</v>
+        <v>-11.7</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -4888,7 +4894,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.1</v>
       </c>
       <c r="S36" s="52" t="inlineStr">
         <is>
@@ -4976,7 +4982,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-4.5</v>
+        <v>-4.8</v>
       </c>
       <c r="S37" s="54" t="inlineStr">
         <is>
@@ -5064,7 +5070,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-12.1</v>
+        <v>-12.7</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -5152,7 +5158,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-12.4</v>
+        <v>-11</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -5240,7 +5246,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.7</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -5328,7 +5334,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-25.8</v>
+        <v>-25.3</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -5416,7 +5422,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-1.9</v>
+        <v>-2.1</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -5623,7 +5629,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>3.1</v>
+        <v>4.1</v>
       </c>
       <c r="S46" s="52" t="inlineStr">
         <is>
@@ -5711,7 +5717,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>16.2</v>
+        <v>15.6</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -5798,7 +5804,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R48" s="42" t="n"/>
+      <c r="R48" s="42" t="n">
+        <v>-32.2</v>
+      </c>
       <c r="S48" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -5809,7 +5817,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U48" s="51" t="n"/>
+      <c r="U48" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V48" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -5880,7 +5892,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R49" s="42" t="n"/>
+      <c r="R49" s="42" t="n">
+        <v>15.9</v>
+      </c>
       <c r="S49" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -5891,7 +5905,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U49" s="51" t="n"/>
+      <c r="U49" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V49" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -5962,7 +5980,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R50" s="42" t="n"/>
+      <c r="R50" s="42" t="n">
+        <v>-13.6</v>
+      </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -5973,7 +5993,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U50" s="51" t="n"/>
+      <c r="U50" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V50" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -6045,7 +6069,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-24</v>
+        <v>-23.8</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -6133,7 +6157,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>-2.1</v>
+        <v>-1.5</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -6145,9 +6169,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U52" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U52" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V52" s="53" t="inlineStr">
@@ -6220,7 +6244,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R53" s="42" t="n"/>
+      <c r="R53" s="42" t="n">
+        <v>-4.5</v>
+      </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -6231,7 +6257,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U53" s="51" t="n"/>
+      <c r="U53" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V53" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -6970,7 +7000,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-1.1</v>
+        <v>-0.6</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -7034,7 +7064,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-16.9</v>
+        <v>-15.6</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -7098,7 +7128,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-11.3</v>
+        <v>-10.7</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -7154,7 +7184,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-18.2</v>
+        <v>-18</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -7210,7 +7240,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-0.7</v>
+        <v>-0.5</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -7266,7 +7296,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>18.4</v>
+        <v>18.1</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -7458,7 +7488,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-13.8</v>
+        <v>-14.7</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -7546,7 +7576,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-1.8</v>
+        <v>-1.2</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -7558,9 +7588,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U39" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U39" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V39" s="53" t="inlineStr">
@@ -7634,7 +7664,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="S40" s="52" t="inlineStr">
         <is>
@@ -7722,7 +7752,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -7810,7 +7840,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-14.9</v>
+        <v>-14.5</v>
       </c>
       <c r="S42" s="53" t="inlineStr">
         <is>
@@ -7898,7 +7928,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>-18.8</v>
+        <v>-19.7</v>
       </c>
       <c r="S43" s="53" t="inlineStr">
         <is>
@@ -8104,7 +8134,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R47" s="42" t="n"/>
+      <c r="R47" s="42" t="n">
+        <v>17.7</v>
+      </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -8115,7 +8147,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U47" s="51" t="n"/>
+      <c r="U47" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V47" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -8187,7 +8223,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>-12.8</v>
+        <v>-12.3</v>
       </c>
       <c r="S48" s="52" t="inlineStr">
         <is>
@@ -8363,7 +8399,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-13.7</v>
+        <v>-13</v>
       </c>
       <c r="S50" s="53" t="inlineStr">
         <is>
@@ -8450,7 +8486,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R51" s="42" t="n"/>
+      <c r="R51" s="42" t="n">
+        <v>6.2</v>
+      </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -8461,7 +8499,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U51" s="51" t="n"/>
+      <c r="U51" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V51" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -8532,7 +8574,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R52" s="42" t="n"/>
+      <c r="R52" s="42" t="n">
+        <v>-13.1</v>
+      </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -8543,7 +8587,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U52" s="51" t="n"/>
+      <c r="U52" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V52" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -8614,7 +8662,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R53" s="42" t="n"/>
+      <c r="R53" s="42" t="n">
+        <v>-7.8</v>
+      </c>
       <c r="S53" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -8625,7 +8675,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U53" s="51" t="n"/>
+      <c r="U53" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V53" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -9352,7 +9406,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -9472,7 +9526,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-8.6</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -9528,7 +9582,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>9.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -9556,43 +9610,35 @@
       </c>
       <c r="E34" s="42" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="F34" s="42" t="inlineStr">
         <is>
-          <t>Oregon</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="G34" s="42" t="n">
-        <v>-11.4</v>
-      </c>
-      <c r="H34" s="42" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="I34" s="42" t="n">
-        <v>-1.1</v>
-      </c>
+        <v>8.6</v>
+      </c>
+      <c r="H34" s="42" t="n"/>
+      <c r="I34" s="42" t="n"/>
       <c r="J34" s="42" t="n">
-        <v>-18.1</v>
+        <v>8.4</v>
       </c>
       <c r="K34" s="42" t="n">
-        <v>-1.4</v>
+        <v>-7.1</v>
       </c>
       <c r="L34" s="42" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="M34" s="42" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="N34" s="47" t="n">
-        <v>-4.8</v>
-      </c>
+        <v>51.7</v>
+      </c>
+      <c r="M34" s="42" t="n"/>
+      <c r="N34" s="42" t="n"/>
       <c r="O34" s="42" t="n"/>
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-15.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -9620,35 +9666,43 @@
       </c>
       <c r="E35" s="42" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="F35" s="42" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="G35" s="42" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="H35" s="42" t="n"/>
-      <c r="I35" s="42" t="n"/>
+        <v>-5.9</v>
+      </c>
+      <c r="H35" s="42" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="I35" s="47" t="n">
+        <v>2.4</v>
+      </c>
       <c r="J35" s="42" t="n">
-        <v>8.4</v>
+        <v>-5.4</v>
       </c>
       <c r="K35" s="42" t="n">
         <v>-7.1</v>
       </c>
       <c r="L35" s="42" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="M35" s="42" t="n"/>
-      <c r="N35" s="42" t="n"/>
+        <v>44.4</v>
+      </c>
+      <c r="M35" s="42" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="N35" s="47" t="n">
+        <v>-5.1</v>
+      </c>
       <c r="O35" s="42" t="n"/>
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>8.9</v>
+        <v>-7.8</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -9661,7 +9715,7 @@
       </c>
       <c r="B36" s="42" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="C36" s="42" t="inlineStr">
@@ -9676,43 +9730,43 @@
       </c>
       <c r="E36" s="42" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="F36" s="42" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Oregon</t>
         </is>
       </c>
       <c r="G36" s="42" t="n">
-        <v>-5.9</v>
+        <v>-11.4</v>
       </c>
       <c r="H36" s="42" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="I36" s="47" t="n">
-        <v>2.4</v>
+        <v>-12.5</v>
+      </c>
+      <c r="I36" s="42" t="n">
+        <v>-1.1</v>
       </c>
       <c r="J36" s="42" t="n">
-        <v>-5.4</v>
+        <v>-18.1</v>
       </c>
       <c r="K36" s="42" t="n">
-        <v>-7.1</v>
+        <v>-1.4</v>
       </c>
       <c r="L36" s="42" t="n">
-        <v>44.4</v>
+        <v>53.7</v>
       </c>
       <c r="M36" s="42" t="n">
-        <v>49.5</v>
+        <v>58.5</v>
       </c>
       <c r="N36" s="47" t="n">
-        <v>-5.1</v>
+        <v>-4.8</v>
       </c>
       <c r="O36" s="42" t="n"/>
       <c r="P36" s="42" t="n"/>
       <c r="Q36" s="42" t="n"/>
       <c r="R36" s="42" t="n">
-        <v>-7.6</v>
+        <v>-15.2</v>
       </c>
       <c r="S36" s="51" t="n"/>
       <c r="T36" s="51" t="n"/>
@@ -9903,7 +9957,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="S40" s="52" t="inlineStr">
         <is>
@@ -9991,7 +10045,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>14.1</v>
+        <v>14.3</v>
       </c>
       <c r="S41" s="52" t="inlineStr">
         <is>
@@ -10079,7 +10133,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-24.1</v>
+        <v>-26.2</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -10255,7 +10309,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-24.6</v>
+        <v>-25.6</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -10343,7 +10397,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -10431,7 +10485,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-0.3</v>
+        <v>0.2</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -10519,7 +10573,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>11</v>
+        <v>10.1</v>
       </c>
       <c r="S47" s="52" t="inlineStr">
         <is>
@@ -10726,7 +10780,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.3</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -10814,7 +10868,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -10902,7 +10956,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="S53" s="53" t="inlineStr">
         <is>
@@ -10990,7 +11044,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-11.2</v>
+        <v>-11.3</v>
       </c>
       <c r="S54" s="53" t="inlineStr">
         <is>
@@ -11078,7 +11132,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="S55" s="52" t="inlineStr">
         <is>
@@ -11165,7 +11219,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R56" s="42" t="n"/>
+      <c r="R56" s="42" t="n">
+        <v>-4.7</v>
+      </c>
       <c r="S56" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -11176,7 +11232,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U56" s="51" t="n"/>
+      <c r="U56" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V56" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -11248,7 +11308,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>-6</v>
+        <v>-6.2</v>
       </c>
       <c r="S57" s="52" t="inlineStr">
         <is>
@@ -11335,7 +11395,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R58" s="42" t="n"/>
+      <c r="R58" s="42" t="n">
+        <v>16.8</v>
+      </c>
       <c r="S58" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -11346,7 +11408,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U58" s="51" t="n"/>
+      <c r="U58" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V58" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -11897,7 +11963,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -11961,7 +12027,7 @@
       <c r="P23" s="42" t="n"/>
       <c r="Q23" s="42" t="n"/>
       <c r="R23" s="42" t="n">
-        <v>-11.4</v>
+        <v>-12.2</v>
       </c>
       <c r="S23" s="51" t="n"/>
       <c r="T23" s="51" t="n"/>
@@ -12025,7 +12091,7 @@
       <c r="P24" s="42" t="n"/>
       <c r="Q24" s="42" t="n"/>
       <c r="R24" s="42" t="n">
-        <v>-1.7</v>
+        <v>-1.9</v>
       </c>
       <c r="S24" s="51" t="n"/>
       <c r="T24" s="51" t="n"/>
@@ -12089,7 +12155,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -12281,7 +12347,7 @@
         </is>
       </c>
       <c r="R29" s="42" t="n">
-        <v>-9.800000000000001</v>
+        <v>-9.6</v>
       </c>
       <c r="S29" s="52" t="inlineStr">
         <is>
@@ -12369,7 +12435,7 @@
         </is>
       </c>
       <c r="R30" s="42" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="S30" s="52" t="inlineStr">
         <is>
@@ -12457,7 +12523,7 @@
         </is>
       </c>
       <c r="R31" s="42" t="n">
-        <v>-13.2</v>
+        <v>-11.8</v>
       </c>
       <c r="S31" s="53" t="inlineStr">
         <is>
@@ -12469,9 +12535,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U31" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U31" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V31" s="52" t="inlineStr">
@@ -12545,7 +12611,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>-9.300000000000001</v>
+        <v>-8.5</v>
       </c>
       <c r="S32" s="53" t="inlineStr">
         <is>
@@ -12752,7 +12818,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-13.7</v>
+        <v>-13</v>
       </c>
       <c r="S36" s="53" t="inlineStr">
         <is>
@@ -12840,7 +12906,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="S37" s="52" t="inlineStr">
         <is>
@@ -12928,7 +12994,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="S38" s="52" t="inlineStr">
         <is>
@@ -13506,7 +13572,7 @@
         </is>
       </c>
       <c r="R18" s="42" t="n">
-        <v>-1.9</v>
+        <v>-2.1</v>
       </c>
       <c r="S18" s="52" t="inlineStr">
         <is>
@@ -13594,7 +13660,7 @@
         </is>
       </c>
       <c r="R19" s="42" t="n">
-        <v>-37.8</v>
+        <v>-36.9</v>
       </c>
       <c r="S19" s="52" t="inlineStr">
         <is>
@@ -13606,9 +13672,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U19" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U19" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V19" s="52" t="inlineStr">
@@ -13801,7 +13867,7 @@
         </is>
       </c>
       <c r="R23" s="42" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="S23" s="52" t="inlineStr">
         <is>
@@ -13889,7 +13955,7 @@
         </is>
       </c>
       <c r="R24" s="42" t="n">
-        <v>-6.2</v>
+        <v>-6.8</v>
       </c>
       <c r="S24" s="53" t="inlineStr">
         <is>
@@ -14514,7 +14580,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>-15.7</v>
+        <v>-14.8</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -14570,7 +14636,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.7</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -14626,7 +14692,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>-14.8</v>
+        <v>-14</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -14682,7 +14748,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>6</v>
+        <v>6.8</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -14738,7 +14804,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -14794,7 +14860,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-10.3</v>
+        <v>-11</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -14850,7 +14916,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>18.8</v>
+        <v>19.1</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -15042,7 +15108,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-24.1</v>
+        <v>-26.2</v>
       </c>
       <c r="S35" s="52" t="inlineStr">
         <is>
@@ -15130,7 +15196,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
       <c r="S36" s="53" t="inlineStr">
         <is>
@@ -15218,7 +15284,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-9.1</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -15306,7 +15372,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="S38" s="52" t="inlineStr">
         <is>
@@ -15482,7 +15548,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-14.4</v>
+        <v>-13.6</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -15570,7 +15636,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-15.7</v>
+        <v>-15.5</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -15777,7 +15843,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>15.3</v>
+        <v>13.7</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -15865,7 +15931,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="S46" s="52" t="inlineStr">
         <is>
@@ -15953,7 +16019,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-7.2</v>
+        <v>-7.3</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -16041,7 +16107,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>15.2</v>
+        <v>15</v>
       </c>
       <c r="S48" s="52" t="inlineStr">
         <is>
@@ -16129,7 +16195,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -16217,7 +16283,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-11</v>
+        <v>-11.1</v>
       </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
@@ -16776,7 +16842,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>-0.5</v>
+        <v>0.6</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -16832,7 +16898,7 @@
       <c r="P23" s="42" t="n"/>
       <c r="Q23" s="42" t="n"/>
       <c r="R23" s="42" t="n">
-        <v>-18.2</v>
+        <v>-19</v>
       </c>
       <c r="S23" s="51" t="n"/>
       <c r="T23" s="51" t="n"/>
@@ -16888,7 +16954,7 @@
       <c r="P24" s="42" t="n"/>
       <c r="Q24" s="42" t="n"/>
       <c r="R24" s="42" t="n">
-        <v>-6.6</v>
+        <v>-6.3</v>
       </c>
       <c r="S24" s="51" t="n"/>
       <c r="T24" s="51" t="n"/>
@@ -16944,7 +17010,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>9.699999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -17000,7 +17066,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -17192,7 +17258,7 @@
         </is>
       </c>
       <c r="R30" s="42" t="n">
-        <v>-14.9</v>
+        <v>-14.5</v>
       </c>
       <c r="S30" s="53" t="inlineStr">
         <is>
@@ -17280,7 +17346,7 @@
         </is>
       </c>
       <c r="R31" s="42" t="n">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
       <c r="S31" s="53" t="inlineStr">
         <is>
@@ -17368,7 +17434,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="S32" s="52" t="inlineStr">
         <is>
@@ -17456,7 +17522,7 @@
         </is>
       </c>
       <c r="R33" s="42" t="n">
-        <v>4.1</v>
+        <v>4.6</v>
       </c>
       <c r="S33" s="52" t="inlineStr">
         <is>
@@ -17515,7 +17581,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="I34" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="J34" s="42" t="n">
         <v>5</v>
@@ -17544,7 +17610,7 @@
         </is>
       </c>
       <c r="R34" s="42" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="S34" s="53" t="inlineStr">
         <is>
@@ -17751,7 +17817,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-2.1</v>
+        <v>-1.5</v>
       </c>
       <c r="S38" s="52" t="inlineStr">
         <is>
@@ -17763,9 +17829,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U38" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U38" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V38" s="53" t="inlineStr">
@@ -17839,7 +17905,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-20.7</v>
+        <v>-22</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -17927,7 +17993,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-21.1</v>
+        <v>-21.8</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -18015,7 +18081,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-6.8</v>
+        <v>-7</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -18102,7 +18168,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R42" s="42" t="n"/>
+      <c r="R42" s="42" t="n">
+        <v>-7.3</v>
+      </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -18113,7 +18181,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U42" s="51" t="n"/>
+      <c r="U42" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V42" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -18620,7 +18692,7 @@
       <c r="P20" s="42" t="n"/>
       <c r="Q20" s="42" t="n"/>
       <c r="R20" s="42" t="n">
-        <v>-14.5</v>
+        <v>-15.2</v>
       </c>
       <c r="S20" s="51" t="n"/>
       <c r="T20" s="51" t="n"/>
@@ -18676,7 +18748,7 @@
       <c r="P21" s="42" t="n"/>
       <c r="Q21" s="42" t="n"/>
       <c r="R21" s="42" t="n">
-        <v>-3.4</v>
+        <v>-3.6</v>
       </c>
       <c r="S21" s="51" t="n"/>
       <c r="T21" s="51" t="n"/>
@@ -18732,7 +18804,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>3.2</v>
+        <v>2.2</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -18924,7 +18996,7 @@
         </is>
       </c>
       <c r="R26" s="42" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="S26" s="52" t="inlineStr">
         <is>
@@ -19012,7 +19084,7 @@
         </is>
       </c>
       <c r="R27" s="42" t="n">
-        <v>-2.6</v>
+        <v>-1.5</v>
       </c>
       <c r="S27" s="53" t="inlineStr">
         <is>
@@ -19100,7 +19172,7 @@
         </is>
       </c>
       <c r="R28" s="42" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="S28" s="53" t="inlineStr">
         <is>
@@ -19306,7 +19378,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R32" s="42" t="n"/>
+      <c r="R32" s="42" t="n">
+        <v>-15</v>
+      </c>
       <c r="S32" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -19317,7 +19391,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U32" s="51" t="n"/>
+      <c r="U32" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V32" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -19388,7 +19466,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R33" s="42" t="n"/>
+      <c r="R33" s="42" t="n">
+        <v>-2.4</v>
+      </c>
       <c r="S33" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -19399,7 +19479,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U33" s="51" t="n"/>
+      <c r="U33" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V33" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -19470,7 +19554,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R34" s="42" t="n"/>
+      <c r="R34" s="42" t="n">
+        <v>1.5</v>
+      </c>
       <c r="S34" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -19481,7 +19567,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U34" s="51" t="n"/>
+      <c r="U34" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V34" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -19552,7 +19642,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R35" s="42" t="n"/>
+      <c r="R35" s="42" t="n">
+        <v>1.3</v>
+      </c>
       <c r="S35" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -19563,7 +19655,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U35" s="51" t="n"/>
+      <c r="U35" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V35" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -20246,7 +20342,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -20310,7 +20406,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-10.5</v>
+        <v>-10.6</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -20374,7 +20470,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-15</v>
+        <v>-14.7</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -20438,7 +20534,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-10.1</v>
+        <v>-10.2</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -20502,7 +20598,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -20566,7 +20662,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-15.4</v>
+        <v>-16.2</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -20622,7 +20718,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-33.1</v>
+        <v>-33.4</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -20678,7 +20774,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>-11.7</v>
+        <v>-11.5</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -20870,7 +20966,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -20958,7 +21054,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="S40" s="52" t="inlineStr">
         <is>
@@ -21046,7 +21142,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -21134,7 +21230,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -21222,7 +21318,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>-0.1</v>
+        <v>0.7</v>
       </c>
       <c r="S43" s="52" t="inlineStr">
         <is>
@@ -21310,7 +21406,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>11.4</v>
+        <v>10.7</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -21398,7 +21494,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -21605,7 +21701,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-15.5</v>
+        <v>-16.4</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -21692,7 +21788,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R50" s="42" t="n"/>
+      <c r="R50" s="42" t="n">
+        <v>-40.5</v>
+      </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -21703,7 +21801,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U50" s="51" t="n"/>
+      <c r="U50" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V50" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -21775,7 +21877,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>16.1</v>
+        <v>15.4</v>
       </c>
       <c r="S51" s="53" t="inlineStr">
         <is>
@@ -21863,7 +21965,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>-3.4</v>
+        <v>-3.3</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -21951,7 +22053,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>-5.5</v>
+        <v>-4.9</v>
       </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
@@ -22039,7 +22141,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-13.5</v>
+        <v>-13.3</v>
       </c>
       <c r="S54" s="53" t="inlineStr">
         <is>
@@ -22126,7 +22228,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R55" s="42" t="n"/>
+      <c r="R55" s="42" t="n">
+        <v>-13.8</v>
+      </c>
       <c r="S55" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -22137,7 +22241,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U55" s="51" t="n"/>
+      <c r="U55" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V55" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -22872,7 +22980,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>-3.5</v>
+        <v>-2.5</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -22928,7 +23036,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -22984,7 +23092,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-24</v>
+        <v>-23.7</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -23040,7 +23148,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-4</v>
+        <v>-3.5</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -23096,7 +23204,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -23152,7 +23260,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>15.8</v>
+        <v>15</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -23344,7 +23452,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-8.199999999999999</v>
+        <v>-7.6</v>
       </c>
       <c r="S35" s="52" t="inlineStr">
         <is>
@@ -23432,7 +23540,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>0.1</v>
+        <v>-1.6</v>
       </c>
       <c r="S36" s="52" t="inlineStr">
         <is>
@@ -23520,7 +23628,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-5.8</v>
+        <v>-5.1</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -23608,7 +23716,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>16.7</v>
+        <v>17.6</v>
       </c>
       <c r="S38" s="52" t="inlineStr">
         <is>
@@ -23696,7 +23804,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -23784,7 +23892,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-14.1</v>
+        <v>-13.2</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -23990,7 +24098,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R44" s="42" t="n"/>
+      <c r="R44" s="42" t="n">
+        <v>2.2</v>
+      </c>
       <c r="S44" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -24001,7 +24111,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U44" s="51" t="n"/>
+      <c r="U44" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V44" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -24161,7 +24275,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-14.2</v>
+        <v>-14.4</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -24248,7 +24362,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R47" s="42" t="n"/>
+      <c r="R47" s="42" t="n">
+        <v>-4.5</v>
+      </c>
       <c r="S47" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -24259,7 +24375,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U47" s="51" t="n"/>
+      <c r="U47" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V47" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -24330,7 +24450,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R48" s="42" t="n"/>
+      <c r="R48" s="42" t="n">
+        <v>-19</v>
+      </c>
       <c r="S48" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -24341,7 +24463,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U48" s="51" t="n"/>
+      <c r="U48" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V48" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -24412,7 +24538,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R49" s="42" t="n"/>
+      <c r="R49" s="42" t="n">
+        <v>-5.1</v>
+      </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -24423,7 +24551,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U49" s="51" t="n"/>
+      <c r="U49" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V49" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -35381,7 +35513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -59866,7 +59998,7 @@
       <c r="P9" s="42" t="n"/>
       <c r="Q9" s="42" t="n"/>
       <c r="R9" s="42" t="n">
-        <v>8.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="S9" s="51" t="n"/>
       <c r="T9" s="51" t="n"/>
@@ -59922,7 +60054,7 @@
       <c r="P10" s="42" t="n"/>
       <c r="Q10" s="42" t="n"/>
       <c r="R10" s="42" t="n">
-        <v>-33.1</v>
+        <v>-33.4</v>
       </c>
       <c r="S10" s="51" t="n"/>
       <c r="T10" s="51" t="n"/>
@@ -59986,7 +60118,7 @@
       <c r="P11" s="42" t="n"/>
       <c r="Q11" s="42" t="n"/>
       <c r="R11" s="42" t="n">
-        <v>-9.300000000000001</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S11" s="51" t="n"/>
       <c r="T11" s="51" t="n"/>
@@ -60050,7 +60182,7 @@
       <c r="P12" s="42" t="n"/>
       <c r="Q12" s="42" t="n"/>
       <c r="R12" s="42" t="n">
-        <v>-17.6</v>
+        <v>-16.9</v>
       </c>
       <c r="S12" s="51" t="n"/>
       <c r="T12" s="51" t="n"/>
@@ -60106,7 +60238,7 @@
       <c r="P13" s="42" t="n"/>
       <c r="Q13" s="42" t="n"/>
       <c r="R13" s="42" t="n">
-        <v>-13.2</v>
+        <v>-13</v>
       </c>
       <c r="S13" s="51" t="n"/>
       <c r="T13" s="51" t="n"/>
@@ -60162,7 +60294,7 @@
       <c r="P14" s="42" t="n"/>
       <c r="Q14" s="42" t="n"/>
       <c r="R14" s="42" t="n">
-        <v>-30.3</v>
+        <v>-29.9</v>
       </c>
       <c r="S14" s="51" t="n"/>
       <c r="T14" s="51" t="n"/>
@@ -60218,7 +60350,7 @@
       <c r="P15" s="42" t="n"/>
       <c r="Q15" s="42" t="n"/>
       <c r="R15" s="42" t="n">
-        <v>8.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="S15" s="51" t="n"/>
       <c r="T15" s="51" t="n"/>
@@ -60330,7 +60462,7 @@
       <c r="P17" s="42" t="n"/>
       <c r="Q17" s="42" t="n"/>
       <c r="R17" s="42" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="S17" s="51" t="n"/>
       <c r="T17" s="51" t="n"/>
@@ -60386,7 +60518,7 @@
       <c r="P18" s="42" t="n"/>
       <c r="Q18" s="42" t="n"/>
       <c r="R18" s="42" t="n">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="S18" s="51" t="n"/>
       <c r="T18" s="51" t="n"/>
@@ -60442,7 +60574,7 @@
       <c r="P19" s="42" t="n"/>
       <c r="Q19" s="42" t="n"/>
       <c r="R19" s="42" t="n">
-        <v>-2.4</v>
+        <v>-2.6</v>
       </c>
       <c r="S19" s="51" t="n"/>
       <c r="T19" s="51" t="n"/>
@@ -60498,7 +60630,7 @@
       <c r="P20" s="42" t="n"/>
       <c r="Q20" s="42" t="n"/>
       <c r="R20" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S20" s="51" t="n"/>
       <c r="T20" s="51" t="n"/>
@@ -60554,7 +60686,7 @@
       <c r="P21" s="42" t="n"/>
       <c r="Q21" s="42" t="n"/>
       <c r="R21" s="42" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="S21" s="51" t="n"/>
       <c r="T21" s="51" t="n"/>
@@ -60610,7 +60742,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>-15.7</v>
+        <v>-14.8</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -60666,7 +60798,7 @@
       <c r="P23" s="42" t="n"/>
       <c r="Q23" s="42" t="n"/>
       <c r="R23" s="42" t="n">
-        <v>-11.4</v>
+        <v>-10.9</v>
       </c>
       <c r="S23" s="51" t="n"/>
       <c r="T23" s="51" t="n"/>
@@ -60722,7 +60854,7 @@
       <c r="P24" s="42" t="n"/>
       <c r="Q24" s="42" t="n"/>
       <c r="R24" s="42" t="n">
-        <v>-11</v>
+        <v>-11.7</v>
       </c>
       <c r="S24" s="51" t="n"/>
       <c r="T24" s="51" t="n"/>
@@ -60842,7 +60974,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>-1.1</v>
+        <v>-0.6</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -60906,7 +61038,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>-16.9</v>
+        <v>-15.6</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -60970,7 +61102,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-11.3</v>
+        <v>-10.7</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -61026,7 +61158,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-18.2</v>
+        <v>-18</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -61082,7 +61214,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-0.7</v>
+        <v>-0.5</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -61138,7 +61270,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>18.4</v>
+        <v>18.1</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -61202,7 +61334,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -61322,7 +61454,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-8.6</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -61378,7 +61510,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>9.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -61406,43 +61538,35 @@
       </c>
       <c r="E36" s="42" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="F36" s="42" t="inlineStr">
         <is>
-          <t>Oregon</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="G36" s="42" t="n">
-        <v>-11.4</v>
-      </c>
-      <c r="H36" s="42" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="I36" s="42" t="n">
-        <v>-1.1</v>
-      </c>
+        <v>8.6</v>
+      </c>
+      <c r="H36" s="42" t="n"/>
+      <c r="I36" s="42" t="n"/>
       <c r="J36" s="42" t="n">
-        <v>-18.1</v>
+        <v>8.4</v>
       </c>
       <c r="K36" s="42" t="n">
-        <v>-1.4</v>
+        <v>-7.1</v>
       </c>
       <c r="L36" s="42" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="M36" s="42" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="N36" s="47" t="n">
-        <v>-4.8</v>
-      </c>
+        <v>51.7</v>
+      </c>
+      <c r="M36" s="42" t="n"/>
+      <c r="N36" s="42" t="n"/>
       <c r="O36" s="42" t="n"/>
       <c r="P36" s="42" t="n"/>
       <c r="Q36" s="42" t="n"/>
       <c r="R36" s="42" t="n">
-        <v>-15.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="S36" s="51" t="n"/>
       <c r="T36" s="51" t="n"/>
@@ -61470,35 +61594,43 @@
       </c>
       <c r="E37" s="42" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="F37" s="42" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="G37" s="42" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="H37" s="42" t="n"/>
-      <c r="I37" s="42" t="n"/>
+        <v>-5.9</v>
+      </c>
+      <c r="H37" s="42" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="I37" s="47" t="n">
+        <v>2.4</v>
+      </c>
       <c r="J37" s="42" t="n">
-        <v>8.4</v>
+        <v>-5.4</v>
       </c>
       <c r="K37" s="42" t="n">
         <v>-7.1</v>
       </c>
       <c r="L37" s="42" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="M37" s="42" t="n"/>
-      <c r="N37" s="42" t="n"/>
+        <v>44.4</v>
+      </c>
+      <c r="M37" s="42" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="N37" s="47" t="n">
+        <v>-5.1</v>
+      </c>
       <c r="O37" s="42" t="n"/>
       <c r="P37" s="42" t="n"/>
       <c r="Q37" s="42" t="n"/>
       <c r="R37" s="42" t="n">
-        <v>8.9</v>
+        <v>-7.8</v>
       </c>
       <c r="S37" s="51" t="n"/>
       <c r="T37" s="51" t="n"/>
@@ -61511,7 +61643,7 @@
       </c>
       <c r="B38" s="42" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="C38" s="42" t="inlineStr">
@@ -61526,43 +61658,43 @@
       </c>
       <c r="E38" s="42" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="F38" s="42" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Oregon</t>
         </is>
       </c>
       <c r="G38" s="42" t="n">
-        <v>-5.9</v>
+        <v>-11.4</v>
       </c>
       <c r="H38" s="42" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="I38" s="47" t="n">
-        <v>2.4</v>
+        <v>-12.5</v>
+      </c>
+      <c r="I38" s="42" t="n">
+        <v>-1.1</v>
       </c>
       <c r="J38" s="42" t="n">
-        <v>-5.4</v>
+        <v>-18.1</v>
       </c>
       <c r="K38" s="42" t="n">
-        <v>-7.1</v>
+        <v>-1.4</v>
       </c>
       <c r="L38" s="42" t="n">
-        <v>44.4</v>
+        <v>53.7</v>
       </c>
       <c r="M38" s="42" t="n">
-        <v>49.5</v>
+        <v>58.5</v>
       </c>
       <c r="N38" s="47" t="n">
-        <v>-5.1</v>
+        <v>-4.8</v>
       </c>
       <c r="O38" s="42" t="n"/>
       <c r="P38" s="42" t="n"/>
       <c r="Q38" s="42" t="n"/>
       <c r="R38" s="42" t="n">
-        <v>-7.6</v>
+        <v>-15.2</v>
       </c>
       <c r="S38" s="51" t="n"/>
       <c r="T38" s="51" t="n"/>
@@ -61626,7 +61758,7 @@
       <c r="P39" s="42" t="n"/>
       <c r="Q39" s="42" t="n"/>
       <c r="R39" s="42" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="S39" s="51" t="n"/>
       <c r="T39" s="51" t="n"/>
@@ -61690,7 +61822,7 @@
       <c r="P40" s="42" t="n"/>
       <c r="Q40" s="42" t="n"/>
       <c r="R40" s="42" t="n">
-        <v>-11.4</v>
+        <v>-12.2</v>
       </c>
       <c r="S40" s="51" t="n"/>
       <c r="T40" s="51" t="n"/>
@@ -61754,7 +61886,7 @@
       <c r="P41" s="42" t="n"/>
       <c r="Q41" s="42" t="n"/>
       <c r="R41" s="42" t="n">
-        <v>-1.7</v>
+        <v>-1.9</v>
       </c>
       <c r="S41" s="51" t="n"/>
       <c r="T41" s="51" t="n"/>
@@ -61818,7 +61950,7 @@
       <c r="P42" s="42" t="n"/>
       <c r="Q42" s="42" t="n"/>
       <c r="R42" s="42" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="S42" s="51" t="n"/>
       <c r="T42" s="51" t="n"/>
@@ -61874,7 +62006,7 @@
       <c r="P43" s="42" t="n"/>
       <c r="Q43" s="42" t="n"/>
       <c r="R43" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.7</v>
       </c>
       <c r="S43" s="51" t="n"/>
       <c r="T43" s="51" t="n"/>
@@ -61930,7 +62062,7 @@
       <c r="P44" s="42" t="n"/>
       <c r="Q44" s="42" t="n"/>
       <c r="R44" s="42" t="n">
-        <v>-14.8</v>
+        <v>-14</v>
       </c>
       <c r="S44" s="51" t="n"/>
       <c r="T44" s="51" t="n"/>
@@ -61986,7 +62118,7 @@
       <c r="P45" s="42" t="n"/>
       <c r="Q45" s="42" t="n"/>
       <c r="R45" s="42" t="n">
-        <v>6</v>
+        <v>6.8</v>
       </c>
       <c r="S45" s="51" t="n"/>
       <c r="T45" s="51" t="n"/>
@@ -62042,7 +62174,7 @@
       <c r="P46" s="42" t="n"/>
       <c r="Q46" s="42" t="n"/>
       <c r="R46" s="42" t="n">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="S46" s="51" t="n"/>
       <c r="T46" s="51" t="n"/>
@@ -62098,7 +62230,7 @@
       <c r="P47" s="42" t="n"/>
       <c r="Q47" s="42" t="n"/>
       <c r="R47" s="42" t="n">
-        <v>-10.3</v>
+        <v>-11</v>
       </c>
       <c r="S47" s="51" t="n"/>
       <c r="T47" s="51" t="n"/>
@@ -62154,7 +62286,7 @@
       <c r="P48" s="42" t="n"/>
       <c r="Q48" s="42" t="n"/>
       <c r="R48" s="42" t="n">
-        <v>18.8</v>
+        <v>19.1</v>
       </c>
       <c r="S48" s="51" t="n"/>
       <c r="T48" s="51" t="n"/>
@@ -62210,7 +62342,7 @@
       <c r="P49" s="42" t="n"/>
       <c r="Q49" s="42" t="n"/>
       <c r="R49" s="42" t="n">
-        <v>-0.5</v>
+        <v>0.6</v>
       </c>
       <c r="S49" s="51" t="n"/>
       <c r="T49" s="51" t="n"/>
@@ -62266,7 +62398,7 @@
       <c r="P50" s="42" t="n"/>
       <c r="Q50" s="42" t="n"/>
       <c r="R50" s="42" t="n">
-        <v>-18.2</v>
+        <v>-19</v>
       </c>
       <c r="S50" s="51" t="n"/>
       <c r="T50" s="51" t="n"/>
@@ -62322,7 +62454,7 @@
       <c r="P51" s="42" t="n"/>
       <c r="Q51" s="42" t="n"/>
       <c r="R51" s="42" t="n">
-        <v>-6.6</v>
+        <v>-6.3</v>
       </c>
       <c r="S51" s="51" t="n"/>
       <c r="T51" s="51" t="n"/>
@@ -62378,7 +62510,7 @@
       <c r="P52" s="42" t="n"/>
       <c r="Q52" s="42" t="n"/>
       <c r="R52" s="42" t="n">
-        <v>9.699999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="S52" s="51" t="n"/>
       <c r="T52" s="51" t="n"/>
@@ -62434,7 +62566,7 @@
       <c r="P53" s="42" t="n"/>
       <c r="Q53" s="42" t="n"/>
       <c r="R53" s="42" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="S53" s="51" t="n"/>
       <c r="T53" s="51" t="n"/>
@@ -62498,7 +62630,7 @@
       <c r="P54" s="42" t="n"/>
       <c r="Q54" s="42" t="n"/>
       <c r="R54" s="42" t="n">
-        <v>-14.5</v>
+        <v>-15.2</v>
       </c>
       <c r="S54" s="51" t="n"/>
       <c r="T54" s="51" t="n"/>
@@ -62554,7 +62686,7 @@
       <c r="P55" s="42" t="n"/>
       <c r="Q55" s="42" t="n"/>
       <c r="R55" s="42" t="n">
-        <v>-3.4</v>
+        <v>-3.6</v>
       </c>
       <c r="S55" s="51" t="n"/>
       <c r="T55" s="51" t="n"/>
@@ -62610,7 +62742,7 @@
       <c r="P56" s="42" t="n"/>
       <c r="Q56" s="42" t="n"/>
       <c r="R56" s="42" t="n">
-        <v>3.2</v>
+        <v>2.2</v>
       </c>
       <c r="S56" s="51" t="n"/>
       <c r="T56" s="51" t="n"/>
@@ -62674,7 +62806,7 @@
       <c r="P57" s="42" t="n"/>
       <c r="Q57" s="42" t="n"/>
       <c r="R57" s="42" t="n">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="S57" s="51" t="n"/>
       <c r="T57" s="51" t="n"/>
@@ -62738,7 +62870,7 @@
       <c r="P58" s="42" t="n"/>
       <c r="Q58" s="42" t="n"/>
       <c r="R58" s="42" t="n">
-        <v>-10.5</v>
+        <v>-10.6</v>
       </c>
       <c r="S58" s="51" t="n"/>
       <c r="T58" s="51" t="n"/>
@@ -62802,7 +62934,7 @@
       <c r="P59" s="42" t="n"/>
       <c r="Q59" s="42" t="n"/>
       <c r="R59" s="42" t="n">
-        <v>-15</v>
+        <v>-14.7</v>
       </c>
       <c r="S59" s="51" t="n"/>
       <c r="T59" s="51" t="n"/>
@@ -62866,7 +62998,7 @@
       <c r="P60" s="42" t="n"/>
       <c r="Q60" s="42" t="n"/>
       <c r="R60" s="42" t="n">
-        <v>-10.1</v>
+        <v>-10.2</v>
       </c>
       <c r="S60" s="51" t="n"/>
       <c r="T60" s="51" t="n"/>
@@ -62930,7 +63062,7 @@
       <c r="P61" s="42" t="n"/>
       <c r="Q61" s="42" t="n"/>
       <c r="R61" s="42" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="S61" s="51" t="n"/>
       <c r="T61" s="51" t="n"/>
@@ -62994,7 +63126,7 @@
       <c r="P62" s="42" t="n"/>
       <c r="Q62" s="42" t="n"/>
       <c r="R62" s="42" t="n">
-        <v>-15.4</v>
+        <v>-16.2</v>
       </c>
       <c r="S62" s="51" t="n"/>
       <c r="T62" s="51" t="n"/>
@@ -63050,7 +63182,7 @@
       <c r="P63" s="42" t="n"/>
       <c r="Q63" s="42" t="n"/>
       <c r="R63" s="42" t="n">
-        <v>-33.1</v>
+        <v>-33.4</v>
       </c>
       <c r="S63" s="51" t="n"/>
       <c r="T63" s="51" t="n"/>
@@ -63106,7 +63238,7 @@
       <c r="P64" s="42" t="n"/>
       <c r="Q64" s="42" t="n"/>
       <c r="R64" s="42" t="n">
-        <v>-11.7</v>
+        <v>-11.5</v>
       </c>
       <c r="S64" s="51" t="n"/>
       <c r="T64" s="51" t="n"/>
@@ -63162,7 +63294,7 @@
       <c r="P65" s="42" t="n"/>
       <c r="Q65" s="42" t="n"/>
       <c r="R65" s="42" t="n">
-        <v>-3.5</v>
+        <v>-2.5</v>
       </c>
       <c r="S65" s="51" t="n"/>
       <c r="T65" s="51" t="n"/>
@@ -63218,7 +63350,7 @@
       <c r="P66" s="42" t="n"/>
       <c r="Q66" s="42" t="n"/>
       <c r="R66" s="42" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="S66" s="51" t="n"/>
       <c r="T66" s="51" t="n"/>
@@ -63274,7 +63406,7 @@
       <c r="P67" s="42" t="n"/>
       <c r="Q67" s="42" t="n"/>
       <c r="R67" s="42" t="n">
-        <v>-24</v>
+        <v>-23.7</v>
       </c>
       <c r="S67" s="51" t="n"/>
       <c r="T67" s="51" t="n"/>
@@ -63330,7 +63462,7 @@
       <c r="P68" s="42" t="n"/>
       <c r="Q68" s="42" t="n"/>
       <c r="R68" s="42" t="n">
-        <v>-4</v>
+        <v>-3.5</v>
       </c>
       <c r="S68" s="51" t="n"/>
       <c r="T68" s="51" t="n"/>
@@ -63386,7 +63518,7 @@
       <c r="P69" s="42" t="n"/>
       <c r="Q69" s="42" t="n"/>
       <c r="R69" s="42" t="n">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="S69" s="51" t="n"/>
       <c r="T69" s="51" t="n"/>
@@ -63442,7 +63574,7 @@
       <c r="P70" s="42" t="n"/>
       <c r="Q70" s="42" t="n"/>
       <c r="R70" s="42" t="n">
-        <v>15.8</v>
+        <v>15</v>
       </c>
       <c r="S70" s="51" t="n"/>
       <c r="T70" s="51" t="n"/>
@@ -63633,7 +63765,7 @@
         </is>
       </c>
       <c r="R74" s="42" t="n">
-        <v>-4.5</v>
+        <v>-5.4</v>
       </c>
       <c r="S74" s="53" t="inlineStr">
         <is>
@@ -63721,7 +63853,7 @@
         </is>
       </c>
       <c r="R75" s="42" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="S75" s="53" t="inlineStr">
         <is>
@@ -63809,7 +63941,7 @@
         </is>
       </c>
       <c r="R76" s="42" t="n">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
       <c r="S76" s="52" t="inlineStr">
         <is>
@@ -63897,7 +64029,7 @@
         </is>
       </c>
       <c r="R77" s="42" t="n">
-        <v>-1.3</v>
+        <v>-1.7</v>
       </c>
       <c r="S77" s="53" t="inlineStr">
         <is>
@@ -63985,7 +64117,7 @@
         </is>
       </c>
       <c r="R78" s="42" t="n">
-        <v>-13.4</v>
+        <v>-13.5</v>
       </c>
       <c r="S78" s="52" t="inlineStr">
         <is>
@@ -64073,7 +64205,7 @@
         </is>
       </c>
       <c r="R79" s="42" t="n">
-        <v>-4.7</v>
+        <v>-4.8</v>
       </c>
       <c r="S79" s="52" t="inlineStr">
         <is>
@@ -64161,7 +64293,7 @@
         </is>
       </c>
       <c r="R80" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.1</v>
       </c>
       <c r="S80" s="52" t="inlineStr">
         <is>
@@ -64249,7 +64381,7 @@
         </is>
       </c>
       <c r="R81" s="42" t="n">
-        <v>-4.5</v>
+        <v>-4.8</v>
       </c>
       <c r="S81" s="54" t="inlineStr">
         <is>
@@ -64337,7 +64469,7 @@
         </is>
       </c>
       <c r="R82" s="42" t="n">
-        <v>-12.1</v>
+        <v>-12.7</v>
       </c>
       <c r="S82" s="53" t="inlineStr">
         <is>
@@ -64425,7 +64557,7 @@
         </is>
       </c>
       <c r="R83" s="42" t="n">
-        <v>-12.4</v>
+        <v>-11</v>
       </c>
       <c r="S83" s="53" t="inlineStr">
         <is>
@@ -64513,7 +64645,7 @@
         </is>
       </c>
       <c r="R84" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.7</v>
       </c>
       <c r="S84" s="53" t="inlineStr">
         <is>
@@ -64601,7 +64733,7 @@
         </is>
       </c>
       <c r="R85" s="42" t="n">
-        <v>-25.8</v>
+        <v>-25.3</v>
       </c>
       <c r="S85" s="53" t="inlineStr">
         <is>
@@ -64689,7 +64821,7 @@
         </is>
       </c>
       <c r="R86" s="42" t="n">
-        <v>-1.9</v>
+        <v>-2.1</v>
       </c>
       <c r="S86" s="52" t="inlineStr">
         <is>
@@ -64777,7 +64909,7 @@
         </is>
       </c>
       <c r="R87" s="42" t="n">
-        <v>-13.8</v>
+        <v>-14.7</v>
       </c>
       <c r="S87" s="53" t="inlineStr">
         <is>
@@ -64865,7 +64997,7 @@
         </is>
       </c>
       <c r="R88" s="42" t="n">
-        <v>-1.8</v>
+        <v>-1.2</v>
       </c>
       <c r="S88" s="52" t="inlineStr">
         <is>
@@ -64877,9 +65009,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U88" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U88" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V88" s="53" t="inlineStr">
@@ -64953,7 +65085,7 @@
         </is>
       </c>
       <c r="R89" s="42" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="S89" s="52" t="inlineStr">
         <is>
@@ -65041,7 +65173,7 @@
         </is>
       </c>
       <c r="R90" s="42" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="S90" s="53" t="inlineStr">
         <is>
@@ -65129,7 +65261,7 @@
         </is>
       </c>
       <c r="R91" s="42" t="n">
-        <v>-14.9</v>
+        <v>-14.5</v>
       </c>
       <c r="S91" s="53" t="inlineStr">
         <is>
@@ -65217,7 +65349,7 @@
         </is>
       </c>
       <c r="R92" s="42" t="n">
-        <v>-18.8</v>
+        <v>-19.7</v>
       </c>
       <c r="S92" s="53" t="inlineStr">
         <is>
@@ -65305,7 +65437,7 @@
         </is>
       </c>
       <c r="R93" s="42" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="S93" s="52" t="inlineStr">
         <is>
@@ -65393,7 +65525,7 @@
         </is>
       </c>
       <c r="R94" s="42" t="n">
-        <v>14.1</v>
+        <v>14.3</v>
       </c>
       <c r="S94" s="52" t="inlineStr">
         <is>
@@ -65481,7 +65613,7 @@
         </is>
       </c>
       <c r="R95" s="42" t="n">
-        <v>-24.1</v>
+        <v>-26.2</v>
       </c>
       <c r="S95" s="52" t="inlineStr">
         <is>
@@ -65657,7 +65789,7 @@
         </is>
       </c>
       <c r="R97" s="42" t="n">
-        <v>-24.6</v>
+        <v>-25.6</v>
       </c>
       <c r="S97" s="52" t="inlineStr">
         <is>
@@ -65745,7 +65877,7 @@
         </is>
       </c>
       <c r="R98" s="42" t="n">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="S98" s="52" t="inlineStr">
         <is>
@@ -65833,7 +65965,7 @@
         </is>
       </c>
       <c r="R99" s="42" t="n">
-        <v>-0.3</v>
+        <v>0.2</v>
       </c>
       <c r="S99" s="53" t="inlineStr">
         <is>
@@ -65921,7 +66053,7 @@
         </is>
       </c>
       <c r="R100" s="42" t="n">
-        <v>11</v>
+        <v>10.1</v>
       </c>
       <c r="S100" s="52" t="inlineStr">
         <is>
@@ -66009,7 +66141,7 @@
         </is>
       </c>
       <c r="R101" s="42" t="n">
-        <v>-9.800000000000001</v>
+        <v>-9.6</v>
       </c>
       <c r="S101" s="52" t="inlineStr">
         <is>
@@ -66097,7 +66229,7 @@
         </is>
       </c>
       <c r="R102" s="42" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="S102" s="52" t="inlineStr">
         <is>
@@ -66185,7 +66317,7 @@
         </is>
       </c>
       <c r="R103" s="42" t="n">
-        <v>-13.2</v>
+        <v>-11.8</v>
       </c>
       <c r="S103" s="53" t="inlineStr">
         <is>
@@ -66197,9 +66329,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U103" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U103" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V103" s="52" t="inlineStr">
@@ -66273,7 +66405,7 @@
         </is>
       </c>
       <c r="R104" s="42" t="n">
-        <v>-9.300000000000001</v>
+        <v>-8.5</v>
       </c>
       <c r="S104" s="53" t="inlineStr">
         <is>
@@ -66361,7 +66493,7 @@
         </is>
       </c>
       <c r="R105" s="42" t="n">
-        <v>-37.8</v>
+        <v>-36.9</v>
       </c>
       <c r="S105" s="52" t="inlineStr">
         <is>
@@ -66373,9 +66505,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U105" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U105" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V105" s="52" t="inlineStr">
@@ -66449,7 +66581,7 @@
         </is>
       </c>
       <c r="R106" s="42" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
       <c r="S106" s="53" t="inlineStr">
         <is>
@@ -66537,7 +66669,7 @@
         </is>
       </c>
       <c r="R107" s="42" t="n">
-        <v>-9.1</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="S107" s="53" t="inlineStr">
         <is>
@@ -66625,7 +66757,7 @@
         </is>
       </c>
       <c r="R108" s="42" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="S108" s="52" t="inlineStr">
         <is>
@@ -66801,7 +66933,7 @@
         </is>
       </c>
       <c r="R110" s="42" t="n">
-        <v>-14.4</v>
+        <v>-13.6</v>
       </c>
       <c r="S110" s="53" t="inlineStr">
         <is>
@@ -66889,7 +67021,7 @@
         </is>
       </c>
       <c r="R111" s="42" t="n">
-        <v>-15.7</v>
+        <v>-15.5</v>
       </c>
       <c r="S111" s="53" t="inlineStr">
         <is>
@@ -66977,7 +67109,7 @@
         </is>
       </c>
       <c r="R112" s="42" t="n">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
       <c r="S112" s="53" t="inlineStr">
         <is>
@@ -67065,7 +67197,7 @@
         </is>
       </c>
       <c r="R113" s="42" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="S113" s="52" t="inlineStr">
         <is>
@@ -67153,7 +67285,7 @@
         </is>
       </c>
       <c r="R114" s="42" t="n">
-        <v>4.1</v>
+        <v>4.6</v>
       </c>
       <c r="S114" s="52" t="inlineStr">
         <is>
@@ -67212,7 +67344,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="I115" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="J115" s="42" t="n">
         <v>5</v>
@@ -67241,7 +67373,7 @@
         </is>
       </c>
       <c r="R115" s="42" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="S115" s="53" t="inlineStr">
         <is>
@@ -67329,7 +67461,7 @@
         </is>
       </c>
       <c r="R116" s="42" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="S116" s="52" t="inlineStr">
         <is>
@@ -67417,7 +67549,7 @@
         </is>
       </c>
       <c r="R117" s="42" t="n">
-        <v>-2.6</v>
+        <v>-1.5</v>
       </c>
       <c r="S117" s="53" t="inlineStr">
         <is>
@@ -67505,7 +67637,7 @@
         </is>
       </c>
       <c r="R118" s="42" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="S118" s="53" t="inlineStr">
         <is>
@@ -67593,7 +67725,7 @@
         </is>
       </c>
       <c r="R119" s="42" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="S119" s="53" t="inlineStr">
         <is>
@@ -67681,7 +67813,7 @@
         </is>
       </c>
       <c r="R120" s="42" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="S120" s="52" t="inlineStr">
         <is>
@@ -67769,7 +67901,7 @@
         </is>
       </c>
       <c r="R121" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="S121" s="53" t="inlineStr">
         <is>
@@ -67857,7 +67989,7 @@
         </is>
       </c>
       <c r="R122" s="42" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="S122" s="52" t="inlineStr">
         <is>
@@ -67945,7 +68077,7 @@
         </is>
       </c>
       <c r="R123" s="42" t="n">
-        <v>-0.1</v>
+        <v>0.7</v>
       </c>
       <c r="S123" s="52" t="inlineStr">
         <is>
@@ -68033,7 +68165,7 @@
         </is>
       </c>
       <c r="R124" s="42" t="n">
-        <v>11.4</v>
+        <v>10.7</v>
       </c>
       <c r="S124" s="52" t="inlineStr">
         <is>
@@ -68121,7 +68253,7 @@
         </is>
       </c>
       <c r="R125" s="42" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="S125" s="52" t="inlineStr">
         <is>
@@ -68209,7 +68341,7 @@
         </is>
       </c>
       <c r="R126" s="42" t="n">
-        <v>-8.199999999999999</v>
+        <v>-7.6</v>
       </c>
       <c r="S126" s="52" t="inlineStr">
         <is>
@@ -68297,7 +68429,7 @@
         </is>
       </c>
       <c r="R127" s="42" t="n">
-        <v>0.1</v>
+        <v>-1.6</v>
       </c>
       <c r="S127" s="52" t="inlineStr">
         <is>
@@ -68385,7 +68517,7 @@
         </is>
       </c>
       <c r="R128" s="42" t="n">
-        <v>-5.8</v>
+        <v>-5.1</v>
       </c>
       <c r="S128" s="53" t="inlineStr">
         <is>
@@ -68473,7 +68605,7 @@
         </is>
       </c>
       <c r="R129" s="42" t="n">
-        <v>16.7</v>
+        <v>17.6</v>
       </c>
       <c r="S129" s="52" t="inlineStr">
         <is>
@@ -68561,7 +68693,7 @@
         </is>
       </c>
       <c r="R130" s="42" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="S130" s="52" t="inlineStr">
         <is>
@@ -68649,7 +68781,7 @@
         </is>
       </c>
       <c r="R131" s="42" t="n">
-        <v>-14.1</v>
+        <v>-13.2</v>
       </c>
       <c r="S131" s="53" t="inlineStr">
         <is>
@@ -68856,7 +68988,7 @@
         </is>
       </c>
       <c r="R135" s="42" t="n">
-        <v>-1.1</v>
+        <v>-0.3</v>
       </c>
       <c r="S135" s="53" t="inlineStr">
         <is>
@@ -68868,9 +69000,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U135" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U135" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V135" s="53" t="inlineStr">
@@ -68943,7 +69075,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R136" s="42" t="n"/>
+      <c r="R136" s="42" t="n">
+        <v>6.7</v>
+      </c>
       <c r="S136" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -68954,7 +69088,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U136" s="51" t="n"/>
+      <c r="U136" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V136" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -69026,7 +69164,7 @@
         </is>
       </c>
       <c r="R137" s="42" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="S137" s="52" t="inlineStr">
         <is>
@@ -69114,7 +69252,7 @@
         </is>
       </c>
       <c r="R138" s="42" t="n">
-        <v>-1.3</v>
+        <v>-1.4</v>
       </c>
       <c r="S138" s="52" t="inlineStr">
         <is>
@@ -69202,7 +69340,7 @@
         </is>
       </c>
       <c r="R139" s="42" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="S139" s="52" t="inlineStr">
         <is>
@@ -69290,7 +69428,7 @@
         </is>
       </c>
       <c r="R140" s="42" t="n">
-        <v>-20.8</v>
+        <v>-20.1</v>
       </c>
       <c r="S140" s="52" t="inlineStr">
         <is>
@@ -69302,9 +69440,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U140" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U140" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V140" s="53" t="inlineStr">
@@ -69378,7 +69516,7 @@
         </is>
       </c>
       <c r="R141" s="42" t="n">
-        <v>-8</v>
+        <v>-8.1</v>
       </c>
       <c r="S141" s="53" t="inlineStr">
         <is>
@@ -69466,7 +69604,7 @@
         </is>
       </c>
       <c r="R142" s="42" t="n">
-        <v>3.1</v>
+        <v>4.1</v>
       </c>
       <c r="S142" s="52" t="inlineStr">
         <is>
@@ -69554,7 +69692,7 @@
         </is>
       </c>
       <c r="R143" s="42" t="n">
-        <v>16.2</v>
+        <v>15.6</v>
       </c>
       <c r="S143" s="53" t="inlineStr">
         <is>
@@ -69641,7 +69779,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R144" s="42" t="n"/>
+      <c r="R144" s="42" t="n">
+        <v>-32.2</v>
+      </c>
       <c r="S144" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -69652,7 +69792,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U144" s="51" t="n"/>
+      <c r="U144" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V144" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -69723,7 +69867,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R145" s="42" t="n"/>
+      <c r="R145" s="42" t="n">
+        <v>15.9</v>
+      </c>
       <c r="S145" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -69734,7 +69880,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U145" s="51" t="n"/>
+      <c r="U145" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V145" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -69805,7 +69955,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R146" s="42" t="n"/>
+      <c r="R146" s="42" t="n">
+        <v>-13.6</v>
+      </c>
       <c r="S146" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -69816,7 +69968,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U146" s="51" t="n"/>
+      <c r="U146" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V146" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -69888,7 +70044,7 @@
         </is>
       </c>
       <c r="R147" s="42" t="n">
-        <v>-24</v>
+        <v>-23.8</v>
       </c>
       <c r="S147" s="52" t="inlineStr">
         <is>
@@ -69975,7 +70131,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R148" s="42" t="n"/>
+      <c r="R148" s="42" t="n">
+        <v>17.7</v>
+      </c>
       <c r="S148" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -69986,7 +70144,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U148" s="51" t="n"/>
+      <c r="U148" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V148" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -70058,7 +70220,7 @@
         </is>
       </c>
       <c r="R149" s="42" t="n">
-        <v>-12.8</v>
+        <v>-12.3</v>
       </c>
       <c r="S149" s="52" t="inlineStr">
         <is>
@@ -70234,7 +70396,7 @@
         </is>
       </c>
       <c r="R151" s="42" t="n">
-        <v>-13.7</v>
+        <v>-13</v>
       </c>
       <c r="S151" s="53" t="inlineStr">
         <is>
@@ -70321,7 +70483,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R152" s="42" t="n"/>
+      <c r="R152" s="42" t="n">
+        <v>6.2</v>
+      </c>
       <c r="S152" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -70332,7 +70496,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U152" s="51" t="n"/>
+      <c r="U152" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V152" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -70403,7 +70571,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R153" s="42" t="n"/>
+      <c r="R153" s="42" t="n">
+        <v>-13.1</v>
+      </c>
       <c r="S153" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -70414,7 +70584,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U153" s="51" t="n"/>
+      <c r="U153" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V153" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -70485,7 +70659,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R154" s="42" t="n"/>
+      <c r="R154" s="42" t="n">
+        <v>-7.8</v>
+      </c>
       <c r="S154" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -70496,7 +70672,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U154" s="51" t="n"/>
+      <c r="U154" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V154" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -70568,7 +70748,7 @@
         </is>
       </c>
       <c r="R155" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.3</v>
       </c>
       <c r="S155" s="52" t="inlineStr">
         <is>
@@ -70656,7 +70836,7 @@
         </is>
       </c>
       <c r="R156" s="42" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="S156" s="52" t="inlineStr">
         <is>
@@ -70744,7 +70924,7 @@
         </is>
       </c>
       <c r="R157" s="42" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="S157" s="53" t="inlineStr">
         <is>
@@ -70832,7 +71012,7 @@
         </is>
       </c>
       <c r="R158" s="42" t="n">
-        <v>-11.2</v>
+        <v>-11.3</v>
       </c>
       <c r="S158" s="53" t="inlineStr">
         <is>
@@ -70920,7 +71100,7 @@
         </is>
       </c>
       <c r="R159" s="42" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="S159" s="52" t="inlineStr">
         <is>
@@ -71007,7 +71187,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R160" s="42" t="n"/>
+      <c r="R160" s="42" t="n">
+        <v>-4.7</v>
+      </c>
       <c r="S160" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -71018,7 +71200,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U160" s="51" t="n"/>
+      <c r="U160" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V160" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -71090,7 +71276,7 @@
         </is>
       </c>
       <c r="R161" s="42" t="n">
-        <v>-6</v>
+        <v>-6.2</v>
       </c>
       <c r="S161" s="52" t="inlineStr">
         <is>
@@ -71177,7 +71363,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R162" s="42" t="n"/>
+      <c r="R162" s="42" t="n">
+        <v>16.8</v>
+      </c>
       <c r="S162" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -71188,7 +71376,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U162" s="51" t="n"/>
+      <c r="U162" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V162" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -71260,7 +71452,7 @@
         </is>
       </c>
       <c r="R163" s="42" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="S163" s="52" t="inlineStr">
         <is>
@@ -71348,7 +71540,7 @@
         </is>
       </c>
       <c r="R164" s="42" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="S164" s="52" t="inlineStr">
         <is>
@@ -71436,7 +71628,7 @@
         </is>
       </c>
       <c r="R165" s="42" t="n">
-        <v>-6.2</v>
+        <v>-6.8</v>
       </c>
       <c r="S165" s="53" t="inlineStr">
         <is>
@@ -71524,7 +71716,7 @@
         </is>
       </c>
       <c r="R166" s="42" t="n">
-        <v>15.3</v>
+        <v>13.7</v>
       </c>
       <c r="S166" s="52" t="inlineStr">
         <is>
@@ -71612,7 +71804,7 @@
         </is>
       </c>
       <c r="R167" s="42" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="S167" s="52" t="inlineStr">
         <is>
@@ -71700,7 +71892,7 @@
         </is>
       </c>
       <c r="R168" s="42" t="n">
-        <v>-7.2</v>
+        <v>-7.3</v>
       </c>
       <c r="S168" s="53" t="inlineStr">
         <is>
@@ -71788,7 +71980,7 @@
         </is>
       </c>
       <c r="R169" s="42" t="n">
-        <v>15.2</v>
+        <v>15</v>
       </c>
       <c r="S169" s="52" t="inlineStr">
         <is>
@@ -71876,7 +72068,7 @@
         </is>
       </c>
       <c r="R170" s="42" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="S170" s="53" t="inlineStr">
         <is>
@@ -71964,7 +72156,7 @@
         </is>
       </c>
       <c r="R171" s="42" t="n">
-        <v>-11</v>
+        <v>-11.1</v>
       </c>
       <c r="S171" s="52" t="inlineStr">
         <is>
@@ -72052,7 +72244,7 @@
         </is>
       </c>
       <c r="R172" s="42" t="n">
-        <v>-2.1</v>
+        <v>-1.5</v>
       </c>
       <c r="S172" s="52" t="inlineStr">
         <is>
@@ -72064,9 +72256,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U172" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U172" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V172" s="53" t="inlineStr">
@@ -72140,7 +72332,7 @@
         </is>
       </c>
       <c r="R173" s="42" t="n">
-        <v>-20.7</v>
+        <v>-22</v>
       </c>
       <c r="S173" s="53" t="inlineStr">
         <is>
@@ -72228,7 +72420,7 @@
         </is>
       </c>
       <c r="R174" s="42" t="n">
-        <v>-21.1</v>
+        <v>-21.8</v>
       </c>
       <c r="S174" s="53" t="inlineStr">
         <is>
@@ -72316,7 +72508,7 @@
         </is>
       </c>
       <c r="R175" s="42" t="n">
-        <v>-6.8</v>
+        <v>-7</v>
       </c>
       <c r="S175" s="53" t="inlineStr">
         <is>
@@ -72403,7 +72595,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R176" s="42" t="n"/>
+      <c r="R176" s="42" t="n">
+        <v>-7.3</v>
+      </c>
       <c r="S176" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -72414,7 +72608,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U176" s="51" t="n"/>
+      <c r="U176" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V176" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -72485,7 +72683,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R177" s="42" t="n"/>
+      <c r="R177" s="42" t="n">
+        <v>-15</v>
+      </c>
       <c r="S177" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -72496,7 +72696,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U177" s="51" t="n"/>
+      <c r="U177" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V177" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -72567,7 +72771,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R178" s="42" t="n"/>
+      <c r="R178" s="42" t="n">
+        <v>-2.4</v>
+      </c>
       <c r="S178" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -72578,7 +72784,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U178" s="51" t="n"/>
+      <c r="U178" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V178" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -72649,7 +72859,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R179" s="42" t="n"/>
+      <c r="R179" s="42" t="n">
+        <v>1.5</v>
+      </c>
       <c r="S179" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -72660,7 +72872,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U179" s="51" t="n"/>
+      <c r="U179" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V179" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -72731,7 +72947,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R180" s="42" t="n"/>
+      <c r="R180" s="42" t="n">
+        <v>1.3</v>
+      </c>
       <c r="S180" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -72742,7 +72960,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U180" s="51" t="n"/>
+      <c r="U180" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V180" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -72814,7 +73036,7 @@
         </is>
       </c>
       <c r="R181" s="42" t="n">
-        <v>-15.5</v>
+        <v>-16.4</v>
       </c>
       <c r="S181" s="53" t="inlineStr">
         <is>
@@ -72901,7 +73123,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R182" s="42" t="n"/>
+      <c r="R182" s="42" t="n">
+        <v>-40.5</v>
+      </c>
       <c r="S182" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -72912,7 +73136,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U182" s="51" t="n"/>
+      <c r="U182" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V182" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -72984,7 +73212,7 @@
         </is>
       </c>
       <c r="R183" s="42" t="n">
-        <v>16.1</v>
+        <v>15.4</v>
       </c>
       <c r="S183" s="53" t="inlineStr">
         <is>
@@ -73072,7 +73300,7 @@
         </is>
       </c>
       <c r="R184" s="42" t="n">
-        <v>-3.4</v>
+        <v>-3.3</v>
       </c>
       <c r="S184" s="52" t="inlineStr">
         <is>
@@ -73160,7 +73388,7 @@
         </is>
       </c>
       <c r="R185" s="42" t="n">
-        <v>-5.5</v>
+        <v>-4.9</v>
       </c>
       <c r="S185" s="52" t="inlineStr">
         <is>
@@ -73248,7 +73476,7 @@
         </is>
       </c>
       <c r="R186" s="42" t="n">
-        <v>-13.5</v>
+        <v>-13.3</v>
       </c>
       <c r="S186" s="53" t="inlineStr">
         <is>
@@ -73335,7 +73563,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R187" s="42" t="n"/>
+      <c r="R187" s="42" t="n">
+        <v>-13.8</v>
+      </c>
       <c r="S187" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -73346,7 +73576,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U187" s="51" t="n"/>
+      <c r="U187" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V187" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -73417,7 +73651,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R188" s="42" t="n"/>
+      <c r="R188" s="42" t="n">
+        <v>2.2</v>
+      </c>
       <c r="S188" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -73428,7 +73664,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U188" s="51" t="n"/>
+      <c r="U188" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V188" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -73588,7 +73828,7 @@
         </is>
       </c>
       <c r="R190" s="42" t="n">
-        <v>-14.2</v>
+        <v>-14.4</v>
       </c>
       <c r="S190" s="53" t="inlineStr">
         <is>
@@ -73675,7 +73915,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="R191" s="42" t="n"/>
+      <c r="R191" s="42" t="n">
+        <v>-4.5</v>
+      </c>
       <c r="S191" s="52" t="inlineStr">
         <is>
           <t>Loss</t>
@@ -73686,7 +73928,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U191" s="51" t="n"/>
+      <c r="U191" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V191" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -73757,7 +74003,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R192" s="42" t="n"/>
+      <c r="R192" s="42" t="n">
+        <v>-19</v>
+      </c>
       <c r="S192" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -73768,7 +74016,11 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U192" s="51" t="n"/>
+      <c r="U192" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="V192" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -73839,7 +74091,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="R193" s="42" t="n"/>
+      <c r="R193" s="42" t="n">
+        <v>-5.1</v>
+      </c>
       <c r="S193" s="53" t="inlineStr">
         <is>
           <t>Win</t>
@@ -73850,7 +74104,11 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U193" s="51" t="n"/>
+      <c r="U193" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="V193" s="52" t="inlineStr">
         <is>
           <t>Loss</t>

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-10-15 14:42 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -1632,7 +1632,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>9.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -1688,7 +1688,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-33.7</v>
+        <v>-33.4</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -1752,7 +1752,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-9.5</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -1816,7 +1816,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-17</v>
+        <v>-17.6</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -1880,7 +1880,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-12.4</v>
+        <v>-12.5</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -1936,7 +1936,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-30.1</v>
+        <v>-29.9</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -2000,7 +2000,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>9.9</v>
+        <v>9.5</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -2064,7 +2064,7 @@
       <c r="P36" s="42" t="n"/>
       <c r="Q36" s="42" t="n"/>
       <c r="R36" s="42" t="n">
-        <v>-5.7</v>
+        <v>-5.8</v>
       </c>
       <c r="S36" s="51" t="n"/>
       <c r="T36" s="51" t="n"/>
@@ -2128,7 +2128,7 @@
       <c r="P37" s="42" t="n"/>
       <c r="Q37" s="42" t="n"/>
       <c r="R37" s="42" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="S37" s="51" t="n"/>
       <c r="T37" s="51" t="n"/>
@@ -2320,7 +2320,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-5.4</v>
+        <v>-5.6</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -2496,7 +2496,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="S43" s="52" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-1.7</v>
+        <v>-1.5</v>
       </c>
       <c r="S44" s="53" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>-13.5</v>
+        <v>-13.2</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-4.8</v>
+        <v>-4.3</v>
       </c>
       <c r="S46" s="52" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-36.9</v>
+        <v>-37.5</v>
       </c>
       <c r="S47" s="52" t="inlineStr">
         <is>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-0.3</v>
+        <v>-1.1</v>
       </c>
       <c r="S51" s="53" t="inlineStr">
         <is>
@@ -3067,9 +3067,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U51" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U51" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V51" s="53" t="inlineStr">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="S52" s="53" t="inlineStr">
         <is>
@@ -3319,7 +3319,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-1.4</v>
+        <v>-0.8</v>
       </c>
       <c r="S54" s="52" t="inlineStr">
         <is>
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>18.9</v>
+        <v>18.7</v>
       </c>
       <c r="S55" s="52" t="inlineStr">
         <is>
@@ -3495,7 +3495,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>-20.1</v>
+        <v>-20.8</v>
       </c>
       <c r="S56" s="52" t="inlineStr">
         <is>
@@ -3507,9 +3507,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U56" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U56" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V56" s="53" t="inlineStr">
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>-8.1</v>
+        <v>-7.6</v>
       </c>
       <c r="S57" s="53" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.1</v>
       </c>
       <c r="S58" s="53" t="inlineStr">
         <is>
@@ -3759,7 +3759,7 @@
         </is>
       </c>
       <c r="R59" s="42" t="n">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="S59" s="53" t="inlineStr">
         <is>
@@ -4414,7 +4414,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>8.9</v>
+        <v>7.9</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -4542,7 +4542,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-8.9</v>
+        <v>-7.5</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -4606,7 +4606,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -4670,7 +4670,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-14.7</v>
+        <v>-14.9</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -4734,7 +4734,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-11.5</v>
+        <v>-11.9</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -4798,7 +4798,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-11</v>
+        <v>-11.4</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -4990,7 +4990,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-6.1</v>
+        <v>-6.8</v>
       </c>
       <c r="S36" s="52" t="inlineStr">
         <is>
@@ -5078,7 +5078,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-4.8</v>
+        <v>-4.4</v>
       </c>
       <c r="S37" s="54" t="inlineStr">
         <is>
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-12.7</v>
+        <v>-12.5</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-11</v>
+        <v>-12.1</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -5342,7 +5342,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-6.7</v>
+        <v>-6.6</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -5430,7 +5430,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-25.3</v>
+        <v>-24.3</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -5518,7 +5518,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-2.1</v>
+        <v>-1.7</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -5813,7 +5813,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>15.6</v>
+        <v>16.5</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -5989,7 +5989,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>15.9</v>
+        <v>15</v>
       </c>
       <c r="S49" s="52" t="inlineStr">
         <is>
@@ -6077,7 +6077,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-13.6</v>
+        <v>-13</v>
       </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
@@ -6165,7 +6165,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-23.8</v>
+        <v>-24.1</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -6253,7 +6253,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>-1.5</v>
+        <v>-1.8</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -6265,9 +6265,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U52" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U52" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V52" s="53" t="inlineStr">
@@ -6341,7 +6341,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>-4.5</v>
+        <v>-4.9</v>
       </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
@@ -7040,7 +7040,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-1</v>
+        <v>-0.6</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -7168,7 +7168,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-16.6</v>
+        <v>-16.8</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -7232,7 +7232,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-11</v>
+        <v>-10.7</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -7296,7 +7296,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-18.5</v>
+        <v>-18</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -7360,7 +7360,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-0.6</v>
+        <v>-0.8</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -7424,7 +7424,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>17.2</v>
+        <v>18.7</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -7704,7 +7704,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-1.2</v>
+        <v>-1.4</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -7792,7 +7792,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="S40" s="52" t="inlineStr">
         <is>
@@ -7880,7 +7880,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-14.5</v>
+        <v>-15.5</v>
       </c>
       <c r="S42" s="53" t="inlineStr">
         <is>
@@ -8056,7 +8056,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>-19.7</v>
+        <v>-19.2</v>
       </c>
       <c r="S43" s="53" t="inlineStr">
         <is>
@@ -8263,7 +8263,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>17.7</v>
+        <v>17.9</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -8351,7 +8351,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>-12.3</v>
+        <v>-13.6</v>
       </c>
       <c r="S48" s="52" t="inlineStr">
         <is>
@@ -8439,7 +8439,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-5.8</v>
+        <v>-6.2</v>
       </c>
       <c r="S49" s="54" t="inlineStr">
         <is>
@@ -8527,7 +8527,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-13</v>
+        <v>-13.2</v>
       </c>
       <c r="S50" s="53" t="inlineStr">
         <is>
@@ -8615,7 +8615,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>6.2</v>
+        <v>4.9</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -8703,7 +8703,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>-13.1</v>
+        <v>-13</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -8791,7 +8791,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>-7.8</v>
+        <v>-7.1</v>
       </c>
       <c r="S53" s="53" t="inlineStr">
         <is>
@@ -9534,7 +9534,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -9598,7 +9598,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -9662,7 +9662,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-7.7</v>
+        <v>-8.4</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -9726,7 +9726,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>9</v>
+        <v>8.4</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -9790,7 +9790,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>10.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -9854,7 +9854,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>-7.4</v>
+        <v>-7.1</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -9918,7 +9918,7 @@
       <c r="P36" s="42" t="n"/>
       <c r="Q36" s="42" t="n"/>
       <c r="R36" s="42" t="n">
-        <v>-15.8</v>
+        <v>-15.5</v>
       </c>
       <c r="S36" s="51" t="n"/>
       <c r="T36" s="51" t="n"/>
@@ -10109,7 +10109,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="S40" s="52" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>14.3</v>
+        <v>13.8</v>
       </c>
       <c r="S41" s="52" t="inlineStr">
         <is>
@@ -10285,7 +10285,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-26.2</v>
+        <v>-26</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -10461,7 +10461,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-25.6</v>
+        <v>-25.3</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -10549,7 +10549,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -10637,7 +10637,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>0.2</v>
+        <v>-0.6</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -10725,7 +10725,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>10.1</v>
+        <v>10.4</v>
       </c>
       <c r="S47" s="52" t="inlineStr">
         <is>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-12.3</v>
+        <v>-12.8</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="S53" s="53" t="inlineStr">
         <is>
@@ -11196,7 +11196,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-11.3</v>
+        <v>-11.1</v>
       </c>
       <c r="S54" s="53" t="inlineStr">
         <is>
@@ -11284,7 +11284,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="S55" s="52" t="inlineStr">
         <is>
@@ -11372,7 +11372,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>-4.7</v>
+        <v>-4.6</v>
       </c>
       <c r="S56" s="53" t="inlineStr">
         <is>
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>-6.2</v>
+        <v>-6.5</v>
       </c>
       <c r="S57" s="52" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>16.8</v>
+        <v>15.5</v>
       </c>
       <c r="S58" s="53" t="inlineStr">
         <is>
@@ -12123,7 +12123,7 @@
         </is>
       </c>
       <c r="R22" s="42" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="S22" s="52" t="inlineStr">
         <is>
@@ -12211,7 +12211,7 @@
         </is>
       </c>
       <c r="R23" s="42" t="n">
-        <v>-11.6</v>
+        <v>-11.3</v>
       </c>
       <c r="S23" s="54" t="inlineStr">
         <is>
@@ -12299,7 +12299,7 @@
         </is>
       </c>
       <c r="R24" s="42" t="n">
-        <v>-1.7</v>
+        <v>-1.9</v>
       </c>
       <c r="S24" s="53" t="inlineStr">
         <is>
@@ -12387,7 +12387,7 @@
         </is>
       </c>
       <c r="R25" s="42" t="n">
-        <v>9.1</v>
+        <v>8.9</v>
       </c>
       <c r="S25" s="53" t="inlineStr">
         <is>
@@ -12595,7 +12595,7 @@
         </is>
       </c>
       <c r="R29" s="42" t="n">
-        <v>-9.6</v>
+        <v>-9.9</v>
       </c>
       <c r="S29" s="52" t="inlineStr">
         <is>
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="R30" s="42" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="S30" s="52" t="inlineStr">
         <is>
@@ -12771,7 +12771,7 @@
         </is>
       </c>
       <c r="R31" s="42" t="n">
-        <v>-11.8</v>
+        <v>-11.6</v>
       </c>
       <c r="S31" s="53" t="inlineStr">
         <is>
@@ -12859,7 +12859,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>-8.5</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S32" s="53" t="inlineStr">
         <is>
@@ -13066,7 +13066,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-13</v>
+        <v>-13.2</v>
       </c>
       <c r="S36" s="53" t="inlineStr">
         <is>
@@ -13242,7 +13242,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="S38" s="52" t="inlineStr">
         <is>
@@ -13629,7 +13629,7 @@
       <c r="P14" s="42" t="n"/>
       <c r="Q14" s="42" t="n"/>
       <c r="R14" s="42" t="n">
-        <v>-1</v>
+        <v>-0.6</v>
       </c>
       <c r="S14" s="51" t="n"/>
       <c r="T14" s="51" t="n"/>
@@ -13820,7 +13820,7 @@
         </is>
       </c>
       <c r="R18" s="42" t="n">
-        <v>-2.1</v>
+        <v>-1.7</v>
       </c>
       <c r="S18" s="52" t="inlineStr">
         <is>
@@ -13908,7 +13908,7 @@
         </is>
       </c>
       <c r="R19" s="42" t="n">
-        <v>-36.9</v>
+        <v>-37.5</v>
       </c>
       <c r="S19" s="52" t="inlineStr">
         <is>
@@ -14115,7 +14115,7 @@
         </is>
       </c>
       <c r="R23" s="42" t="n">
-        <v>18.9</v>
+        <v>18.7</v>
       </c>
       <c r="S23" s="52" t="inlineStr">
         <is>
@@ -14203,7 +14203,7 @@
         </is>
       </c>
       <c r="R24" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.1</v>
       </c>
       <c r="S24" s="53" t="inlineStr">
         <is>
@@ -14836,7 +14836,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>-14.7</v>
+        <v>-14.9</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -14964,7 +14964,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>-14.4</v>
+        <v>-14.6</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -15028,7 +15028,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -15092,7 +15092,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -15156,7 +15156,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-10.3</v>
+        <v>-10.8</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -15220,7 +15220,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>19.5</v>
+        <v>19.2</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -15412,7 +15412,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-26.2</v>
+        <v>-26</v>
       </c>
       <c r="S35" s="52" t="inlineStr">
         <is>
@@ -15500,7 +15500,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="S36" s="53" t="inlineStr">
         <is>
@@ -15588,7 +15588,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.4</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -15764,7 +15764,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-7</v>
+        <v>-7.4</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -15852,7 +15852,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-13.6</v>
+        <v>-13.9</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -15940,7 +15940,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-15.5</v>
+        <v>-15.8</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -16147,7 +16147,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>13.7</v>
+        <v>15.4</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -16235,7 +16235,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="S46" s="52" t="inlineStr">
         <is>
@@ -16323,7 +16323,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-7.3</v>
+        <v>-7.5</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -16411,7 +16411,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>15</v>
+        <v>15.6</v>
       </c>
       <c r="S48" s="52" t="inlineStr">
         <is>
@@ -16499,7 +16499,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -16587,7 +16587,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-11.1</v>
+        <v>-10.9</v>
       </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
@@ -17154,7 +17154,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -17218,7 +17218,7 @@
       <c r="P23" s="42" t="n"/>
       <c r="Q23" s="42" t="n"/>
       <c r="R23" s="42" t="n">
-        <v>-18.8</v>
+        <v>-19.5</v>
       </c>
       <c r="S23" s="51" t="n"/>
       <c r="T23" s="51" t="n"/>
@@ -17282,7 +17282,7 @@
       <c r="P24" s="42" t="n"/>
       <c r="Q24" s="42" t="n"/>
       <c r="R24" s="42" t="n">
-        <v>-6.6</v>
+        <v>-6.9</v>
       </c>
       <c r="S24" s="51" t="n"/>
       <c r="T24" s="51" t="n"/>
@@ -17346,7 +17346,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>9.4</v>
+        <v>8.9</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -17410,7 +17410,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -17602,7 +17602,7 @@
         </is>
       </c>
       <c r="R30" s="42" t="n">
-        <v>-14.5</v>
+        <v>-15.5</v>
       </c>
       <c r="S30" s="53" t="inlineStr">
         <is>
@@ -17690,7 +17690,7 @@
         </is>
       </c>
       <c r="R31" s="42" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="S31" s="53" t="inlineStr">
         <is>
@@ -17778,7 +17778,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="S32" s="52" t="inlineStr">
         <is>
@@ -17866,7 +17866,7 @@
         </is>
       </c>
       <c r="R33" s="42" t="n">
-        <v>4.6</v>
+        <v>3.9</v>
       </c>
       <c r="S33" s="52" t="inlineStr">
         <is>
@@ -17925,7 +17925,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="I34" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="J34" s="42" t="n">
         <v>5</v>
@@ -17954,7 +17954,7 @@
         </is>
       </c>
       <c r="R34" s="42" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="S34" s="53" t="inlineStr">
         <is>
@@ -18161,7 +18161,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-1.5</v>
+        <v>-1.8</v>
       </c>
       <c r="S38" s="52" t="inlineStr">
         <is>
@@ -18173,9 +18173,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U38" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U38" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V38" s="53" t="inlineStr">
@@ -18249,7 +18249,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-22</v>
+        <v>-21.7</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -18337,7 +18337,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-21.8</v>
+        <v>-21.3</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -18425,7 +18425,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -18513,7 +18513,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-7.3</v>
+        <v>-7.6</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -19036,7 +19036,7 @@
       <c r="P20" s="42" t="n"/>
       <c r="Q20" s="42" t="n"/>
       <c r="R20" s="42" t="n">
-        <v>-14.6</v>
+        <v>-14.5</v>
       </c>
       <c r="S20" s="51" t="n"/>
       <c r="T20" s="51" t="n"/>
@@ -19100,7 +19100,7 @@
       <c r="P21" s="42" t="n"/>
       <c r="Q21" s="42" t="n"/>
       <c r="R21" s="42" t="n">
-        <v>-3.5</v>
+        <v>-3.3</v>
       </c>
       <c r="S21" s="51" t="n"/>
       <c r="T21" s="51" t="n"/>
@@ -19164,7 +19164,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -19356,7 +19356,7 @@
         </is>
       </c>
       <c r="R26" s="42" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="S26" s="52" t="inlineStr">
         <is>
@@ -19444,7 +19444,7 @@
         </is>
       </c>
       <c r="R27" s="42" t="n">
-        <v>-1.5</v>
+        <v>-2.2</v>
       </c>
       <c r="S27" s="53" t="inlineStr">
         <is>
@@ -19532,7 +19532,7 @@
         </is>
       </c>
       <c r="R28" s="42" t="n">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="S28" s="53" t="inlineStr">
         <is>
@@ -19739,7 +19739,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>-15</v>
+        <v>-15.7</v>
       </c>
       <c r="S32" s="53" t="inlineStr">
         <is>
@@ -19915,7 +19915,7 @@
         </is>
       </c>
       <c r="R34" s="42" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="S34" s="53" t="inlineStr">
         <is>
@@ -20003,7 +20003,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="S35" s="52" t="inlineStr">
         <is>
@@ -20702,7 +20702,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-23.7</v>
+        <v>-22.2</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -20766,7 +20766,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-10.6</v>
+        <v>-10.4</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -20830,7 +20830,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-14.1</v>
+        <v>-14.3</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -20894,7 +20894,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-10.7</v>
+        <v>-10.5</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -20958,7 +20958,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -21022,7 +21022,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-15.4</v>
+        <v>-16.2</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -21078,7 +21078,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-33.9</v>
+        <v>-33.2</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -21142,7 +21142,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>-11.7</v>
+        <v>-11.8</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -21334,7 +21334,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -21422,7 +21422,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="S40" s="52" t="inlineStr">
         <is>
@@ -21510,7 +21510,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-8.300000000000001</v>
+        <v>-8.4</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -21686,7 +21686,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="S43" s="52" t="inlineStr">
         <is>
@@ -21774,7 +21774,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>10.7</v>
+        <v>12.1</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -21862,7 +21862,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>8.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -21874,9 +21874,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U45" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U45" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V45" s="52" t="inlineStr">
@@ -22157,7 +22157,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-40.5</v>
+        <v>-40.4</v>
       </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
@@ -22245,7 +22245,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
       <c r="S51" s="53" t="inlineStr">
         <is>
@@ -22333,7 +22333,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>-3.3</v>
+        <v>-2.6</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -22421,7 +22421,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>-4.9</v>
+        <v>-5.4</v>
       </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
@@ -22509,7 +22509,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-13.3</v>
+        <v>-13.4</v>
       </c>
       <c r="S54" s="53" t="inlineStr">
         <is>
@@ -22597,7 +22597,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>-13.8</v>
+        <v>-13.2</v>
       </c>
       <c r="S55" s="53" t="inlineStr">
         <is>
@@ -23356,7 +23356,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>-2.8</v>
+        <v>-3</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -23420,7 +23420,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -23484,7 +23484,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-24.1</v>
+        <v>-24.3</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -23548,7 +23548,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-3.6</v>
+        <v>-4.1</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -23612,7 +23612,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -23676,7 +23676,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>14.1</v>
+        <v>15.9</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -23868,7 +23868,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-7.6</v>
+        <v>-7.5</v>
       </c>
       <c r="S35" s="52" t="inlineStr">
         <is>
@@ -23956,7 +23956,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-1.6</v>
+        <v>-0.9</v>
       </c>
       <c r="S36" s="52" t="inlineStr">
         <is>
@@ -24044,7 +24044,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-5.1</v>
+        <v>-5.3</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -24132,7 +24132,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>17.6</v>
+        <v>16.5</v>
       </c>
       <c r="S38" s="52" t="inlineStr">
         <is>
@@ -24220,7 +24220,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -24308,7 +24308,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-13.2</v>
+        <v>-13.8</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -24515,7 +24515,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="S44" s="53" t="inlineStr">
         <is>
@@ -24603,7 +24603,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -24691,7 +24691,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-14.4</v>
+        <v>-14.6</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -24779,7 +24779,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-4.5</v>
+        <v>-4.9</v>
       </c>
       <c r="S47" s="52" t="inlineStr">
         <is>
@@ -24867,7 +24867,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>-19</v>
+        <v>-18.2</v>
       </c>
       <c r="S48" s="53" t="inlineStr">
         <is>
@@ -24955,7 +24955,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-5.1</v>
+        <v>-6.3</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -35929,7 +35929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -60872,7 +60872,7 @@
       <c r="P9" s="42" t="n"/>
       <c r="Q9" s="42" t="n"/>
       <c r="R9" s="42" t="n">
-        <v>9.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="S9" s="51" t="n"/>
       <c r="T9" s="51" t="n"/>
@@ -60928,7 +60928,7 @@
       <c r="P10" s="42" t="n"/>
       <c r="Q10" s="42" t="n"/>
       <c r="R10" s="42" t="n">
-        <v>-33.7</v>
+        <v>-33.4</v>
       </c>
       <c r="S10" s="51" t="n"/>
       <c r="T10" s="51" t="n"/>
@@ -60992,7 +60992,7 @@
       <c r="P11" s="42" t="n"/>
       <c r="Q11" s="42" t="n"/>
       <c r="R11" s="42" t="n">
-        <v>-9.5</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="S11" s="51" t="n"/>
       <c r="T11" s="51" t="n"/>
@@ -61056,7 +61056,7 @@
       <c r="P12" s="42" t="n"/>
       <c r="Q12" s="42" t="n"/>
       <c r="R12" s="42" t="n">
-        <v>-17</v>
+        <v>-17.6</v>
       </c>
       <c r="S12" s="51" t="n"/>
       <c r="T12" s="51" t="n"/>
@@ -61120,7 +61120,7 @@
       <c r="P13" s="42" t="n"/>
       <c r="Q13" s="42" t="n"/>
       <c r="R13" s="42" t="n">
-        <v>-12.4</v>
+        <v>-12.5</v>
       </c>
       <c r="S13" s="51" t="n"/>
       <c r="T13" s="51" t="n"/>
@@ -61176,7 +61176,7 @@
       <c r="P14" s="42" t="n"/>
       <c r="Q14" s="42" t="n"/>
       <c r="R14" s="42" t="n">
-        <v>-30.1</v>
+        <v>-29.9</v>
       </c>
       <c r="S14" s="51" t="n"/>
       <c r="T14" s="51" t="n"/>
@@ -61240,7 +61240,7 @@
       <c r="P15" s="42" t="n"/>
       <c r="Q15" s="42" t="n"/>
       <c r="R15" s="42" t="n">
-        <v>9.9</v>
+        <v>9.5</v>
       </c>
       <c r="S15" s="51" t="n"/>
       <c r="T15" s="51" t="n"/>
@@ -61304,7 +61304,7 @@
       <c r="P16" s="42" t="n"/>
       <c r="Q16" s="42" t="n"/>
       <c r="R16" s="42" t="n">
-        <v>-5.7</v>
+        <v>-5.8</v>
       </c>
       <c r="S16" s="51" t="n"/>
       <c r="T16" s="51" t="n"/>
@@ -61368,7 +61368,7 @@
       <c r="P17" s="42" t="n"/>
       <c r="Q17" s="42" t="n"/>
       <c r="R17" s="42" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="S17" s="51" t="n"/>
       <c r="T17" s="51" t="n"/>
@@ -61432,7 +61432,7 @@
       <c r="P18" s="42" t="n"/>
       <c r="Q18" s="42" t="n"/>
       <c r="R18" s="42" t="n">
-        <v>8.9</v>
+        <v>7.9</v>
       </c>
       <c r="S18" s="51" t="n"/>
       <c r="T18" s="51" t="n"/>
@@ -61560,7 +61560,7 @@
       <c r="P20" s="42" t="n"/>
       <c r="Q20" s="42" t="n"/>
       <c r="R20" s="42" t="n">
-        <v>-8.9</v>
+        <v>-7.5</v>
       </c>
       <c r="S20" s="51" t="n"/>
       <c r="T20" s="51" t="n"/>
@@ -61624,7 +61624,7 @@
       <c r="P21" s="42" t="n"/>
       <c r="Q21" s="42" t="n"/>
       <c r="R21" s="42" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="S21" s="51" t="n"/>
       <c r="T21" s="51" t="n"/>
@@ -61688,7 +61688,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>-14.7</v>
+        <v>-14.9</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -61752,7 +61752,7 @@
       <c r="P23" s="42" t="n"/>
       <c r="Q23" s="42" t="n"/>
       <c r="R23" s="42" t="n">
-        <v>-11.5</v>
+        <v>-11.9</v>
       </c>
       <c r="S23" s="51" t="n"/>
       <c r="T23" s="51" t="n"/>
@@ -61816,7 +61816,7 @@
       <c r="P24" s="42" t="n"/>
       <c r="Q24" s="42" t="n"/>
       <c r="R24" s="42" t="n">
-        <v>-11</v>
+        <v>-11.4</v>
       </c>
       <c r="S24" s="51" t="n"/>
       <c r="T24" s="51" t="n"/>
@@ -61880,7 +61880,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>-1</v>
+        <v>-0.6</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -62008,7 +62008,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>-16.6</v>
+        <v>-16.8</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -62072,7 +62072,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-11</v>
+        <v>-10.7</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -62136,7 +62136,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-18.5</v>
+        <v>-18</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -62200,7 +62200,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-0.6</v>
+        <v>-0.8</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -62264,7 +62264,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>17.2</v>
+        <v>18.7</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -62328,7 +62328,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -62392,7 +62392,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -62456,7 +62456,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-7.7</v>
+        <v>-8.4</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -62520,7 +62520,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>9</v>
+        <v>8.4</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -62584,7 +62584,7 @@
       <c r="P36" s="42" t="n"/>
       <c r="Q36" s="42" t="n"/>
       <c r="R36" s="42" t="n">
-        <v>10.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="S36" s="51" t="n"/>
       <c r="T36" s="51" t="n"/>
@@ -62648,7 +62648,7 @@
       <c r="P37" s="42" t="n"/>
       <c r="Q37" s="42" t="n"/>
       <c r="R37" s="42" t="n">
-        <v>-7.4</v>
+        <v>-7.1</v>
       </c>
       <c r="S37" s="51" t="n"/>
       <c r="T37" s="51" t="n"/>
@@ -62712,7 +62712,7 @@
       <c r="P38" s="42" t="n"/>
       <c r="Q38" s="42" t="n"/>
       <c r="R38" s="42" t="n">
-        <v>-15.8</v>
+        <v>-15.5</v>
       </c>
       <c r="S38" s="51" t="n"/>
       <c r="T38" s="51" t="n"/>
@@ -62784,7 +62784,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -62872,7 +62872,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-11.6</v>
+        <v>-11.3</v>
       </c>
       <c r="S40" s="54" t="inlineStr">
         <is>
@@ -62960,7 +62960,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-1.7</v>
+        <v>-1.9</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -63048,7 +63048,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>9.1</v>
+        <v>8.9</v>
       </c>
       <c r="S42" s="53" t="inlineStr">
         <is>
@@ -63192,7 +63192,7 @@
       <c r="P44" s="42" t="n"/>
       <c r="Q44" s="42" t="n"/>
       <c r="R44" s="42" t="n">
-        <v>-14.4</v>
+        <v>-14.6</v>
       </c>
       <c r="S44" s="51" t="n"/>
       <c r="T44" s="51" t="n"/>
@@ -63256,7 +63256,7 @@
       <c r="P45" s="42" t="n"/>
       <c r="Q45" s="42" t="n"/>
       <c r="R45" s="42" t="n">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="S45" s="51" t="n"/>
       <c r="T45" s="51" t="n"/>
@@ -63320,7 +63320,7 @@
       <c r="P46" s="42" t="n"/>
       <c r="Q46" s="42" t="n"/>
       <c r="R46" s="42" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="S46" s="51" t="n"/>
       <c r="T46" s="51" t="n"/>
@@ -63384,7 +63384,7 @@
       <c r="P47" s="42" t="n"/>
       <c r="Q47" s="42" t="n"/>
       <c r="R47" s="42" t="n">
-        <v>-10.3</v>
+        <v>-10.8</v>
       </c>
       <c r="S47" s="51" t="n"/>
       <c r="T47" s="51" t="n"/>
@@ -63448,7 +63448,7 @@
       <c r="P48" s="42" t="n"/>
       <c r="Q48" s="42" t="n"/>
       <c r="R48" s="42" t="n">
-        <v>19.5</v>
+        <v>19.2</v>
       </c>
       <c r="S48" s="51" t="n"/>
       <c r="T48" s="51" t="n"/>
@@ -63512,7 +63512,7 @@
       <c r="P49" s="42" t="n"/>
       <c r="Q49" s="42" t="n"/>
       <c r="R49" s="42" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="S49" s="51" t="n"/>
       <c r="T49" s="51" t="n"/>
@@ -63576,7 +63576,7 @@
       <c r="P50" s="42" t="n"/>
       <c r="Q50" s="42" t="n"/>
       <c r="R50" s="42" t="n">
-        <v>-18.8</v>
+        <v>-19.5</v>
       </c>
       <c r="S50" s="51" t="n"/>
       <c r="T50" s="51" t="n"/>
@@ -63640,7 +63640,7 @@
       <c r="P51" s="42" t="n"/>
       <c r="Q51" s="42" t="n"/>
       <c r="R51" s="42" t="n">
-        <v>-6.6</v>
+        <v>-6.9</v>
       </c>
       <c r="S51" s="51" t="n"/>
       <c r="T51" s="51" t="n"/>
@@ -63704,7 +63704,7 @@
       <c r="P52" s="42" t="n"/>
       <c r="Q52" s="42" t="n"/>
       <c r="R52" s="42" t="n">
-        <v>9.4</v>
+        <v>8.9</v>
       </c>
       <c r="S52" s="51" t="n"/>
       <c r="T52" s="51" t="n"/>
@@ -63768,7 +63768,7 @@
       <c r="P53" s="42" t="n"/>
       <c r="Q53" s="42" t="n"/>
       <c r="R53" s="42" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="S53" s="51" t="n"/>
       <c r="T53" s="51" t="n"/>
@@ -63832,7 +63832,7 @@
       <c r="P54" s="42" t="n"/>
       <c r="Q54" s="42" t="n"/>
       <c r="R54" s="42" t="n">
-        <v>-14.6</v>
+        <v>-14.5</v>
       </c>
       <c r="S54" s="51" t="n"/>
       <c r="T54" s="51" t="n"/>
@@ -63896,7 +63896,7 @@
       <c r="P55" s="42" t="n"/>
       <c r="Q55" s="42" t="n"/>
       <c r="R55" s="42" t="n">
-        <v>-3.5</v>
+        <v>-3.3</v>
       </c>
       <c r="S55" s="51" t="n"/>
       <c r="T55" s="51" t="n"/>
@@ -63960,7 +63960,7 @@
       <c r="P56" s="42" t="n"/>
       <c r="Q56" s="42" t="n"/>
       <c r="R56" s="42" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="S56" s="51" t="n"/>
       <c r="T56" s="51" t="n"/>
@@ -64024,7 +64024,7 @@
       <c r="P57" s="42" t="n"/>
       <c r="Q57" s="42" t="n"/>
       <c r="R57" s="42" t="n">
-        <v>-23.7</v>
+        <v>-22.2</v>
       </c>
       <c r="S57" s="51" t="n"/>
       <c r="T57" s="51" t="n"/>
@@ -64088,7 +64088,7 @@
       <c r="P58" s="42" t="n"/>
       <c r="Q58" s="42" t="n"/>
       <c r="R58" s="42" t="n">
-        <v>-10.6</v>
+        <v>-10.4</v>
       </c>
       <c r="S58" s="51" t="n"/>
       <c r="T58" s="51" t="n"/>
@@ -64152,7 +64152,7 @@
       <c r="P59" s="42" t="n"/>
       <c r="Q59" s="42" t="n"/>
       <c r="R59" s="42" t="n">
-        <v>-14.1</v>
+        <v>-14.3</v>
       </c>
       <c r="S59" s="51" t="n"/>
       <c r="T59" s="51" t="n"/>
@@ -64216,7 +64216,7 @@
       <c r="P60" s="42" t="n"/>
       <c r="Q60" s="42" t="n"/>
       <c r="R60" s="42" t="n">
-        <v>-10.7</v>
+        <v>-10.5</v>
       </c>
       <c r="S60" s="51" t="n"/>
       <c r="T60" s="51" t="n"/>
@@ -64280,7 +64280,7 @@
       <c r="P61" s="42" t="n"/>
       <c r="Q61" s="42" t="n"/>
       <c r="R61" s="42" t="n">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
       <c r="S61" s="51" t="n"/>
       <c r="T61" s="51" t="n"/>
@@ -64344,7 +64344,7 @@
       <c r="P62" s="42" t="n"/>
       <c r="Q62" s="42" t="n"/>
       <c r="R62" s="42" t="n">
-        <v>-15.4</v>
+        <v>-16.2</v>
       </c>
       <c r="S62" s="51" t="n"/>
       <c r="T62" s="51" t="n"/>
@@ -64400,7 +64400,7 @@
       <c r="P63" s="42" t="n"/>
       <c r="Q63" s="42" t="n"/>
       <c r="R63" s="42" t="n">
-        <v>-33.9</v>
+        <v>-33.2</v>
       </c>
       <c r="S63" s="51" t="n"/>
       <c r="T63" s="51" t="n"/>
@@ -64464,7 +64464,7 @@
       <c r="P64" s="42" t="n"/>
       <c r="Q64" s="42" t="n"/>
       <c r="R64" s="42" t="n">
-        <v>-11.7</v>
+        <v>-11.8</v>
       </c>
       <c r="S64" s="51" t="n"/>
       <c r="T64" s="51" t="n"/>
@@ -64528,7 +64528,7 @@
       <c r="P65" s="42" t="n"/>
       <c r="Q65" s="42" t="n"/>
       <c r="R65" s="42" t="n">
-        <v>-2.8</v>
+        <v>-3</v>
       </c>
       <c r="S65" s="51" t="n"/>
       <c r="T65" s="51" t="n"/>
@@ -64592,7 +64592,7 @@
       <c r="P66" s="42" t="n"/>
       <c r="Q66" s="42" t="n"/>
       <c r="R66" s="42" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="S66" s="51" t="n"/>
       <c r="T66" s="51" t="n"/>
@@ -64656,7 +64656,7 @@
       <c r="P67" s="42" t="n"/>
       <c r="Q67" s="42" t="n"/>
       <c r="R67" s="42" t="n">
-        <v>-24.1</v>
+        <v>-24.3</v>
       </c>
       <c r="S67" s="51" t="n"/>
       <c r="T67" s="51" t="n"/>
@@ -64720,7 +64720,7 @@
       <c r="P68" s="42" t="n"/>
       <c r="Q68" s="42" t="n"/>
       <c r="R68" s="42" t="n">
-        <v>-3.6</v>
+        <v>-4.1</v>
       </c>
       <c r="S68" s="51" t="n"/>
       <c r="T68" s="51" t="n"/>
@@ -64784,7 +64784,7 @@
       <c r="P69" s="42" t="n"/>
       <c r="Q69" s="42" t="n"/>
       <c r="R69" s="42" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="S69" s="51" t="n"/>
       <c r="T69" s="51" t="n"/>
@@ -64848,7 +64848,7 @@
       <c r="P70" s="42" t="n"/>
       <c r="Q70" s="42" t="n"/>
       <c r="R70" s="42" t="n">
-        <v>14.1</v>
+        <v>15.9</v>
       </c>
       <c r="S70" s="51" t="n"/>
       <c r="T70" s="51" t="n"/>
@@ -65039,7 +65039,7 @@
         </is>
       </c>
       <c r="R74" s="42" t="n">
-        <v>-5.4</v>
+        <v>-5.6</v>
       </c>
       <c r="S74" s="53" t="inlineStr">
         <is>
@@ -65215,7 +65215,7 @@
         </is>
       </c>
       <c r="R76" s="42" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="S76" s="52" t="inlineStr">
         <is>
@@ -65303,7 +65303,7 @@
         </is>
       </c>
       <c r="R77" s="42" t="n">
-        <v>-1.7</v>
+        <v>-1.5</v>
       </c>
       <c r="S77" s="53" t="inlineStr">
         <is>
@@ -65391,7 +65391,7 @@
         </is>
       </c>
       <c r="R78" s="42" t="n">
-        <v>-13.5</v>
+        <v>-13.2</v>
       </c>
       <c r="S78" s="52" t="inlineStr">
         <is>
@@ -65479,7 +65479,7 @@
         </is>
       </c>
       <c r="R79" s="42" t="n">
-        <v>-4.8</v>
+        <v>-4.3</v>
       </c>
       <c r="S79" s="52" t="inlineStr">
         <is>
@@ -65567,7 +65567,7 @@
         </is>
       </c>
       <c r="R80" s="42" t="n">
-        <v>-6.1</v>
+        <v>-6.8</v>
       </c>
       <c r="S80" s="52" t="inlineStr">
         <is>
@@ -65655,7 +65655,7 @@
         </is>
       </c>
       <c r="R81" s="42" t="n">
-        <v>-4.8</v>
+        <v>-4.4</v>
       </c>
       <c r="S81" s="54" t="inlineStr">
         <is>
@@ -65743,7 +65743,7 @@
         </is>
       </c>
       <c r="R82" s="42" t="n">
-        <v>-12.7</v>
+        <v>-12.5</v>
       </c>
       <c r="S82" s="53" t="inlineStr">
         <is>
@@ -65831,7 +65831,7 @@
         </is>
       </c>
       <c r="R83" s="42" t="n">
-        <v>-11</v>
+        <v>-12.1</v>
       </c>
       <c r="S83" s="53" t="inlineStr">
         <is>
@@ -65919,7 +65919,7 @@
         </is>
       </c>
       <c r="R84" s="42" t="n">
-        <v>-6.7</v>
+        <v>-6.6</v>
       </c>
       <c r="S84" s="53" t="inlineStr">
         <is>
@@ -66007,7 +66007,7 @@
         </is>
       </c>
       <c r="R85" s="42" t="n">
-        <v>-25.3</v>
+        <v>-24.3</v>
       </c>
       <c r="S85" s="53" t="inlineStr">
         <is>
@@ -66095,7 +66095,7 @@
         </is>
       </c>
       <c r="R86" s="42" t="n">
-        <v>-2.1</v>
+        <v>-1.7</v>
       </c>
       <c r="S86" s="52" t="inlineStr">
         <is>
@@ -66271,7 +66271,7 @@
         </is>
       </c>
       <c r="R88" s="42" t="n">
-        <v>-1.2</v>
+        <v>-1.4</v>
       </c>
       <c r="S88" s="52" t="inlineStr">
         <is>
@@ -66359,7 +66359,7 @@
         </is>
       </c>
       <c r="R89" s="42" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="S89" s="52" t="inlineStr">
         <is>
@@ -66447,7 +66447,7 @@
         </is>
       </c>
       <c r="R90" s="42" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="S90" s="53" t="inlineStr">
         <is>
@@ -66535,7 +66535,7 @@
         </is>
       </c>
       <c r="R91" s="42" t="n">
-        <v>-14.5</v>
+        <v>-15.5</v>
       </c>
       <c r="S91" s="53" t="inlineStr">
         <is>
@@ -66623,7 +66623,7 @@
         </is>
       </c>
       <c r="R92" s="42" t="n">
-        <v>-19.7</v>
+        <v>-19.2</v>
       </c>
       <c r="S92" s="53" t="inlineStr">
         <is>
@@ -66711,7 +66711,7 @@
         </is>
       </c>
       <c r="R93" s="42" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="S93" s="52" t="inlineStr">
         <is>
@@ -66799,7 +66799,7 @@
         </is>
       </c>
       <c r="R94" s="42" t="n">
-        <v>14.3</v>
+        <v>13.8</v>
       </c>
       <c r="S94" s="52" t="inlineStr">
         <is>
@@ -66887,7 +66887,7 @@
         </is>
       </c>
       <c r="R95" s="42" t="n">
-        <v>-26.2</v>
+        <v>-26</v>
       </c>
       <c r="S95" s="52" t="inlineStr">
         <is>
@@ -67063,7 +67063,7 @@
         </is>
       </c>
       <c r="R97" s="42" t="n">
-        <v>-25.6</v>
+        <v>-25.3</v>
       </c>
       <c r="S97" s="52" t="inlineStr">
         <is>
@@ -67151,7 +67151,7 @@
         </is>
       </c>
       <c r="R98" s="42" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="S98" s="52" t="inlineStr">
         <is>
@@ -67239,7 +67239,7 @@
         </is>
       </c>
       <c r="R99" s="42" t="n">
-        <v>0.2</v>
+        <v>-0.6</v>
       </c>
       <c r="S99" s="53" t="inlineStr">
         <is>
@@ -67327,7 +67327,7 @@
         </is>
       </c>
       <c r="R100" s="42" t="n">
-        <v>10.1</v>
+        <v>10.4</v>
       </c>
       <c r="S100" s="52" t="inlineStr">
         <is>
@@ -67415,7 +67415,7 @@
         </is>
       </c>
       <c r="R101" s="42" t="n">
-        <v>-9.6</v>
+        <v>-9.9</v>
       </c>
       <c r="S101" s="52" t="inlineStr">
         <is>
@@ -67503,7 +67503,7 @@
         </is>
       </c>
       <c r="R102" s="42" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="S102" s="52" t="inlineStr">
         <is>
@@ -67591,7 +67591,7 @@
         </is>
       </c>
       <c r="R103" s="42" t="n">
-        <v>-11.8</v>
+        <v>-11.6</v>
       </c>
       <c r="S103" s="53" t="inlineStr">
         <is>
@@ -67679,7 +67679,7 @@
         </is>
       </c>
       <c r="R104" s="42" t="n">
-        <v>-8.5</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S104" s="53" t="inlineStr">
         <is>
@@ -67767,7 +67767,7 @@
         </is>
       </c>
       <c r="R105" s="42" t="n">
-        <v>-36.9</v>
+        <v>-37.5</v>
       </c>
       <c r="S105" s="52" t="inlineStr">
         <is>
@@ -67855,7 +67855,7 @@
         </is>
       </c>
       <c r="R106" s="42" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="S106" s="53" t="inlineStr">
         <is>
@@ -67943,7 +67943,7 @@
         </is>
       </c>
       <c r="R107" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.4</v>
       </c>
       <c r="S107" s="53" t="inlineStr">
         <is>
@@ -68119,7 +68119,7 @@
         </is>
       </c>
       <c r="R109" s="42" t="n">
-        <v>-7</v>
+        <v>-7.4</v>
       </c>
       <c r="S109" s="53" t="inlineStr">
         <is>
@@ -68207,7 +68207,7 @@
         </is>
       </c>
       <c r="R110" s="42" t="n">
-        <v>-13.6</v>
+        <v>-13.9</v>
       </c>
       <c r="S110" s="53" t="inlineStr">
         <is>
@@ -68295,7 +68295,7 @@
         </is>
       </c>
       <c r="R111" s="42" t="n">
-        <v>-15.5</v>
+        <v>-15.8</v>
       </c>
       <c r="S111" s="53" t="inlineStr">
         <is>
@@ -68383,7 +68383,7 @@
         </is>
       </c>
       <c r="R112" s="42" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="S112" s="53" t="inlineStr">
         <is>
@@ -68471,7 +68471,7 @@
         </is>
       </c>
       <c r="R113" s="42" t="n">
-        <v>0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="S113" s="52" t="inlineStr">
         <is>
@@ -68559,7 +68559,7 @@
         </is>
       </c>
       <c r="R114" s="42" t="n">
-        <v>4.6</v>
+        <v>3.9</v>
       </c>
       <c r="S114" s="52" t="inlineStr">
         <is>
@@ -68618,7 +68618,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="I115" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="J115" s="42" t="n">
         <v>5</v>
@@ -68647,7 +68647,7 @@
         </is>
       </c>
       <c r="R115" s="42" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="S115" s="53" t="inlineStr">
         <is>
@@ -68735,7 +68735,7 @@
         </is>
       </c>
       <c r="R116" s="42" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="S116" s="52" t="inlineStr">
         <is>
@@ -68823,7 +68823,7 @@
         </is>
       </c>
       <c r="R117" s="42" t="n">
-        <v>-1.5</v>
+        <v>-2.2</v>
       </c>
       <c r="S117" s="53" t="inlineStr">
         <is>
@@ -68911,7 +68911,7 @@
         </is>
       </c>
       <c r="R118" s="42" t="n">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="S118" s="53" t="inlineStr">
         <is>
@@ -68999,7 +68999,7 @@
         </is>
       </c>
       <c r="R119" s="42" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="S119" s="53" t="inlineStr">
         <is>
@@ -69087,7 +69087,7 @@
         </is>
       </c>
       <c r="R120" s="42" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="S120" s="52" t="inlineStr">
         <is>
@@ -69175,7 +69175,7 @@
         </is>
       </c>
       <c r="R121" s="42" t="n">
-        <v>-8.300000000000001</v>
+        <v>-8.4</v>
       </c>
       <c r="S121" s="53" t="inlineStr">
         <is>
@@ -69351,7 +69351,7 @@
         </is>
       </c>
       <c r="R123" s="42" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="S123" s="52" t="inlineStr">
         <is>
@@ -69439,7 +69439,7 @@
         </is>
       </c>
       <c r="R124" s="42" t="n">
-        <v>10.7</v>
+        <v>12.1</v>
       </c>
       <c r="S124" s="52" t="inlineStr">
         <is>
@@ -69527,7 +69527,7 @@
         </is>
       </c>
       <c r="R125" s="42" t="n">
-        <v>8.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="S125" s="52" t="inlineStr">
         <is>
@@ -69539,9 +69539,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U125" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U125" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V125" s="52" t="inlineStr">
@@ -69615,7 +69615,7 @@
         </is>
       </c>
       <c r="R126" s="42" t="n">
-        <v>-7.6</v>
+        <v>-7.5</v>
       </c>
       <c r="S126" s="52" t="inlineStr">
         <is>
@@ -69703,7 +69703,7 @@
         </is>
       </c>
       <c r="R127" s="42" t="n">
-        <v>-1.6</v>
+        <v>-0.9</v>
       </c>
       <c r="S127" s="52" t="inlineStr">
         <is>
@@ -69791,7 +69791,7 @@
         </is>
       </c>
       <c r="R128" s="42" t="n">
-        <v>-5.1</v>
+        <v>-5.3</v>
       </c>
       <c r="S128" s="53" t="inlineStr">
         <is>
@@ -69879,7 +69879,7 @@
         </is>
       </c>
       <c r="R129" s="42" t="n">
-        <v>17.6</v>
+        <v>16.5</v>
       </c>
       <c r="S129" s="52" t="inlineStr">
         <is>
@@ -69967,7 +69967,7 @@
         </is>
       </c>
       <c r="R130" s="42" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="S130" s="52" t="inlineStr">
         <is>
@@ -70055,7 +70055,7 @@
         </is>
       </c>
       <c r="R131" s="42" t="n">
-        <v>-13.2</v>
+        <v>-13.8</v>
       </c>
       <c r="S131" s="53" t="inlineStr">
         <is>
@@ -70262,7 +70262,7 @@
         </is>
       </c>
       <c r="R135" s="42" t="n">
-        <v>-0.3</v>
+        <v>-1.1</v>
       </c>
       <c r="S135" s="53" t="inlineStr">
         <is>
@@ -70274,9 +70274,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U135" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U135" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V135" s="53" t="inlineStr">
@@ -70350,7 +70350,7 @@
         </is>
       </c>
       <c r="R136" s="42" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="S136" s="53" t="inlineStr">
         <is>
@@ -70526,7 +70526,7 @@
         </is>
       </c>
       <c r="R138" s="42" t="n">
-        <v>-1.4</v>
+        <v>-0.8</v>
       </c>
       <c r="S138" s="52" t="inlineStr">
         <is>
@@ -70614,7 +70614,7 @@
         </is>
       </c>
       <c r="R139" s="42" t="n">
-        <v>18.9</v>
+        <v>18.7</v>
       </c>
       <c r="S139" s="52" t="inlineStr">
         <is>
@@ -70702,7 +70702,7 @@
         </is>
       </c>
       <c r="R140" s="42" t="n">
-        <v>-20.1</v>
+        <v>-20.8</v>
       </c>
       <c r="S140" s="52" t="inlineStr">
         <is>
@@ -70714,9 +70714,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U140" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U140" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V140" s="53" t="inlineStr">
@@ -70790,7 +70790,7 @@
         </is>
       </c>
       <c r="R141" s="42" t="n">
-        <v>-8.1</v>
+        <v>-7.6</v>
       </c>
       <c r="S141" s="53" t="inlineStr">
         <is>
@@ -70966,7 +70966,7 @@
         </is>
       </c>
       <c r="R143" s="42" t="n">
-        <v>15.6</v>
+        <v>16.5</v>
       </c>
       <c r="S143" s="53" t="inlineStr">
         <is>
@@ -71142,7 +71142,7 @@
         </is>
       </c>
       <c r="R145" s="42" t="n">
-        <v>15.9</v>
+        <v>15</v>
       </c>
       <c r="S145" s="52" t="inlineStr">
         <is>
@@ -71230,7 +71230,7 @@
         </is>
       </c>
       <c r="R146" s="42" t="n">
-        <v>-13.6</v>
+        <v>-13</v>
       </c>
       <c r="S146" s="52" t="inlineStr">
         <is>
@@ -71318,7 +71318,7 @@
         </is>
       </c>
       <c r="R147" s="42" t="n">
-        <v>-23.8</v>
+        <v>-24.1</v>
       </c>
       <c r="S147" s="52" t="inlineStr">
         <is>
@@ -71406,7 +71406,7 @@
         </is>
       </c>
       <c r="R148" s="42" t="n">
-        <v>17.7</v>
+        <v>17.9</v>
       </c>
       <c r="S148" s="53" t="inlineStr">
         <is>
@@ -71494,7 +71494,7 @@
         </is>
       </c>
       <c r="R149" s="42" t="n">
-        <v>-12.3</v>
+        <v>-13.6</v>
       </c>
       <c r="S149" s="52" t="inlineStr">
         <is>
@@ -71582,7 +71582,7 @@
         </is>
       </c>
       <c r="R150" s="42" t="n">
-        <v>-5.8</v>
+        <v>-6.2</v>
       </c>
       <c r="S150" s="54" t="inlineStr">
         <is>
@@ -71670,7 +71670,7 @@
         </is>
       </c>
       <c r="R151" s="42" t="n">
-        <v>-13</v>
+        <v>-13.2</v>
       </c>
       <c r="S151" s="53" t="inlineStr">
         <is>
@@ -71758,7 +71758,7 @@
         </is>
       </c>
       <c r="R152" s="42" t="n">
-        <v>6.2</v>
+        <v>4.9</v>
       </c>
       <c r="S152" s="52" t="inlineStr">
         <is>
@@ -71846,7 +71846,7 @@
         </is>
       </c>
       <c r="R153" s="42" t="n">
-        <v>-13.1</v>
+        <v>-13</v>
       </c>
       <c r="S153" s="52" t="inlineStr">
         <is>
@@ -71934,7 +71934,7 @@
         </is>
       </c>
       <c r="R154" s="42" t="n">
-        <v>-7.8</v>
+        <v>-7.1</v>
       </c>
       <c r="S154" s="53" t="inlineStr">
         <is>
@@ -72022,7 +72022,7 @@
         </is>
       </c>
       <c r="R155" s="42" t="n">
-        <v>-12.3</v>
+        <v>-12.8</v>
       </c>
       <c r="S155" s="52" t="inlineStr">
         <is>
@@ -72198,7 +72198,7 @@
         </is>
       </c>
       <c r="R157" s="42" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="S157" s="53" t="inlineStr">
         <is>
@@ -72286,7 +72286,7 @@
         </is>
       </c>
       <c r="R158" s="42" t="n">
-        <v>-11.3</v>
+        <v>-11.1</v>
       </c>
       <c r="S158" s="53" t="inlineStr">
         <is>
@@ -72374,7 +72374,7 @@
         </is>
       </c>
       <c r="R159" s="42" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="S159" s="52" t="inlineStr">
         <is>
@@ -72462,7 +72462,7 @@
         </is>
       </c>
       <c r="R160" s="42" t="n">
-        <v>-4.7</v>
+        <v>-4.6</v>
       </c>
       <c r="S160" s="53" t="inlineStr">
         <is>
@@ -72550,7 +72550,7 @@
         </is>
       </c>
       <c r="R161" s="42" t="n">
-        <v>-6.2</v>
+        <v>-6.5</v>
       </c>
       <c r="S161" s="52" t="inlineStr">
         <is>
@@ -72638,7 +72638,7 @@
         </is>
       </c>
       <c r="R162" s="42" t="n">
-        <v>16.8</v>
+        <v>15.5</v>
       </c>
       <c r="S162" s="53" t="inlineStr">
         <is>
@@ -72814,7 +72814,7 @@
         </is>
       </c>
       <c r="R164" s="42" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="S164" s="52" t="inlineStr">
         <is>
@@ -72902,7 +72902,7 @@
         </is>
       </c>
       <c r="R165" s="42" t="n">
-        <v>-6.8</v>
+        <v>-6.1</v>
       </c>
       <c r="S165" s="53" t="inlineStr">
         <is>
@@ -72990,7 +72990,7 @@
         </is>
       </c>
       <c r="R166" s="42" t="n">
-        <v>13.7</v>
+        <v>15.4</v>
       </c>
       <c r="S166" s="52" t="inlineStr">
         <is>
@@ -73078,7 +73078,7 @@
         </is>
       </c>
       <c r="R167" s="42" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="S167" s="52" t="inlineStr">
         <is>
@@ -73166,7 +73166,7 @@
         </is>
       </c>
       <c r="R168" s="42" t="n">
-        <v>-7.3</v>
+        <v>-7.5</v>
       </c>
       <c r="S168" s="53" t="inlineStr">
         <is>
@@ -73254,7 +73254,7 @@
         </is>
       </c>
       <c r="R169" s="42" t="n">
-        <v>15</v>
+        <v>15.6</v>
       </c>
       <c r="S169" s="52" t="inlineStr">
         <is>
@@ -73342,7 +73342,7 @@
         </is>
       </c>
       <c r="R170" s="42" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="S170" s="53" t="inlineStr">
         <is>
@@ -73430,7 +73430,7 @@
         </is>
       </c>
       <c r="R171" s="42" t="n">
-        <v>-11.1</v>
+        <v>-10.9</v>
       </c>
       <c r="S171" s="52" t="inlineStr">
         <is>
@@ -73518,7 +73518,7 @@
         </is>
       </c>
       <c r="R172" s="42" t="n">
-        <v>-1.5</v>
+        <v>-1.8</v>
       </c>
       <c r="S172" s="52" t="inlineStr">
         <is>
@@ -73530,9 +73530,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U172" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U172" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V172" s="53" t="inlineStr">
@@ -73606,7 +73606,7 @@
         </is>
       </c>
       <c r="R173" s="42" t="n">
-        <v>-22</v>
+        <v>-21.7</v>
       </c>
       <c r="S173" s="53" t="inlineStr">
         <is>
@@ -73694,7 +73694,7 @@
         </is>
       </c>
       <c r="R174" s="42" t="n">
-        <v>-21.8</v>
+        <v>-21.3</v>
       </c>
       <c r="S174" s="53" t="inlineStr">
         <is>
@@ -73782,7 +73782,7 @@
         </is>
       </c>
       <c r="R175" s="42" t="n">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="S175" s="53" t="inlineStr">
         <is>
@@ -73870,7 +73870,7 @@
         </is>
       </c>
       <c r="R176" s="42" t="n">
-        <v>-7.3</v>
+        <v>-7.6</v>
       </c>
       <c r="S176" s="52" t="inlineStr">
         <is>
@@ -73958,7 +73958,7 @@
         </is>
       </c>
       <c r="R177" s="42" t="n">
-        <v>-15</v>
+        <v>-15.7</v>
       </c>
       <c r="S177" s="53" t="inlineStr">
         <is>
@@ -74134,7 +74134,7 @@
         </is>
       </c>
       <c r="R179" s="42" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="S179" s="53" t="inlineStr">
         <is>
@@ -74222,7 +74222,7 @@
         </is>
       </c>
       <c r="R180" s="42" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="S180" s="52" t="inlineStr">
         <is>
@@ -74398,7 +74398,7 @@
         </is>
       </c>
       <c r="R182" s="42" t="n">
-        <v>-40.5</v>
+        <v>-40.4</v>
       </c>
       <c r="S182" s="52" t="inlineStr">
         <is>
@@ -74486,7 +74486,7 @@
         </is>
       </c>
       <c r="R183" s="42" t="n">
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
       <c r="S183" s="53" t="inlineStr">
         <is>
@@ -74574,7 +74574,7 @@
         </is>
       </c>
       <c r="R184" s="42" t="n">
-        <v>-3.3</v>
+        <v>-2.6</v>
       </c>
       <c r="S184" s="52" t="inlineStr">
         <is>
@@ -74662,7 +74662,7 @@
         </is>
       </c>
       <c r="R185" s="42" t="n">
-        <v>-4.9</v>
+        <v>-5.4</v>
       </c>
       <c r="S185" s="52" t="inlineStr">
         <is>
@@ -74750,7 +74750,7 @@
         </is>
       </c>
       <c r="R186" s="42" t="n">
-        <v>-13.3</v>
+        <v>-13.4</v>
       </c>
       <c r="S186" s="53" t="inlineStr">
         <is>
@@ -74838,7 +74838,7 @@
         </is>
       </c>
       <c r="R187" s="42" t="n">
-        <v>-13.8</v>
+        <v>-13.2</v>
       </c>
       <c r="S187" s="53" t="inlineStr">
         <is>
@@ -74926,7 +74926,7 @@
         </is>
       </c>
       <c r="R188" s="42" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="S188" s="53" t="inlineStr">
         <is>
@@ -75014,7 +75014,7 @@
         </is>
       </c>
       <c r="R189" s="42" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="S189" s="52" t="inlineStr">
         <is>
@@ -75102,7 +75102,7 @@
         </is>
       </c>
       <c r="R190" s="42" t="n">
-        <v>-14.4</v>
+        <v>-14.6</v>
       </c>
       <c r="S190" s="53" t="inlineStr">
         <is>
@@ -75190,7 +75190,7 @@
         </is>
       </c>
       <c r="R191" s="42" t="n">
-        <v>-4.5</v>
+        <v>-4.9</v>
       </c>
       <c r="S191" s="52" t="inlineStr">
         <is>
@@ -75278,7 +75278,7 @@
         </is>
       </c>
       <c r="R192" s="42" t="n">
-        <v>-19</v>
+        <v>-18.2</v>
       </c>
       <c r="S192" s="53" t="inlineStr">
         <is>
@@ -75366,7 +75366,7 @@
         </is>
       </c>
       <c r="R193" s="42" t="n">
-        <v>-5.1</v>
+        <v>-6.3</v>
       </c>
       <c r="S193" s="53" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Live odds + game results + model refresh 2026-10-23 16:24 UTC
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -1632,7 +1632,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -1696,7 +1696,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.4</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -1760,7 +1760,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-7.5</v>
+        <v>-7.3</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -1824,7 +1824,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-14.5</v>
+        <v>-14.6</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -1888,7 +1888,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-7.6</v>
+        <v>-7.8</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -1952,7 +1952,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-15.9</v>
+        <v>-15.7</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -2016,7 +2016,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -2288,7 +2288,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-35</v>
+        <v>-35.3</v>
       </c>
       <c r="S40" s="51" t="n"/>
       <c r="T40" s="51" t="n"/>
@@ -2360,7 +2360,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-7.8</v>
+        <v>-8.6</v>
       </c>
       <c r="S41" s="52" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-17.3</v>
+        <v>-17.5</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -2536,7 +2536,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.7</v>
       </c>
       <c r="S43" s="52" t="inlineStr">
         <is>
@@ -2616,7 +2616,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-25.1</v>
+        <v>-26.2</v>
       </c>
       <c r="S44" s="51" t="n"/>
       <c r="T44" s="51" t="n"/>
@@ -2688,7 +2688,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -2776,7 +2776,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-5.1</v>
+        <v>-5.4</v>
       </c>
       <c r="S46" s="54" t="inlineStr">
         <is>
@@ -2864,7 +2864,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -3071,7 +3071,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-6</v>
+        <v>-5.4</v>
       </c>
       <c r="S51" s="53" t="inlineStr">
         <is>
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>3.2</v>
+        <v>5.5</v>
       </c>
       <c r="S52" s="53" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
@@ -3259,9 +3259,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U53" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U53" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V53" s="52" t="inlineStr">
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-1</v>
+        <v>-2.5</v>
       </c>
       <c r="S54" s="53" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>-13.2</v>
+        <v>-12.2</v>
       </c>
       <c r="S55" s="52" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>-4.6</v>
+        <v>-1.1</v>
       </c>
       <c r="S56" s="52" t="inlineStr">
         <is>
@@ -3599,7 +3599,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>-38.3</v>
+        <v>-39.8</v>
       </c>
       <c r="S57" s="52" t="inlineStr">
         <is>
@@ -3806,7 +3806,7 @@
         </is>
       </c>
       <c r="R61" s="42" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="S61" s="53" t="inlineStr">
         <is>
@@ -3818,9 +3818,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U61" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U61" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V61" s="53" t="inlineStr">
@@ -3894,7 +3894,7 @@
         </is>
       </c>
       <c r="R62" s="42" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="S62" s="53" t="inlineStr">
         <is>
@@ -3982,7 +3982,7 @@
         </is>
       </c>
       <c r="R63" s="42" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="S63" s="52" t="inlineStr">
         <is>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="R64" s="42" t="n">
-        <v>-1.8</v>
+        <v>-1.7</v>
       </c>
       <c r="S64" s="52" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="R65" s="42" t="n">
-        <v>18.8</v>
+        <v>19.7</v>
       </c>
       <c r="S65" s="52" t="inlineStr">
         <is>
@@ -4246,7 +4246,7 @@
         </is>
       </c>
       <c r="R66" s="42" t="n">
-        <v>-20.5</v>
+        <v>-20.1</v>
       </c>
       <c r="S66" s="52" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
         </is>
       </c>
       <c r="R67" s="42" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.8</v>
       </c>
       <c r="S67" s="53" t="inlineStr">
         <is>
@@ -4422,7 +4422,7 @@
         </is>
       </c>
       <c r="R68" s="42" t="n">
-        <v>-6.8</v>
+        <v>-7.2</v>
       </c>
       <c r="S68" s="53" t="inlineStr">
         <is>
@@ -4510,7 +4510,7 @@
         </is>
       </c>
       <c r="R69" s="42" t="n">
-        <v>-7.2</v>
+        <v>-6.6</v>
       </c>
       <c r="S69" s="53" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="R26" s="42" t="n">
-        <v>-4.7</v>
+        <v>-5.6</v>
       </c>
       <c r="S26" s="53" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>-7.7</v>
+        <v>-7.6</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -5317,7 +5317,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -5381,7 +5381,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -5445,7 +5445,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-0.3</v>
+        <v>-0.5</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -5636,7 +5636,7 @@
         </is>
       </c>
       <c r="R34" s="42" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="S34" s="52" t="inlineStr">
         <is>
@@ -5724,7 +5724,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-1.9</v>
+        <v>-2.1</v>
       </c>
       <c r="S35" s="53" t="inlineStr">
         <is>
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-8.1</v>
+        <v>-8.4</v>
       </c>
       <c r="S36" s="53" t="inlineStr">
         <is>
@@ -5900,7 +5900,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-15.7</v>
+        <v>-15.4</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -6076,7 +6076,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-11.4</v>
+        <v>-10.6</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-10.6</v>
+        <v>-9.9</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-6.6</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -6459,7 +6459,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>-4.9</v>
+        <v>-2.1</v>
       </c>
       <c r="S45" s="54" t="inlineStr">
         <is>
@@ -6547,7 +6547,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-12.1</v>
+        <v>-9.9</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -6635,7 +6635,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-11.5</v>
+        <v>-12.5</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>-5.7</v>
+        <v>-6.1</v>
       </c>
       <c r="S48" s="53" t="inlineStr">
         <is>
@@ -6811,7 +6811,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-26.2</v>
+        <v>-26.4</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -6899,7 +6899,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
@@ -6911,9 +6911,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U50" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U50" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V50" s="53" t="inlineStr">
@@ -7106,7 +7106,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="S54" s="52" t="inlineStr">
         <is>
@@ -7194,7 +7194,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="S55" s="53" t="inlineStr">
         <is>
@@ -7282,7 +7282,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>-32.6</v>
+        <v>-32.4</v>
       </c>
       <c r="S56" s="52" t="inlineStr">
         <is>
@@ -7370,7 +7370,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>15.4</v>
+        <v>15.9</v>
       </c>
       <c r="S57" s="52" t="inlineStr">
         <is>
@@ -7458,7 +7458,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.7</v>
       </c>
       <c r="S58" s="52" t="inlineStr">
         <is>
@@ -7546,7 +7546,7 @@
         </is>
       </c>
       <c r="R59" s="42" t="n">
-        <v>-23.9</v>
+        <v>-24.2</v>
       </c>
       <c r="S59" s="52" t="inlineStr">
         <is>
@@ -7722,7 +7722,7 @@
         </is>
       </c>
       <c r="R61" s="42" t="n">
-        <v>-4.3</v>
+        <v>-5.1</v>
       </c>
       <c r="S61" s="52" t="inlineStr">
         <is>
@@ -8421,7 +8421,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-13.4</v>
+        <v>-13.6</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -8549,7 +8549,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>14.2</v>
+        <v>15.1</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -8613,7 +8613,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -8677,7 +8677,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-3.2</v>
+        <v>-3.8</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -8741,7 +8741,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-8.9</v>
+        <v>-9.4</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -8805,7 +8805,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -8869,7 +8869,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>-7.1</v>
+        <v>-7.7</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -9149,7 +9149,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-1.3</v>
+        <v>-1.5</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -9237,7 +9237,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-16.9</v>
+        <v>-16.5</v>
       </c>
       <c r="S41" s="52" t="inlineStr">
         <is>
@@ -9413,7 +9413,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>-18.7</v>
+        <v>-18.3</v>
       </c>
       <c r="S43" s="53" t="inlineStr">
         <is>
@@ -9501,7 +9501,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>18.9</v>
+        <v>18.3</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -9797,7 +9797,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-14.7</v>
+        <v>-15.6</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -9885,7 +9885,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-1.7</v>
+        <v>-2.9</v>
       </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
@@ -9973,7 +9973,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>1.9</v>
+        <v>3.1</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -10061,7 +10061,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="S52" s="53" t="inlineStr">
         <is>
@@ -10149,7 +10149,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>-14.6</v>
+        <v>-16.2</v>
       </c>
       <c r="S53" s="53" t="inlineStr">
         <is>
@@ -10237,7 +10237,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>-19.6</v>
+        <v>-18.6</v>
       </c>
       <c r="S54" s="53" t="inlineStr">
         <is>
@@ -10444,7 +10444,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
       <c r="S58" s="53" t="inlineStr">
         <is>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="R59" s="42" t="n">
-        <v>-12.9</v>
+        <v>-12.1</v>
       </c>
       <c r="S59" s="52" t="inlineStr">
         <is>
@@ -10620,7 +10620,7 @@
         </is>
       </c>
       <c r="R60" s="42" t="n">
-        <v>-5.9</v>
+        <v>-6.3</v>
       </c>
       <c r="S60" s="54" t="inlineStr">
         <is>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="R61" s="42" t="n">
-        <v>-13.3</v>
+        <v>-12.7</v>
       </c>
       <c r="S61" s="53" t="inlineStr">
         <is>
@@ -10796,7 +10796,7 @@
         </is>
       </c>
       <c r="R62" s="42" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="S62" s="52" t="inlineStr">
         <is>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="R63" s="42" t="n">
-        <v>-13.1</v>
+        <v>-13</v>
       </c>
       <c r="S63" s="52" t="inlineStr">
         <is>
@@ -10972,7 +10972,7 @@
         </is>
       </c>
       <c r="R64" s="42" t="n">
-        <v>-7.9</v>
+        <v>-7.7</v>
       </c>
       <c r="S64" s="53" t="inlineStr">
         <is>
@@ -11715,7 +11715,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>10.3</v>
+        <v>9.9</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -11843,7 +11843,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -11907,7 +11907,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-12</v>
+        <v>-11.9</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -11971,7 +11971,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>-15.8</v>
+        <v>-16.2</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -12035,7 +12035,7 @@
       <c r="P35" s="42" t="n"/>
       <c r="Q35" s="42" t="n"/>
       <c r="R35" s="42" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="S35" s="51" t="n"/>
       <c r="T35" s="51" t="n"/>
@@ -12226,7 +12226,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -12402,7 +12402,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>-7.9</v>
+        <v>-7.6</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -12490,7 +12490,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>8.199999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -12578,7 +12578,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>9.6</v>
+        <v>10.2</v>
       </c>
       <c r="S43" s="53" t="inlineStr">
         <is>
@@ -12666,7 +12666,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-7</v>
+        <v>-7.1</v>
       </c>
       <c r="S44" s="53" t="inlineStr">
         <is>
@@ -12754,7 +12754,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>-15.9</v>
+        <v>-15.2</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -12961,7 +12961,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="S49" s="52" t="inlineStr">
         <is>
@@ -13049,7 +13049,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>13.9</v>
+        <v>11.7</v>
       </c>
       <c r="S50" s="52" t="inlineStr">
         <is>
@@ -13137,7 +13137,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-26.5</v>
+        <v>-25.7</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -13225,7 +13225,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>-29.7</v>
+        <v>-30.3</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -13313,7 +13313,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>-24.2</v>
+        <v>-23.8</v>
       </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
@@ -13401,7 +13401,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="S54" s="52" t="inlineStr">
         <is>
@@ -13489,7 +13489,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>-0.6</v>
+        <v>-0.1</v>
       </c>
       <c r="S55" s="53" t="inlineStr">
         <is>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="S56" s="52" t="inlineStr">
         <is>
@@ -13784,7 +13784,7 @@
         </is>
       </c>
       <c r="R60" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.4</v>
       </c>
       <c r="S60" s="52" t="inlineStr">
         <is>
@@ -13872,7 +13872,7 @@
         </is>
       </c>
       <c r="R61" s="42" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="S61" s="52" t="inlineStr">
         <is>
@@ -13960,7 +13960,7 @@
         </is>
       </c>
       <c r="R62" s="42" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="S62" s="53" t="inlineStr">
         <is>
@@ -14048,7 +14048,7 @@
         </is>
       </c>
       <c r="R63" s="42" t="n">
-        <v>-11.3</v>
+        <v>-11.1</v>
       </c>
       <c r="S63" s="53" t="inlineStr">
         <is>
@@ -14224,7 +14224,7 @@
         </is>
       </c>
       <c r="R65" s="42" t="n">
-        <v>-5.3</v>
+        <v>-4.6</v>
       </c>
       <c r="S65" s="53" t="inlineStr">
         <is>
@@ -14312,7 +14312,7 @@
         </is>
       </c>
       <c r="R66" s="42" t="n">
-        <v>-6.1</v>
+        <v>-6.3</v>
       </c>
       <c r="S66" s="52" t="inlineStr">
         <is>
@@ -14400,7 +14400,7 @@
         </is>
       </c>
       <c r="R67" s="42" t="n">
-        <v>15.6</v>
+        <v>16.5</v>
       </c>
       <c r="S67" s="53" t="inlineStr">
         <is>
@@ -14975,7 +14975,7 @@
         </is>
       </c>
       <c r="R22" s="42" t="n">
-        <v>-7.7</v>
+        <v>-7.8</v>
       </c>
       <c r="S22" s="53" t="inlineStr">
         <is>
@@ -15151,7 +15151,7 @@
         </is>
       </c>
       <c r="R24" s="42" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="S24" s="52" t="inlineStr">
         <is>
@@ -15239,7 +15239,7 @@
         </is>
       </c>
       <c r="R25" s="42" t="n">
-        <v>-2.1</v>
+        <v>-2.2</v>
       </c>
       <c r="S25" s="53" t="inlineStr">
         <is>
@@ -15447,7 +15447,7 @@
         </is>
       </c>
       <c r="R29" s="42" t="n">
-        <v>5.2</v>
+        <v>5.9</v>
       </c>
       <c r="S29" s="52" t="inlineStr">
         <is>
@@ -15535,7 +15535,7 @@
         </is>
       </c>
       <c r="R30" s="42" t="n">
-        <v>-12.1</v>
+        <v>-11.9</v>
       </c>
       <c r="S30" s="54" t="inlineStr">
         <is>
@@ -15623,7 +15623,7 @@
         </is>
       </c>
       <c r="R31" s="42" t="n">
-        <v>-2.2</v>
+        <v>-2</v>
       </c>
       <c r="S31" s="53" t="inlineStr">
         <is>
@@ -15711,7 +15711,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="S32" s="53" t="inlineStr">
         <is>
@@ -15918,7 +15918,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-9.9</v>
+        <v>-10</v>
       </c>
       <c r="S36" s="53" t="inlineStr">
         <is>
@@ -16006,7 +16006,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>10.6</v>
+        <v>10.9</v>
       </c>
       <c r="S37" s="52" t="inlineStr">
         <is>
@@ -16094,7 +16094,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-11.7</v>
+        <v>-13.8</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -16106,9 +16106,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U38" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U38" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V38" s="52" t="inlineStr">
@@ -16182,7 +16182,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.5</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -16389,7 +16389,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>-13.3</v>
+        <v>-12.7</v>
       </c>
       <c r="S43" s="53" t="inlineStr">
         <is>
@@ -16477,7 +16477,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -16565,7 +16565,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>12.2</v>
+        <v>11.7</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -16952,7 +16952,7 @@
       <c r="P14" s="42" t="n"/>
       <c r="Q14" s="42" t="n"/>
       <c r="R14" s="42" t="n">
-        <v>-22.4</v>
+        <v>-21.7</v>
       </c>
       <c r="S14" s="51" t="n"/>
       <c r="T14" s="51" t="n"/>
@@ -17350,7 +17350,7 @@
         </is>
       </c>
       <c r="R22" s="42" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="S22" s="52" t="inlineStr">
         <is>
@@ -17362,9 +17362,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U22" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U22" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V22" s="53" t="inlineStr">
@@ -17438,7 +17438,7 @@
         </is>
       </c>
       <c r="R23" s="42" t="n">
-        <v>-38.3</v>
+        <v>-39.8</v>
       </c>
       <c r="S23" s="52" t="inlineStr">
         <is>
@@ -17645,7 +17645,7 @@
         </is>
       </c>
       <c r="R27" s="42" t="n">
-        <v>18.8</v>
+        <v>19.7</v>
       </c>
       <c r="S27" s="52" t="inlineStr">
         <is>
@@ -17733,7 +17733,7 @@
         </is>
       </c>
       <c r="R28" s="42" t="n">
-        <v>-6.8</v>
+        <v>-7.2</v>
       </c>
       <c r="S28" s="53" t="inlineStr">
         <is>
@@ -18366,7 +18366,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>-22.4</v>
+        <v>-21.7</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -18430,7 +18430,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>-7.6</v>
+        <v>-7.7</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -18494,7 +18494,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>-6</v>
+        <v>-5.4</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -18558,7 +18558,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -18601,7 +18601,7 @@
         <v>-3</v>
       </c>
       <c r="I29" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="J29" s="42" t="n">
         <v>-3.8</v>
@@ -18622,7 +18622,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-1.9</v>
+        <v>-2.9</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -18686,7 +18686,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-11.6</v>
+        <v>-12.5</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -18750,7 +18750,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>3</v>
+        <v>4.1</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -18942,7 +18942,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-15.7</v>
+        <v>-15.4</v>
       </c>
       <c r="S35" s="53" t="inlineStr">
         <is>
@@ -19030,7 +19030,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>-6.9</v>
+        <v>-6.7</v>
       </c>
       <c r="S36" s="52" t="inlineStr">
         <is>
@@ -19118,7 +19118,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-14.6</v>
+        <v>-14.8</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -19206,7 +19206,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -19294,7 +19294,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="S39" s="53" t="inlineStr">
         <is>
@@ -19382,7 +19382,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-9.4</v>
+        <v>-9.5</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -19470,7 +19470,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>18.7</v>
+        <v>19.2</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -19677,7 +19677,7 @@
         </is>
       </c>
       <c r="R45" s="42" t="n">
-        <v>-26.5</v>
+        <v>-25.7</v>
       </c>
       <c r="S45" s="52" t="inlineStr">
         <is>
@@ -19765,7 +19765,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -19853,7 +19853,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-9</v>
+        <v>-10.1</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -19941,7 +19941,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>8.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="S48" s="52" t="inlineStr">
         <is>
@@ -20029,7 +20029,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-7.7</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -20117,7 +20117,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-13.6</v>
+        <v>-14.7</v>
       </c>
       <c r="S50" s="53" t="inlineStr">
         <is>
@@ -20205,7 +20205,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>-16.2</v>
+        <v>-17.4</v>
       </c>
       <c r="S51" s="53" t="inlineStr">
         <is>
@@ -20412,7 +20412,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>14.7</v>
+        <v>14.2</v>
       </c>
       <c r="S55" s="52" t="inlineStr">
         <is>
@@ -20500,7 +20500,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
       <c r="S56" s="52" t="inlineStr">
         <is>
@@ -20588,7 +20588,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>-7.5</v>
+        <v>-7.2</v>
       </c>
       <c r="S57" s="53" t="inlineStr">
         <is>
@@ -20676,7 +20676,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>14.9</v>
+        <v>14.3</v>
       </c>
       <c r="S58" s="52" t="inlineStr">
         <is>
@@ -20764,7 +20764,7 @@
         </is>
       </c>
       <c r="R59" s="42" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="S59" s="53" t="inlineStr">
         <is>
@@ -20852,7 +20852,7 @@
         </is>
       </c>
       <c r="R60" s="42" t="n">
-        <v>-11.8</v>
+        <v>-11.9</v>
       </c>
       <c r="S60" s="52" t="inlineStr">
         <is>
@@ -21483,7 +21483,7 @@
       <c r="P23" s="42" t="n"/>
       <c r="Q23" s="42" t="n"/>
       <c r="R23" s="42" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="S23" s="51" t="n"/>
       <c r="T23" s="51" t="n"/>
@@ -21547,7 +21547,7 @@
       <c r="P24" s="42" t="n"/>
       <c r="Q24" s="42" t="n"/>
       <c r="R24" s="42" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="S24" s="51" t="n"/>
       <c r="T24" s="51" t="n"/>
@@ -21611,7 +21611,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -21802,7 +21802,7 @@
         </is>
       </c>
       <c r="R29" s="42" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="S29" s="52" t="inlineStr">
         <is>
@@ -21890,7 +21890,7 @@
         </is>
       </c>
       <c r="R30" s="42" t="n">
-        <v>-21.9</v>
+        <v>-22.4</v>
       </c>
       <c r="S30" s="52" t="inlineStr">
         <is>
@@ -21978,7 +21978,7 @@
         </is>
       </c>
       <c r="R31" s="42" t="n">
-        <v>-6.3</v>
+        <v>-5.9</v>
       </c>
       <c r="S31" s="53" t="inlineStr">
         <is>
@@ -22066,7 +22066,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>8.5</v>
+        <v>7.9</v>
       </c>
       <c r="S32" s="52" t="inlineStr">
         <is>
@@ -22154,7 +22154,7 @@
         </is>
       </c>
       <c r="R33" s="42" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
       <c r="S33" s="53" t="inlineStr">
         <is>
@@ -22361,7 +22361,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-14.6</v>
+        <v>-16.2</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -22449,7 +22449,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>3.6</v>
+        <v>2.3</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -22537,7 +22537,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>0.2</v>
+        <v>-2.2</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -22625,7 +22625,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="S40" s="52" t="inlineStr">
         <is>
@@ -22713,7 +22713,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>5.7</v>
+        <v>6.5</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -23008,7 +23008,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-22.2</v>
+        <v>-22</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -23096,7 +23096,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>-21.5</v>
+        <v>-20.8</v>
       </c>
       <c r="S47" s="53" t="inlineStr">
         <is>
@@ -23184,7 +23184,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>-7.2</v>
+        <v>-6.6</v>
       </c>
       <c r="S48" s="53" t="inlineStr">
         <is>
@@ -23272,7 +23272,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-7.2</v>
+        <v>-6.2</v>
       </c>
       <c r="S49" s="52" t="inlineStr">
         <is>
@@ -23795,7 +23795,7 @@
       <c r="P20" s="42" t="n"/>
       <c r="Q20" s="42" t="n"/>
       <c r="R20" s="42" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="S20" s="51" t="n"/>
       <c r="T20" s="51" t="n"/>
@@ -23923,7 +23923,7 @@
       <c r="P22" s="42" t="n"/>
       <c r="Q22" s="42" t="n"/>
       <c r="R22" s="42" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="S22" s="51" t="n"/>
       <c r="T22" s="51" t="n"/>
@@ -24115,7 +24115,7 @@
         </is>
       </c>
       <c r="R26" s="42" t="n">
-        <v>-14.4</v>
+        <v>-15.2</v>
       </c>
       <c r="S26" s="53" t="inlineStr">
         <is>
@@ -24203,7 +24203,7 @@
         </is>
       </c>
       <c r="R27" s="42" t="n">
-        <v>-3.4</v>
+        <v>-2.4</v>
       </c>
       <c r="S27" s="53" t="inlineStr">
         <is>
@@ -24498,7 +24498,7 @@
         </is>
       </c>
       <c r="R32" s="42" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
       <c r="S32" s="52" t="inlineStr">
         <is>
@@ -24586,7 +24586,7 @@
         </is>
       </c>
       <c r="R33" s="42" t="n">
-        <v>-1.8</v>
+        <v>-1.5</v>
       </c>
       <c r="S33" s="53" t="inlineStr">
         <is>
@@ -24674,7 +24674,7 @@
         </is>
       </c>
       <c r="R34" s="42" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
       <c r="S34" s="53" t="inlineStr">
         <is>
@@ -24881,7 +24881,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-15.6</v>
+        <v>-15.1</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -24969,7 +24969,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-2.4</v>
+        <v>-2.3</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -25057,7 +25057,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -25145,7 +25145,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="S41" s="52" t="inlineStr">
         <is>
@@ -25844,7 +25844,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-9</v>
+        <v>-8.5</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -25908,7 +25908,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>10</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -25972,7 +25972,7 @@
       <c r="P30" s="42" t="n"/>
       <c r="Q30" s="42" t="n"/>
       <c r="R30" s="42" t="n">
-        <v>-1.2</v>
+        <v>-2.4</v>
       </c>
       <c r="S30" s="51" t="n"/>
       <c r="T30" s="51" t="n"/>
@@ -26036,7 +26036,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -26100,7 +26100,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -26137,7 +26137,7 @@
         </is>
       </c>
       <c r="G33" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="H33" s="42" t="n">
         <v>-3.2</v>
@@ -26164,7 +26164,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-4.8</v>
+        <v>-5</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -26355,7 +26355,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-22.3</v>
+        <v>-25</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -26443,7 +26443,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-11</v>
+        <v>-10.6</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -26531,7 +26531,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>-13.8</v>
+        <v>-13.5</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -26619,7 +26619,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>-10.5</v>
+        <v>-10.9</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -26707,7 +26707,7 @@
         </is>
       </c>
       <c r="R41" s="42" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="S41" s="53" t="inlineStr">
         <is>
@@ -26795,7 +26795,7 @@
         </is>
       </c>
       <c r="R42" s="42" t="n">
-        <v>-15.4</v>
+        <v>-15.2</v>
       </c>
       <c r="S42" s="52" t="inlineStr">
         <is>
@@ -26875,7 +26875,7 @@
         </is>
       </c>
       <c r="R43" s="42" t="n">
-        <v>-30.4</v>
+        <v>-31.3</v>
       </c>
       <c r="S43" s="51" t="n"/>
       <c r="T43" s="51" t="n"/>
@@ -26947,7 +26947,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-11.7</v>
+        <v>-11.5</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="S48" s="53" t="inlineStr">
         <is>
@@ -27242,7 +27242,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>14.3</v>
+        <v>13.3</v>
       </c>
       <c r="S49" s="52" t="inlineStr">
         <is>
@@ -27330,7 +27330,7 @@
         </is>
       </c>
       <c r="R50" s="42" t="n">
-        <v>-8.5</v>
+        <v>-10.3</v>
       </c>
       <c r="S50" s="53" t="inlineStr">
         <is>
@@ -27342,9 +27342,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U50" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U50" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V50" s="53" t="inlineStr">
@@ -27418,7 +27418,7 @@
         </is>
       </c>
       <c r="R51" s="42" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="S51" s="52" t="inlineStr">
         <is>
@@ -27506,7 +27506,7 @@
         </is>
       </c>
       <c r="R52" s="42" t="n">
-        <v>0.7</v>
+        <v>-0.7</v>
       </c>
       <c r="S52" s="52" t="inlineStr">
         <is>
@@ -27594,7 +27594,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>10.9</v>
+        <v>12.8</v>
       </c>
       <c r="S53" s="52" t="inlineStr">
         <is>
@@ -27682,7 +27682,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>7.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="S54" s="52" t="inlineStr">
         <is>
@@ -27694,9 +27694,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U54" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U54" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V54" s="52" t="inlineStr">
@@ -27889,7 +27889,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>-16.4</v>
+        <v>-16.3</v>
       </c>
       <c r="S58" s="53" t="inlineStr">
         <is>
@@ -27977,7 +27977,7 @@
         </is>
       </c>
       <c r="R59" s="42" t="n">
-        <v>-40.6</v>
+        <v>-40.5</v>
       </c>
       <c r="S59" s="52" t="inlineStr">
         <is>
@@ -28065,7 +28065,7 @@
         </is>
       </c>
       <c r="R60" s="42" t="n">
-        <v>15.9</v>
+        <v>15.2</v>
       </c>
       <c r="S60" s="53" t="inlineStr">
         <is>
@@ -28153,7 +28153,7 @@
         </is>
       </c>
       <c r="R61" s="42" t="n">
-        <v>-2.5</v>
+        <v>-3.2</v>
       </c>
       <c r="S61" s="52" t="inlineStr">
         <is>
@@ -28241,7 +28241,7 @@
         </is>
       </c>
       <c r="R62" s="42" t="n">
-        <v>-5.8</v>
+        <v>-5.3</v>
       </c>
       <c r="S62" s="52" t="inlineStr">
         <is>
@@ -28329,7 +28329,7 @@
         </is>
       </c>
       <c r="R63" s="42" t="n">
-        <v>-13.3</v>
+        <v>-12.9</v>
       </c>
       <c r="S63" s="53" t="inlineStr">
         <is>
@@ -28417,7 +28417,7 @@
         </is>
       </c>
       <c r="R64" s="42" t="n">
-        <v>-13.1</v>
+        <v>-12.8</v>
       </c>
       <c r="S64" s="53" t="inlineStr">
         <is>
@@ -28429,9 +28429,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U64" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U64" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V64" s="52" t="inlineStr">
@@ -29184,7 +29184,7 @@
         </is>
       </c>
       <c r="R26" s="42" t="n">
-        <v>-2.8</v>
+        <v>-3.2</v>
       </c>
       <c r="S26" s="53" t="inlineStr">
         <is>
@@ -29272,7 +29272,7 @@
         </is>
       </c>
       <c r="R27" s="42" t="n">
-        <v>10.4</v>
+        <v>9.9</v>
       </c>
       <c r="S27" s="52" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-1.5</v>
+        <v>-1.9</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -29416,7 +29416,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>-5.7</v>
+        <v>-5.5</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -29544,7 +29544,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>-16.2</v>
+        <v>-16.7</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -29736,7 +29736,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-3.6</v>
+        <v>-2.9</v>
       </c>
       <c r="S35" s="52" t="inlineStr">
         <is>
@@ -29824,7 +29824,7 @@
         </is>
       </c>
       <c r="R36" s="42" t="n">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="S36" s="52" t="inlineStr">
         <is>
@@ -29912,7 +29912,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>-23.5</v>
+        <v>-23.6</v>
       </c>
       <c r="S37" s="53" t="inlineStr">
         <is>
@@ -30000,7 +30000,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-4.3</v>
+        <v>-4.4</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -30088,7 +30088,7 @@
         </is>
       </c>
       <c r="R39" s="42" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="S39" s="52" t="inlineStr">
         <is>
@@ -30176,7 +30176,7 @@
         </is>
       </c>
       <c r="R40" s="42" t="n">
-        <v>14.8</v>
+        <v>15.2</v>
       </c>
       <c r="S40" s="53" t="inlineStr">
         <is>
@@ -30383,7 +30383,7 @@
         </is>
       </c>
       <c r="R44" s="42" t="n">
-        <v>-7.6</v>
+        <v>-9.1</v>
       </c>
       <c r="S44" s="52" t="inlineStr">
         <is>
@@ -30395,9 +30395,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U44" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U44" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V44" s="52" t="inlineStr">
@@ -30559,7 +30559,7 @@
         </is>
       </c>
       <c r="R46" s="42" t="n">
-        <v>-5.6</v>
+        <v>-7.2</v>
       </c>
       <c r="S46" s="53" t="inlineStr">
         <is>
@@ -30647,7 +30647,7 @@
         </is>
       </c>
       <c r="R47" s="42" t="n">
-        <v>16.5</v>
+        <v>17.2</v>
       </c>
       <c r="S47" s="52" t="inlineStr">
         <is>
@@ -30735,7 +30735,7 @@
         </is>
       </c>
       <c r="R48" s="42" t="n">
-        <v>4.9</v>
+        <v>5.8</v>
       </c>
       <c r="S48" s="52" t="inlineStr">
         <is>
@@ -30823,7 +30823,7 @@
         </is>
       </c>
       <c r="R49" s="42" t="n">
-        <v>-13.3</v>
+        <v>-14.3</v>
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
@@ -31030,7 +31030,7 @@
         </is>
       </c>
       <c r="R53" s="42" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="S53" s="53" t="inlineStr">
         <is>
@@ -31118,7 +31118,7 @@
         </is>
       </c>
       <c r="R54" s="42" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="S54" s="52" t="inlineStr">
         <is>
@@ -31206,7 +31206,7 @@
         </is>
       </c>
       <c r="R55" s="42" t="n">
-        <v>-14.3</v>
+        <v>-14.6</v>
       </c>
       <c r="S55" s="53" t="inlineStr">
         <is>
@@ -31294,7 +31294,7 @@
         </is>
       </c>
       <c r="R56" s="42" t="n">
-        <v>-4.3</v>
+        <v>-5.1</v>
       </c>
       <c r="S56" s="52" t="inlineStr">
         <is>
@@ -31382,7 +31382,7 @@
         </is>
       </c>
       <c r="R57" s="42" t="n">
-        <v>-18.4</v>
+        <v>-18.9</v>
       </c>
       <c r="S57" s="53" t="inlineStr">
         <is>
@@ -31470,7 +31470,7 @@
         </is>
       </c>
       <c r="R58" s="42" t="n">
-        <v>-5.3</v>
+        <v>-5.7</v>
       </c>
       <c r="S58" s="52" t="inlineStr">
         <is>
@@ -42814,7 +42814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -64804,7 +64804,7 @@
         </is>
       </c>
       <c r="C92" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D92" s="42" t="n">
         <v>87</v>
@@ -69126,7 +69126,7 @@
       <c r="P9" s="42" t="n"/>
       <c r="Q9" s="42" t="n"/>
       <c r="R9" s="42" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="S9" s="51" t="n"/>
       <c r="T9" s="51" t="n"/>
@@ -69190,7 +69190,7 @@
       <c r="P10" s="42" t="n"/>
       <c r="Q10" s="42" t="n"/>
       <c r="R10" s="42" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.4</v>
       </c>
       <c r="S10" s="51" t="n"/>
       <c r="T10" s="51" t="n"/>
@@ -69254,7 +69254,7 @@
       <c r="P11" s="42" t="n"/>
       <c r="Q11" s="42" t="n"/>
       <c r="R11" s="42" t="n">
-        <v>-7.5</v>
+        <v>-7.3</v>
       </c>
       <c r="S11" s="51" t="n"/>
       <c r="T11" s="51" t="n"/>
@@ -69318,7 +69318,7 @@
       <c r="P12" s="42" t="n"/>
       <c r="Q12" s="42" t="n"/>
       <c r="R12" s="42" t="n">
-        <v>-14.5</v>
+        <v>-14.6</v>
       </c>
       <c r="S12" s="51" t="n"/>
       <c r="T12" s="51" t="n"/>
@@ -69382,7 +69382,7 @@
       <c r="P13" s="42" t="n"/>
       <c r="Q13" s="42" t="n"/>
       <c r="R13" s="42" t="n">
-        <v>-7.6</v>
+        <v>-7.8</v>
       </c>
       <c r="S13" s="51" t="n"/>
       <c r="T13" s="51" t="n"/>
@@ -69446,7 +69446,7 @@
       <c r="P14" s="42" t="n"/>
       <c r="Q14" s="42" t="n"/>
       <c r="R14" s="42" t="n">
-        <v>-15.9</v>
+        <v>-15.7</v>
       </c>
       <c r="S14" s="51" t="n"/>
       <c r="T14" s="51" t="n"/>
@@ -69510,7 +69510,7 @@
       <c r="P15" s="42" t="n"/>
       <c r="Q15" s="42" t="n"/>
       <c r="R15" s="42" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="S15" s="51" t="n"/>
       <c r="T15" s="51" t="n"/>
@@ -69582,7 +69582,7 @@
         </is>
       </c>
       <c r="R16" s="42" t="n">
-        <v>-4.7</v>
+        <v>-5.6</v>
       </c>
       <c r="S16" s="53" t="inlineStr">
         <is>
@@ -69662,7 +69662,7 @@
       <c r="P17" s="42" t="n"/>
       <c r="Q17" s="42" t="n"/>
       <c r="R17" s="42" t="n">
-        <v>-7.7</v>
+        <v>-7.6</v>
       </c>
       <c r="S17" s="51" t="n"/>
       <c r="T17" s="51" t="n"/>
@@ -69726,7 +69726,7 @@
       <c r="P18" s="42" t="n"/>
       <c r="Q18" s="42" t="n"/>
       <c r="R18" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="S18" s="51" t="n"/>
       <c r="T18" s="51" t="n"/>
@@ -69790,7 +69790,7 @@
       <c r="P19" s="42" t="n"/>
       <c r="Q19" s="42" t="n"/>
       <c r="R19" s="42" t="n">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="S19" s="51" t="n"/>
       <c r="T19" s="51" t="n"/>
@@ -69854,7 +69854,7 @@
       <c r="P20" s="42" t="n"/>
       <c r="Q20" s="42" t="n"/>
       <c r="R20" s="42" t="n">
-        <v>-0.3</v>
+        <v>-0.5</v>
       </c>
       <c r="S20" s="51" t="n"/>
       <c r="T20" s="51" t="n"/>
@@ -69918,7 +69918,7 @@
       <c r="P21" s="42" t="n"/>
       <c r="Q21" s="42" t="n"/>
       <c r="R21" s="42" t="n">
-        <v>-13.4</v>
+        <v>-13.6</v>
       </c>
       <c r="S21" s="51" t="n"/>
       <c r="T21" s="51" t="n"/>
@@ -70046,7 +70046,7 @@
       <c r="P23" s="42" t="n"/>
       <c r="Q23" s="42" t="n"/>
       <c r="R23" s="42" t="n">
-        <v>14.2</v>
+        <v>15.1</v>
       </c>
       <c r="S23" s="51" t="n"/>
       <c r="T23" s="51" t="n"/>
@@ -70110,7 +70110,7 @@
       <c r="P24" s="42" t="n"/>
       <c r="Q24" s="42" t="n"/>
       <c r="R24" s="42" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="S24" s="51" t="n"/>
       <c r="T24" s="51" t="n"/>
@@ -70174,7 +70174,7 @@
       <c r="P25" s="42" t="n"/>
       <c r="Q25" s="42" t="n"/>
       <c r="R25" s="42" t="n">
-        <v>-3.2</v>
+        <v>-3.8</v>
       </c>
       <c r="S25" s="51" t="n"/>
       <c r="T25" s="51" t="n"/>
@@ -70238,7 +70238,7 @@
       <c r="P26" s="42" t="n"/>
       <c r="Q26" s="42" t="n"/>
       <c r="R26" s="42" t="n">
-        <v>-8.9</v>
+        <v>-9.4</v>
       </c>
       <c r="S26" s="51" t="n"/>
       <c r="T26" s="51" t="n"/>
@@ -70302,7 +70302,7 @@
       <c r="P27" s="42" t="n"/>
       <c r="Q27" s="42" t="n"/>
       <c r="R27" s="42" t="n">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="S27" s="51" t="n"/>
       <c r="T27" s="51" t="n"/>
@@ -70366,7 +70366,7 @@
       <c r="P28" s="42" t="n"/>
       <c r="Q28" s="42" t="n"/>
       <c r="R28" s="42" t="n">
-        <v>-7.1</v>
+        <v>-7.7</v>
       </c>
       <c r="S28" s="51" t="n"/>
       <c r="T28" s="51" t="n"/>
@@ -70430,7 +70430,7 @@
       <c r="P29" s="42" t="n"/>
       <c r="Q29" s="42" t="n"/>
       <c r="R29" s="42" t="n">
-        <v>10.3</v>
+        <v>9.9</v>
       </c>
       <c r="S29" s="51" t="n"/>
       <c r="T29" s="51" t="n"/>
@@ -70558,7 +70558,7 @@
       <c r="P31" s="42" t="n"/>
       <c r="Q31" s="42" t="n"/>
       <c r="R31" s="42" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="S31" s="51" t="n"/>
       <c r="T31" s="51" t="n"/>
@@ -70622,7 +70622,7 @@
       <c r="P32" s="42" t="n"/>
       <c r="Q32" s="42" t="n"/>
       <c r="R32" s="42" t="n">
-        <v>-12</v>
+        <v>-11.9</v>
       </c>
       <c r="S32" s="51" t="n"/>
       <c r="T32" s="51" t="n"/>
@@ -70686,7 +70686,7 @@
       <c r="P33" s="42" t="n"/>
       <c r="Q33" s="42" t="n"/>
       <c r="R33" s="42" t="n">
-        <v>-15.8</v>
+        <v>-16.2</v>
       </c>
       <c r="S33" s="51" t="n"/>
       <c r="T33" s="51" t="n"/>
@@ -70750,7 +70750,7 @@
       <c r="P34" s="42" t="n"/>
       <c r="Q34" s="42" t="n"/>
       <c r="R34" s="42" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="S34" s="51" t="n"/>
       <c r="T34" s="51" t="n"/>
@@ -70822,7 +70822,7 @@
         </is>
       </c>
       <c r="R35" s="42" t="n">
-        <v>-7.7</v>
+        <v>-7.8</v>
       </c>
       <c r="S35" s="53" t="inlineStr">
         <is>
@@ -70998,7 +70998,7 @@
         </is>
       </c>
       <c r="R37" s="42" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="S37" s="52" t="inlineStr">
         <is>
@@ -71086,7 +71086,7 @@
         </is>
       </c>
       <c r="R38" s="42" t="n">
-        <v>-2.1</v>
+        <v>-2.2</v>
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
@@ -71166,7 +71166,7 @@
       <c r="P39" s="42" t="n"/>
       <c r="Q39" s="42" t="n"/>
       <c r="R39" s="42" t="n">
-        <v>-22.4</v>
+        <v>-21.7</v>
       </c>
       <c r="S39" s="51" t="n"/>
       <c r="T39" s="51" t="n"/>
@@ -71230,7 +71230,7 @@
       <c r="P40" s="42" t="n"/>
       <c r="Q40" s="42" t="n"/>
       <c r="R40" s="42" t="n">
-        <v>-7.6</v>
+        <v>-7.7</v>
       </c>
       <c r="S40" s="51" t="n"/>
       <c r="T40" s="51" t="n"/>
@@ -71294,7 +71294,7 @@
       <c r="P41" s="42" t="n"/>
       <c r="Q41" s="42" t="n"/>
       <c r="R41" s="42" t="n">
-        <v>-6</v>
+        <v>-5.4</v>
       </c>
       <c r="S41" s="51" t="n"/>
       <c r="T41" s="51" t="n"/>
@@ -71358,7 +71358,7 @@
       <c r="P42" s="42" t="n"/>
       <c r="Q42" s="42" t="n"/>
       <c r="R42" s="42" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="S42" s="51" t="n"/>
       <c r="T42" s="51" t="n"/>
@@ -71401,7 +71401,7 @@
         <v>-3</v>
       </c>
       <c r="I43" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="J43" s="42" t="n">
         <v>-3.8</v>
@@ -71422,7 +71422,7 @@
       <c r="P43" s="42" t="n"/>
       <c r="Q43" s="42" t="n"/>
       <c r="R43" s="42" t="n">
-        <v>-1.9</v>
+        <v>-2.9</v>
       </c>
       <c r="S43" s="51" t="n"/>
       <c r="T43" s="51" t="n"/>
@@ -71486,7 +71486,7 @@
       <c r="P44" s="42" t="n"/>
       <c r="Q44" s="42" t="n"/>
       <c r="R44" s="42" t="n">
-        <v>-11.6</v>
+        <v>-12.5</v>
       </c>
       <c r="S44" s="51" t="n"/>
       <c r="T44" s="51" t="n"/>
@@ -71550,7 +71550,7 @@
       <c r="P45" s="42" t="n"/>
       <c r="Q45" s="42" t="n"/>
       <c r="R45" s="42" t="n">
-        <v>3</v>
+        <v>4.1</v>
       </c>
       <c r="S45" s="51" t="n"/>
       <c r="T45" s="51" t="n"/>
@@ -71678,7 +71678,7 @@
       <c r="P47" s="42" t="n"/>
       <c r="Q47" s="42" t="n"/>
       <c r="R47" s="42" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="S47" s="51" t="n"/>
       <c r="T47" s="51" t="n"/>
@@ -71742,7 +71742,7 @@
       <c r="P48" s="42" t="n"/>
       <c r="Q48" s="42" t="n"/>
       <c r="R48" s="42" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="S48" s="51" t="n"/>
       <c r="T48" s="51" t="n"/>
@@ -71806,7 +71806,7 @@
       <c r="P49" s="42" t="n"/>
       <c r="Q49" s="42" t="n"/>
       <c r="R49" s="42" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="S49" s="51" t="n"/>
       <c r="T49" s="51" t="n"/>
@@ -71870,7 +71870,7 @@
       <c r="P50" s="42" t="n"/>
       <c r="Q50" s="42" t="n"/>
       <c r="R50" s="42" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="S50" s="51" t="n"/>
       <c r="T50" s="51" t="n"/>
@@ -71998,7 +71998,7 @@
       <c r="P52" s="42" t="n"/>
       <c r="Q52" s="42" t="n"/>
       <c r="R52" s="42" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="S52" s="51" t="n"/>
       <c r="T52" s="51" t="n"/>
@@ -72062,7 +72062,7 @@
       <c r="P53" s="42" t="n"/>
       <c r="Q53" s="42" t="n"/>
       <c r="R53" s="42" t="n">
-        <v>-9</v>
+        <v>-8.5</v>
       </c>
       <c r="S53" s="51" t="n"/>
       <c r="T53" s="51" t="n"/>
@@ -72126,7 +72126,7 @@
       <c r="P54" s="42" t="n"/>
       <c r="Q54" s="42" t="n"/>
       <c r="R54" s="42" t="n">
-        <v>10</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="S54" s="51" t="n"/>
       <c r="T54" s="51" t="n"/>
@@ -72190,7 +72190,7 @@
       <c r="P55" s="42" t="n"/>
       <c r="Q55" s="42" t="n"/>
       <c r="R55" s="42" t="n">
-        <v>-1.2</v>
+        <v>-2.4</v>
       </c>
       <c r="S55" s="51" t="n"/>
       <c r="T55" s="51" t="n"/>
@@ -72254,7 +72254,7 @@
       <c r="P56" s="42" t="n"/>
       <c r="Q56" s="42" t="n"/>
       <c r="R56" s="42" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="S56" s="51" t="n"/>
       <c r="T56" s="51" t="n"/>
@@ -72318,7 +72318,7 @@
       <c r="P57" s="42" t="n"/>
       <c r="Q57" s="42" t="n"/>
       <c r="R57" s="42" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="S57" s="51" t="n"/>
       <c r="T57" s="51" t="n"/>
@@ -72355,7 +72355,7 @@
         </is>
       </c>
       <c r="G58" s="42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="H58" s="42" t="n">
         <v>-3.2</v>
@@ -72382,7 +72382,7 @@
       <c r="P58" s="42" t="n"/>
       <c r="Q58" s="42" t="n"/>
       <c r="R58" s="42" t="n">
-        <v>-4.8</v>
+        <v>-5</v>
       </c>
       <c r="S58" s="51" t="n"/>
       <c r="T58" s="51" t="n"/>
@@ -72454,7 +72454,7 @@
         </is>
       </c>
       <c r="R59" s="42" t="n">
-        <v>-2.8</v>
+        <v>-3.2</v>
       </c>
       <c r="S59" s="53" t="inlineStr">
         <is>
@@ -72542,7 +72542,7 @@
         </is>
       </c>
       <c r="R60" s="42" t="n">
-        <v>10.4</v>
+        <v>9.9</v>
       </c>
       <c r="S60" s="52" t="inlineStr">
         <is>
@@ -72622,7 +72622,7 @@
       <c r="P61" s="42" t="n"/>
       <c r="Q61" s="42" t="n"/>
       <c r="R61" s="42" t="n">
-        <v>-1.5</v>
+        <v>-1.9</v>
       </c>
       <c r="S61" s="51" t="n"/>
       <c r="T61" s="51" t="n"/>
@@ -72686,7 +72686,7 @@
       <c r="P62" s="42" t="n"/>
       <c r="Q62" s="42" t="n"/>
       <c r="R62" s="42" t="n">
-        <v>-5.7</v>
+        <v>-5.5</v>
       </c>
       <c r="S62" s="51" t="n"/>
       <c r="T62" s="51" t="n"/>
@@ -72814,7 +72814,7 @@
       <c r="P64" s="42" t="n"/>
       <c r="Q64" s="42" t="n"/>
       <c r="R64" s="42" t="n">
-        <v>-16.2</v>
+        <v>-16.7</v>
       </c>
       <c r="S64" s="51" t="n"/>
       <c r="T64" s="51" t="n"/>
@@ -73005,7 +73005,7 @@
         </is>
       </c>
       <c r="R68" s="42" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="S68" s="52" t="inlineStr">
         <is>
@@ -73085,7 +73085,7 @@
         </is>
       </c>
       <c r="R69" s="42" t="n">
-        <v>-35</v>
+        <v>-35.3</v>
       </c>
       <c r="S69" s="51" t="n"/>
       <c r="T69" s="51" t="n"/>
@@ -73157,7 +73157,7 @@
         </is>
       </c>
       <c r="R70" s="42" t="n">
-        <v>-7.8</v>
+        <v>-8.6</v>
       </c>
       <c r="S70" s="52" t="inlineStr">
         <is>
@@ -73245,7 +73245,7 @@
         </is>
       </c>
       <c r="R71" s="42" t="n">
-        <v>-17.3</v>
+        <v>-17.5</v>
       </c>
       <c r="S71" s="52" t="inlineStr">
         <is>
@@ -73333,7 +73333,7 @@
         </is>
       </c>
       <c r="R72" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.7</v>
       </c>
       <c r="S72" s="52" t="inlineStr">
         <is>
@@ -73413,7 +73413,7 @@
         </is>
       </c>
       <c r="R73" s="42" t="n">
-        <v>-25.1</v>
+        <v>-26.2</v>
       </c>
       <c r="S73" s="51" t="n"/>
       <c r="T73" s="51" t="n"/>
@@ -73485,7 +73485,7 @@
         </is>
       </c>
       <c r="R74" s="42" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="S74" s="52" t="inlineStr">
         <is>
@@ -73573,7 +73573,7 @@
         </is>
       </c>
       <c r="R75" s="42" t="n">
-        <v>-5.1</v>
+        <v>-5.4</v>
       </c>
       <c r="S75" s="54" t="inlineStr">
         <is>
@@ -73661,7 +73661,7 @@
         </is>
       </c>
       <c r="R76" s="42" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="S76" s="53" t="inlineStr">
         <is>
@@ -73749,7 +73749,7 @@
         </is>
       </c>
       <c r="R77" s="42" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="S77" s="52" t="inlineStr">
         <is>
@@ -73837,7 +73837,7 @@
         </is>
       </c>
       <c r="R78" s="42" t="n">
-        <v>-1.9</v>
+        <v>-2.1</v>
       </c>
       <c r="S78" s="53" t="inlineStr">
         <is>
@@ -73925,7 +73925,7 @@
         </is>
       </c>
       <c r="R79" s="42" t="n">
-        <v>-8.1</v>
+        <v>-8.4</v>
       </c>
       <c r="S79" s="53" t="inlineStr">
         <is>
@@ -74013,7 +74013,7 @@
         </is>
       </c>
       <c r="R80" s="42" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="S80" s="53" t="inlineStr">
         <is>
@@ -74101,7 +74101,7 @@
         </is>
       </c>
       <c r="R81" s="42" t="n">
-        <v>-15.7</v>
+        <v>-15.4</v>
       </c>
       <c r="S81" s="53" t="inlineStr">
         <is>
@@ -74189,7 +74189,7 @@
         </is>
       </c>
       <c r="R82" s="42" t="n">
-        <v>-11.4</v>
+        <v>-10.6</v>
       </c>
       <c r="S82" s="52" t="inlineStr">
         <is>
@@ -74277,7 +74277,7 @@
         </is>
       </c>
       <c r="R83" s="42" t="n">
-        <v>-10.6</v>
+        <v>-9.9</v>
       </c>
       <c r="S83" s="53" t="inlineStr">
         <is>
@@ -74453,7 +74453,7 @@
         </is>
       </c>
       <c r="R85" s="42" t="n">
-        <v>-1.3</v>
+        <v>-1.5</v>
       </c>
       <c r="S85" s="53" t="inlineStr">
         <is>
@@ -74541,7 +74541,7 @@
         </is>
       </c>
       <c r="R86" s="42" t="n">
-        <v>-16.9</v>
+        <v>-16.5</v>
       </c>
       <c r="S86" s="52" t="inlineStr">
         <is>
@@ -74717,7 +74717,7 @@
         </is>
       </c>
       <c r="R88" s="42" t="n">
-        <v>-18.7</v>
+        <v>-18.3</v>
       </c>
       <c r="S88" s="53" t="inlineStr">
         <is>
@@ -74805,7 +74805,7 @@
         </is>
       </c>
       <c r="R89" s="42" t="n">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="S89" s="52" t="inlineStr">
         <is>
@@ -74893,7 +74893,7 @@
         </is>
       </c>
       <c r="R90" s="42" t="n">
-        <v>18.9</v>
+        <v>18.3</v>
       </c>
       <c r="S90" s="52" t="inlineStr">
         <is>
@@ -74981,7 +74981,7 @@
         </is>
       </c>
       <c r="R91" s="42" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="S91" s="52" t="inlineStr">
         <is>
@@ -75069,7 +75069,7 @@
         </is>
       </c>
       <c r="R92" s="42" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="S92" s="53" t="inlineStr">
         <is>
@@ -75157,7 +75157,7 @@
         </is>
       </c>
       <c r="R93" s="42" t="n">
-        <v>-7.9</v>
+        <v>-7.6</v>
       </c>
       <c r="S93" s="53" t="inlineStr">
         <is>
@@ -75245,7 +75245,7 @@
         </is>
       </c>
       <c r="R94" s="42" t="n">
-        <v>8.199999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="S94" s="52" t="inlineStr">
         <is>
@@ -75333,7 +75333,7 @@
         </is>
       </c>
       <c r="R95" s="42" t="n">
-        <v>9.6</v>
+        <v>10.2</v>
       </c>
       <c r="S95" s="53" t="inlineStr">
         <is>
@@ -75421,7 +75421,7 @@
         </is>
       </c>
       <c r="R96" s="42" t="n">
-        <v>-7</v>
+        <v>-7.1</v>
       </c>
       <c r="S96" s="53" t="inlineStr">
         <is>
@@ -75509,7 +75509,7 @@
         </is>
       </c>
       <c r="R97" s="42" t="n">
-        <v>-15.9</v>
+        <v>-15.2</v>
       </c>
       <c r="S97" s="52" t="inlineStr">
         <is>
@@ -75597,7 +75597,7 @@
         </is>
       </c>
       <c r="R98" s="42" t="n">
-        <v>5.2</v>
+        <v>5.9</v>
       </c>
       <c r="S98" s="52" t="inlineStr">
         <is>
@@ -75685,7 +75685,7 @@
         </is>
       </c>
       <c r="R99" s="42" t="n">
-        <v>-12.1</v>
+        <v>-11.9</v>
       </c>
       <c r="S99" s="54" t="inlineStr">
         <is>
@@ -75773,7 +75773,7 @@
         </is>
       </c>
       <c r="R100" s="42" t="n">
-        <v>-2.2</v>
+        <v>-2</v>
       </c>
       <c r="S100" s="53" t="inlineStr">
         <is>
@@ -75861,7 +75861,7 @@
         </is>
       </c>
       <c r="R101" s="42" t="n">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="S101" s="53" t="inlineStr">
         <is>
@@ -75949,7 +75949,7 @@
         </is>
       </c>
       <c r="R102" s="42" t="n">
-        <v>-6.9</v>
+        <v>-6.7</v>
       </c>
       <c r="S102" s="52" t="inlineStr">
         <is>
@@ -76037,7 +76037,7 @@
         </is>
       </c>
       <c r="R103" s="42" t="n">
-        <v>-14.6</v>
+        <v>-14.8</v>
       </c>
       <c r="S103" s="53" t="inlineStr">
         <is>
@@ -76125,7 +76125,7 @@
         </is>
       </c>
       <c r="R104" s="42" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="S104" s="53" t="inlineStr">
         <is>
@@ -76213,7 +76213,7 @@
         </is>
       </c>
       <c r="R105" s="42" t="n">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="S105" s="53" t="inlineStr">
         <is>
@@ -76301,7 +76301,7 @@
         </is>
       </c>
       <c r="R106" s="42" t="n">
-        <v>-9.4</v>
+        <v>-9.5</v>
       </c>
       <c r="S106" s="53" t="inlineStr">
         <is>
@@ -76389,7 +76389,7 @@
         </is>
       </c>
       <c r="R107" s="42" t="n">
-        <v>18.7</v>
+        <v>19.2</v>
       </c>
       <c r="S107" s="53" t="inlineStr">
         <is>
@@ -76477,7 +76477,7 @@
         </is>
       </c>
       <c r="R108" s="42" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="S108" s="52" t="inlineStr">
         <is>
@@ -76565,7 +76565,7 @@
         </is>
       </c>
       <c r="R109" s="42" t="n">
-        <v>-21.9</v>
+        <v>-22.4</v>
       </c>
       <c r="S109" s="52" t="inlineStr">
         <is>
@@ -76653,7 +76653,7 @@
         </is>
       </c>
       <c r="R110" s="42" t="n">
-        <v>-6.3</v>
+        <v>-5.9</v>
       </c>
       <c r="S110" s="53" t="inlineStr">
         <is>
@@ -76741,7 +76741,7 @@
         </is>
       </c>
       <c r="R111" s="42" t="n">
-        <v>8.5</v>
+        <v>7.9</v>
       </c>
       <c r="S111" s="52" t="inlineStr">
         <is>
@@ -76829,7 +76829,7 @@
         </is>
       </c>
       <c r="R112" s="42" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
       <c r="S112" s="53" t="inlineStr">
         <is>
@@ -76917,7 +76917,7 @@
         </is>
       </c>
       <c r="R113" s="42" t="n">
-        <v>-14.4</v>
+        <v>-15.2</v>
       </c>
       <c r="S113" s="53" t="inlineStr">
         <is>
@@ -77005,7 +77005,7 @@
         </is>
       </c>
       <c r="R114" s="42" t="n">
-        <v>-3.4</v>
+        <v>-2.4</v>
       </c>
       <c r="S114" s="53" t="inlineStr">
         <is>
@@ -77181,7 +77181,7 @@
         </is>
       </c>
       <c r="R116" s="42" t="n">
-        <v>-22.3</v>
+        <v>-25</v>
       </c>
       <c r="S116" s="53" t="inlineStr">
         <is>
@@ -77269,7 +77269,7 @@
         </is>
       </c>
       <c r="R117" s="42" t="n">
-        <v>-11</v>
+        <v>-10.6</v>
       </c>
       <c r="S117" s="53" t="inlineStr">
         <is>
@@ -77357,7 +77357,7 @@
         </is>
       </c>
       <c r="R118" s="42" t="n">
-        <v>-13.8</v>
+        <v>-13.5</v>
       </c>
       <c r="S118" s="52" t="inlineStr">
         <is>
@@ -77445,7 +77445,7 @@
         </is>
       </c>
       <c r="R119" s="42" t="n">
-        <v>-10.5</v>
+        <v>-10.9</v>
       </c>
       <c r="S119" s="53" t="inlineStr">
         <is>
@@ -77533,7 +77533,7 @@
         </is>
       </c>
       <c r="R120" s="42" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="S120" s="53" t="inlineStr">
         <is>
@@ -77621,7 +77621,7 @@
         </is>
       </c>
       <c r="R121" s="42" t="n">
-        <v>-15.4</v>
+        <v>-15.2</v>
       </c>
       <c r="S121" s="52" t="inlineStr">
         <is>
@@ -77701,7 +77701,7 @@
         </is>
       </c>
       <c r="R122" s="42" t="n">
-        <v>-30.4</v>
+        <v>-31.3</v>
       </c>
       <c r="S122" s="51" t="n"/>
       <c r="T122" s="51" t="n"/>
@@ -77773,7 +77773,7 @@
         </is>
       </c>
       <c r="R123" s="42" t="n">
-        <v>-11.7</v>
+        <v>-11.5</v>
       </c>
       <c r="S123" s="52" t="inlineStr">
         <is>
@@ -77861,7 +77861,7 @@
         </is>
       </c>
       <c r="R124" s="42" t="n">
-        <v>-3.6</v>
+        <v>-2.9</v>
       </c>
       <c r="S124" s="52" t="inlineStr">
         <is>
@@ -77949,7 +77949,7 @@
         </is>
       </c>
       <c r="R125" s="42" t="n">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="S125" s="52" t="inlineStr">
         <is>
@@ -78037,7 +78037,7 @@
         </is>
       </c>
       <c r="R126" s="42" t="n">
-        <v>-23.5</v>
+        <v>-23.6</v>
       </c>
       <c r="S126" s="53" t="inlineStr">
         <is>
@@ -78125,7 +78125,7 @@
         </is>
       </c>
       <c r="R127" s="42" t="n">
-        <v>-4.3</v>
+        <v>-4.4</v>
       </c>
       <c r="S127" s="53" t="inlineStr">
         <is>
@@ -78213,7 +78213,7 @@
         </is>
       </c>
       <c r="R128" s="42" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="S128" s="52" t="inlineStr">
         <is>
@@ -78301,7 +78301,7 @@
         </is>
       </c>
       <c r="R129" s="42" t="n">
-        <v>14.8</v>
+        <v>15.2</v>
       </c>
       <c r="S129" s="53" t="inlineStr">
         <is>
@@ -78508,7 +78508,7 @@
         </is>
       </c>
       <c r="R133" s="42" t="n">
-        <v>-6</v>
+        <v>-5.4</v>
       </c>
       <c r="S133" s="53" t="inlineStr">
         <is>
@@ -78596,7 +78596,7 @@
         </is>
       </c>
       <c r="R134" s="42" t="n">
-        <v>3.2</v>
+        <v>5.5</v>
       </c>
       <c r="S134" s="53" t="inlineStr">
         <is>
@@ -78684,7 +78684,7 @@
         </is>
       </c>
       <c r="R135" s="42" t="n">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="S135" s="52" t="inlineStr">
         <is>
@@ -78696,9 +78696,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U135" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U135" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V135" s="52" t="inlineStr">
@@ -78772,7 +78772,7 @@
         </is>
       </c>
       <c r="R136" s="42" t="n">
-        <v>-1</v>
+        <v>-2.5</v>
       </c>
       <c r="S136" s="53" t="inlineStr">
         <is>
@@ -78860,7 +78860,7 @@
         </is>
       </c>
       <c r="R137" s="42" t="n">
-        <v>-13.2</v>
+        <v>-12.2</v>
       </c>
       <c r="S137" s="52" t="inlineStr">
         <is>
@@ -78948,7 +78948,7 @@
         </is>
       </c>
       <c r="R138" s="42" t="n">
-        <v>-4.6</v>
+        <v>-1.1</v>
       </c>
       <c r="S138" s="52" t="inlineStr">
         <is>
@@ -79036,7 +79036,7 @@
         </is>
       </c>
       <c r="R139" s="42" t="n">
-        <v>-6.6</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="S139" s="52" t="inlineStr">
         <is>
@@ -79124,7 +79124,7 @@
         </is>
       </c>
       <c r="R140" s="42" t="n">
-        <v>-4.9</v>
+        <v>-2.1</v>
       </c>
       <c r="S140" s="54" t="inlineStr">
         <is>
@@ -79212,7 +79212,7 @@
         </is>
       </c>
       <c r="R141" s="42" t="n">
-        <v>-12.1</v>
+        <v>-9.9</v>
       </c>
       <c r="S141" s="53" t="inlineStr">
         <is>
@@ -79300,7 +79300,7 @@
         </is>
       </c>
       <c r="R142" s="42" t="n">
-        <v>-11.5</v>
+        <v>-12.5</v>
       </c>
       <c r="S142" s="53" t="inlineStr">
         <is>
@@ -79388,7 +79388,7 @@
         </is>
       </c>
       <c r="R143" s="42" t="n">
-        <v>-5.7</v>
+        <v>-6.1</v>
       </c>
       <c r="S143" s="53" t="inlineStr">
         <is>
@@ -79476,7 +79476,7 @@
         </is>
       </c>
       <c r="R144" s="42" t="n">
-        <v>-26.2</v>
+        <v>-26.4</v>
       </c>
       <c r="S144" s="53" t="inlineStr">
         <is>
@@ -79564,7 +79564,7 @@
         </is>
       </c>
       <c r="R145" s="42" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="S145" s="52" t="inlineStr">
         <is>
@@ -79576,9 +79576,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U145" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U145" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V145" s="53" t="inlineStr">
@@ -79652,7 +79652,7 @@
         </is>
       </c>
       <c r="R146" s="42" t="n">
-        <v>-14.7</v>
+        <v>-15.6</v>
       </c>
       <c r="S146" s="53" t="inlineStr">
         <is>
@@ -79740,7 +79740,7 @@
         </is>
       </c>
       <c r="R147" s="42" t="n">
-        <v>-1.7</v>
+        <v>-2.9</v>
       </c>
       <c r="S147" s="52" t="inlineStr">
         <is>
@@ -79828,7 +79828,7 @@
         </is>
       </c>
       <c r="R148" s="42" t="n">
-        <v>1.9</v>
+        <v>3.1</v>
       </c>
       <c r="S148" s="52" t="inlineStr">
         <is>
@@ -79916,7 +79916,7 @@
         </is>
       </c>
       <c r="R149" s="42" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="S149" s="53" t="inlineStr">
         <is>
@@ -80004,7 +80004,7 @@
         </is>
       </c>
       <c r="R150" s="42" t="n">
-        <v>-14.6</v>
+        <v>-16.2</v>
       </c>
       <c r="S150" s="53" t="inlineStr">
         <is>
@@ -80092,7 +80092,7 @@
         </is>
       </c>
       <c r="R151" s="42" t="n">
-        <v>-19.6</v>
+        <v>-18.6</v>
       </c>
       <c r="S151" s="53" t="inlineStr">
         <is>
@@ -80180,7 +80180,7 @@
         </is>
       </c>
       <c r="R152" s="42" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="S152" s="52" t="inlineStr">
         <is>
@@ -80268,7 +80268,7 @@
         </is>
       </c>
       <c r="R153" s="42" t="n">
-        <v>13.9</v>
+        <v>11.7</v>
       </c>
       <c r="S153" s="52" t="inlineStr">
         <is>
@@ -80356,7 +80356,7 @@
         </is>
       </c>
       <c r="R154" s="42" t="n">
-        <v>-26.5</v>
+        <v>-25.7</v>
       </c>
       <c r="S154" s="52" t="inlineStr">
         <is>
@@ -80444,7 +80444,7 @@
         </is>
       </c>
       <c r="R155" s="42" t="n">
-        <v>-29.7</v>
+        <v>-30.3</v>
       </c>
       <c r="S155" s="52" t="inlineStr">
         <is>
@@ -80532,7 +80532,7 @@
         </is>
       </c>
       <c r="R156" s="42" t="n">
-        <v>-24.2</v>
+        <v>-23.8</v>
       </c>
       <c r="S156" s="52" t="inlineStr">
         <is>
@@ -80620,7 +80620,7 @@
         </is>
       </c>
       <c r="R157" s="42" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="S157" s="52" t="inlineStr">
         <is>
@@ -80708,7 +80708,7 @@
         </is>
       </c>
       <c r="R158" s="42" t="n">
-        <v>-0.6</v>
+        <v>-0.1</v>
       </c>
       <c r="S158" s="53" t="inlineStr">
         <is>
@@ -80796,7 +80796,7 @@
         </is>
       </c>
       <c r="R159" s="42" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="S159" s="52" t="inlineStr">
         <is>
@@ -80884,7 +80884,7 @@
         </is>
       </c>
       <c r="R160" s="42" t="n">
-        <v>-9.9</v>
+        <v>-10</v>
       </c>
       <c r="S160" s="53" t="inlineStr">
         <is>
@@ -80972,7 +80972,7 @@
         </is>
       </c>
       <c r="R161" s="42" t="n">
-        <v>10.6</v>
+        <v>10.9</v>
       </c>
       <c r="S161" s="52" t="inlineStr">
         <is>
@@ -81060,7 +81060,7 @@
         </is>
       </c>
       <c r="R162" s="42" t="n">
-        <v>-11.7</v>
+        <v>-13.8</v>
       </c>
       <c r="S162" s="53" t="inlineStr">
         <is>
@@ -81072,9 +81072,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U162" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U162" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V162" s="52" t="inlineStr">
@@ -81148,7 +81148,7 @@
         </is>
       </c>
       <c r="R163" s="42" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.5</v>
       </c>
       <c r="S163" s="53" t="inlineStr">
         <is>
@@ -81236,7 +81236,7 @@
         </is>
       </c>
       <c r="R164" s="42" t="n">
-        <v>-38.3</v>
+        <v>-39.8</v>
       </c>
       <c r="S164" s="52" t="inlineStr">
         <is>
@@ -81324,7 +81324,7 @@
         </is>
       </c>
       <c r="R165" s="42" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="S165" s="53" t="inlineStr">
         <is>
@@ -81412,7 +81412,7 @@
         </is>
       </c>
       <c r="R166" s="42" t="n">
-        <v>-9</v>
+        <v>-10.1</v>
       </c>
       <c r="S166" s="53" t="inlineStr">
         <is>
@@ -81500,7 +81500,7 @@
         </is>
       </c>
       <c r="R167" s="42" t="n">
-        <v>8.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="S167" s="52" t="inlineStr">
         <is>
@@ -81588,7 +81588,7 @@
         </is>
       </c>
       <c r="R168" s="42" t="n">
-        <v>-7.7</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="S168" s="53" t="inlineStr">
         <is>
@@ -81676,7 +81676,7 @@
         </is>
       </c>
       <c r="R169" s="42" t="n">
-        <v>-13.6</v>
+        <v>-14.7</v>
       </c>
       <c r="S169" s="53" t="inlineStr">
         <is>
@@ -81764,7 +81764,7 @@
         </is>
       </c>
       <c r="R170" s="42" t="n">
-        <v>-16.2</v>
+        <v>-17.4</v>
       </c>
       <c r="S170" s="53" t="inlineStr">
         <is>
@@ -81852,7 +81852,7 @@
         </is>
       </c>
       <c r="R171" s="42" t="n">
-        <v>3.6</v>
+        <v>2.3</v>
       </c>
       <c r="S171" s="53" t="inlineStr">
         <is>
@@ -81940,7 +81940,7 @@
         </is>
       </c>
       <c r="R172" s="42" t="n">
-        <v>0.2</v>
+        <v>-2.2</v>
       </c>
       <c r="S172" s="52" t="inlineStr">
         <is>
@@ -82028,7 +82028,7 @@
         </is>
       </c>
       <c r="R173" s="42" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="S173" s="52" t="inlineStr">
         <is>
@@ -82116,7 +82116,7 @@
         </is>
       </c>
       <c r="R174" s="42" t="n">
-        <v>5.7</v>
+        <v>6.5</v>
       </c>
       <c r="S174" s="53" t="inlineStr">
         <is>
@@ -82204,7 +82204,7 @@
         </is>
       </c>
       <c r="R175" s="42" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
       <c r="S175" s="52" t="inlineStr">
         <is>
@@ -82292,7 +82292,7 @@
         </is>
       </c>
       <c r="R176" s="42" t="n">
-        <v>-1.8</v>
+        <v>-1.5</v>
       </c>
       <c r="S176" s="53" t="inlineStr">
         <is>
@@ -82380,7 +82380,7 @@
         </is>
       </c>
       <c r="R177" s="42" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
       <c r="S177" s="53" t="inlineStr">
         <is>
@@ -82468,7 +82468,7 @@
         </is>
       </c>
       <c r="R178" s="42" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="S178" s="53" t="inlineStr">
         <is>
@@ -82556,7 +82556,7 @@
         </is>
       </c>
       <c r="R179" s="42" t="n">
-        <v>14.3</v>
+        <v>13.3</v>
       </c>
       <c r="S179" s="52" t="inlineStr">
         <is>
@@ -82644,7 +82644,7 @@
         </is>
       </c>
       <c r="R180" s="42" t="n">
-        <v>-8.5</v>
+        <v>-10.3</v>
       </c>
       <c r="S180" s="53" t="inlineStr">
         <is>
@@ -82656,9 +82656,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U180" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U180" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V180" s="53" t="inlineStr">
@@ -82732,7 +82732,7 @@
         </is>
       </c>
       <c r="R181" s="42" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="S181" s="52" t="inlineStr">
         <is>
@@ -82820,7 +82820,7 @@
         </is>
       </c>
       <c r="R182" s="42" t="n">
-        <v>0.7</v>
+        <v>-0.7</v>
       </c>
       <c r="S182" s="52" t="inlineStr">
         <is>
@@ -82908,7 +82908,7 @@
         </is>
       </c>
       <c r="R183" s="42" t="n">
-        <v>10.9</v>
+        <v>12.8</v>
       </c>
       <c r="S183" s="52" t="inlineStr">
         <is>
@@ -82996,7 +82996,7 @@
         </is>
       </c>
       <c r="R184" s="42" t="n">
-        <v>7.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="S184" s="52" t="inlineStr">
         <is>
@@ -83008,9 +83008,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U184" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U184" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V184" s="52" t="inlineStr">
@@ -83084,7 +83084,7 @@
         </is>
       </c>
       <c r="R185" s="42" t="n">
-        <v>-7.6</v>
+        <v>-9.1</v>
       </c>
       <c r="S185" s="52" t="inlineStr">
         <is>
@@ -83096,9 +83096,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U185" s="52" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="U185" s="53" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="V185" s="52" t="inlineStr">
@@ -83260,7 +83260,7 @@
         </is>
       </c>
       <c r="R187" s="42" t="n">
-        <v>-5.6</v>
+        <v>-7.2</v>
       </c>
       <c r="S187" s="53" t="inlineStr">
         <is>
@@ -83348,7 +83348,7 @@
         </is>
       </c>
       <c r="R188" s="42" t="n">
-        <v>16.5</v>
+        <v>17.2</v>
       </c>
       <c r="S188" s="52" t="inlineStr">
         <is>
@@ -83436,7 +83436,7 @@
         </is>
       </c>
       <c r="R189" s="42" t="n">
-        <v>4.9</v>
+        <v>5.8</v>
       </c>
       <c r="S189" s="52" t="inlineStr">
         <is>
@@ -83524,7 +83524,7 @@
         </is>
       </c>
       <c r="R190" s="42" t="n">
-        <v>-13.3</v>
+        <v>-14.3</v>
       </c>
       <c r="S190" s="53" t="inlineStr">
         <is>
@@ -83731,7 +83731,7 @@
         </is>
       </c>
       <c r="R194" s="42" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="S194" s="53" t="inlineStr">
         <is>
@@ -83743,9 +83743,9 @@
           <t>Loss</t>
         </is>
       </c>
-      <c r="U194" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U194" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V194" s="53" t="inlineStr">
@@ -83819,7 +83819,7 @@
         </is>
       </c>
       <c r="R195" s="42" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="S195" s="53" t="inlineStr">
         <is>
@@ -83907,7 +83907,7 @@
         </is>
       </c>
       <c r="R196" s="42" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="S196" s="52" t="inlineStr">
         <is>
@@ -83995,7 +83995,7 @@
         </is>
       </c>
       <c r="R197" s="42" t="n">
-        <v>-1.8</v>
+        <v>-1.7</v>
       </c>
       <c r="S197" s="52" t="inlineStr">
         <is>
@@ -84083,7 +84083,7 @@
         </is>
       </c>
       <c r="R198" s="42" t="n">
-        <v>18.8</v>
+        <v>19.7</v>
       </c>
       <c r="S198" s="52" t="inlineStr">
         <is>
@@ -84171,7 +84171,7 @@
         </is>
       </c>
       <c r="R199" s="42" t="n">
-        <v>-20.5</v>
+        <v>-20.1</v>
       </c>
       <c r="S199" s="52" t="inlineStr">
         <is>
@@ -84259,7 +84259,7 @@
         </is>
       </c>
       <c r="R200" s="42" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.8</v>
       </c>
       <c r="S200" s="53" t="inlineStr">
         <is>
@@ -84347,7 +84347,7 @@
         </is>
       </c>
       <c r="R201" s="42" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="S201" s="52" t="inlineStr">
         <is>
@@ -84435,7 +84435,7 @@
         </is>
       </c>
       <c r="R202" s="42" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="S202" s="53" t="inlineStr">
         <is>
@@ -84523,7 +84523,7 @@
         </is>
       </c>
       <c r="R203" s="42" t="n">
-        <v>-32.6</v>
+        <v>-32.4</v>
       </c>
       <c r="S203" s="52" t="inlineStr">
         <is>
@@ -84611,7 +84611,7 @@
         </is>
       </c>
       <c r="R204" s="42" t="n">
-        <v>15.4</v>
+        <v>15.9</v>
       </c>
       <c r="S204" s="52" t="inlineStr">
         <is>
@@ -84699,7 +84699,7 @@
         </is>
       </c>
       <c r="R205" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.7</v>
       </c>
       <c r="S205" s="52" t="inlineStr">
         <is>
@@ -84787,7 +84787,7 @@
         </is>
       </c>
       <c r="R206" s="42" t="n">
-        <v>-23.9</v>
+        <v>-24.2</v>
       </c>
       <c r="S206" s="52" t="inlineStr">
         <is>
@@ -84875,7 +84875,7 @@
         </is>
       </c>
       <c r="R207" s="42" t="n">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
       <c r="S207" s="53" t="inlineStr">
         <is>
@@ -84963,7 +84963,7 @@
         </is>
       </c>
       <c r="R208" s="42" t="n">
-        <v>-12.9</v>
+        <v>-12.1</v>
       </c>
       <c r="S208" s="52" t="inlineStr">
         <is>
@@ -85051,7 +85051,7 @@
         </is>
       </c>
       <c r="R209" s="42" t="n">
-        <v>-5.9</v>
+        <v>-6.3</v>
       </c>
       <c r="S209" s="54" t="inlineStr">
         <is>
@@ -85139,7 +85139,7 @@
         </is>
       </c>
       <c r="R210" s="42" t="n">
-        <v>-13.3</v>
+        <v>-12.7</v>
       </c>
       <c r="S210" s="53" t="inlineStr">
         <is>
@@ -85227,7 +85227,7 @@
         </is>
       </c>
       <c r="R211" s="42" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="S211" s="52" t="inlineStr">
         <is>
@@ -85315,7 +85315,7 @@
         </is>
       </c>
       <c r="R212" s="42" t="n">
-        <v>-13.1</v>
+        <v>-13</v>
       </c>
       <c r="S212" s="52" t="inlineStr">
         <is>
@@ -85403,7 +85403,7 @@
         </is>
       </c>
       <c r="R213" s="42" t="n">
-        <v>-7.9</v>
+        <v>-7.7</v>
       </c>
       <c r="S213" s="53" t="inlineStr">
         <is>
@@ -85491,7 +85491,7 @@
         </is>
       </c>
       <c r="R214" s="42" t="n">
-        <v>-12.5</v>
+        <v>-12.4</v>
       </c>
       <c r="S214" s="52" t="inlineStr">
         <is>
@@ -85579,7 +85579,7 @@
         </is>
       </c>
       <c r="R215" s="42" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="S215" s="52" t="inlineStr">
         <is>
@@ -85667,7 +85667,7 @@
         </is>
       </c>
       <c r="R216" s="42" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="S216" s="53" t="inlineStr">
         <is>
@@ -85755,7 +85755,7 @@
         </is>
       </c>
       <c r="R217" s="42" t="n">
-        <v>-11.3</v>
+        <v>-11.1</v>
       </c>
       <c r="S217" s="53" t="inlineStr">
         <is>
@@ -85931,7 +85931,7 @@
         </is>
       </c>
       <c r="R219" s="42" t="n">
-        <v>-5.3</v>
+        <v>-4.6</v>
       </c>
       <c r="S219" s="53" t="inlineStr">
         <is>
@@ -86019,7 +86019,7 @@
         </is>
       </c>
       <c r="R220" s="42" t="n">
-        <v>-6.1</v>
+        <v>-6.3</v>
       </c>
       <c r="S220" s="52" t="inlineStr">
         <is>
@@ -86107,7 +86107,7 @@
         </is>
       </c>
       <c r="R221" s="42" t="n">
-        <v>15.6</v>
+        <v>16.5</v>
       </c>
       <c r="S221" s="53" t="inlineStr">
         <is>
@@ -86195,7 +86195,7 @@
         </is>
       </c>
       <c r="R222" s="42" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="S222" s="52" t="inlineStr">
         <is>
@@ -86283,7 +86283,7 @@
         </is>
       </c>
       <c r="R223" s="42" t="n">
-        <v>12.2</v>
+        <v>11.7</v>
       </c>
       <c r="S223" s="52" t="inlineStr">
         <is>
@@ -86371,7 +86371,7 @@
         </is>
       </c>
       <c r="R224" s="42" t="n">
-        <v>-6.8</v>
+        <v>-7.2</v>
       </c>
       <c r="S224" s="53" t="inlineStr">
         <is>
@@ -86459,7 +86459,7 @@
         </is>
       </c>
       <c r="R225" s="42" t="n">
-        <v>14.7</v>
+        <v>14.2</v>
       </c>
       <c r="S225" s="52" t="inlineStr">
         <is>
@@ -86547,7 +86547,7 @@
         </is>
       </c>
       <c r="R226" s="42" t="n">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
       <c r="S226" s="52" t="inlineStr">
         <is>
@@ -86635,7 +86635,7 @@
         </is>
       </c>
       <c r="R227" s="42" t="n">
-        <v>-7.5</v>
+        <v>-7.2</v>
       </c>
       <c r="S227" s="53" t="inlineStr">
         <is>
@@ -86723,7 +86723,7 @@
         </is>
       </c>
       <c r="R228" s="42" t="n">
-        <v>14.9</v>
+        <v>14.3</v>
       </c>
       <c r="S228" s="52" t="inlineStr">
         <is>
@@ -86811,7 +86811,7 @@
         </is>
       </c>
       <c r="R229" s="42" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="S229" s="53" t="inlineStr">
         <is>
@@ -86899,7 +86899,7 @@
         </is>
       </c>
       <c r="R230" s="42" t="n">
-        <v>-11.8</v>
+        <v>-11.9</v>
       </c>
       <c r="S230" s="52" t="inlineStr">
         <is>
@@ -87075,7 +87075,7 @@
         </is>
       </c>
       <c r="R232" s="42" t="n">
-        <v>-22.2</v>
+        <v>-22</v>
       </c>
       <c r="S232" s="53" t="inlineStr">
         <is>
@@ -87163,7 +87163,7 @@
         </is>
       </c>
       <c r="R233" s="42" t="n">
-        <v>-21.5</v>
+        <v>-20.8</v>
       </c>
       <c r="S233" s="53" t="inlineStr">
         <is>
@@ -87251,7 +87251,7 @@
         </is>
       </c>
       <c r="R234" s="42" t="n">
-        <v>-7.2</v>
+        <v>-6.6</v>
       </c>
       <c r="S234" s="53" t="inlineStr">
         <is>
@@ -87339,7 +87339,7 @@
         </is>
       </c>
       <c r="R235" s="42" t="n">
-        <v>-7.2</v>
+        <v>-6.2</v>
       </c>
       <c r="S235" s="52" t="inlineStr">
         <is>
@@ -87427,7 +87427,7 @@
         </is>
       </c>
       <c r="R236" s="42" t="n">
-        <v>-15.6</v>
+        <v>-15.1</v>
       </c>
       <c r="S236" s="53" t="inlineStr">
         <is>
@@ -87515,7 +87515,7 @@
         </is>
       </c>
       <c r="R237" s="42" t="n">
-        <v>-2.4</v>
+        <v>-2.3</v>
       </c>
       <c r="S237" s="52" t="inlineStr">
         <is>
@@ -87603,7 +87603,7 @@
         </is>
       </c>
       <c r="R238" s="42" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="S238" s="53" t="inlineStr">
         <is>
@@ -87691,7 +87691,7 @@
         </is>
       </c>
       <c r="R239" s="42" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="S239" s="52" t="inlineStr">
         <is>
@@ -87779,7 +87779,7 @@
         </is>
       </c>
       <c r="R240" s="42" t="n">
-        <v>-16.4</v>
+        <v>-16.3</v>
       </c>
       <c r="S240" s="53" t="inlineStr">
         <is>
@@ -87867,7 +87867,7 @@
         </is>
       </c>
       <c r="R241" s="42" t="n">
-        <v>-40.6</v>
+        <v>-40.5</v>
       </c>
       <c r="S241" s="52" t="inlineStr">
         <is>
@@ -87955,7 +87955,7 @@
         </is>
       </c>
       <c r="R242" s="42" t="n">
-        <v>15.9</v>
+        <v>15.2</v>
       </c>
       <c r="S242" s="53" t="inlineStr">
         <is>
@@ -88043,7 +88043,7 @@
         </is>
       </c>
       <c r="R243" s="42" t="n">
-        <v>-2.5</v>
+        <v>-3.2</v>
       </c>
       <c r="S243" s="52" t="inlineStr">
         <is>
@@ -88131,7 +88131,7 @@
         </is>
       </c>
       <c r="R244" s="42" t="n">
-        <v>-5.8</v>
+        <v>-5.3</v>
       </c>
       <c r="S244" s="52" t="inlineStr">
         <is>
@@ -88219,7 +88219,7 @@
         </is>
       </c>
       <c r="R245" s="42" t="n">
-        <v>-13.3</v>
+        <v>-12.9</v>
       </c>
       <c r="S245" s="53" t="inlineStr">
         <is>
@@ -88307,7 +88307,7 @@
         </is>
       </c>
       <c r="R246" s="42" t="n">
-        <v>-13.1</v>
+        <v>-12.8</v>
       </c>
       <c r="S246" s="53" t="inlineStr">
         <is>
@@ -88319,9 +88319,9 @@
           <t>Win</t>
         </is>
       </c>
-      <c r="U246" s="53" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="U246" s="52" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="V246" s="52" t="inlineStr">
@@ -88395,7 +88395,7 @@
         </is>
       </c>
       <c r="R247" s="42" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="S247" s="53" t="inlineStr">
         <is>
@@ -88483,7 +88483,7 @@
         </is>
       </c>
       <c r="R248" s="42" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="S248" s="52" t="inlineStr">
         <is>
@@ -88571,7 +88571,7 @@
         </is>
       </c>
       <c r="R249" s="42" t="n">
-        <v>-14.3</v>
+        <v>-14.6</v>
       </c>
       <c r="S249" s="53" t="inlineStr">
         <is>
@@ -88659,7 +88659,7 @@
         </is>
       </c>
       <c r="R250" s="42" t="n">
-        <v>-4.3</v>
+        <v>-5.1</v>
       </c>
       <c r="S250" s="52" t="inlineStr">
         <is>
@@ -88747,7 +88747,7 @@
         </is>
       </c>
       <c r="R251" s="42" t="n">
-        <v>-18.4</v>
+        <v>-18.9</v>
       </c>
       <c r="S251" s="53" t="inlineStr">
         <is>
@@ -88835,7 +88835,7 @@
         </is>
       </c>
       <c r="R252" s="42" t="n">
-        <v>-5.3</v>
+        <v>-5.7</v>
       </c>
       <c r="S252" s="52" t="inlineStr">
         <is>

</xml_diff>